<commit_message>
Update standings 2026-09-13 00:16 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -619,16 +619,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -643,16 +643,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -1099,16 +1099,16 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>sakalaka</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -1123,16 +1123,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>sakalaka</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
@@ -1682,14 +1682,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C8" t="n">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="D8" t="n">
         <v>54</v>
@@ -1698,14 +1698,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C9" t="n">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="D9" t="n">
         <v>54</v>
@@ -2002,33 +2002,33 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="C28" t="n">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D28" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="C29" t="n">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="D29" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30">
@@ -2908,7 +2908,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2919,7 +2919,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -3642,30 +3642,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E8" t="n">
-        <v>545267</v>
+        <v>31543</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>604934</v>
+        <v>820692</v>
       </c>
       <c r="H8" t="n">
-        <v>545267</v>
+        <v>1637750</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -3679,30 +3679,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>31543</v>
+        <v>545267</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>820692</v>
+        <v>604934</v>
       </c>
       <c r="H9" t="n">
-        <v>1637750</v>
+        <v>545267</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -4382,30 +4382,30 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>sakalaka</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E28" t="n">
-        <v>117338</v>
+        <v>1615102</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>4684930</v>
+        <v>4234674</v>
       </c>
       <c r="H28" t="n">
-        <v>117338</v>
+        <v>6092784</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -4419,30 +4419,30 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>sakalaka</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E29" t="n">
-        <v>1615102</v>
+        <v>117338</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>4234674</v>
+        <v>4684930</v>
       </c>
       <c r="H29" t="n">
-        <v>6092784</v>
+        <v>117338</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -4708,7 +4708,7 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O2" t="n">
         <v>101.2</v>
@@ -4720,7 +4720,7 @@
         <v>0.4</v>
       </c>
       <c r="R2" t="n">
-        <v>2897</v>
+        <v>4395</v>
       </c>
       <c r="S2" t="n">
         <v>270274</v>
@@ -4779,7 +4779,7 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="O3" t="n">
         <v>100.4</v>
@@ -4791,7 +4791,7 @@
         <v>0.4</v>
       </c>
       <c r="R3" t="n">
-        <v>314091</v>
+        <v>90138</v>
       </c>
       <c r="S3" t="n">
         <v>166751</v>
@@ -4850,7 +4850,7 @@
         <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="O4" t="n">
         <v>100.3</v>
@@ -4862,7 +4862,7 @@
         <v>0.6</v>
       </c>
       <c r="R4" t="n">
-        <v>110721</v>
+        <v>159696</v>
       </c>
       <c r="S4" t="n">
         <v>637992</v>
@@ -4921,7 +4921,7 @@
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="O5" t="n">
         <v>101.1</v>
@@ -4933,7 +4933,7 @@
         <v>1.1</v>
       </c>
       <c r="R5" t="n">
-        <v>743639</v>
+        <v>433216</v>
       </c>
       <c r="S5" t="n">
         <v>101935</v>
@@ -4992,7 +4992,7 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="O6" t="n">
         <v>100.6</v>
@@ -5004,7 +5004,7 @@
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>408916</v>
+        <v>433216</v>
       </c>
       <c r="S6" t="n">
         <v>3039834</v>
@@ -5063,7 +5063,7 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="O7" t="n">
         <v>100.7</v>
@@ -5075,7 +5075,7 @@
         <v>0.7</v>
       </c>
       <c r="R7" t="n">
-        <v>314091</v>
+        <v>444016</v>
       </c>
       <c r="S7" t="n">
         <v>617418</v>
@@ -5092,28 +5092,28 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>275</v>
       </c>
       <c r="D8" t="n">
-        <v>69.7</v>
+        <v>75.7</v>
       </c>
       <c r="E8" t="n">
         <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>48</v>
+        <v>95</v>
       </c>
       <c r="G8" t="n">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="H8" t="n">
         <v>2</v>
@@ -5134,53 +5134,57 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="O8" t="n">
-        <v>100.2</v>
+        <v>100.5</v>
       </c>
       <c r="P8" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>1384256</v>
+        <v>464779</v>
       </c>
       <c r="S8" t="n">
-        <v>1461471</v>
+        <v>1066412</v>
       </c>
       <c r="T8" t="n">
         <v>2</v>
       </c>
-      <c r="U8" t="inlineStr"/>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>3xc, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>275</v>
       </c>
       <c r="D9" t="n">
-        <v>75.7</v>
+        <v>69.7</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>95</v>
+        <v>48</v>
       </c>
       <c r="G9" t="n">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="H9" t="n">
         <v>2</v>
@@ -5201,31 +5205,27 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="O9" t="n">
-        <v>100.5</v>
+        <v>100.2</v>
       </c>
       <c r="P9" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="R9" t="n">
-        <v>375042</v>
+        <v>464779</v>
       </c>
       <c r="S9" t="n">
-        <v>1066412</v>
+        <v>1461471</v>
       </c>
       <c r="T9" t="n">
         <v>2</v>
       </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>3xc, wildcard</t>
-        </is>
-      </c>
+      <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5272,7 +5272,7 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="O10" t="n">
         <v>101</v>
@@ -5284,7 +5284,7 @@
         <v>0.2</v>
       </c>
       <c r="R10" t="n">
-        <v>717233</v>
+        <v>537731</v>
       </c>
       <c r="S10" t="n">
         <v>878473</v>
@@ -5343,7 +5343,7 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="O11" t="n">
         <v>101</v>
@@ -5355,7 +5355,7 @@
         <v>0.2</v>
       </c>
       <c r="R11" t="n">
-        <v>1472197</v>
+        <v>613815</v>
       </c>
       <c r="S11" t="n">
         <v>1034411</v>
@@ -5414,7 +5414,7 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="O12" t="n">
         <v>101.1</v>
@@ -5426,7 +5426,7 @@
         <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>544926</v>
+        <v>783160</v>
       </c>
       <c r="S12" t="n">
         <v>24105</v>
@@ -5485,7 +5485,7 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="O13" t="n">
         <v>101.4</v>
@@ -5497,7 +5497,7 @@
         <v>0.2</v>
       </c>
       <c r="R13" t="n">
-        <v>994664</v>
+        <v>877134</v>
       </c>
       <c r="S13" t="n">
         <v>88386</v>
@@ -5556,7 +5556,7 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="O14" t="n">
         <v>100.2</v>
@@ -5568,7 +5568,7 @@
         <v>0.6</v>
       </c>
       <c r="R14" t="n">
-        <v>801253</v>
+        <v>960518</v>
       </c>
       <c r="S14" t="n">
         <v>4399137</v>
@@ -5623,7 +5623,7 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="O15" t="n">
         <v>100.5</v>
@@ -5635,7 +5635,7 @@
         <v>0.5</v>
       </c>
       <c r="R15" t="n">
-        <v>1516623</v>
+        <v>1178342</v>
       </c>
       <c r="S15" t="n">
         <v>5250200</v>
@@ -5694,7 +5694,7 @@
         <v>-4</v>
       </c>
       <c r="N16" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="O16" t="n">
         <v>101</v>
@@ -5706,7 +5706,7 @@
         <v>1.4</v>
       </c>
       <c r="R16" t="n">
-        <v>1496797</v>
+        <v>1197866</v>
       </c>
       <c r="S16" t="n">
         <v>670758</v>
@@ -5765,7 +5765,7 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="O17" t="n">
         <v>100.4</v>
@@ -5777,7 +5777,7 @@
         <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>1322832</v>
+        <v>1370522</v>
       </c>
       <c r="S17" t="n">
         <v>3046343</v>
@@ -5836,7 +5836,7 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="O18" t="n">
         <v>100.5</v>
@@ -5848,7 +5848,7 @@
         <v>0.6</v>
       </c>
       <c r="R18" t="n">
-        <v>1065607</v>
+        <v>1506462</v>
       </c>
       <c r="S18" t="n">
         <v>5881370</v>
@@ -5907,7 +5907,7 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O19" t="n">
         <v>100.4</v>
@@ -5919,7 +5919,7 @@
         <v>0.5</v>
       </c>
       <c r="R19" t="n">
-        <v>961038</v>
+        <v>1760710</v>
       </c>
       <c r="S19" t="n">
         <v>3009015</v>
@@ -5978,7 +5978,7 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="O20" t="n">
         <v>100.6</v>
@@ -5990,7 +5990,7 @@
         <v>1</v>
       </c>
       <c r="R20" t="n">
-        <v>1609623</v>
+        <v>1760710</v>
       </c>
       <c r="S20" t="n">
         <v>4185865</v>
@@ -6061,7 +6061,7 @@
         <v>1</v>
       </c>
       <c r="R21" t="n">
-        <v>2700348</v>
+        <v>2129676</v>
       </c>
       <c r="S21" t="n">
         <v>3395267</v>
@@ -6120,7 +6120,7 @@
         <v>-4</v>
       </c>
       <c r="N22" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="O22" t="n">
         <v>100.4</v>
@@ -6132,7 +6132,7 @@
         <v>0.2</v>
       </c>
       <c r="R22" t="n">
-        <v>2393668</v>
+        <v>2408926</v>
       </c>
       <c r="S22" t="n">
         <v>3048395</v>
@@ -6191,7 +6191,7 @@
         <v>-4</v>
       </c>
       <c r="N23" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="O23" t="n">
         <v>100.7</v>
@@ -6203,7 +6203,7 @@
         <v>0.1</v>
       </c>
       <c r="R23" t="n">
-        <v>2279669</v>
+        <v>2603542</v>
       </c>
       <c r="S23" t="n">
         <v>1948104</v>
@@ -6262,7 +6262,7 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="O24" t="n">
         <v>100.9</v>
@@ -6274,7 +6274,7 @@
         <v>1</v>
       </c>
       <c r="R24" t="n">
-        <v>3198740</v>
+        <v>3089001</v>
       </c>
       <c r="S24" t="n">
         <v>453361</v>
@@ -6329,7 +6329,7 @@
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="O25" t="n">
         <v>101.3</v>
@@ -6341,7 +6341,7 @@
         <v>0.4</v>
       </c>
       <c r="R25" t="n">
-        <v>4175402</v>
+        <v>4279947</v>
       </c>
       <c r="S25" t="n">
         <v>2735246</v>
@@ -6400,7 +6400,7 @@
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="O26" t="n">
         <v>101.2</v>
@@ -6412,7 +6412,7 @@
         <v>1.5</v>
       </c>
       <c r="R26" t="n">
-        <v>5267498</v>
+        <v>4497875</v>
       </c>
       <c r="S26" t="n">
         <v>1396363</v>
@@ -6471,7 +6471,7 @@
         <v>-4</v>
       </c>
       <c r="N27" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="O27" t="n">
         <v>100.4</v>
@@ -6483,7 +6483,7 @@
         <v>0.7</v>
       </c>
       <c r="R27" t="n">
-        <v>7314821</v>
+        <v>4737183</v>
       </c>
       <c r="U27" t="inlineStr">
         <is>
@@ -6494,34 +6494,34 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>sakalaka</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="C28" t="n">
         <v>222</v>
       </c>
       <c r="D28" t="n">
-        <v>59.3</v>
+        <v>61.7</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="G28" t="n">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="H28" t="n">
         <v>2</v>
       </c>
       <c r="I28" t="n">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="J28" t="n">
         <v>1</v>
@@ -6536,63 +6536,63 @@
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="O28" t="n">
-        <v>100.2</v>
+        <v>100</v>
       </c>
       <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q28" t="n">
-        <v>0</v>
-      </c>
       <c r="R28" t="n">
-        <v>5141430</v>
+        <v>4818275</v>
       </c>
       <c r="S28" t="n">
-        <v>3963132</v>
+        <v>1595922</v>
       </c>
       <c r="T28" t="n">
         <v>2</v>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>bboost, 3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>sakalaka</t>
         </is>
       </c>
       <c r="C29" t="n">
         <v>222</v>
       </c>
       <c r="D29" t="n">
-        <v>61.7</v>
+        <v>59.3</v>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="G29" t="n">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="H29" t="n">
         <v>2</v>
       </c>
       <c r="I29" t="n">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="J29" t="n">
         <v>1</v>
@@ -6607,29 +6607,29 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="O29" t="n">
-        <v>100</v>
+        <v>100.2</v>
       </c>
       <c r="P29" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="R29" t="n">
-        <v>4237077</v>
+        <v>4818275</v>
       </c>
       <c r="S29" t="n">
-        <v>1595922</v>
+        <v>3963132</v>
       </c>
       <c r="T29" t="n">
         <v>2</v>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>bboost, 3xc, wildcard</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
@@ -6678,7 +6678,7 @@
         <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="O30" t="n">
         <v>101.2</v>
@@ -6690,7 +6690,7 @@
         <v>0.7</v>
       </c>
       <c r="R30" t="n">
-        <v>4044609</v>
+        <v>5027559</v>
       </c>
       <c r="U30" t="inlineStr">
         <is>
@@ -6743,7 +6743,7 @@
         <v>-8</v>
       </c>
       <c r="N31" t="n">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="O31" t="n">
         <v>100.9</v>
@@ -6755,7 +6755,7 @@
         <v>1</v>
       </c>
       <c r="R31" t="n">
-        <v>8329113</v>
+        <v>7436422</v>
       </c>
       <c r="S31" t="n">
         <v>140252</v>
@@ -6826,7 +6826,7 @@
         <v>2.2</v>
       </c>
       <c r="R32" t="n">
-        <v>8835494</v>
+        <v>8382065</v>
       </c>
       <c r="S32" t="n">
         <v>216389</v>

</xml_diff>

<commit_message>
Update standings 2026-09-13 02:11 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -619,16 +619,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -643,16 +643,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -1682,14 +1682,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C8" t="n">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="D8" t="n">
         <v>54</v>
@@ -1698,14 +1698,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C9" t="n">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="D9" t="n">
         <v>54</v>
@@ -3642,30 +3642,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E8" t="n">
-        <v>31543</v>
+        <v>545267</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>820692</v>
+        <v>604934</v>
       </c>
       <c r="H8" t="n">
-        <v>1637750</v>
+        <v>545267</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -3679,30 +3679,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E9" t="n">
-        <v>545267</v>
+        <v>31543</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>604934</v>
+        <v>820692</v>
       </c>
       <c r="H9" t="n">
-        <v>545267</v>
+        <v>1637750</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -5092,28 +5092,28 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>275</v>
       </c>
       <c r="D8" t="n">
-        <v>75.7</v>
+        <v>69.7</v>
       </c>
       <c r="E8" t="n">
         <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>95</v>
+        <v>48</v>
       </c>
       <c r="G8" t="n">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="H8" t="n">
         <v>2</v>
@@ -5134,57 +5134,53 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="O8" t="n">
-        <v>100.5</v>
+        <v>100.2</v>
       </c>
       <c r="P8" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="R8" t="n">
         <v>464779</v>
       </c>
       <c r="S8" t="n">
-        <v>1066412</v>
+        <v>1461471</v>
       </c>
       <c r="T8" t="n">
         <v>2</v>
       </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>3xc, wildcard</t>
-        </is>
-      </c>
+      <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>275</v>
       </c>
       <c r="D9" t="n">
-        <v>69.7</v>
+        <v>75.7</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>48</v>
+        <v>95</v>
       </c>
       <c r="G9" t="n">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="H9" t="n">
         <v>2</v>
@@ -5205,27 +5201,31 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="O9" t="n">
-        <v>100.2</v>
+        <v>100.5</v>
       </c>
       <c r="P9" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
         <v>464779</v>
       </c>
       <c r="S9" t="n">
-        <v>1461471</v>
+        <v>1066412</v>
       </c>
       <c r="T9" t="n">
         <v>2</v>
       </c>
-      <c r="U9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>3xc, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-14 06:16 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -835,16 +835,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -1810,33 +1810,33 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="C17" t="n">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="D17" t="n">
-        <v>54</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18">
@@ -3938,30 +3938,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>31543</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>820692</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>1637750</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -3975,30 +3975,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E17" t="n">
-        <v>31543</v>
+        <v>453230</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>820692</v>
+        <v>5483351</v>
       </c>
       <c r="H17" t="n">
-        <v>1637750</v>
+        <v>8188106</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -5656,37 +5656,37 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C16" t="n">
         <v>284</v>
       </c>
       <c r="D16" t="n">
-        <v>71.7</v>
+        <v>75.7</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5698,66 +5698,66 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>100.5</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="R16" t="n">
-        <v>1264459</v>
+        <v>1327109</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>1066412</v>
       </c>
       <c r="T16" t="n">
         <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C17" t="n">
         <v>284</v>
       </c>
       <c r="D17" t="n">
-        <v>75.7</v>
+        <v>71.7</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="G17" t="n">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="H17" t="n">
         <v>2</v>
       </c>
       <c r="I17" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="J17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K17" t="n">
         <v>2</v>
@@ -5769,29 +5769,29 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="O17" t="n">
-        <v>100.5</v>
+        <v>100.4</v>
       </c>
       <c r="P17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="Q17" t="n">
         <v>0.5</v>
       </c>
-      <c r="Q17" t="n">
-        <v>0</v>
-      </c>
       <c r="R17" t="n">
-        <v>1327109</v>
+        <v>1264459</v>
       </c>
       <c r="S17" t="n">
-        <v>1066412</v>
+        <v>3009015</v>
       </c>
       <c r="T17" t="n">
         <v>2</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>3xc, freehit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-14 08:13 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -571,19 +571,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>101</v>
+        <v>76</v>
       </c>
       <c r="E6" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
         <v>305</v>
@@ -595,19 +595,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>76</v>
+        <v>101</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F7" t="n">
         <v>305</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -835,16 +835,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -1650,33 +1650,33 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C6" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D6" t="n">
-        <v>43</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C7" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D7" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8">
@@ -1810,33 +1810,33 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>54</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="C17" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="D17" t="n">
-        <v>67</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18">
@@ -2389,7 +2389,11 @@
       <c r="B16" t="n">
         <v>57</v>
       </c>
-      <c r="C16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2485,11 +2489,7 @@
       <c r="B24" t="n">
         <v>48</v>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="C24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2649,7 +2649,11 @@
       <c r="B4" t="n">
         <v>2</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2767,11 +2771,7 @@
       <c r="B14" t="n">
         <v>1</v>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3568,30 +3568,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E6" t="n">
-        <v>281617</v>
+        <v>6474</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1051323</v>
+        <v>1177681</v>
       </c>
       <c r="H6" t="n">
-        <v>1076546</v>
+        <v>6474</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -3605,30 +3605,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E7" t="n">
-        <v>6474</v>
+        <v>281617</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1177681</v>
+        <v>1051323</v>
       </c>
       <c r="H7" t="n">
-        <v>6474</v>
+        <v>1076546</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -3938,30 +3938,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>31543</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>820692</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>1637750</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -3975,30 +3975,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E17" t="n">
-        <v>453230</v>
+        <v>31543</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>5483351</v>
+        <v>820692</v>
       </c>
       <c r="H17" t="n">
-        <v>8188106</v>
+        <v>1637750</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4946,34 +4946,34 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>305</v>
       </c>
       <c r="D6" t="n">
-        <v>69.3</v>
+        <v>76.3</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G6" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H6" t="n">
         <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="J6" t="n">
         <v>3</v>
@@ -4982,69 +4982,69 @@
         <v>3</v>
       </c>
       <c r="L6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N6" t="n">
         <v>47</v>
       </c>
       <c r="O6" t="n">
-        <v>101</v>
+        <v>100.7</v>
       </c>
       <c r="P6" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="Q6" t="n">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="R6" t="n">
         <v>394418</v>
       </c>
       <c r="S6" t="n">
-        <v>670758</v>
+        <v>617418</v>
       </c>
       <c r="T6" t="n">
         <v>2</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>305</v>
       </c>
       <c r="D7" t="n">
-        <v>76.3</v>
+        <v>69.3</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="G7" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H7" t="n">
         <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="J7" t="n">
         <v>3</v>
@@ -5053,35 +5053,35 @@
         <v>3</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N7" t="n">
         <v>47</v>
       </c>
       <c r="O7" t="n">
-        <v>100.7</v>
+        <v>101</v>
       </c>
       <c r="P7" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.7</v>
+        <v>1.4</v>
       </c>
       <c r="R7" t="n">
         <v>394418</v>
       </c>
       <c r="S7" t="n">
-        <v>617418</v>
+        <v>670758</v>
       </c>
       <c r="T7" t="n">
         <v>2</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
@@ -5656,37 +5656,37 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
         <v>284</v>
       </c>
       <c r="D16" t="n">
-        <v>75.7</v>
+        <v>71.7</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" t="n">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="G16" t="n">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5698,66 +5698,66 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="O16" t="n">
-        <v>100.5</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="Q16" t="n">
         <v>0.5</v>
       </c>
-      <c r="Q16" t="n">
-        <v>0</v>
-      </c>
       <c r="R16" t="n">
-        <v>1327109</v>
+        <v>1264459</v>
       </c>
       <c r="S16" t="n">
-        <v>1066412</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
         <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>3xc, freehit</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C17" t="n">
         <v>284</v>
       </c>
       <c r="D17" t="n">
-        <v>71.7</v>
+        <v>75.7</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="G17" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="H17" t="n">
         <v>2</v>
       </c>
       <c r="I17" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="J17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K17" t="n">
         <v>2</v>
@@ -5769,29 +5769,29 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="O17" t="n">
-        <v>100.4</v>
+        <v>100.5</v>
       </c>
       <c r="P17" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>1264459</v>
+        <v>1327109</v>
       </c>
       <c r="S17" t="n">
-        <v>3009015</v>
+        <v>1066412</v>
       </c>
       <c r="T17" t="n">
         <v>2</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>3xc, freehit</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-14 10:12 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -571,19 +571,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>76</v>
+        <v>101</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F6" t="n">
         <v>305</v>
@@ -595,19 +595,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>101</v>
+        <v>76</v>
       </c>
       <c r="E7" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
         <v>305</v>
@@ -1650,33 +1650,33 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C6" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D6" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C7" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D7" t="n">
-        <v>43</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8">
@@ -2389,11 +2389,7 @@
       <c r="B16" t="n">
         <v>57</v>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2489,7 +2485,11 @@
       <c r="B24" t="n">
         <v>48</v>
       </c>
-      <c r="C24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2649,11 +2649,7 @@
       <c r="B4" t="n">
         <v>2</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2771,7 +2767,11 @@
       <c r="B14" t="n">
         <v>1</v>
       </c>
-      <c r="C14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3568,30 +3568,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E6" t="n">
-        <v>6474</v>
+        <v>281617</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1177681</v>
+        <v>1051323</v>
       </c>
       <c r="H6" t="n">
-        <v>6474</v>
+        <v>1076546</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -3605,30 +3605,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E7" t="n">
-        <v>281617</v>
+        <v>6474</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1051323</v>
+        <v>1177681</v>
       </c>
       <c r="H7" t="n">
-        <v>1076546</v>
+        <v>6474</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -4946,34 +4946,34 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>305</v>
       </c>
       <c r="D6" t="n">
-        <v>76.3</v>
+        <v>69.3</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="G6" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H6" t="n">
         <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="J6" t="n">
         <v>3</v>
@@ -4982,69 +4982,69 @@
         <v>3</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N6" t="n">
         <v>47</v>
       </c>
       <c r="O6" t="n">
-        <v>100.7</v>
+        <v>101</v>
       </c>
       <c r="P6" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.7</v>
+        <v>1.4</v>
       </c>
       <c r="R6" t="n">
         <v>394418</v>
       </c>
       <c r="S6" t="n">
-        <v>617418</v>
+        <v>670758</v>
       </c>
       <c r="T6" t="n">
         <v>2</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>305</v>
       </c>
       <c r="D7" t="n">
-        <v>69.3</v>
+        <v>76.3</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G7" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H7" t="n">
         <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="J7" t="n">
         <v>3</v>
@@ -5053,35 +5053,35 @@
         <v>3</v>
       </c>
       <c r="L7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N7" t="n">
         <v>47</v>
       </c>
       <c r="O7" t="n">
-        <v>101</v>
+        <v>100.7</v>
       </c>
       <c r="P7" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="Q7" t="n">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="R7" t="n">
         <v>394418</v>
       </c>
       <c r="S7" t="n">
-        <v>670758</v>
+        <v>617418</v>
       </c>
       <c r="T7" t="n">
         <v>2</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-14 12:15 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -571,19 +571,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>101</v>
+        <v>76</v>
       </c>
       <c r="E6" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
         <v>305</v>
@@ -595,19 +595,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>76</v>
+        <v>101</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F7" t="n">
         <v>305</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -835,16 +835,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -1650,33 +1650,33 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C6" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D6" t="n">
-        <v>43</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C7" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D7" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8">
@@ -1810,33 +1810,33 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="C17" t="n">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="D17" t="n">
-        <v>54</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18">
@@ -2389,7 +2389,11 @@
       <c r="B16" t="n">
         <v>57</v>
       </c>
-      <c r="C16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2485,11 +2489,7 @@
       <c r="B24" t="n">
         <v>48</v>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="C24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2649,7 +2649,11 @@
       <c r="B4" t="n">
         <v>2</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2767,11 +2771,7 @@
       <c r="B14" t="n">
         <v>1</v>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3568,30 +3568,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E6" t="n">
-        <v>281617</v>
+        <v>6474</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1051323</v>
+        <v>1177681</v>
       </c>
       <c r="H6" t="n">
-        <v>1076546</v>
+        <v>6474</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -3605,30 +3605,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E7" t="n">
-        <v>6474</v>
+        <v>281617</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1177681</v>
+        <v>1051323</v>
       </c>
       <c r="H7" t="n">
-        <v>6474</v>
+        <v>1076546</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -3938,30 +3938,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>31543</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>820692</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>1637750</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -3975,30 +3975,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E17" t="n">
-        <v>31543</v>
+        <v>453230</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>820692</v>
+        <v>5483351</v>
       </c>
       <c r="H17" t="n">
-        <v>1637750</v>
+        <v>8188106</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4946,34 +4946,34 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>305</v>
       </c>
       <c r="D6" t="n">
-        <v>69.3</v>
+        <v>76.3</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G6" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H6" t="n">
         <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="J6" t="n">
         <v>3</v>
@@ -4982,69 +4982,69 @@
         <v>3</v>
       </c>
       <c r="L6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N6" t="n">
         <v>47</v>
       </c>
       <c r="O6" t="n">
-        <v>101</v>
+        <v>100.7</v>
       </c>
       <c r="P6" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="Q6" t="n">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="R6" t="n">
         <v>394418</v>
       </c>
       <c r="S6" t="n">
-        <v>670758</v>
+        <v>617418</v>
       </c>
       <c r="T6" t="n">
         <v>2</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>305</v>
       </c>
       <c r="D7" t="n">
-        <v>76.3</v>
+        <v>69.3</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="G7" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H7" t="n">
         <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="J7" t="n">
         <v>3</v>
@@ -5053,35 +5053,35 @@
         <v>3</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N7" t="n">
         <v>47</v>
       </c>
       <c r="O7" t="n">
-        <v>100.7</v>
+        <v>101</v>
       </c>
       <c r="P7" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.7</v>
+        <v>1.4</v>
       </c>
       <c r="R7" t="n">
         <v>394418</v>
       </c>
       <c r="S7" t="n">
-        <v>617418</v>
+        <v>670758</v>
       </c>
       <c r="T7" t="n">
         <v>2</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
@@ -5656,37 +5656,37 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C16" t="n">
         <v>284</v>
       </c>
       <c r="D16" t="n">
-        <v>71.7</v>
+        <v>75.7</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5698,66 +5698,66 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>100.5</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="R16" t="n">
-        <v>1264459</v>
+        <v>1327109</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>1066412</v>
       </c>
       <c r="T16" t="n">
         <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C17" t="n">
         <v>284</v>
       </c>
       <c r="D17" t="n">
-        <v>75.7</v>
+        <v>71.7</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="G17" t="n">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="H17" t="n">
         <v>2</v>
       </c>
       <c r="I17" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="J17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K17" t="n">
         <v>2</v>
@@ -5769,29 +5769,29 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="O17" t="n">
-        <v>100.5</v>
+        <v>100.4</v>
       </c>
       <c r="P17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="Q17" t="n">
         <v>0.5</v>
       </c>
-      <c r="Q17" t="n">
-        <v>0</v>
-      </c>
       <c r="R17" t="n">
-        <v>1327109</v>
+        <v>1264459</v>
       </c>
       <c r="S17" t="n">
-        <v>1066412</v>
+        <v>3009015</v>
       </c>
       <c r="T17" t="n">
         <v>2</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>3xc, freehit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-14 16:11 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -571,19 +571,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>76</v>
+        <v>101</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F6" t="n">
         <v>305</v>
@@ -595,19 +595,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>101</v>
+        <v>76</v>
       </c>
       <c r="E7" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
         <v>305</v>
@@ -1650,33 +1650,33 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C6" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D6" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C7" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D7" t="n">
-        <v>43</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8">
@@ -2389,11 +2389,7 @@
       <c r="B16" t="n">
         <v>57</v>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2489,7 +2485,11 @@
       <c r="B24" t="n">
         <v>48</v>
       </c>
-      <c r="C24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2649,11 +2649,7 @@
       <c r="B4" t="n">
         <v>2</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2771,7 +2767,11 @@
       <c r="B14" t="n">
         <v>1</v>
       </c>
-      <c r="C14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3568,30 +3568,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E6" t="n">
-        <v>6474</v>
+        <v>281617</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1177681</v>
+        <v>1051323</v>
       </c>
       <c r="H6" t="n">
-        <v>6474</v>
+        <v>1076546</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -3605,30 +3605,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E7" t="n">
-        <v>281617</v>
+        <v>6474</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1051323</v>
+        <v>1177681</v>
       </c>
       <c r="H7" t="n">
-        <v>1076546</v>
+        <v>6474</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -4946,34 +4946,34 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>305</v>
       </c>
       <c r="D6" t="n">
-        <v>76.3</v>
+        <v>69.3</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="G6" t="n">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H6" t="n">
         <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="J6" t="n">
         <v>3</v>
@@ -4982,69 +4982,69 @@
         <v>3</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N6" t="n">
         <v>47</v>
       </c>
       <c r="O6" t="n">
-        <v>100.7</v>
+        <v>101</v>
       </c>
       <c r="P6" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.7</v>
+        <v>1.4</v>
       </c>
       <c r="R6" t="n">
         <v>394418</v>
       </c>
       <c r="S6" t="n">
-        <v>617418</v>
+        <v>670758</v>
       </c>
       <c r="T6" t="n">
         <v>2</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>305</v>
       </c>
       <c r="D7" t="n">
-        <v>69.3</v>
+        <v>76.3</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G7" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H7" t="n">
         <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="J7" t="n">
         <v>3</v>
@@ -5053,35 +5053,35 @@
         <v>3</v>
       </c>
       <c r="L7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N7" t="n">
         <v>47</v>
       </c>
       <c r="O7" t="n">
-        <v>101</v>
+        <v>100.7</v>
       </c>
       <c r="P7" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="Q7" t="n">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="R7" t="n">
         <v>394418</v>
       </c>
       <c r="S7" t="n">
-        <v>670758</v>
+        <v>617418</v>
       </c>
       <c r="T7" t="n">
         <v>2</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-14 20:12 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -484,13 +484,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="3">
@@ -508,13 +508,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>315</v>
+        <v>325</v>
       </c>
     </row>
     <row r="4">
@@ -523,22 +523,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F4" t="n">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="5">
@@ -547,22 +547,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="6">
@@ -571,27 +571,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E6" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>305</v>
+        <v>312</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -628,13 +628,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="9">
@@ -700,13 +700,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="12">
@@ -715,22 +715,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>287</v>
+        <v>293</v>
       </c>
     </row>
     <row r="13">
@@ -739,22 +739,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="E13" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="14">
@@ -763,22 +763,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="15">
@@ -787,22 +787,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F15" t="n">
-        <v>284</v>
+        <v>287</v>
       </c>
     </row>
     <row r="16">
@@ -811,46 +811,46 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="18">
@@ -859,22 +859,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="19">
@@ -883,22 +883,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="20">
@@ -907,22 +907,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="21">
@@ -964,13 +964,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="23">
@@ -1027,22 +1027,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="26">
@@ -1051,46 +1051,46 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="E26" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>260</v>
+        <v>266</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F27" t="n">
-        <v>259</v>
+        <v>266</v>
       </c>
     </row>
     <row r="28">
@@ -1099,22 +1099,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="29">
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="30">
@@ -1156,13 +1156,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E30" t="n">
         <v>-4</v>
       </c>
       <c r="F30" t="n">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="31">
@@ -1180,13 +1180,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E31" t="n">
         <v>-8</v>
       </c>
       <c r="F31" t="n">
-        <v>215</v>
+        <v>225</v>
       </c>
     </row>
     <row r="32">
@@ -1618,49 +1618,49 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C4" t="n">
         <v>103</v>
       </c>
       <c r="D4" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C5" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D5" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="C6" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D6" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7">
@@ -1746,145 +1746,145 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>73</v>
+        <v>48</v>
       </c>
       <c r="C12" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="D12" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="C13" t="n">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="D13" t="n">
-        <v>60</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="C14" t="n">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="D14" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C15" t="n">
-        <v>118</v>
+        <v>97</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="C16" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D16" t="n">
-        <v>54</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="C17" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="D17" t="n">
-        <v>67</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C18" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D18" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C19" t="n">
-        <v>120</v>
+        <v>101</v>
       </c>
       <c r="D19" t="n">
-        <v>49</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="C20" t="n">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D20" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21">
@@ -1954,65 +1954,65 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="C25" t="n">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="D25" t="n">
-        <v>78</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="C26" t="n">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="D26" t="n">
-        <v>46</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C27" t="n">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="D27" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>59</v>
       </c>
       <c r="C28" t="n">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="D28" t="n">
-        <v>38</v>
+        <v>47</v>
       </c>
     </row>
     <row r="29">
@@ -2339,7 +2339,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2350,7 +2350,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2361,7 +2361,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2516,7 +2516,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2527,7 +2527,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2538,7 +2538,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2731,7 +2731,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2746,7 +2746,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2761,7 +2761,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2798,7 +2798,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2809,7 +2809,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -2820,7 +2820,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -2831,7 +2831,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -2842,7 +2842,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -2853,7 +2853,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -2897,7 +2897,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -2908,7 +2908,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -3209,12 +3209,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Wissa</t>
+          <t>Ballard</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -3224,18 +3224,18 @@
         <v>8</v>
       </c>
       <c r="E10" t="n">
-        <v>3.7</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Ballard</t>
+          <t>Wissa</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -3245,13 +3245,13 @@
         <v>8</v>
       </c>
       <c r="E11" t="n">
-        <v>4.9</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3272,7 +3272,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3494,30 +3494,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E4" t="n">
-        <v>71857</v>
+        <v>281617</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1929309</v>
+        <v>1051323</v>
       </c>
       <c r="H4" t="n">
-        <v>297407</v>
+        <v>1076546</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -3531,30 +3531,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E5" t="n">
-        <v>27153</v>
+        <v>71857</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>606381</v>
+        <v>1929309</v>
       </c>
       <c r="H5" t="n">
-        <v>240451</v>
+        <v>297407</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -3568,30 +3568,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E6" t="n">
-        <v>281617</v>
+        <v>27153</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1051323</v>
+        <v>606381</v>
       </c>
       <c r="H6" t="n">
-        <v>1076546</v>
+        <v>240451</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -3601,7 +3601,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -3790,30 +3790,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E12" t="n">
-        <v>37120</v>
+        <v>60517</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2015/16</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1571193</v>
+        <v>1414622</v>
       </c>
       <c r="H12" t="n">
-        <v>3349378</v>
+        <v>339763</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -3827,30 +3827,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E13" t="n">
-        <v>1128645</v>
+        <v>8917</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>3434302</v>
+        <v>2118382</v>
       </c>
       <c r="H13" t="n">
-        <v>1128645</v>
+        <v>9146930</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -3864,30 +3864,30 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E14" t="n">
-        <v>189374</v>
+        <v>37120</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>1757289</v>
+        <v>1571193</v>
       </c>
       <c r="H14" t="n">
-        <v>250879</v>
+        <v>3349378</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -3901,30 +3901,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E15" t="n">
-        <v>273503</v>
+        <v>1128645</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1994005</v>
+        <v>3434302</v>
       </c>
       <c r="H15" t="n">
-        <v>1917309</v>
+        <v>1128645</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -3938,30 +3938,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>31543</v>
+        <v>189374</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>820692</v>
+        <v>1757289</v>
       </c>
       <c r="H16" t="n">
-        <v>1637750</v>
+        <v>250879</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -3971,34 +3971,34 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E17" t="n">
-        <v>453230</v>
+        <v>31543</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>5483351</v>
+        <v>820692</v>
       </c>
       <c r="H17" t="n">
-        <v>8188106</v>
+        <v>1637750</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4012,19 +4012,19 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E18" t="n">
-        <v>486041</v>
+        <v>273503</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4032,10 +4032,10 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>2415786</v>
+        <v>1994005</v>
       </c>
       <c r="H18" t="n">
-        <v>1206623</v>
+        <v>1917309</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -4049,30 +4049,30 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E19" t="n">
-        <v>60517</v>
+        <v>453230</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2015/16</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>1414622</v>
+        <v>5483351</v>
       </c>
       <c r="H19" t="n">
-        <v>339763</v>
+        <v>8188106</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -4086,30 +4086,30 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>8917</v>
+        <v>486041</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>2118382</v>
+        <v>2415786</v>
       </c>
       <c r="H20" t="n">
-        <v>9146930</v>
+        <v>1206623</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -4271,19 +4271,19 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E25" t="n">
-        <v>15288</v>
+        <v>334016</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -4291,10 +4291,10 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>329510</v>
+        <v>2156629</v>
       </c>
       <c r="H25" t="n">
-        <v>538046</v>
+        <v>2691725</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -4308,19 +4308,19 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E26" t="n">
-        <v>1320699</v>
+        <v>15288</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -4328,36 +4328,36 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>2490743</v>
+        <v>329510</v>
       </c>
       <c r="H26" t="n">
-        <v>1861933</v>
+        <v>538046</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E27" t="n">
-        <v>81907</v>
+        <v>1320699</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -4365,14 +4365,14 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>3252487</v>
+        <v>2490743</v>
       </c>
       <c r="H27" t="n">
-        <v>11118394</v>
+        <v>1861933</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2024/25</t>
         </is>
       </c>
     </row>
@@ -4382,19 +4382,19 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E28" t="n">
-        <v>334016</v>
+        <v>81907</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -4402,10 +4402,10 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>2156629</v>
+        <v>3252487</v>
       </c>
       <c r="H28" t="n">
-        <v>2691725</v>
+        <v>11118394</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -4675,7 +4675,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="D2" t="n">
         <v>87.7</v>
@@ -4746,7 +4746,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>315</v>
+        <v>325</v>
       </c>
       <c r="D3" t="n">
         <v>69.7</v>
@@ -4804,25 +4804,25 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="D4" t="n">
-        <v>74</v>
+        <v>69.3</v>
       </c>
       <c r="E4" t="n">
         <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>68</v>
+        <v>48</v>
       </c>
       <c r="G4" t="n">
         <v>103</v>
@@ -4831,37 +4831,37 @@
         <v>2</v>
       </c>
       <c r="I4" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="J4" t="n">
         <v>3</v>
       </c>
       <c r="K4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N4" t="n">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="O4" t="n">
-        <v>101.1</v>
+        <v>101</v>
       </c>
       <c r="P4" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="R4" t="n">
-        <v>223959</v>
+        <v>394418</v>
       </c>
       <c r="S4" t="n">
-        <v>24105</v>
+        <v>670758</v>
       </c>
       <c r="T4" t="n">
         <v>2</v>
@@ -4875,40 +4875,40 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D5" t="n">
-        <v>76.3</v>
+        <v>74</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="G5" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="H5" t="n">
         <v>2</v>
       </c>
       <c r="I5" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="J5" t="n">
         <v>3</v>
       </c>
       <c r="K5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -4917,63 +4917,63 @@
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="O5" t="n">
-        <v>100.4</v>
+        <v>101.1</v>
       </c>
       <c r="P5" t="n">
-        <v>0.4</v>
+        <v>1.1</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>252786</v>
+        <v>223959</v>
       </c>
       <c r="S5" t="n">
-        <v>166751</v>
+        <v>24105</v>
       </c>
       <c r="T5" t="n">
         <v>2</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="D6" t="n">
-        <v>69.3</v>
+        <v>76.3</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="G6" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="H6" t="n">
         <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="J6" t="n">
         <v>3</v>
@@ -4982,35 +4982,35 @@
         <v>3</v>
       </c>
       <c r="L6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="O6" t="n">
-        <v>101</v>
+        <v>100.4</v>
       </c>
       <c r="P6" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="Q6" t="n">
-        <v>1.4</v>
+        <v>0.4</v>
       </c>
       <c r="R6" t="n">
-        <v>394418</v>
+        <v>252786</v>
       </c>
       <c r="S6" t="n">
-        <v>670758</v>
+        <v>166751</v>
       </c>
       <c r="T6" t="n">
         <v>2</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>
@@ -5097,7 +5097,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D8" t="n">
         <v>71.3</v>
@@ -5310,7 +5310,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D11" t="n">
         <v>75.3</v>
@@ -5372,41 +5372,41 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="D12" t="n">
-        <v>72.7</v>
+        <v>72.3</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="G12" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="H12" t="n">
         <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
         <v>3</v>
       </c>
-      <c r="K12" t="n">
-        <v>2</v>
-      </c>
       <c r="L12" t="n">
         <v>0</v>
       </c>
@@ -5414,140 +5414,136 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="O12" t="n">
-        <v>101.1</v>
+        <v>100.2</v>
       </c>
       <c r="P12" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
       <c r="Q12" t="n">
-        <v>1.1</v>
+        <v>0.6</v>
       </c>
       <c r="R12" t="n">
-        <v>1088487</v>
+        <v>1411981</v>
       </c>
       <c r="S12" t="n">
-        <v>101935</v>
+        <v>4399137</v>
       </c>
       <c r="T12" t="n">
-        <v>3</v>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>bboost</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D13" t="n">
-        <v>66.7</v>
+        <v>73</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="G13" t="n">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="H13" t="n">
         <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>33</v>
+        <v>63</v>
       </c>
       <c r="O13" t="n">
-        <v>100.4</v>
+        <v>101</v>
       </c>
       <c r="P13" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="Q13" t="n">
         <v>0.2</v>
       </c>
       <c r="R13" t="n">
-        <v>1163981</v>
+        <v>1458203</v>
       </c>
       <c r="S13" t="n">
-        <v>3048395</v>
+        <v>878473</v>
       </c>
       <c r="T13" t="n">
         <v>2</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="D14" t="n">
-        <v>70</v>
+        <v>72.7</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14" t="n">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="G14" t="n">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="H14" t="n">
         <v>2</v>
       </c>
       <c r="I14" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="J14" t="n">
         <v>3</v>
       </c>
       <c r="K14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -5556,93 +5552,93 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="O14" t="n">
-        <v>100.4</v>
+        <v>101.1</v>
       </c>
       <c r="P14" t="n">
-        <v>0.4</v>
+        <v>1.1</v>
       </c>
       <c r="Q14" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="R14" t="n">
-        <v>1257108</v>
+        <v>1088487</v>
       </c>
       <c r="S14" t="n">
-        <v>3046343</v>
+        <v>101935</v>
       </c>
       <c r="T14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="D15" t="n">
-        <v>71</v>
+        <v>66.7</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="G15" t="n">
-        <v>118</v>
+        <v>97</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="J15" t="n">
         <v>1</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N15" t="n">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="O15" t="n">
-        <v>100.5</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="R15" t="n">
-        <v>1375721</v>
+        <v>1163981</v>
       </c>
       <c r="S15" t="n">
-        <v>5881370</v>
+        <v>3048395</v>
       </c>
       <c r="T15" t="n">
         <v>2</v>
@@ -5656,40 +5652,40 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D16" t="n">
-        <v>75.7</v>
+        <v>70</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>95</v>
+        <v>68</v>
       </c>
       <c r="G16" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="J16" t="n">
         <v>3</v>
       </c>
       <c r="K16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
@@ -5698,66 +5694,66 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="O16" t="n">
-        <v>100.5</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
         <v>0</v>
       </c>
       <c r="R16" t="n">
-        <v>1327109</v>
+        <v>1257108</v>
       </c>
       <c r="S16" t="n">
-        <v>1066412</v>
+        <v>3046343</v>
       </c>
       <c r="T16" t="n">
         <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D17" t="n">
-        <v>71.7</v>
+        <v>75.7</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="G17" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="H17" t="n">
         <v>2</v>
       </c>
       <c r="I17" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="J17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K17" t="n">
         <v>2</v>
@@ -5769,69 +5765,69 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="O17" t="n">
-        <v>100.4</v>
+        <v>100.5</v>
       </c>
       <c r="P17" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>1264459</v>
+        <v>1327109</v>
       </c>
       <c r="S17" t="n">
-        <v>3009015</v>
+        <v>1066412</v>
       </c>
       <c r="T17" t="n">
         <v>2</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>3xc, freehit</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D18" t="n">
-        <v>69.3</v>
+        <v>71</v>
       </c>
       <c r="E18" t="n">
         <v>2</v>
       </c>
       <c r="F18" t="n">
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="G18" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="H18" t="n">
         <v>2</v>
       </c>
       <c r="I18" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J18" t="n">
         <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
         <v>0</v>
@@ -5840,7 +5836,7 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="O18" t="n">
         <v>100.5</v>
@@ -5849,13 +5845,13 @@
         <v>0.5</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="R18" t="n">
-        <v>1391545</v>
+        <v>1375721</v>
       </c>
       <c r="S18" t="n">
-        <v>5250200</v>
+        <v>5881370</v>
       </c>
       <c r="T18" t="n">
         <v>2</v>
@@ -5869,40 +5865,40 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D19" t="n">
-        <v>72.3</v>
+        <v>71.7</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="G19" t="n">
-        <v>120</v>
+        <v>101</v>
       </c>
       <c r="H19" t="n">
         <v>2</v>
       </c>
       <c r="I19" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J19" t="n">
         <v>1</v>
       </c>
       <c r="K19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L19" t="n">
         <v>0</v>
@@ -5911,62 +5907,66 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>56</v>
+        <v>26</v>
       </c>
       <c r="O19" t="n">
-        <v>100.2</v>
+        <v>100.4</v>
       </c>
       <c r="P19" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="R19" t="n">
-        <v>1411981</v>
+        <v>1264459</v>
       </c>
       <c r="S19" t="n">
-        <v>4399137</v>
+        <v>3009015</v>
       </c>
       <c r="T19" t="n">
         <v>2</v>
       </c>
-      <c r="U19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>3xc, freehit</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D20" t="n">
-        <v>73</v>
+        <v>69.3</v>
       </c>
       <c r="E20" t="n">
         <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="G20" t="n">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="H20" t="n">
         <v>2</v>
       </c>
       <c r="I20" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="J20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
         <v>2</v>
@@ -5978,29 +5978,29 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="O20" t="n">
-        <v>101</v>
+        <v>100.5</v>
       </c>
       <c r="P20" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="R20" t="n">
-        <v>1458203</v>
+        <v>1391545</v>
       </c>
       <c r="S20" t="n">
-        <v>878473</v>
+        <v>5250200</v>
       </c>
       <c r="T20" t="n">
         <v>2</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
@@ -6087,7 +6087,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D22" t="n">
         <v>61.7</v>
@@ -6291,40 +6291,40 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D25" t="n">
-        <v>65.7</v>
+        <v>64.3</v>
       </c>
       <c r="E25" t="n">
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="G25" t="n">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="H25" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" t="n">
+        <v>38</v>
+      </c>
+      <c r="J25" t="n">
         <v>3</v>
       </c>
-      <c r="I25" t="n">
-        <v>41</v>
-      </c>
-      <c r="J25" t="n">
-        <v>1</v>
-      </c>
       <c r="K25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
@@ -6333,119 +6333,115 @@
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="O25" t="n">
-        <v>100.6</v>
+        <v>100.9</v>
       </c>
       <c r="P25" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="Q25" t="n">
         <v>1</v>
       </c>
       <c r="R25" t="n">
-        <v>2758639</v>
+        <v>3583946</v>
       </c>
       <c r="S25" t="n">
-        <v>3395267</v>
+        <v>453361</v>
       </c>
       <c r="T25" t="n">
-        <v>3</v>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>3xc</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="D26" t="n">
-        <v>67</v>
+        <v>65.7</v>
       </c>
       <c r="E26" t="n">
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G26" t="n">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="H26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I26" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="J26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K26" t="n">
         <v>3</v>
       </c>
       <c r="L26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="O26" t="n">
-        <v>100.7</v>
+        <v>100.6</v>
       </c>
       <c r="P26" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="R26" t="n">
-        <v>3318900</v>
+        <v>2758639</v>
       </c>
       <c r="S26" t="n">
-        <v>1948104</v>
+        <v>3395267</v>
       </c>
       <c r="T26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>3xc</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="D27" t="n">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E27" t="n">
         <v>1</v>
@@ -6454,40 +6450,46 @@
         <v>48</v>
       </c>
       <c r="G27" t="n">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="H27" t="n">
         <v>2</v>
       </c>
       <c r="I27" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J27" t="n">
         <v>3</v>
       </c>
       <c r="K27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N27" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="O27" t="n">
-        <v>101.2</v>
+        <v>100.7</v>
       </c>
       <c r="P27" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="R27" t="n">
-        <v>3390269</v>
+        <v>3318900</v>
+      </c>
+      <c r="S27" t="n">
+        <v>1948104</v>
+      </c>
+      <c r="T27" t="n">
+        <v>2</v>
       </c>
       <c r="U27" t="inlineStr">
         <is>
@@ -6498,19 +6500,19 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="D28" t="n">
-        <v>64.3</v>
+        <v>62</v>
       </c>
       <c r="E28" t="n">
         <v>1</v>
@@ -6519,13 +6521,13 @@
         <v>48</v>
       </c>
       <c r="G28" t="n">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="H28" t="n">
         <v>2</v>
       </c>
       <c r="I28" t="n">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="J28" t="n">
         <v>3</v>
@@ -6540,27 +6542,25 @@
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="O28" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P28" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q28" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="R28" t="n">
-        <v>3583946</v>
-      </c>
-      <c r="S28" t="n">
-        <v>453361</v>
-      </c>
-      <c r="T28" t="n">
-        <v>2</v>
-      </c>
-      <c r="U28" t="inlineStr"/>
+        <v>3390269</v>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6574,7 +6574,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D29" t="n">
         <v>59.3</v>
@@ -6645,7 +6645,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D30" t="n">
         <v>52.7</v>
@@ -6710,7 +6710,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="D31" t="n">
         <v>47.7</v>

</xml_diff>

<commit_message>
Update standings 2026-09-14 22:11 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -484,13 +484,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="3">
@@ -556,13 +556,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="6">
@@ -580,13 +580,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="7">
@@ -595,16 +595,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -619,22 +619,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="9">
@@ -700,13 +700,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="12">
@@ -748,13 +748,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="14">
@@ -763,16 +763,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
@@ -787,19 +787,19 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="E15" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
         <v>287</v>
@@ -811,22 +811,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F16" t="n">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="17">
@@ -964,13 +964,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="23">
@@ -1051,43 +1051,43 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F26" t="n">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E27" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
         <v>266</v>
@@ -1108,13 +1108,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="29">
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="30">
@@ -1147,22 +1147,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Slumber FC</t>
+          <t>Redsbay</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="E30" t="n">
-        <v>-4</v>
+        <v>-8</v>
       </c>
       <c r="F30" t="n">
-        <v>225</v>
+        <v>232</v>
       </c>
     </row>
     <row r="31">
@@ -1171,22 +1171,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Redsbay</t>
+          <t>Slumber FC</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="E31" t="n">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="F31" t="n">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="32">
@@ -1666,33 +1666,33 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="C7" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D7" t="n">
-        <v>60</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="C8" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D8" t="n">
-        <v>37</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9">
@@ -1778,49 +1778,49 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="C14" t="n">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="D14" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="C16" t="n">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="D16" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17">
@@ -1970,33 +1970,33 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="C26" t="n">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="D26" t="n">
-        <v>78</v>
+        <v>46</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="C27" t="n">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="D27" t="n">
-        <v>46</v>
+        <v>78</v>
       </c>
     </row>
     <row r="28">
@@ -2034,33 +2034,33 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="C30" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D30" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="C31" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D31" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="32">
@@ -2820,7 +2820,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -2831,7 +2831,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -3605,30 +3605,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E7" t="n">
-        <v>6474</v>
+        <v>28582</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1177681</v>
+        <v>881388</v>
       </c>
       <c r="H7" t="n">
-        <v>6474</v>
+        <v>239490</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -3642,30 +3642,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E8" t="n">
-        <v>28582</v>
+        <v>6474</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>881388</v>
+        <v>1177681</v>
       </c>
       <c r="H8" t="n">
-        <v>239490</v>
+        <v>6474</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -3864,30 +3864,30 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E14" t="n">
-        <v>37120</v>
+        <v>189374</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>1571193</v>
+        <v>1757289</v>
       </c>
       <c r="H14" t="n">
-        <v>3349378</v>
+        <v>250879</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -3901,30 +3901,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>1128645</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>3434302</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>1128645</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -3938,30 +3938,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E16" t="n">
-        <v>189374</v>
+        <v>1128645</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1757289</v>
+        <v>3434302</v>
       </c>
       <c r="H16" t="n">
-        <v>250879</v>
+        <v>1128645</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -4308,19 +4308,19 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E26" t="n">
-        <v>15288</v>
+        <v>1320699</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -4328,36 +4328,36 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>329510</v>
+        <v>2490743</v>
       </c>
       <c r="H26" t="n">
-        <v>538046</v>
+        <v>1861933</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2024/25</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E27" t="n">
-        <v>1320699</v>
+        <v>15288</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -4365,14 +4365,14 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>2490743</v>
+        <v>329510</v>
       </c>
       <c r="H27" t="n">
-        <v>1861933</v>
+        <v>538046</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
     </row>
@@ -4456,19 +4456,19 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Slumber FC</t>
+          <t>Redsbay</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E30" t="n">
-        <v>676529</v>
+        <v>4884220</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -4476,10 +4476,10 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>998938</v>
+        <v>4884220</v>
       </c>
       <c r="H30" t="n">
-        <v>676529</v>
+        <v>4884220</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -4493,19 +4493,19 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Redsbay</t>
+          <t>Slumber FC</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E31" t="n">
-        <v>4884220</v>
+        <v>676529</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -4513,10 +4513,10 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>4884220</v>
+        <v>998938</v>
       </c>
       <c r="H31" t="n">
-        <v>4884220</v>
+        <v>676529</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -4675,7 +4675,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D2" t="n">
         <v>87.7</v>
@@ -4884,7 +4884,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D5" t="n">
         <v>74</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D6" t="n">
         <v>76.3</v>
@@ -5017,40 +5017,40 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>305</v>
       </c>
       <c r="D7" t="n">
-        <v>76.3</v>
+        <v>71.3</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="G7" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H7" t="n">
         <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="J7" t="n">
         <v>3</v>
       </c>
       <c r="K7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -5059,69 +5059,69 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="O7" t="n">
-        <v>100.7</v>
+        <v>101.4</v>
       </c>
       <c r="P7" t="n">
-        <v>0.7</v>
+        <v>1.4</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="R7" t="n">
-        <v>394418</v>
+        <v>434425</v>
       </c>
       <c r="S7" t="n">
-        <v>617418</v>
+        <v>88386</v>
       </c>
       <c r="T7" t="n">
         <v>2</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D8" t="n">
-        <v>71.3</v>
+        <v>76.3</v>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="G8" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H8" t="n">
         <v>2</v>
       </c>
       <c r="I8" t="n">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="J8" t="n">
         <v>3</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -5130,29 +5130,29 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="O8" t="n">
-        <v>101.4</v>
+        <v>100.7</v>
       </c>
       <c r="P8" t="n">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="R8" t="n">
-        <v>434425</v>
+        <v>394418</v>
       </c>
       <c r="S8" t="n">
-        <v>88386</v>
+        <v>617418</v>
       </c>
       <c r="T8" t="n">
         <v>2</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>
@@ -5310,7 +5310,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D11" t="n">
         <v>75.3</v>
@@ -5448,7 +5448,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D13" t="n">
         <v>73</v>
@@ -5510,40 +5510,40 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="C14" t="n">
         <v>287</v>
       </c>
       <c r="D14" t="n">
-        <v>72.7</v>
+        <v>70</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="G14" t="n">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="H14" t="n">
         <v>2</v>
       </c>
       <c r="I14" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="J14" t="n">
         <v>3</v>
       </c>
       <c r="K14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -5552,149 +5552,149 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="O14" t="n">
-        <v>101.1</v>
+        <v>100.4</v>
       </c>
       <c r="P14" t="n">
-        <v>1.1</v>
+        <v>0.4</v>
       </c>
       <c r="Q14" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>1088487</v>
+        <v>1257108</v>
       </c>
       <c r="S14" t="n">
-        <v>101935</v>
+        <v>3046343</v>
       </c>
       <c r="T14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
         <v>287</v>
       </c>
       <c r="D15" t="n">
-        <v>66.7</v>
+        <v>72.7</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G15" t="n">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>35</v>
+      </c>
+      <c r="O15" t="n">
+        <v>101.1</v>
+      </c>
+      <c r="P15" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="R15" t="n">
+        <v>1088487</v>
+      </c>
+      <c r="S15" t="n">
+        <v>101935</v>
+      </c>
+      <c r="T15" t="n">
         <v>3</v>
       </c>
-      <c r="L15" t="n">
-        <v>1</v>
-      </c>
-      <c r="M15" t="n">
-        <v>-4</v>
-      </c>
-      <c r="N15" t="n">
-        <v>33</v>
-      </c>
-      <c r="O15" t="n">
-        <v>100.4</v>
-      </c>
-      <c r="P15" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="R15" t="n">
-        <v>1163981</v>
-      </c>
-      <c r="S15" t="n">
-        <v>3048395</v>
-      </c>
-      <c r="T15" t="n">
-        <v>2</v>
-      </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D16" t="n">
-        <v>70</v>
+        <v>66.7</v>
       </c>
       <c r="E16" t="n">
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="G16" t="n">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="J16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" t="n">
         <v>3</v>
       </c>
-      <c r="K16" t="n">
-        <v>1</v>
-      </c>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M16" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N16" t="n">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="O16" t="n">
         <v>100.4</v>
@@ -5703,20 +5703,20 @@
         <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="R16" t="n">
-        <v>1257108</v>
+        <v>1163981</v>
       </c>
       <c r="S16" t="n">
-        <v>3046343</v>
+        <v>3048395</v>
       </c>
       <c r="T16" t="n">
         <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
@@ -6087,7 +6087,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D22" t="n">
         <v>61.7</v>
@@ -6358,142 +6358,142 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D26" t="n">
-        <v>65.7</v>
+        <v>67</v>
       </c>
       <c r="E26" t="n">
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="G26" t="n">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="H26" t="n">
+        <v>2</v>
+      </c>
+      <c r="I26" t="n">
+        <v>46</v>
+      </c>
+      <c r="J26" t="n">
         <v>3</v>
-      </c>
-      <c r="I26" t="n">
-        <v>41</v>
-      </c>
-      <c r="J26" t="n">
-        <v>1</v>
       </c>
       <c r="K26" t="n">
         <v>3</v>
       </c>
       <c r="L26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N26" t="n">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="O26" t="n">
-        <v>100.6</v>
+        <v>100.7</v>
       </c>
       <c r="P26" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="Q26" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="R26" t="n">
-        <v>2758639</v>
+        <v>3318900</v>
       </c>
       <c r="S26" t="n">
-        <v>3395267</v>
+        <v>1948104</v>
       </c>
       <c r="T26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>3xc</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="C27" t="n">
         <v>266</v>
       </c>
       <c r="D27" t="n">
-        <v>67</v>
+        <v>65.7</v>
       </c>
       <c r="E27" t="n">
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G27" t="n">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="H27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I27" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="J27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K27" t="n">
         <v>3</v>
       </c>
       <c r="L27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M27" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="O27" t="n">
-        <v>100.7</v>
+        <v>100.6</v>
       </c>
       <c r="P27" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="R27" t="n">
-        <v>3318900</v>
+        <v>2758639</v>
       </c>
       <c r="S27" t="n">
-        <v>1948104</v>
+        <v>3395267</v>
       </c>
       <c r="T27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>3xc</t>
         </is>
       </c>
     </row>
@@ -6509,7 +6509,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D28" t="n">
         <v>62</v>
@@ -6574,7 +6574,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D29" t="n">
         <v>59.3</v>
@@ -6636,61 +6636,67 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Slumber FC</t>
+          <t>Redsbay</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="D30" t="n">
-        <v>52.7</v>
+        <v>47.7</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G30" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H30" t="n">
         <v>2</v>
       </c>
       <c r="I30" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="J30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M30" t="n">
-        <v>-4</v>
+        <v>-8</v>
       </c>
       <c r="N30" t="n">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="O30" t="n">
-        <v>100.4</v>
+        <v>100.9</v>
       </c>
       <c r="P30" t="n">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="R30" t="n">
-        <v>6572720</v>
+        <v>7330374</v>
+      </c>
+      <c r="S30" t="n">
+        <v>140252</v>
+      </c>
+      <c r="T30" t="n">
+        <v>2</v>
       </c>
       <c r="U30" t="inlineStr">
         <is>
@@ -6701,67 +6707,61 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Redsbay</t>
+          <t>Slumber FC</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D31" t="n">
-        <v>47.7</v>
+        <v>52.7</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G31" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="H31" t="n">
         <v>2</v>
       </c>
       <c r="I31" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="J31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="N31" t="n">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="O31" t="n">
-        <v>100.9</v>
+        <v>100.4</v>
       </c>
       <c r="P31" t="n">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
       <c r="Q31" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="R31" t="n">
-        <v>7330374</v>
-      </c>
-      <c r="S31" t="n">
-        <v>140252</v>
-      </c>
-      <c r="T31" t="n">
-        <v>2</v>
+        <v>6572720</v>
       </c>
       <c r="U31" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update standings 2026-09-15 00:16 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -4720,7 +4720,7 @@
         <v>0.4</v>
       </c>
       <c r="R2" t="n">
-        <v>9993</v>
+        <v>9971</v>
       </c>
       <c r="S2" t="n">
         <v>270274</v>
@@ -4791,7 +4791,7 @@
         <v>0.2</v>
       </c>
       <c r="R3" t="n">
-        <v>176788</v>
+        <v>105685</v>
       </c>
       <c r="S3" t="n">
         <v>1461471</v>
@@ -4858,7 +4858,7 @@
         <v>1.4</v>
       </c>
       <c r="R4" t="n">
-        <v>394418</v>
+        <v>258869</v>
       </c>
       <c r="S4" t="n">
         <v>670758</v>
@@ -4929,7 +4929,7 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>223959</v>
+        <v>269558</v>
       </c>
       <c r="S5" t="n">
         <v>24105</v>
@@ -5000,7 +5000,7 @@
         <v>0.4</v>
       </c>
       <c r="R6" t="n">
-        <v>252786</v>
+        <v>301918</v>
       </c>
       <c r="S6" t="n">
         <v>166751</v>
@@ -5071,7 +5071,7 @@
         <v>0.2</v>
       </c>
       <c r="R7" t="n">
-        <v>434425</v>
+        <v>510595</v>
       </c>
       <c r="S7" t="n">
         <v>88386</v>
@@ -5130,7 +5130,7 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="O8" t="n">
         <v>100.7</v>
@@ -5142,7 +5142,7 @@
         <v>0.7</v>
       </c>
       <c r="R8" t="n">
-        <v>394418</v>
+        <v>530348</v>
       </c>
       <c r="S8" t="n">
         <v>617418</v>
@@ -5201,7 +5201,7 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="O9" t="n">
         <v>100.3</v>
@@ -5213,7 +5213,7 @@
         <v>0.6</v>
       </c>
       <c r="R9" t="n">
-        <v>516440</v>
+        <v>719732</v>
       </c>
       <c r="S9" t="n">
         <v>637992</v>
@@ -5272,7 +5272,7 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O10" t="n">
         <v>101</v>
@@ -5284,7 +5284,7 @@
         <v>0.2</v>
       </c>
       <c r="R10" t="n">
-        <v>575726</v>
+        <v>747829</v>
       </c>
       <c r="S10" t="n">
         <v>1034411</v>
@@ -5355,7 +5355,7 @@
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>831682</v>
+        <v>836186</v>
       </c>
       <c r="S11" t="n">
         <v>3039834</v>
@@ -5426,7 +5426,7 @@
         <v>0.6</v>
       </c>
       <c r="R12" t="n">
-        <v>1411981</v>
+        <v>1050933</v>
       </c>
       <c r="S12" t="n">
         <v>4399137</v>
@@ -5493,7 +5493,7 @@
         <v>0.2</v>
       </c>
       <c r="R13" t="n">
-        <v>1458203</v>
+        <v>1258971</v>
       </c>
       <c r="S13" t="n">
         <v>878473</v>
@@ -5564,7 +5564,7 @@
         <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>1257108</v>
+        <v>1374667</v>
       </c>
       <c r="S14" t="n">
         <v>3046343</v>
@@ -5635,7 +5635,7 @@
         <v>1.1</v>
       </c>
       <c r="R15" t="n">
-        <v>1088487</v>
+        <v>1382146</v>
       </c>
       <c r="S15" t="n">
         <v>101935</v>
@@ -5706,7 +5706,7 @@
         <v>0.2</v>
       </c>
       <c r="R16" t="n">
-        <v>1163981</v>
+        <v>1402141</v>
       </c>
       <c r="S16" t="n">
         <v>3048395</v>
@@ -5777,7 +5777,7 @@
         <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>1327109</v>
+        <v>1512514</v>
       </c>
       <c r="S17" t="n">
         <v>1066412</v>
@@ -5836,7 +5836,7 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="O18" t="n">
         <v>100.5</v>
@@ -5848,7 +5848,7 @@
         <v>0.6</v>
       </c>
       <c r="R18" t="n">
-        <v>1375721</v>
+        <v>1563918</v>
       </c>
       <c r="S18" t="n">
         <v>5881370</v>
@@ -5907,7 +5907,7 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O19" t="n">
         <v>100.4</v>
@@ -5919,7 +5919,7 @@
         <v>0.5</v>
       </c>
       <c r="R19" t="n">
-        <v>1264459</v>
+        <v>1580919</v>
       </c>
       <c r="S19" t="n">
         <v>3009015</v>
@@ -5990,7 +5990,7 @@
         <v>0.5</v>
       </c>
       <c r="R20" t="n">
-        <v>1391545</v>
+        <v>1650086</v>
       </c>
       <c r="S20" t="n">
         <v>5250200</v>
@@ -6061,7 +6061,7 @@
         <v>1</v>
       </c>
       <c r="R21" t="n">
-        <v>1595374</v>
+        <v>1867826</v>
       </c>
       <c r="S21" t="n">
         <v>4185865</v>
@@ -6132,7 +6132,7 @@
         <v>0.4</v>
       </c>
       <c r="R22" t="n">
-        <v>2129786</v>
+        <v>2260007</v>
       </c>
       <c r="S22" t="n">
         <v>2735246</v>
@@ -6191,7 +6191,7 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="O23" t="n">
         <v>101.2</v>
@@ -6203,7 +6203,7 @@
         <v>1.5</v>
       </c>
       <c r="R23" t="n">
-        <v>2381160</v>
+        <v>2682180</v>
       </c>
       <c r="S23" t="n">
         <v>1396363</v>
@@ -6274,7 +6274,7 @@
         <v>0.2</v>
       </c>
       <c r="R24" t="n">
-        <v>2467563</v>
+        <v>2769665</v>
       </c>
       <c r="S24" t="n">
         <v>1595922</v>
@@ -6345,7 +6345,7 @@
         <v>1</v>
       </c>
       <c r="R25" t="n">
-        <v>3583946</v>
+        <v>2949027</v>
       </c>
       <c r="S25" t="n">
         <v>453361</v>
@@ -6412,7 +6412,7 @@
         <v>0.1</v>
       </c>
       <c r="R26" t="n">
-        <v>3318900</v>
+        <v>2973583</v>
       </c>
       <c r="S26" t="n">
         <v>1948104</v>
@@ -6483,7 +6483,7 @@
         <v>1</v>
       </c>
       <c r="R27" t="n">
-        <v>2758639</v>
+        <v>3064196</v>
       </c>
       <c r="S27" t="n">
         <v>3395267</v>
@@ -6554,7 +6554,7 @@
         <v>0.7</v>
       </c>
       <c r="R28" t="n">
-        <v>3390269</v>
+        <v>3317256</v>
       </c>
       <c r="U28" t="inlineStr">
         <is>
@@ -6619,7 +6619,7 @@
         <v>0</v>
       </c>
       <c r="R29" t="n">
-        <v>4757632</v>
+        <v>4839833</v>
       </c>
       <c r="S29" t="n">
         <v>3963132</v>
@@ -6690,7 +6690,7 @@
         <v>1</v>
       </c>
       <c r="R30" t="n">
-        <v>7330374</v>
+        <v>6223274</v>
       </c>
       <c r="S30" t="n">
         <v>140252</v>
@@ -6761,7 +6761,7 @@
         <v>0.7</v>
       </c>
       <c r="R31" t="n">
-        <v>6572720</v>
+        <v>6606759</v>
       </c>
       <c r="U31" t="inlineStr">
         <is>
@@ -6826,7 +6826,7 @@
         <v>2.2</v>
       </c>
       <c r="R32" t="n">
-        <v>8752145</v>
+        <v>8850751</v>
       </c>
       <c r="S32" t="n">
         <v>216389</v>

</xml_diff>

<commit_message>
Update standings 2026-09-15 10:12 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -835,22 +835,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="18">
@@ -859,22 +859,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="19">
@@ -883,16 +883,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -999,26 +999,26 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="25">
@@ -1027,22 +1027,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="26">
@@ -1826,49 +1826,49 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="C17" t="n">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="D17" t="n">
-        <v>54</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="C18" t="n">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="D18" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C19" t="n">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="D19" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20">
@@ -1922,49 +1922,49 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C23" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D23" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="n">
+        <v>45</v>
+      </c>
+      <c r="C24" t="n">
+        <v>86</v>
+      </c>
+      <c r="D24" t="n">
         <v>46</v>
-      </c>
-      <c r="C24" t="n">
-        <v>89</v>
-      </c>
-      <c r="D24" t="n">
-        <v>50</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="C25" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="D25" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26">
@@ -2243,7 +2243,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -2254,7 +2254,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -2505,7 +2505,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -2516,7 +2516,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2687,7 +2687,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -2698,7 +2698,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -2875,7 +2875,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2886,7 +2886,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2897,7 +2897,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -3975,30 +3975,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E17" t="n">
-        <v>31543</v>
+        <v>453230</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>820692</v>
+        <v>5483351</v>
       </c>
       <c r="H17" t="n">
-        <v>1637750</v>
+        <v>8188106</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4012,30 +4012,30 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E18" t="n">
-        <v>273503</v>
+        <v>31543</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>1994005</v>
+        <v>820692</v>
       </c>
       <c r="H18" t="n">
-        <v>1917309</v>
+        <v>1637750</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -4049,30 +4049,30 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E19" t="n">
-        <v>453230</v>
+        <v>273503</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>5483351</v>
+        <v>1994005</v>
       </c>
       <c r="H19" t="n">
-        <v>8188106</v>
+        <v>1917309</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -4197,30 +4197,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H23" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4230,34 +4230,34 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>1615102</v>
+        <v>95791</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>4234674</v>
+        <v>2404119</v>
       </c>
       <c r="H24" t="n">
-        <v>6092784</v>
+        <v>5124417</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -4271,30 +4271,30 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E25" t="n">
-        <v>334016</v>
+        <v>1615102</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>2156629</v>
+        <v>4234674</v>
       </c>
       <c r="H25" t="n">
-        <v>2691725</v>
+        <v>6092784</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -4720,7 +4720,7 @@
         <v>0.4</v>
       </c>
       <c r="R2" t="n">
-        <v>9971</v>
+        <v>10250</v>
       </c>
       <c r="S2" t="n">
         <v>270274</v>
@@ -4791,7 +4791,7 @@
         <v>0.2</v>
       </c>
       <c r="R3" t="n">
-        <v>105685</v>
+        <v>109108</v>
       </c>
       <c r="S3" t="n">
         <v>1461471</v>
@@ -4858,7 +4858,7 @@
         <v>1.4</v>
       </c>
       <c r="R4" t="n">
-        <v>258869</v>
+        <v>267533</v>
       </c>
       <c r="S4" t="n">
         <v>670758</v>
@@ -4929,7 +4929,7 @@
         <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>269558</v>
+        <v>278598</v>
       </c>
       <c r="S5" t="n">
         <v>24105</v>
@@ -5000,7 +5000,7 @@
         <v>0.4</v>
       </c>
       <c r="R6" t="n">
-        <v>301918</v>
+        <v>312178</v>
       </c>
       <c r="S6" t="n">
         <v>166751</v>
@@ -5071,7 +5071,7 @@
         <v>0.2</v>
       </c>
       <c r="R7" t="n">
-        <v>510595</v>
+        <v>528537</v>
       </c>
       <c r="S7" t="n">
         <v>88386</v>
@@ -5142,7 +5142,7 @@
         <v>0.7</v>
       </c>
       <c r="R8" t="n">
-        <v>530348</v>
+        <v>549095</v>
       </c>
       <c r="S8" t="n">
         <v>617418</v>
@@ -5213,7 +5213,7 @@
         <v>0.6</v>
       </c>
       <c r="R9" t="n">
-        <v>719732</v>
+        <v>745361</v>
       </c>
       <c r="S9" t="n">
         <v>637992</v>
@@ -5284,7 +5284,7 @@
         <v>0.2</v>
       </c>
       <c r="R10" t="n">
-        <v>747829</v>
+        <v>774645</v>
       </c>
       <c r="S10" t="n">
         <v>1034411</v>
@@ -5355,7 +5355,7 @@
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>836186</v>
+        <v>866801</v>
       </c>
       <c r="S11" t="n">
         <v>3039834</v>
@@ -5426,7 +5426,7 @@
         <v>0.6</v>
       </c>
       <c r="R12" t="n">
-        <v>1050933</v>
+        <v>1089861</v>
       </c>
       <c r="S12" t="n">
         <v>4399137</v>
@@ -5493,7 +5493,7 @@
         <v>0.2</v>
       </c>
       <c r="R13" t="n">
-        <v>1258971</v>
+        <v>1306162</v>
       </c>
       <c r="S13" t="n">
         <v>878473</v>
@@ -5564,7 +5564,7 @@
         <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>1374667</v>
+        <v>1426049</v>
       </c>
       <c r="S14" t="n">
         <v>3046343</v>
@@ -5635,7 +5635,7 @@
         <v>1.1</v>
       </c>
       <c r="R15" t="n">
-        <v>1382146</v>
+        <v>1433794</v>
       </c>
       <c r="S15" t="n">
         <v>101935</v>
@@ -5706,7 +5706,7 @@
         <v>0.2</v>
       </c>
       <c r="R16" t="n">
-        <v>1402141</v>
+        <v>1454432</v>
       </c>
       <c r="S16" t="n">
         <v>3048395</v>
@@ -5723,37 +5723,37 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D17" t="n">
-        <v>75.7</v>
+        <v>71.7</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="G17" t="n">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="H17" t="n">
         <v>2</v>
       </c>
       <c r="I17" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="J17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K17" t="n">
         <v>2</v>
@@ -5765,69 +5765,69 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="O17" t="n">
-        <v>100.5</v>
+        <v>100.4</v>
       </c>
       <c r="P17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="Q17" t="n">
         <v>0.5</v>
       </c>
-      <c r="Q17" t="n">
-        <v>0</v>
-      </c>
       <c r="R17" t="n">
-        <v>1512514</v>
+        <v>1501110</v>
       </c>
       <c r="S17" t="n">
-        <v>1066412</v>
+        <v>3009015</v>
       </c>
       <c r="T17" t="n">
         <v>2</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>3xc, freehit</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D18" t="n">
-        <v>71</v>
+        <v>75.7</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="G18" t="n">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="H18" t="n">
         <v>2</v>
       </c>
       <c r="I18" t="n">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L18" t="n">
         <v>0</v>
@@ -5836,7 +5836,7 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="O18" t="n">
         <v>100.5</v>
@@ -5845,13 +5845,13 @@
         <v>0.5</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="R18" t="n">
-        <v>1563918</v>
+        <v>1569102</v>
       </c>
       <c r="S18" t="n">
-        <v>5881370</v>
+        <v>1066412</v>
       </c>
       <c r="T18" t="n">
         <v>2</v>
@@ -5865,19 +5865,19 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="C19" t="n">
         <v>284</v>
       </c>
       <c r="D19" t="n">
-        <v>71.7</v>
+        <v>71</v>
       </c>
       <c r="E19" t="n">
         <v>2</v>
@@ -5886,19 +5886,19 @@
         <v>77</v>
       </c>
       <c r="G19" t="n">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="H19" t="n">
         <v>2</v>
       </c>
       <c r="I19" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="J19" t="n">
         <v>1</v>
       </c>
       <c r="K19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
         <v>0</v>
@@ -5907,29 +5907,29 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="O19" t="n">
-        <v>100.4</v>
+        <v>100.5</v>
       </c>
       <c r="P19" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="R19" t="n">
-        <v>1580919</v>
+        <v>1622014</v>
       </c>
       <c r="S19" t="n">
-        <v>3009015</v>
+        <v>5881370</v>
       </c>
       <c r="T19" t="n">
         <v>2</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>3xc, freehit</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5990,7 @@
         <v>0.5</v>
       </c>
       <c r="R20" t="n">
-        <v>1650086</v>
+        <v>1711492</v>
       </c>
       <c r="S20" t="n">
         <v>5250200</v>
@@ -6061,7 +6061,7 @@
         <v>1</v>
       </c>
       <c r="R21" t="n">
-        <v>1867826</v>
+        <v>1936996</v>
       </c>
       <c r="S21" t="n">
         <v>4185865</v>
@@ -6132,7 +6132,7 @@
         <v>0.4</v>
       </c>
       <c r="R22" t="n">
-        <v>2260007</v>
+        <v>2343465</v>
       </c>
       <c r="S22" t="n">
         <v>2735246</v>
@@ -6149,37 +6149,37 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C23" t="n">
         <v>270</v>
       </c>
       <c r="D23" t="n">
-        <v>59</v>
+        <v>64.3</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
         <v>48</v>
       </c>
       <c r="G23" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="H23" t="n">
         <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K23" t="n">
         <v>2</v>
@@ -6191,63 +6191,59 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="O23" t="n">
-        <v>101.2</v>
+        <v>100.9</v>
       </c>
       <c r="P23" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="Q23" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="R23" t="n">
-        <v>2682180</v>
+        <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>1396363</v>
+        <v>453361</v>
       </c>
       <c r="T23" t="n">
         <v>2</v>
       </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D24" t="n">
-        <v>61.7</v>
+        <v>59</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="G24" t="n">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="H24" t="n">
         <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J24" t="n">
         <v>1</v>
@@ -6262,66 +6258,66 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="O24" t="n">
-        <v>100</v>
+        <v>101.2</v>
       </c>
       <c r="P24" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.2</v>
+        <v>1.5</v>
       </c>
       <c r="R24" t="n">
-        <v>2769665</v>
+        <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>1595922</v>
+        <v>1396363</v>
       </c>
       <c r="T24" t="n">
         <v>2</v>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>bboost, 3xc, wildcard</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D25" t="n">
-        <v>64.3</v>
+        <v>61.7</v>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G25" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="H25" t="n">
         <v>2</v>
       </c>
       <c r="I25" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="J25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K25" t="n">
         <v>2</v>
@@ -6333,27 +6329,31 @@
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="O25" t="n">
-        <v>100.9</v>
+        <v>100</v>
       </c>
       <c r="P25" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="R25" t="n">
-        <v>2949027</v>
+        <v>2868689</v>
       </c>
       <c r="S25" t="n">
-        <v>453361</v>
+        <v>1595922</v>
       </c>
       <c r="T25" t="n">
         <v>2</v>
       </c>
-      <c r="U25" t="inlineStr"/>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>bboost, 3xc, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6412,7 +6412,7 @@
         <v>0.1</v>
       </c>
       <c r="R26" t="n">
-        <v>2973583</v>
+        <v>3077476</v>
       </c>
       <c r="S26" t="n">
         <v>1948104</v>
@@ -6483,7 +6483,7 @@
         <v>1</v>
       </c>
       <c r="R27" t="n">
-        <v>3064196</v>
+        <v>3170793</v>
       </c>
       <c r="S27" t="n">
         <v>3395267</v>
@@ -6554,7 +6554,7 @@
         <v>0.7</v>
       </c>
       <c r="R28" t="n">
-        <v>3317256</v>
+        <v>3430081</v>
       </c>
       <c r="U28" t="inlineStr">
         <is>
@@ -6619,7 +6619,7 @@
         <v>0</v>
       </c>
       <c r="R29" t="n">
-        <v>4839833</v>
+        <v>4982912</v>
       </c>
       <c r="S29" t="n">
         <v>3963132</v>
@@ -6690,7 +6690,7 @@
         <v>1</v>
       </c>
       <c r="R30" t="n">
-        <v>6223274</v>
+        <v>6376870</v>
       </c>
       <c r="S30" t="n">
         <v>140252</v>
@@ -6761,7 +6761,7 @@
         <v>0.7</v>
       </c>
       <c r="R31" t="n">
-        <v>6606759</v>
+        <v>6761783</v>
       </c>
       <c r="U31" t="inlineStr">
         <is>
@@ -6826,7 +6826,7 @@
         <v>2.2</v>
       </c>
       <c r="R32" t="n">
-        <v>8850751</v>
+        <v>8951568</v>
       </c>
       <c r="S32" t="n">
         <v>216389</v>

</xml_diff>

<commit_message>
Update standings 2026-09-15 12:14 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1922,33 +1922,33 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C23" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25">
@@ -2505,7 +2505,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -2516,7 +2516,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2875,7 +2875,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2886,7 +2886,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -4197,30 +4197,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H23" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4234,30 +4234,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H24" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6149,37 +6149,37 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C23" t="n">
         <v>270</v>
       </c>
       <c r="D23" t="n">
-        <v>64.3</v>
+        <v>59</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F23" t="n">
         <v>48</v>
       </c>
       <c r="G23" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="H23" t="n">
         <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
         <v>2</v>
@@ -6191,62 +6191,66 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O23" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P23" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>453361</v>
+        <v>1396363</v>
       </c>
       <c r="T23" t="n">
         <v>2</v>
       </c>
-      <c r="U23" t="inlineStr"/>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C24" t="n">
         <v>270</v>
       </c>
       <c r="D24" t="n">
-        <v>59</v>
+        <v>64.3</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F24" t="n">
         <v>48</v>
       </c>
       <c r="G24" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="H24" t="n">
         <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K24" t="n">
         <v>2</v>
@@ -6258,31 +6262,27 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="O24" t="n">
-        <v>101.2</v>
+        <v>100.9</v>
       </c>
       <c r="P24" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="Q24" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>1396363</v>
+        <v>453361</v>
       </c>
       <c r="T24" t="n">
         <v>2</v>
       </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-15 14:12 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1558,7 +1558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1582,6 +1582,11 @@
           <t>GW3</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>GW4</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1598,6 +1603,9 @@
       <c r="D2" t="n">
         <v>63</v>
       </c>
+      <c r="E2" t="n">
+        <v>81</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1614,6 +1622,9 @@
       <c r="D3" t="n">
         <v>54</v>
       </c>
+      <c r="E3" t="n">
+        <v>116</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1630,6 +1641,9 @@
       <c r="D4" t="n">
         <v>43</v>
       </c>
+      <c r="E4" t="n">
+        <v>107</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1646,6 +1660,9 @@
       <c r="D5" t="n">
         <v>45</v>
       </c>
+      <c r="E5" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1662,6 +1679,9 @@
       <c r="D6" t="n">
         <v>51</v>
       </c>
+      <c r="E6" t="n">
+        <v>84</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1678,6 +1698,9 @@
       <c r="D7" t="n">
         <v>37</v>
       </c>
+      <c r="E7" t="n">
+        <v>91</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1694,6 +1717,9 @@
       <c r="D8" t="n">
         <v>60</v>
       </c>
+      <c r="E8" t="n">
+        <v>76</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1710,6 +1736,9 @@
       <c r="D9" t="n">
         <v>61</v>
       </c>
+      <c r="E9" t="n">
+        <v>62</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1726,6 +1755,9 @@
       <c r="D10" t="n">
         <v>40</v>
       </c>
+      <c r="E10" t="n">
+        <v>91</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1742,6 +1774,9 @@
       <c r="D11" t="n">
         <v>55</v>
       </c>
+      <c r="E11" t="n">
+        <v>71</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1758,6 +1793,9 @@
       <c r="D12" t="n">
         <v>49</v>
       </c>
+      <c r="E12" t="n">
+        <v>76</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1774,6 +1812,9 @@
       <c r="D13" t="n">
         <v>47</v>
       </c>
+      <c r="E13" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1790,6 +1831,9 @@
       <c r="D14" t="n">
         <v>45</v>
       </c>
+      <c r="E14" t="n">
+        <v>77</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1806,6 +1850,9 @@
       <c r="D15" t="n">
         <v>55</v>
       </c>
+      <c r="E15" t="n">
+        <v>69</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1822,6 +1869,9 @@
       <c r="D16" t="n">
         <v>60</v>
       </c>
+      <c r="E16" t="n">
+        <v>87</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1838,6 +1888,9 @@
       <c r="D17" t="n">
         <v>67</v>
       </c>
+      <c r="E17" t="n">
+        <v>71</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1854,6 +1907,9 @@
       <c r="D18" t="n">
         <v>54</v>
       </c>
+      <c r="E18" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1870,6 +1926,9 @@
       <c r="D19" t="n">
         <v>55</v>
       </c>
+      <c r="E19" t="n">
+        <v>71</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1886,6 +1945,9 @@
       <c r="D20" t="n">
         <v>52</v>
       </c>
+      <c r="E20" t="n">
+        <v>75</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1902,6 +1964,9 @@
       <c r="D21" t="n">
         <v>56</v>
       </c>
+      <c r="E21" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1918,37 +1983,46 @@
       <c r="D22" t="n">
         <v>50</v>
       </c>
+      <c r="E22" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C23" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D23" t="n">
-        <v>46</v>
+        <v>38</v>
+      </c>
+      <c r="E23" t="n">
+        <v>77</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D24" t="n">
-        <v>38</v>
+        <v>46</v>
+      </c>
+      <c r="E24" t="n">
+        <v>93</v>
       </c>
     </row>
     <row r="25">
@@ -1966,6 +2040,9 @@
       <c r="D25" t="n">
         <v>50</v>
       </c>
+      <c r="E25" t="n">
+        <v>84</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1982,6 +2059,9 @@
       <c r="D26" t="n">
         <v>46</v>
       </c>
+      <c r="E26" t="n">
+        <v>66</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1998,6 +2078,9 @@
       <c r="D27" t="n">
         <v>78</v>
       </c>
+      <c r="E27" t="n">
+        <v>69</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2014,6 +2097,9 @@
       <c r="D28" t="n">
         <v>47</v>
       </c>
+      <c r="E28" t="n">
+        <v>77</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2030,6 +2116,9 @@
       <c r="D29" t="n">
         <v>48</v>
       </c>
+      <c r="E29" t="n">
+        <v>69</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2046,6 +2135,9 @@
       <c r="D30" t="n">
         <v>37</v>
       </c>
+      <c r="E30" t="n">
+        <v>89</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2062,6 +2154,9 @@
       <c r="D31" t="n">
         <v>32</v>
       </c>
+      <c r="E31" t="n">
+        <v>69</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2077,6 +2172,9 @@
       </c>
       <c r="D32" t="n">
         <v>52</v>
+      </c>
+      <c r="E32" t="n">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -2159,14 +2257,14 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -2177,14 +2275,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Abhay Rawat</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -2225,88 +2323,84 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Abhay Rawat</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>68</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Abhay Rawat</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -2317,254 +2411,258 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>68</v>
-      </c>
-      <c r="C10" t="inlineStr"/>
+        <v>78</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>57</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
+        <v>77</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>57</v>
-      </c>
-      <c r="C18" t="inlineStr"/>
+        <v>72</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>57</v>
-      </c>
-      <c r="C19" t="inlineStr"/>
+        <v>72</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>53</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="C21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="C22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>48</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="C23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>48</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="C24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="C25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="C27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="C28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="C29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="C30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>36</v>
+        <v>57</v>
       </c>
       <c r="C31" t="inlineStr"/>
     </row>
@@ -2575,7 +2673,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="C32" t="inlineStr"/>
     </row>
@@ -2613,11 +2711,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Abhay Rawat</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -2628,66 +2726,78 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhay Rawat</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>2</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>2</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>2</v>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>2</v>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -2698,7 +2808,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -2709,7 +2819,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -2720,7 +2830,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -2731,140 +2841,128 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2875,7 +2973,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2886,7 +2984,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2897,7 +2995,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -2908,7 +3006,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2919,7 +3017,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2930,7 +3028,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2941,7 +3039,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Pranav Thomas</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -2952,22 +3050,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Pranav Thomas</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C32" t="inlineStr"/>
     </row>
@@ -3062,232 +3160,232 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Kayode</t>
+          <t>Schade</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>3.2</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Schade</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E4" t="n">
-        <v>4.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Bogle</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E5" t="n">
-        <v>4.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Davis</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>4.5</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Schade</t>
+          <t>Kayode</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E7" t="n">
-        <v>3.5</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Abhay Rawat</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Suzuki</t>
+          <t>White</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E8" t="n">
-        <v>1.1</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Abhay Rawat</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ballard</t>
+          <t>White</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E9" t="n">
-        <v>4.9</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Ballard</t>
+          <t>White</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E10" t="n">
-        <v>4.9</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Wissa</t>
+          <t>Schade</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E11" t="n">
-        <v>3.7</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Abhay Rawat</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Ballard</t>
+          <t>Suzuki</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>4.9</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ballard</t>
+          <t>Jacquet</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E13" t="n">
-        <v>4.9</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="14">
@@ -3298,59 +3396,59 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Ballard</t>
         </is>
       </c>
       <c r="C14" t="n">
         <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E14" t="n">
-        <v>6.8</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Ballard</t>
         </is>
       </c>
       <c r="C15" t="n">
         <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>6.8</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Wissa</t>
         </is>
       </c>
       <c r="C16" t="n">
         <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>6.8</v>
+        <v>3.7</v>
       </c>
     </row>
   </sheetData>
@@ -4197,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H23" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4234,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H24" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -4678,13 +4776,13 @@
         <v>344</v>
       </c>
       <c r="D2" t="n">
-        <v>87.7</v>
+        <v>86</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G2" t="n">
         <v>126</v>
@@ -4749,19 +4847,19 @@
         <v>325</v>
       </c>
       <c r="D3" t="n">
-        <v>69.7</v>
+        <v>81.2</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I3" t="n">
         <v>54</v>
@@ -4816,19 +4914,19 @@
         <v>315</v>
       </c>
       <c r="D4" t="n">
-        <v>69.3</v>
+        <v>78.8</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="G4" t="n">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I4" t="n">
         <v>43</v>
@@ -4861,10 +4959,10 @@
         <v>267533</v>
       </c>
       <c r="S4" t="n">
-        <v>670758</v>
+        <v>1229264</v>
       </c>
       <c r="T4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
@@ -4887,13 +4985,13 @@
         <v>314</v>
       </c>
       <c r="D5" t="n">
-        <v>74</v>
+        <v>78.5</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G5" t="n">
         <v>103</v>
@@ -4932,10 +5030,10 @@
         <v>278598</v>
       </c>
       <c r="S5" t="n">
-        <v>24105</v>
+        <v>266328</v>
       </c>
       <c r="T5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
@@ -4958,13 +5056,13 @@
         <v>313</v>
       </c>
       <c r="D6" t="n">
-        <v>76.3</v>
+        <v>78.2</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="G6" t="n">
         <v>106</v>
@@ -5029,13 +5127,13 @@
         <v>305</v>
       </c>
       <c r="D7" t="n">
-        <v>71.3</v>
+        <v>76.2</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G7" t="n">
         <v>104</v>
@@ -5074,10 +5172,10 @@
         <v>528537</v>
       </c>
       <c r="S7" t="n">
-        <v>88386</v>
+        <v>466127</v>
       </c>
       <c r="T7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
@@ -5100,13 +5198,13 @@
         <v>305</v>
       </c>
       <c r="D8" t="n">
-        <v>76.3</v>
+        <v>76.2</v>
       </c>
       <c r="E8" t="n">
         <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="G8" t="n">
         <v>105</v>
@@ -5171,13 +5269,13 @@
         <v>300</v>
       </c>
       <c r="D9" t="n">
-        <v>79.3</v>
+        <v>75</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="G9" t="n">
         <v>111</v>
@@ -5242,13 +5340,13 @@
         <v>299</v>
       </c>
       <c r="D10" t="n">
-        <v>69.3</v>
+        <v>74.8</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G10" t="n">
         <v>107</v>
@@ -5313,13 +5411,13 @@
         <v>297</v>
       </c>
       <c r="D11" t="n">
-        <v>75.3</v>
+        <v>74.2</v>
       </c>
       <c r="E11" t="n">
         <v>2</v>
       </c>
       <c r="F11" t="n">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G11" t="n">
         <v>118</v>
@@ -5384,13 +5482,13 @@
         <v>293</v>
       </c>
       <c r="D12" t="n">
-        <v>72.3</v>
+        <v>73.2</v>
       </c>
       <c r="E12" t="n">
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G12" t="n">
         <v>120</v>
@@ -5451,13 +5549,13 @@
         <v>289</v>
       </c>
       <c r="D13" t="n">
-        <v>73</v>
+        <v>72.2</v>
       </c>
       <c r="E13" t="n">
         <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G13" t="n">
         <v>109</v>
@@ -5522,13 +5620,13 @@
         <v>287</v>
       </c>
       <c r="D14" t="n">
-        <v>70</v>
+        <v>71.8</v>
       </c>
       <c r="E14" t="n">
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G14" t="n">
         <v>113</v>
@@ -5593,13 +5691,13 @@
         <v>287</v>
       </c>
       <c r="D15" t="n">
-        <v>72.7</v>
+        <v>71.8</v>
       </c>
       <c r="E15" t="n">
         <v>2</v>
       </c>
       <c r="F15" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="G15" t="n">
         <v>90</v>
@@ -5664,13 +5762,13 @@
         <v>287</v>
       </c>
       <c r="D16" t="n">
-        <v>66.7</v>
+        <v>71.8</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F16" t="n">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="G16" t="n">
         <v>97</v>
@@ -5735,13 +5833,13 @@
         <v>286</v>
       </c>
       <c r="D17" t="n">
-        <v>71.7</v>
+        <v>71.5</v>
       </c>
       <c r="E17" t="n">
         <v>2</v>
       </c>
       <c r="F17" t="n">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="G17" t="n">
         <v>101</v>
@@ -5806,13 +5904,13 @@
         <v>285</v>
       </c>
       <c r="D18" t="n">
-        <v>75.7</v>
+        <v>71.2</v>
       </c>
       <c r="E18" t="n">
         <v>3</v>
       </c>
       <c r="F18" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="G18" t="n">
         <v>111</v>
@@ -5883,7 +5981,7 @@
         <v>2</v>
       </c>
       <c r="F19" t="n">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="G19" t="n">
         <v>118</v>
@@ -5948,13 +6046,13 @@
         <v>283</v>
       </c>
       <c r="D20" t="n">
-        <v>69.3</v>
+        <v>70.8</v>
       </c>
       <c r="E20" t="n">
         <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G20" t="n">
         <v>114</v>
@@ -6019,13 +6117,13 @@
         <v>280</v>
       </c>
       <c r="D21" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E21" t="n">
         <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G21" t="n">
         <v>107</v>
@@ -6090,13 +6188,13 @@
         <v>275</v>
       </c>
       <c r="D22" t="n">
-        <v>61.7</v>
+        <v>68.8</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="G22" t="n">
         <v>93</v>
@@ -6149,108 +6247,104 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C23" t="n">
         <v>270</v>
       </c>
       <c r="D23" t="n">
-        <v>59</v>
+        <v>67.5</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="G23" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="H23" t="n">
         <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J23" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>51</v>
+      </c>
+      <c r="O23" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q23" t="n">
         <v>1</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>61</v>
-      </c>
-      <c r="O23" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P23" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>1396363</v>
+        <v>453361</v>
       </c>
       <c r="T23" t="n">
         <v>2</v>
       </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C24" t="n">
         <v>270</v>
       </c>
       <c r="D24" t="n">
-        <v>64.3</v>
+        <v>67.5</v>
       </c>
       <c r="E24" t="n">
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="G24" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
         <v>2</v>
@@ -6262,27 +6356,31 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O24" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P24" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T24" t="n">
-        <v>2</v>
-      </c>
-      <c r="U24" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6299,13 +6397,13 @@
         <v>269</v>
       </c>
       <c r="D25" t="n">
-        <v>61.7</v>
+        <v>67.2</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="G25" t="n">
         <v>89</v>
@@ -6370,13 +6468,13 @@
         <v>267</v>
       </c>
       <c r="D26" t="n">
-        <v>67</v>
+        <v>66.8</v>
       </c>
       <c r="E26" t="n">
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="G26" t="n">
         <v>102</v>
@@ -6441,13 +6539,13 @@
         <v>266</v>
       </c>
       <c r="D27" t="n">
-        <v>65.7</v>
+        <v>66.5</v>
       </c>
       <c r="E27" t="n">
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>57</v>
+        <v>81</v>
       </c>
       <c r="G27" t="n">
         <v>78</v>
@@ -6512,13 +6610,13 @@
         <v>263</v>
       </c>
       <c r="D28" t="n">
-        <v>62</v>
+        <v>65.8</v>
       </c>
       <c r="E28" t="n">
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="G28" t="n">
         <v>80</v>
@@ -6556,6 +6654,12 @@
       <c r="R28" t="n">
         <v>3430081</v>
       </c>
+      <c r="S28" t="n">
+        <v>614528</v>
+      </c>
+      <c r="T28" t="n">
+        <v>4</v>
+      </c>
       <c r="U28" t="inlineStr">
         <is>
           <t>wildcard</t>
@@ -6577,13 +6681,13 @@
         <v>247</v>
       </c>
       <c r="D29" t="n">
-        <v>59.3</v>
+        <v>61.8</v>
       </c>
       <c r="E29" t="n">
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G29" t="n">
         <v>101</v>
@@ -6648,19 +6752,19 @@
         <v>232</v>
       </c>
       <c r="D30" t="n">
-        <v>47.7</v>
+        <v>58</v>
       </c>
       <c r="E30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="G30" t="n">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="H30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I30" t="n">
         <v>37</v>
@@ -6693,10 +6797,10 @@
         <v>6376870</v>
       </c>
       <c r="S30" t="n">
-        <v>140252</v>
+        <v>1952243</v>
       </c>
       <c r="T30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U30" t="inlineStr">
         <is>
@@ -6719,13 +6823,13 @@
         <v>227</v>
       </c>
       <c r="D31" t="n">
-        <v>52.7</v>
+        <v>56.8</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>38</v>
+        <v>62</v>
       </c>
       <c r="G31" t="n">
         <v>73</v>
@@ -6763,6 +6867,12 @@
       <c r="R31" t="n">
         <v>6761783</v>
       </c>
+      <c r="S31" t="n">
+        <v>553038</v>
+      </c>
+      <c r="T31" t="n">
+        <v>4</v>
+      </c>
       <c r="U31" t="inlineStr">
         <is>
           <t>wildcard</t>
@@ -6784,19 +6894,19 @@
         <v>187</v>
       </c>
       <c r="D32" t="n">
-        <v>44</v>
+        <v>46.8</v>
       </c>
       <c r="E32" t="n">
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="G32" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I32" t="n">
         <v>35</v>

</xml_diff>

<commit_message>
Update standings 2026-09-15 16:11 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C23" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H23" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H24" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,19 +6265,19 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G23" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
         <v>2</v>
@@ -6289,37 +6289,41 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O23" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P23" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T23" t="n">
-        <v>2</v>
-      </c>
-      <c r="U23" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6332,55 +6336,51 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G24" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J24" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>51</v>
+      </c>
+      <c r="O24" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q24" t="n">
         <v>1</v>
-      </c>
-      <c r="K24" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>61</v>
-      </c>
-      <c r="O24" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P24" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T24" t="n">
-        <v>4</v>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-15 18:12 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C23" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D23" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H23" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H24" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,65 +6265,61 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G23" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J23" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>51</v>
+      </c>
+      <c r="O23" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q23" t="n">
         <v>1</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>61</v>
-      </c>
-      <c r="O23" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P23" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T23" t="n">
-        <v>4</v>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6336,19 +6332,19 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G24" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
         <v>2</v>
@@ -6360,27 +6356,31 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O24" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P24" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T24" t="n">
-        <v>2</v>
-      </c>
-      <c r="U24" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-15 20:11 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C23" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H23" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H24" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,19 +6265,19 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G23" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
         <v>2</v>
@@ -6289,37 +6289,41 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O23" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P23" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T23" t="n">
-        <v>2</v>
-      </c>
-      <c r="U23" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6332,55 +6336,51 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G24" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J24" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>51</v>
+      </c>
+      <c r="O24" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q24" t="n">
         <v>1</v>
-      </c>
-      <c r="K24" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>61</v>
-      </c>
-      <c r="O24" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P24" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T24" t="n">
-        <v>4</v>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-16 00:15 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C23" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D23" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H23" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H24" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,65 +6265,61 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G23" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J23" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>51</v>
+      </c>
+      <c r="O23" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q23" t="n">
         <v>1</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>61</v>
-      </c>
-      <c r="O23" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P23" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T23" t="n">
-        <v>4</v>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6336,19 +6332,19 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G24" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
         <v>2</v>
@@ -6360,27 +6356,31 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O24" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P24" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T24" t="n">
-        <v>2</v>
-      </c>
-      <c r="U24" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-16 04:11 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C23" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H23" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H24" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,19 +6265,19 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G23" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
         <v>2</v>
@@ -6289,37 +6289,41 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O23" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P23" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T23" t="n">
-        <v>2</v>
-      </c>
-      <c r="U23" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6332,55 +6336,51 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G24" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J24" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>51</v>
+      </c>
+      <c r="O24" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q24" t="n">
         <v>1</v>
-      </c>
-      <c r="K24" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>61</v>
-      </c>
-      <c r="O24" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P24" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T24" t="n">
-        <v>4</v>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-16 08:12 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C23" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D23" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H23" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H24" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,65 +6265,61 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G23" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J23" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>51</v>
+      </c>
+      <c r="O23" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q23" t="n">
         <v>1</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>61</v>
-      </c>
-      <c r="O23" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P23" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T23" t="n">
-        <v>4</v>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6336,19 +6332,19 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G24" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
         <v>2</v>
@@ -6360,27 +6356,31 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O24" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P24" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T24" t="n">
-        <v>2</v>
-      </c>
-      <c r="U24" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-16 12:15 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C23" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H23" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H24" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,19 +6265,19 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G23" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
         <v>2</v>
@@ -6289,37 +6289,41 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O23" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P23" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T23" t="n">
-        <v>2</v>
-      </c>
-      <c r="U23" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6332,55 +6336,51 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G24" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J24" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>51</v>
+      </c>
+      <c r="O24" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q24" t="n">
         <v>1</v>
-      </c>
-      <c r="K24" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>61</v>
-      </c>
-      <c r="O24" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P24" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T24" t="n">
-        <v>4</v>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-16 14:12 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C23" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D23" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H23" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H24" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,65 +6265,61 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G23" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J23" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>51</v>
+      </c>
+      <c r="O23" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q23" t="n">
         <v>1</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>61</v>
-      </c>
-      <c r="O23" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P23" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T23" t="n">
-        <v>4</v>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6336,19 +6332,19 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G24" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
         <v>2</v>
@@ -6360,27 +6356,31 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O24" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P24" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T24" t="n">
-        <v>2</v>
-      </c>
-      <c r="U24" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-16 16:12 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C23" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H23" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H24" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,19 +6265,19 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G23" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
         <v>2</v>
@@ -6289,37 +6289,41 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O23" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P23" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T23" t="n">
-        <v>2</v>
-      </c>
-      <c r="U23" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6332,55 +6336,51 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G24" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J24" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>51</v>
+      </c>
+      <c r="O24" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q24" t="n">
         <v>1</v>
-      </c>
-      <c r="K24" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>61</v>
-      </c>
-      <c r="O24" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P24" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T24" t="n">
-        <v>4</v>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-16 16:34 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C23" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D23" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H23" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H24" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,65 +6265,61 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G23" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J23" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>51</v>
+      </c>
+      <c r="O23" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q23" t="n">
         <v>1</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>61</v>
-      </c>
-      <c r="O23" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P23" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T23" t="n">
-        <v>4</v>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6336,19 +6332,19 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G24" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
         <v>2</v>
@@ -6360,27 +6356,31 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O24" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P24" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T24" t="n">
-        <v>2</v>
-      </c>
-      <c r="U24" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-16 16:55 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C23" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H23" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H24" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,19 +6265,19 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G23" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
         <v>2</v>
@@ -6289,37 +6289,41 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O23" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P23" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T23" t="n">
-        <v>2</v>
-      </c>
-      <c r="U23" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6332,55 +6336,51 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G24" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J24" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>51</v>
+      </c>
+      <c r="O24" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q24" t="n">
         <v>1</v>
-      </c>
-      <c r="K24" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>61</v>
-      </c>
-      <c r="O24" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P24" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T24" t="n">
-        <v>4</v>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-16 22:10 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C23" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D23" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H23" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H24" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,65 +6265,61 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G23" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J23" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>51</v>
+      </c>
+      <c r="O23" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q23" t="n">
         <v>1</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>61</v>
-      </c>
-      <c r="O23" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P23" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T23" t="n">
-        <v>4</v>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6336,19 +6332,19 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G24" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
         <v>2</v>
@@ -6360,27 +6356,31 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O24" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P24" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T24" t="n">
-        <v>2</v>
-      </c>
-      <c r="U24" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-17 00:14 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C23" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H23" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H24" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,19 +6265,19 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G23" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
         <v>2</v>
@@ -6289,37 +6289,41 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O23" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P23" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T23" t="n">
-        <v>2</v>
-      </c>
-      <c r="U23" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6332,55 +6336,51 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G24" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J24" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>51</v>
+      </c>
+      <c r="O24" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q24" t="n">
         <v>1</v>
-      </c>
-      <c r="K24" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>61</v>
-      </c>
-      <c r="O24" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P24" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T24" t="n">
-        <v>4</v>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-17 02:11 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C23" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D23" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H23" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H24" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,65 +6265,61 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G23" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J23" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>51</v>
+      </c>
+      <c r="O23" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q23" t="n">
         <v>1</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>61</v>
-      </c>
-      <c r="O23" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P23" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T23" t="n">
-        <v>4</v>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6336,19 +6332,19 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G24" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
         <v>2</v>
@@ -6360,27 +6356,31 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O24" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P24" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T24" t="n">
-        <v>2</v>
-      </c>
-      <c r="U24" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-17 04:11 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C23" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H23" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H24" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,19 +6265,19 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G23" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
         <v>2</v>
@@ -6289,37 +6289,41 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O23" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P23" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T23" t="n">
-        <v>2</v>
-      </c>
-      <c r="U23" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6332,55 +6336,51 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G24" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J24" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>51</v>
+      </c>
+      <c r="O24" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q24" t="n">
         <v>1</v>
-      </c>
-      <c r="K24" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>61</v>
-      </c>
-      <c r="O24" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P24" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T24" t="n">
-        <v>4</v>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-17 06:15 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C23" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D23" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H23" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H24" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,65 +6265,61 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G23" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J23" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>51</v>
+      </c>
+      <c r="O23" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q23" t="n">
         <v>1</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>61</v>
-      </c>
-      <c r="O23" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P23" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T23" t="n">
-        <v>4</v>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6336,19 +6332,19 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G24" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
         <v>2</v>
@@ -6360,27 +6356,31 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O24" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P24" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T24" t="n">
-        <v>2</v>
-      </c>
-      <c r="U24" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-17 10:11 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C23" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H23" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H24" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,19 +6265,19 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G23" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
         <v>2</v>
@@ -6289,37 +6289,41 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O23" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P23" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T23" t="n">
-        <v>2</v>
-      </c>
-      <c r="U23" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6332,55 +6336,51 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G24" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J24" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>51</v>
+      </c>
+      <c r="O24" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q24" t="n">
         <v>1</v>
-      </c>
-      <c r="K24" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>61</v>
-      </c>
-      <c r="O24" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P24" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T24" t="n">
-        <v>4</v>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-17 18:13 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C23" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D23" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H23" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H24" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,65 +6265,61 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G23" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J23" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>51</v>
+      </c>
+      <c r="O23" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q23" t="n">
         <v>1</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>61</v>
-      </c>
-      <c r="O23" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P23" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T23" t="n">
-        <v>4</v>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6336,19 +6332,19 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G24" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
         <v>2</v>
@@ -6360,27 +6356,31 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O24" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P24" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T24" t="n">
-        <v>2</v>
-      </c>
-      <c r="U24" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-17 22:11 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C23" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H23" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H24" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,19 +6265,19 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G23" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
         <v>2</v>
@@ -6289,37 +6289,41 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O23" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P23" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T23" t="n">
-        <v>2</v>
-      </c>
-      <c r="U23" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6332,55 +6336,51 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G24" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J24" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>51</v>
+      </c>
+      <c r="O24" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q24" t="n">
         <v>1</v>
-      </c>
-      <c r="K24" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>61</v>
-      </c>
-      <c r="O24" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P24" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T24" t="n">
-        <v>4</v>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-18 00:15 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C23" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D23" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H23" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H24" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,65 +6265,61 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G23" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J23" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>51</v>
+      </c>
+      <c r="O23" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q23" t="n">
         <v>1</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>61</v>
-      </c>
-      <c r="O23" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P23" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T23" t="n">
-        <v>4</v>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6336,19 +6332,19 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G24" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
         <v>2</v>
@@ -6360,27 +6356,31 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O24" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P24" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T24" t="n">
-        <v>2</v>
-      </c>
-      <c r="U24" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-18 02:11 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C23" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H23" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H24" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,19 +6265,19 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G23" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
         <v>2</v>
@@ -6289,37 +6289,41 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O23" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P23" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T23" t="n">
-        <v>2</v>
-      </c>
-      <c r="U23" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6332,55 +6336,51 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G24" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J24" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>51</v>
+      </c>
+      <c r="O24" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q24" t="n">
         <v>1</v>
-      </c>
-      <c r="K24" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>61</v>
-      </c>
-      <c r="O24" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P24" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T24" t="n">
-        <v>4</v>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-18 06:14 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C23" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D23" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H23" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H24" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,65 +6265,61 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G23" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J23" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>51</v>
+      </c>
+      <c r="O23" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q23" t="n">
         <v>1</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>61</v>
-      </c>
-      <c r="O23" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P23" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T23" t="n">
-        <v>4</v>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6336,19 +6332,19 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G24" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
         <v>2</v>
@@ -6360,27 +6356,31 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O24" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P24" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T24" t="n">
-        <v>2</v>
-      </c>
-      <c r="U24" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-18 08:12 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C23" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H23" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H24" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,19 +6265,19 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G23" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
         <v>2</v>
@@ -6289,37 +6289,41 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O23" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P23" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T23" t="n">
-        <v>2</v>
-      </c>
-      <c r="U23" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6332,55 +6336,51 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G24" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J24" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>51</v>
+      </c>
+      <c r="O24" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q24" t="n">
         <v>1</v>
-      </c>
-      <c r="K24" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>61</v>
-      </c>
-      <c r="O24" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P24" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T24" t="n">
-        <v>4</v>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-18 12:14 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1990,39 +1990,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C23" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D23" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E23" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25">
@@ -2896,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H23" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H24" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -6247,12 +6247,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,65 +6265,61 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G23" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J23" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>51</v>
+      </c>
+      <c r="O23" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q23" t="n">
         <v>1</v>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="n">
-        <v>61</v>
-      </c>
-      <c r="O23" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P23" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>1.5</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T23" t="n">
-        <v>4</v>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6336,19 +6332,19 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G24" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
         <v>2</v>
@@ -6360,27 +6356,31 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O24" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P24" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T24" t="n">
-        <v>2</v>
-      </c>
-      <c r="U24" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-09-18 18:13 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -535,7 +535,7 @@
         <v>111</v>
       </c>
       <c r="E4" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>315</v>
@@ -823,7 +823,7 @@
         <v>87</v>
       </c>
       <c r="E16" t="n">
-        <v>-4</v>
+        <v>-8</v>
       </c>
       <c r="F16" t="n">
         <v>287</v>
@@ -979,16 +979,16 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -1003,16 +1003,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1063,7 +1063,7 @@
         <v>66</v>
       </c>
       <c r="E26" t="n">
-        <v>-4</v>
+        <v>-8</v>
       </c>
       <c r="F26" t="n">
         <v>267</v>
@@ -1594,18 +1594,10 @@
           <t>Abhay Rawat</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>74</v>
-      </c>
-      <c r="C2" t="n">
-        <v>126</v>
-      </c>
-      <c r="D2" t="n">
-        <v>63</v>
-      </c>
-      <c r="E2" t="n">
-        <v>81</v>
-      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1613,18 +1605,10 @@
           <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>55</v>
-      </c>
-      <c r="C3" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" t="n">
-        <v>54</v>
-      </c>
-      <c r="E3" t="n">
-        <v>116</v>
-      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1632,18 +1616,10 @@
           <t>Anish Joshi</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>62</v>
-      </c>
-      <c r="C4" t="n">
-        <v>103</v>
-      </c>
-      <c r="D4" t="n">
-        <v>43</v>
-      </c>
-      <c r="E4" t="n">
-        <v>107</v>
-      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1651,18 +1627,10 @@
           <t>Aquib Razack</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>74</v>
-      </c>
-      <c r="C5" t="n">
-        <v>103</v>
-      </c>
-      <c r="D5" t="n">
-        <v>45</v>
-      </c>
-      <c r="E5" t="n">
-        <v>92</v>
-      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1990,39 +1958,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C23" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E23" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25">
@@ -2239,11 +2207,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Abhay Rawat</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>126</v>
+        <v>90</v>
       </c>
       <c r="D3" t="n">
         <v>2</v>
@@ -2711,93 +2679,77 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>3</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C3" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Abhay Rawat</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>2</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>2</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>2</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>2</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -2808,7 +2760,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -2819,7 +2771,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -2830,7 +2782,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -2841,7 +2793,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2852,7 +2804,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2863,7 +2815,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2874,7 +2826,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2885,7 +2837,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2896,7 +2848,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2859,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -2918,51 +2870,51 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2973,7 +2925,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2984,7 +2936,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2995,7 +2947,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -3006,7 +2958,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -3017,7 +2969,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Pranav Thomas</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -3028,46 +2980,62 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Abhay Rawat</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Pranav Thomas</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3527,26 +3495,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
-      </c>
-      <c r="E2" t="n">
-        <v>38561</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2018/19</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>858178</v>
-      </c>
-      <c r="H2" t="n">
-        <v>726260</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2025/26</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -3564,26 +3513,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E3" t="n">
-        <v>545267</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2025/26</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>604934</v>
-      </c>
-      <c r="H3" t="n">
-        <v>545267</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2025/26</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -3601,26 +3531,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>15</v>
-      </c>
-      <c r="E4" t="n">
-        <v>281617</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2019/20</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>1051323</v>
-      </c>
-      <c r="H4" t="n">
-        <v>1076546</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2025/26</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -3638,26 +3549,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>14</v>
-      </c>
-      <c r="E5" t="n">
-        <v>71857</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2020/21</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>1929309</v>
-      </c>
-      <c r="H5" t="n">
-        <v>297407</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2025/26</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -4295,30 +4187,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H23" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4224,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H24" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -4775,29 +4667,14 @@
       <c r="C2" t="n">
         <v>344</v>
       </c>
-      <c r="D2" t="n">
-        <v>86</v>
-      </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
         <v>78</v>
       </c>
-      <c r="G2" t="n">
-        <v>126</v>
-      </c>
-      <c r="H2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I2" t="n">
-        <v>63</v>
-      </c>
-      <c r="J2" t="n">
-        <v>3</v>
-      </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -4806,31 +4683,9 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>48</v>
-      </c>
-      <c r="O2" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P2" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="R2" t="n">
-        <v>10250</v>
-      </c>
-      <c r="S2" t="n">
-        <v>270274</v>
-      </c>
-      <c r="T2" t="n">
-        <v>2</v>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>bboost, freehit, wildcard</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4846,29 +4701,14 @@
       <c r="C3" t="n">
         <v>325</v>
       </c>
-      <c r="D3" t="n">
-        <v>81.2</v>
-      </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
         <v>72</v>
       </c>
-      <c r="G3" t="n">
-        <v>116</v>
-      </c>
-      <c r="H3" t="n">
-        <v>4</v>
-      </c>
-      <c r="I3" t="n">
-        <v>54</v>
-      </c>
-      <c r="J3" t="n">
-        <v>3</v>
-      </c>
       <c r="K3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -4877,25 +4717,7 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>39</v>
-      </c>
-      <c r="O3" t="n">
-        <v>100.2</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="R3" t="n">
-        <v>109108</v>
-      </c>
-      <c r="S3" t="n">
-        <v>1461471</v>
-      </c>
-      <c r="T3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
@@ -4913,62 +4735,25 @@
       <c r="C4" t="n">
         <v>315</v>
       </c>
-      <c r="D4" t="n">
-        <v>78.8</v>
-      </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>72</v>
       </c>
-      <c r="G4" t="n">
-        <v>107</v>
-      </c>
-      <c r="H4" t="n">
-        <v>4</v>
-      </c>
-      <c r="I4" t="n">
-        <v>43</v>
-      </c>
-      <c r="J4" t="n">
-        <v>3</v>
-      </c>
       <c r="K4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>47</v>
-      </c>
-      <c r="O4" t="n">
-        <v>101</v>
-      </c>
-      <c r="P4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="R4" t="n">
-        <v>267533</v>
-      </c>
-      <c r="S4" t="n">
-        <v>1229264</v>
-      </c>
-      <c r="T4" t="n">
-        <v>4</v>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>bboost, wildcard</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4984,29 +4769,14 @@
       <c r="C5" t="n">
         <v>314</v>
       </c>
-      <c r="D5" t="n">
-        <v>78.5</v>
-      </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
         <v>78</v>
       </c>
-      <c r="G5" t="n">
-        <v>103</v>
-      </c>
-      <c r="H5" t="n">
-        <v>2</v>
-      </c>
-      <c r="I5" t="n">
-        <v>45</v>
-      </c>
-      <c r="J5" t="n">
-        <v>3</v>
-      </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -5015,31 +4785,9 @@
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>59</v>
-      </c>
-      <c r="O5" t="n">
-        <v>101.1</v>
-      </c>
-      <c r="P5" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" t="n">
-        <v>278598</v>
-      </c>
-      <c r="S5" t="n">
-        <v>266328</v>
-      </c>
-      <c r="T5" t="n">
-        <v>4</v>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>bboost, wildcard</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5077,7 +4825,7 @@
         <v>3</v>
       </c>
       <c r="K6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
@@ -5089,13 +4837,13 @@
         <v>35</v>
       </c>
       <c r="O6" t="n">
-        <v>100.4</v>
+        <v>100.5</v>
       </c>
       <c r="P6" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.4</v>
+        <v>2.5</v>
       </c>
       <c r="R6" t="n">
         <v>312178</v>
@@ -5148,7 +4896,7 @@
         <v>3</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -5160,10 +4908,10 @@
         <v>21</v>
       </c>
       <c r="O7" t="n">
-        <v>101.4</v>
+        <v>101.8</v>
       </c>
       <c r="P7" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="Q7" t="n">
         <v>0.2</v>
@@ -5201,7 +4949,7 @@
         <v>76.2</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F8" t="n">
         <v>67</v>
@@ -5219,7 +4967,7 @@
         <v>3</v>
       </c>
       <c r="K8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -5231,13 +4979,13 @@
         <v>57</v>
       </c>
       <c r="O8" t="n">
-        <v>100.7</v>
+        <v>101</v>
       </c>
       <c r="P8" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="R8" t="n">
         <v>549095</v>
@@ -5302,10 +5050,10 @@
         <v>48</v>
       </c>
       <c r="O9" t="n">
-        <v>100.3</v>
+        <v>100.4</v>
       </c>
       <c r="P9" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="Q9" t="n">
         <v>0.6</v>
@@ -5373,10 +5121,10 @@
         <v>24</v>
       </c>
       <c r="O10" t="n">
-        <v>101</v>
+        <v>101.3</v>
       </c>
       <c r="P10" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="Q10" t="n">
         <v>0.2</v>
@@ -5414,7 +5162,7 @@
         <v>74.2</v>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
         <v>87</v>
@@ -5444,10 +5192,10 @@
         <v>45</v>
       </c>
       <c r="O11" t="n">
-        <v>100.6</v>
+        <v>101</v>
       </c>
       <c r="P11" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="Q11" t="n">
         <v>0</v>
@@ -5485,7 +5233,7 @@
         <v>73.2</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
         <v>78</v>
@@ -5503,7 +5251,7 @@
         <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -5515,13 +5263,13 @@
         <v>56</v>
       </c>
       <c r="O12" t="n">
-        <v>100.2</v>
+        <v>100.3</v>
       </c>
       <c r="P12" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.6</v>
+        <v>2.7</v>
       </c>
       <c r="R12" t="n">
         <v>1089861</v>
@@ -5582,10 +5330,10 @@
         <v>63</v>
       </c>
       <c r="O13" t="n">
-        <v>101</v>
+        <v>101.4</v>
       </c>
       <c r="P13" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="Q13" t="n">
         <v>0.2</v>
@@ -5623,7 +5371,7 @@
         <v>71.8</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
         <v>78</v>
@@ -5641,7 +5389,7 @@
         <v>3</v>
       </c>
       <c r="K14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -5653,13 +5401,13 @@
         <v>40</v>
       </c>
       <c r="O14" t="n">
-        <v>100.4</v>
+        <v>100.8</v>
       </c>
       <c r="P14" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="Q14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R14" t="n">
         <v>1426049</v>
@@ -5724,10 +5472,10 @@
         <v>35</v>
       </c>
       <c r="O15" t="n">
-        <v>101.1</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
         <v>1.1</v>
@@ -5783,25 +5531,25 @@
         <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M16" t="n">
-        <v>-4</v>
+        <v>-8</v>
       </c>
       <c r="N16" t="n">
         <v>33</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>100.6</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="R16" t="n">
         <v>1454432</v>
@@ -5872,7 +5620,7 @@
         <v>0.4</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.5</v>
+        <v>1.3</v>
       </c>
       <c r="R17" t="n">
         <v>1501110</v>
@@ -5885,7 +5633,7 @@
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>3xc, freehit</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
@@ -5937,10 +5685,10 @@
         <v>58</v>
       </c>
       <c r="O18" t="n">
-        <v>100.5</v>
+        <v>100.9</v>
       </c>
       <c r="P18" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="Q18" t="n">
         <v>0</v>
@@ -6008,10 +5756,10 @@
         <v>50</v>
       </c>
       <c r="O19" t="n">
-        <v>100.5</v>
+        <v>100.9</v>
       </c>
       <c r="P19" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="Q19" t="n">
         <v>0.6</v>
@@ -6079,10 +5827,10 @@
         <v>36</v>
       </c>
       <c r="O20" t="n">
-        <v>100.5</v>
+        <v>101.1</v>
       </c>
       <c r="P20" t="n">
-        <v>0.5</v>
+        <v>1.1</v>
       </c>
       <c r="Q20" t="n">
         <v>0.5</v>
@@ -6156,7 +5904,7 @@
         <v>0.6</v>
       </c>
       <c r="Q21" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="R21" t="n">
         <v>1936996</v>
@@ -6169,7 +5917,7 @@
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>3xc, freehit</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
@@ -6221,10 +5969,10 @@
         <v>33</v>
       </c>
       <c r="O22" t="n">
-        <v>101.3</v>
+        <v>101.7</v>
       </c>
       <c r="P22" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="Q22" t="n">
         <v>0.4</v>
@@ -6247,12 +5995,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -6265,23 +6013,23 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G23" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I23" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J23" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" t="n">
         <v>3</v>
       </c>
-      <c r="K23" t="n">
-        <v>2</v>
-      </c>
       <c r="L23" t="n">
         <v>0</v>
       </c>
@@ -6289,37 +6037,41 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O23" t="n">
-        <v>100.9</v>
+        <v>101.9</v>
       </c>
       <c r="P23" t="n">
-        <v>0.9</v>
+        <v>1.9</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="R23" t="n">
         <v>2778338</v>
       </c>
       <c r="S23" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T23" t="n">
-        <v>2</v>
-      </c>
-      <c r="U23" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -6329,25 +6081,25 @@
         <v>67.5</v>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G24" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
@@ -6356,31 +6108,27 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="O24" t="n">
-        <v>101.2</v>
+        <v>101.1</v>
       </c>
       <c r="P24" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="Q24" t="n">
-        <v>1.5</v>
+        <v>1.1</v>
       </c>
       <c r="R24" t="n">
         <v>2778338</v>
       </c>
       <c r="S24" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T24" t="n">
-        <v>4</v>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6418,7 +6166,7 @@
         <v>1</v>
       </c>
       <c r="K25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
@@ -6430,13 +6178,13 @@
         <v>58</v>
       </c>
       <c r="O25" t="n">
-        <v>100</v>
+        <v>100.2</v>
       </c>
       <c r="P25" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.2</v>
+        <v>1.8</v>
       </c>
       <c r="R25" t="n">
         <v>2868689</v>
@@ -6471,7 +6219,7 @@
         <v>66.8</v>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F26" t="n">
         <v>58</v>
@@ -6489,22 +6237,22 @@
         <v>3</v>
       </c>
       <c r="K26" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M26" t="n">
-        <v>-4</v>
+        <v>-8</v>
       </c>
       <c r="N26" t="n">
         <v>55</v>
       </c>
       <c r="O26" t="n">
-        <v>100.7</v>
+        <v>101.1</v>
       </c>
       <c r="P26" t="n">
-        <v>0.7</v>
+        <v>1.1</v>
       </c>
       <c r="Q26" t="n">
         <v>0.1</v>
@@ -6560,7 +6308,7 @@
         <v>1</v>
       </c>
       <c r="K27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
@@ -6572,13 +6320,13 @@
         <v>33</v>
       </c>
       <c r="O27" t="n">
-        <v>100.6</v>
+        <v>100.8</v>
       </c>
       <c r="P27" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="Q27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R27" t="n">
         <v>3170793</v>
@@ -6613,7 +6361,7 @@
         <v>65.8</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F28" t="n">
         <v>58</v>
@@ -6643,10 +6391,10 @@
         <v>60</v>
       </c>
       <c r="O28" t="n">
-        <v>101.2</v>
+        <v>101.7</v>
       </c>
       <c r="P28" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="Q28" t="n">
         <v>0.7</v>
@@ -6714,10 +6462,10 @@
         <v>62</v>
       </c>
       <c r="O29" t="n">
-        <v>100.2</v>
+        <v>100.7</v>
       </c>
       <c r="P29" t="n">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="Q29" t="n">
         <v>0</v>
@@ -6773,7 +6521,7 @@
         <v>1</v>
       </c>
       <c r="K30" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L30" t="n">
         <v>2</v>
@@ -6785,10 +6533,10 @@
         <v>34</v>
       </c>
       <c r="O30" t="n">
-        <v>100.9</v>
+        <v>101.4</v>
       </c>
       <c r="P30" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="Q30" t="n">
         <v>1</v>
@@ -6826,7 +6574,7 @@
         <v>56.8</v>
       </c>
       <c r="E31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F31" t="n">
         <v>62</v>
@@ -6844,7 +6592,7 @@
         <v>3</v>
       </c>
       <c r="K31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L31" t="n">
         <v>1</v>
@@ -6856,13 +6604,13 @@
         <v>58</v>
       </c>
       <c r="O31" t="n">
-        <v>100.4</v>
+        <v>100.7</v>
       </c>
       <c r="P31" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="Q31" t="n">
-        <v>0.7</v>
+        <v>1.2</v>
       </c>
       <c r="R31" t="n">
         <v>6761783</v>
@@ -6927,10 +6675,10 @@
         <v>9</v>
       </c>
       <c r="O32" t="n">
-        <v>99.40000000000001</v>
+        <v>99.2</v>
       </c>
       <c r="P32" t="n">
-        <v>-0.6</v>
+        <v>-0.8</v>
       </c>
       <c r="Q32" t="n">
         <v>2.2</v>

</xml_diff>

<commit_message>
Update standings 2026-09-18 22:20 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -484,13 +484,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>81</v>
+        <v>4</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3">
@@ -508,13 +508,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>116</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="4">
@@ -523,22 +523,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>111</v>
+        <v>9</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>315</v>
+        <v>322</v>
       </c>
     </row>
     <row r="5">
@@ -547,22 +547,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>92</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F5" t="n">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="6">
@@ -571,22 +571,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>84</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>313</v>
+        <v>316</v>
       </c>
     </row>
     <row r="7">
@@ -595,22 +595,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>91</v>
+        <v>11</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>305</v>
+        <v>310</v>
       </c>
     </row>
     <row r="8">
@@ -619,22 +619,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>76</v>
+        <v>2</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="9">
@@ -643,22 +643,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>300</v>
+        <v>307</v>
       </c>
     </row>
     <row r="10">
@@ -667,22 +667,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>91</v>
+        <v>4</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>299</v>
+        <v>304</v>
       </c>
     </row>
     <row r="11">
@@ -700,13 +700,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>71</v>
+        <v>4</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>297</v>
+        <v>301</v>
       </c>
     </row>
     <row r="12">
@@ -715,46 +715,46 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>76</v>
+        <v>11</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>293</v>
+        <v>298</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>289</v>
+        <v>298</v>
       </c>
     </row>
     <row r="14">
@@ -763,22 +763,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>77</v>
+        <v>4</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>287</v>
+        <v>297</v>
       </c>
     </row>
     <row r="15">
@@ -787,22 +787,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>287</v>
+        <v>293</v>
       </c>
     </row>
     <row r="16">
@@ -811,22 +811,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>87</v>
+        <v>4</v>
       </c>
       <c r="E16" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="17">
@@ -835,22 +835,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>71</v>
+        <v>4</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="18">
@@ -859,22 +859,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>58</v>
+        <v>2</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>285</v>
+        <v>288</v>
       </c>
     </row>
     <row r="19">
@@ -883,22 +883,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>71</v>
+        <v>2</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="20">
@@ -907,22 +907,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>75</v>
+        <v>2</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="F20" t="n">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="21">
@@ -940,13 +940,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>73</v>
+        <v>4</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>280</v>
+        <v>284</v>
       </c>
     </row>
     <row r="22">
@@ -955,22 +955,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>90</v>
+        <v>8</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>275</v>
+        <v>278</v>
       </c>
     </row>
     <row r="23">
@@ -979,46 +979,46 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>2</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>270</v>
+        <v>277</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>77</v>
+        <v>4</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>270</v>
+        <v>274</v>
       </c>
     </row>
     <row r="25">
@@ -1036,13 +1036,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>84</v>
+        <v>2</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="26">
@@ -1051,22 +1051,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="27">
@@ -1075,22 +1075,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>69</v>
+        <v>2</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="28">
@@ -1099,22 +1099,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>77</v>
+        <v>2</v>
       </c>
       <c r="E28" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="F28" t="n">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="29">
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>69</v>
+        <v>2</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="30">
@@ -1156,13 +1156,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>89</v>
+        <v>2</v>
       </c>
       <c r="E30" t="n">
         <v>-8</v>
       </c>
       <c r="F30" t="n">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="31">
@@ -1180,13 +1180,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>69</v>
+        <v>6</v>
       </c>
       <c r="E31" t="n">
         <v>-4</v>
       </c>
       <c r="F31" t="n">
-        <v>227</v>
+        <v>233</v>
       </c>
     </row>
     <row r="32">
@@ -1204,7 +1204,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
@@ -1594,10 +1594,18 @@
           <t>Abhay Rawat</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="B2" t="n">
+        <v>74</v>
+      </c>
+      <c r="C2" t="n">
+        <v>126</v>
+      </c>
+      <c r="D2" t="n">
+        <v>63</v>
+      </c>
+      <c r="E2" t="n">
+        <v>81</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1605,66 +1613,90 @@
           <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+      <c r="B3" t="n">
+        <v>55</v>
+      </c>
+      <c r="C3" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3" t="n">
+        <v>54</v>
+      </c>
+      <c r="E3" t="n">
+        <v>116</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+          <t>Abhinav Premsekhar</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>72</v>
+      </c>
+      <c r="C4" t="n">
+        <v>106</v>
+      </c>
+      <c r="D4" t="n">
+        <v>51</v>
+      </c>
+      <c r="E4" t="n">
+        <v>84</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+          <t>Anish Joshi</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>62</v>
+      </c>
+      <c r="C5" t="n">
+        <v>103</v>
+      </c>
+      <c r="D5" t="n">
+        <v>43</v>
+      </c>
+      <c r="E5" t="n">
+        <v>107</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C6" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D6" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="E6" t="n">
-        <v>84</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="C7" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D7" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E7" t="n">
         <v>91</v>
@@ -1673,58 +1705,58 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="C8" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D8" t="n">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="E8" t="n">
-        <v>76</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C9" t="n">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D9" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E9" t="n">
-        <v>62</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B10" t="n">
+        <v>66</v>
+      </c>
+      <c r="C10" t="n">
+        <v>111</v>
+      </c>
+      <c r="D10" t="n">
         <v>61</v>
       </c>
-      <c r="C10" t="n">
-        <v>107</v>
-      </c>
-      <c r="D10" t="n">
-        <v>40</v>
-      </c>
       <c r="E10" t="n">
-        <v>91</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11">
@@ -1749,112 +1781,112 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>48</v>
+        <v>73</v>
       </c>
       <c r="C12" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="D12" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E12" t="n">
-        <v>76</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="C13" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="D13" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E13" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C14" t="n">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="D14" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E14" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="C16" t="n">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="D16" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="E16" t="n">
-        <v>87</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C17" t="n">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="D17" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E17" t="n">
         <v>71</v>
@@ -1863,58 +1895,58 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="C18" t="n">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="D18" t="n">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="E18" t="n">
-        <v>58</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C19" t="n">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D19" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E19" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C20" t="n">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="D20" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="E20" t="n">
-        <v>75</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21">
@@ -1939,58 +1971,58 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="C22" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D22" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="E22" t="n">
-        <v>90</v>
+        <v>77</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C23" t="n">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="D23" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E23" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E24" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25">
@@ -2015,58 +2047,58 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="C26" t="n">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="D26" t="n">
-        <v>46</v>
+        <v>78</v>
       </c>
       <c r="E26" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="C27" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D27" t="n">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="E27" t="n">
-        <v>69</v>
+        <v>77</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C28" t="n">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="D28" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E28" t="n">
-        <v>77</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29">
@@ -2207,11 +2239,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Abhay Rawat</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>90</v>
+        <v>126</v>
       </c>
       <c r="D3" t="n">
         <v>2</v>
@@ -2394,7 +2426,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -2405,7 +2437,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2416,7 +2448,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2427,7 +2459,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2438,7 +2470,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2604,7 +2636,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2615,7 +2647,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -2679,77 +2711,93 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>3</v>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhay Rawat</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>2</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>2</v>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>2</v>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>2</v>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -2760,7 +2808,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -2771,7 +2819,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -2782,7 +2830,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -2793,7 +2841,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2804,7 +2852,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2815,7 +2863,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2826,7 +2874,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2837,7 +2885,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2848,7 +2896,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2859,7 +2907,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -2870,51 +2918,51 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2925,7 +2973,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2936,7 +2984,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2947,7 +2995,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -2958,7 +3006,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2969,7 +3017,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Pranav Thomas</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2980,62 +3028,46 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Abhay Rawat</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="C29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="C30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0</v>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="C31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Pranav Thomas</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="C32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3401,12 +3433,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Wissa</t>
+          <t>Ballard</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -3416,7 +3448,7 @@
         <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>3.7</v>
+        <v>4.9</v>
       </c>
     </row>
   </sheetData>
@@ -3495,7 +3527,26 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>11</v>
+      </c>
+      <c r="E2" t="n">
+        <v>38561</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2018/19</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>858178</v>
+      </c>
+      <c r="H2" t="n">
+        <v>726260</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2025/26</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -3513,7 +3564,26 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="E3" t="n">
+        <v>545267</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2025/26</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>604934</v>
+      </c>
+      <c r="H3" t="n">
+        <v>545267</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2025/26</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -3522,16 +3592,35 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>12</v>
+      </c>
+      <c r="E4" t="n">
+        <v>27153</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2022/23</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>606381</v>
+      </c>
+      <c r="H4" t="n">
+        <v>240451</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2025/26</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -3540,16 +3629,35 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>281617</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2019/20</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1051323</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1076546</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2025/26</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -3558,30 +3666,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>27153</v>
+        <v>71857</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>606381</v>
+        <v>1929309</v>
       </c>
       <c r="H6" t="n">
-        <v>240451</v>
+        <v>297407</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -3595,30 +3703,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>28582</v>
+        <v>30971</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>881388</v>
+        <v>820221</v>
       </c>
       <c r="H7" t="n">
-        <v>239490</v>
+        <v>58227</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -3632,30 +3740,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E8" t="n">
-        <v>6474</v>
+        <v>28582</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>1177681</v>
+        <v>881388</v>
       </c>
       <c r="H8" t="n">
-        <v>6474</v>
+        <v>239490</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -3669,30 +3777,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E9" t="n">
-        <v>15136</v>
+        <v>6474</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>983840</v>
+        <v>1177681</v>
       </c>
       <c r="H9" t="n">
-        <v>45077</v>
+        <v>6474</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -3706,30 +3814,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E10" t="n">
-        <v>30971</v>
+        <v>15136</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>820221</v>
+        <v>983840</v>
       </c>
       <c r="H10" t="n">
-        <v>58227</v>
+        <v>45077</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -3780,30 +3888,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E12" t="n">
-        <v>60517</v>
+        <v>37120</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2015/16</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1414622</v>
+        <v>1571193</v>
       </c>
       <c r="H12" t="n">
-        <v>339763</v>
+        <v>3349378</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -3813,34 +3921,34 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E13" t="n">
-        <v>8917</v>
+        <v>189374</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>2118382</v>
+        <v>1757289</v>
       </c>
       <c r="H13" t="n">
-        <v>9146930</v>
+        <v>250879</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -3854,30 +3962,30 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E14" t="n">
-        <v>189374</v>
+        <v>60517</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2015/16</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>1757289</v>
+        <v>1414622</v>
       </c>
       <c r="H14" t="n">
-        <v>250879</v>
+        <v>339763</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -3891,30 +3999,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>8917</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>2118382</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>9146930</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -3928,30 +4036,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E16" t="n">
-        <v>1128645</v>
+        <v>31543</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>3434302</v>
+        <v>820692</v>
       </c>
       <c r="H16" t="n">
-        <v>1128645</v>
+        <v>1637750</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -3965,30 +4073,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E17" t="n">
-        <v>453230</v>
+        <v>273503</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>5483351</v>
+        <v>1994005</v>
       </c>
       <c r="H17" t="n">
-        <v>8188106</v>
+        <v>1917309</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4002,30 +4110,30 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E18" t="n">
-        <v>31543</v>
+        <v>453230</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>820692</v>
+        <v>5483351</v>
       </c>
       <c r="H18" t="n">
-        <v>1637750</v>
+        <v>8188106</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -4039,19 +4147,19 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>273503</v>
+        <v>486041</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4059,10 +4167,10 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>1994005</v>
+        <v>2415786</v>
       </c>
       <c r="H19" t="n">
-        <v>1917309</v>
+        <v>1206623</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -4076,30 +4184,30 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E20" t="n">
-        <v>486041</v>
+        <v>1128645</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>2415786</v>
+        <v>3434302</v>
       </c>
       <c r="H20" t="n">
-        <v>1206623</v>
+        <v>1128645</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -4150,30 +4258,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E22" t="n">
-        <v>14603</v>
+        <v>334016</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2016/17</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>949628</v>
+        <v>2156629</v>
       </c>
       <c r="H22" t="n">
-        <v>515830</v>
+        <v>2691725</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -4187,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E23" t="n">
-        <v>95791</v>
+        <v>14603</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2016/17</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2404119</v>
+        <v>949628</v>
       </c>
       <c r="H23" t="n">
-        <v>5124417</v>
+        <v>515830</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4220,34 +4328,34 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H24" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -4298,19 +4406,19 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E26" t="n">
-        <v>1320699</v>
+        <v>15288</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -4318,14 +4426,14 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>2490743</v>
+        <v>329510</v>
       </c>
       <c r="H26" t="n">
-        <v>1861933</v>
+        <v>538046</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
     </row>
@@ -4335,19 +4443,19 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="D27" t="n">
         <v>12</v>
       </c>
       <c r="E27" t="n">
-        <v>15288</v>
+        <v>81907</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -4355,10 +4463,10 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>329510</v>
+        <v>3252487</v>
       </c>
       <c r="H27" t="n">
-        <v>538046</v>
+        <v>11118394</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -4372,19 +4480,19 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E28" t="n">
-        <v>81907</v>
+        <v>1320699</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -4392,14 +4500,14 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>3252487</v>
+        <v>2490743</v>
       </c>
       <c r="H28" t="n">
-        <v>11118394</v>
+        <v>1861933</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2024/25</t>
         </is>
       </c>
     </row>
@@ -4665,16 +4773,31 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>344</v>
+        <v>348</v>
+      </c>
+      <c r="D2" t="n">
+        <v>86</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F2" t="n">
         <v>78</v>
       </c>
+      <c r="G2" t="n">
+        <v>126</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>63</v>
+      </c>
+      <c r="J2" t="n">
+        <v>3</v>
+      </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -4683,9 +4806,31 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U2" t="inlineStr"/>
+        <v>48</v>
+      </c>
+      <c r="O2" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="P2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="R2" t="n">
+        <v>10970</v>
+      </c>
+      <c r="S2" t="n">
+        <v>270274</v>
+      </c>
+      <c r="T2" t="n">
+        <v>2</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>bboost, freehit, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4699,16 +4844,31 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>325</v>
+        <v>327</v>
+      </c>
+      <c r="D3" t="n">
+        <v>81.2</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F3" t="n">
         <v>72</v>
       </c>
+      <c r="G3" t="n">
+        <v>116</v>
+      </c>
+      <c r="H3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I3" t="n">
+        <v>54</v>
+      </c>
+      <c r="J3" t="n">
+        <v>3</v>
+      </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -4717,32 +4877,65 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>39</v>
+      </c>
+      <c r="O3" t="n">
+        <v>100.8</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="R3" t="n">
+        <v>125991</v>
+      </c>
+      <c r="S3" t="n">
+        <v>1461471</v>
+      </c>
+      <c r="T3" t="n">
+        <v>2</v>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>315</v>
+        <v>322</v>
+      </c>
+      <c r="D4" t="n">
+        <v>78.2</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>72</v>
+        <v>77</v>
+      </c>
+      <c r="G4" t="n">
+        <v>106</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>51</v>
+      </c>
+      <c r="J4" t="n">
+        <v>3</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -4751,131 +4944,190 @@
         <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" t="inlineStr"/>
+        <v>35</v>
+      </c>
+      <c r="O4" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="R4" t="n">
+        <v>202778</v>
+      </c>
+      <c r="S4" t="n">
+        <v>166751</v>
+      </c>
+      <c r="T4" t="n">
+        <v>2</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>bboost, 3xc</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>314</v>
+        <v>317</v>
+      </c>
+      <c r="D5" t="n">
+        <v>78.8</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>78</v>
+        <v>72</v>
+      </c>
+      <c r="G5" t="n">
+        <v>107</v>
+      </c>
+      <c r="H5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" t="n">
+        <v>43</v>
+      </c>
+      <c r="J5" t="n">
+        <v>3</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U5" t="inlineStr"/>
+        <v>47</v>
+      </c>
+      <c r="O5" t="n">
+        <v>101.6</v>
+      </c>
+      <c r="P5" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="R5" t="n">
+        <v>298748</v>
+      </c>
+      <c r="S5" t="n">
+        <v>1229264</v>
+      </c>
+      <c r="T5" t="n">
+        <v>4</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>bboost, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="D6" t="n">
-        <v>78.2</v>
+        <v>78.5</v>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G6" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="H6" t="n">
         <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="J6" t="n">
         <v>3</v>
       </c>
       <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>66</v>
+      </c>
+      <c r="O6" t="n">
+        <v>101.6</v>
+      </c>
+      <c r="P6" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>307625</v>
+      </c>
+      <c r="S6" t="n">
+        <v>266328</v>
+      </c>
+      <c r="T6" t="n">
         <v>4</v>
       </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="n">
-        <v>35</v>
-      </c>
-      <c r="O6" t="n">
-        <v>100.5</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="R6" t="n">
-        <v>312178</v>
-      </c>
-      <c r="S6" t="n">
-        <v>166751</v>
-      </c>
-      <c r="T6" t="n">
-        <v>2</v>
-      </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="D7" t="n">
-        <v>76.2</v>
+        <v>74.8</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>
@@ -4884,13 +5136,13 @@
         <v>78</v>
       </c>
       <c r="G7" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="H7" t="n">
         <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="J7" t="n">
         <v>3</v>
@@ -4905,25 +5157,25 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="O7" t="n">
-        <v>101.8</v>
+        <v>101.3</v>
       </c>
       <c r="P7" t="n">
-        <v>1.8</v>
+        <v>1.3</v>
       </c>
       <c r="Q7" t="n">
         <v>0.2</v>
       </c>
       <c r="R7" t="n">
-        <v>528537</v>
+        <v>473776</v>
       </c>
       <c r="S7" t="n">
-        <v>466127</v>
+        <v>1034411</v>
       </c>
       <c r="T7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
@@ -4934,111 +5186,111 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="D8" t="n">
         <v>76.2</v>
       </c>
       <c r="E8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="G8" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H8" t="n">
         <v>2</v>
       </c>
       <c r="I8" t="n">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="J8" t="n">
         <v>3</v>
       </c>
       <c r="K8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>21</v>
+      </c>
+      <c r="O8" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="P8" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="R8" t="n">
+        <v>572309</v>
+      </c>
+      <c r="S8" t="n">
+        <v>466127</v>
+      </c>
+      <c r="T8" t="n">
         <v>4</v>
       </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" t="n">
-        <v>57</v>
-      </c>
-      <c r="O8" t="n">
-        <v>101</v>
-      </c>
-      <c r="P8" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="R8" t="n">
-        <v>549095</v>
-      </c>
-      <c r="S8" t="n">
-        <v>617418</v>
-      </c>
-      <c r="T8" t="n">
-        <v>2</v>
-      </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="D9" t="n">
-        <v>75</v>
+        <v>76.2</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>91</v>
+        <v>67</v>
       </c>
       <c r="G9" t="n">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="H9" t="n">
         <v>2</v>
       </c>
       <c r="I9" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J9" t="n">
         <v>3</v>
       </c>
       <c r="K9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
@@ -5047,22 +5299,22 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="O9" t="n">
-        <v>100.4</v>
+        <v>101</v>
       </c>
       <c r="P9" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="R9" t="n">
-        <v>745361</v>
+        <v>590502</v>
       </c>
       <c r="S9" t="n">
-        <v>637992</v>
+        <v>617418</v>
       </c>
       <c r="T9" t="n">
         <v>2</v>
@@ -5076,40 +5328,40 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="D10" t="n">
-        <v>74.8</v>
+        <v>75</v>
       </c>
       <c r="E10" t="n">
         <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="G10" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="H10" t="n">
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="J10" t="n">
         <v>3</v>
       </c>
       <c r="K10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -5118,29 +5370,29 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="O10" t="n">
-        <v>101.3</v>
+        <v>100.4</v>
       </c>
       <c r="P10" t="n">
-        <v>1.3</v>
+        <v>0.4</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="R10" t="n">
-        <v>774645</v>
+        <v>692220</v>
       </c>
       <c r="S10" t="n">
-        <v>1034411</v>
+        <v>637992</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>
@@ -5156,13 +5408,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="D11" t="n">
         <v>74.2</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
         <v>87</v>
@@ -5201,7 +5453,7 @@
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>866801</v>
+        <v>812371</v>
       </c>
       <c r="S11" t="n">
         <v>3039834</v>
@@ -5218,40 +5470,40 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="D12" t="n">
-        <v>73.2</v>
+        <v>71.8</v>
       </c>
       <c r="E12" t="n">
         <v>2</v>
       </c>
       <c r="F12" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="G12" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="H12" t="n">
         <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="J12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K12" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -5260,59 +5512,63 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="O12" t="n">
-        <v>100.3</v>
+        <v>101.2</v>
       </c>
       <c r="P12" t="n">
-        <v>0.3</v>
+        <v>1.2</v>
       </c>
       <c r="Q12" t="n">
-        <v>2.7</v>
+        <v>1.1</v>
       </c>
       <c r="R12" t="n">
-        <v>1089861</v>
+        <v>954058</v>
       </c>
       <c r="S12" t="n">
-        <v>4399137</v>
+        <v>101935</v>
       </c>
       <c r="T12" t="n">
-        <v>2</v>
-      </c>
-      <c r="U12" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>bboost</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="D13" t="n">
-        <v>72.2</v>
+        <v>71.8</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
         <v>78</v>
       </c>
       <c r="G13" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="H13" t="n">
         <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="J13" t="n">
         <v>3</v>
@@ -5327,69 +5583,69 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="O13" t="n">
-        <v>101.4</v>
+        <v>100.8</v>
       </c>
       <c r="P13" t="n">
-        <v>1.4</v>
+        <v>0.8</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="R13" t="n">
-        <v>1306162</v>
+        <v>954058</v>
       </c>
       <c r="S13" t="n">
-        <v>878473</v>
+        <v>3046343</v>
       </c>
       <c r="T13" t="n">
         <v>2</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>287</v>
+        <v>297</v>
       </c>
       <c r="D14" t="n">
-        <v>71.8</v>
+        <v>73.2</v>
       </c>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F14" t="n">
         <v>78</v>
       </c>
       <c r="G14" t="n">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="H14" t="n">
         <v>2</v>
       </c>
       <c r="I14" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -5398,63 +5654,59 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="O14" t="n">
-        <v>100.8</v>
+        <v>100.3</v>
       </c>
       <c r="P14" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="Q14" t="n">
-        <v>1</v>
+        <v>2.7</v>
       </c>
       <c r="R14" t="n">
-        <v>1426049</v>
+        <v>1029186</v>
       </c>
       <c r="S14" t="n">
-        <v>3046343</v>
+        <v>4399137</v>
       </c>
       <c r="T14" t="n">
         <v>2</v>
       </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+      <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="D15" t="n">
-        <v>71.8</v>
+        <v>72.2</v>
       </c>
       <c r="E15" t="n">
         <v>2</v>
       </c>
       <c r="F15" t="n">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
         <v>3</v>
@@ -5469,93 +5721,93 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>35</v>
+        <v>63</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>101.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
       <c r="R15" t="n">
-        <v>1433794</v>
+        <v>1225258</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>878473</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D16" t="n">
-        <v>71.8</v>
+        <v>71.2</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>67</v>
+        <v>105</v>
       </c>
       <c r="G16" t="n">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K16" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="O16" t="n">
-        <v>100.6</v>
+        <v>100.9</v>
       </c>
       <c r="P16" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="R16" t="n">
-        <v>1454432</v>
+        <v>1474436</v>
       </c>
       <c r="S16" t="n">
-        <v>3048395</v>
+        <v>1066412</v>
       </c>
       <c r="T16" t="n">
         <v>2</v>
@@ -5569,40 +5821,40 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="D17" t="n">
-        <v>71.5</v>
+        <v>71</v>
       </c>
       <c r="E17" t="n">
         <v>2</v>
       </c>
       <c r="F17" t="n">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="G17" t="n">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="H17" t="n">
         <v>2</v>
       </c>
       <c r="I17" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="J17" t="n">
         <v>1</v>
       </c>
       <c r="K17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
@@ -5611,66 +5863,66 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="O17" t="n">
-        <v>100.4</v>
+        <v>100.9</v>
       </c>
       <c r="P17" t="n">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
       <c r="Q17" t="n">
-        <v>1.3</v>
+        <v>0.6</v>
       </c>
       <c r="R17" t="n">
-        <v>1501110</v>
+        <v>1531344</v>
       </c>
       <c r="S17" t="n">
-        <v>3009015</v>
+        <v>5881370</v>
       </c>
       <c r="T17" t="n">
         <v>2</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="D18" t="n">
-        <v>71.2</v>
+        <v>71.5</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="G18" t="n">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="H18" t="n">
         <v>2</v>
       </c>
       <c r="I18" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="J18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K18" t="n">
         <v>2</v>
@@ -5682,69 +5934,69 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="O18" t="n">
-        <v>100.9</v>
+        <v>100.4</v>
       </c>
       <c r="P18" t="n">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
       <c r="Q18" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="R18" t="n">
-        <v>1569102</v>
+        <v>1540621</v>
       </c>
       <c r="S18" t="n">
-        <v>1066412</v>
+        <v>3009015</v>
       </c>
       <c r="T18" t="n">
         <v>2</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D19" t="n">
-        <v>71</v>
+        <v>70.8</v>
       </c>
       <c r="E19" t="n">
         <v>2</v>
       </c>
       <c r="F19" t="n">
-        <v>95</v>
+        <v>57</v>
       </c>
       <c r="G19" t="n">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="H19" t="n">
         <v>2</v>
       </c>
       <c r="I19" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J19" t="n">
         <v>1</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L19" t="n">
         <v>0</v>
@@ -5753,22 +6005,22 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="O19" t="n">
-        <v>100.9</v>
+        <v>101.1</v>
       </c>
       <c r="P19" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="R19" t="n">
-        <v>1622014</v>
+        <v>1750901</v>
       </c>
       <c r="S19" t="n">
-        <v>5881370</v>
+        <v>5250200</v>
       </c>
       <c r="T19" t="n">
         <v>2</v>
@@ -5782,64 +6034,64 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="D20" t="n">
-        <v>70.8</v>
+        <v>71.8</v>
       </c>
       <c r="E20" t="n">
         <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="G20" t="n">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="H20" t="n">
         <v>2</v>
       </c>
       <c r="I20" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J20" t="n">
         <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M20" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="N20" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="O20" t="n">
-        <v>101.1</v>
+        <v>100.6</v>
       </c>
       <c r="P20" t="n">
-        <v>1.1</v>
+        <v>0.6</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="R20" t="n">
-        <v>1711492</v>
+        <v>1804176</v>
       </c>
       <c r="S20" t="n">
-        <v>5250200</v>
+        <v>3048395</v>
       </c>
       <c r="T20" t="n">
         <v>2</v>
@@ -5862,7 +6114,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="D21" t="n">
         <v>70</v>
@@ -5907,7 +6159,7 @@
         <v>0.4</v>
       </c>
       <c r="R21" t="n">
-        <v>1936996</v>
+        <v>1824720</v>
       </c>
       <c r="S21" t="n">
         <v>4185865</v>
@@ -5924,40 +6176,40 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="D22" t="n">
-        <v>68.8</v>
+        <v>67.5</v>
       </c>
       <c r="E22" t="n">
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G22" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H22" t="n">
         <v>2</v>
       </c>
       <c r="I22" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
@@ -5966,48 +6218,44 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="O22" t="n">
-        <v>101.7</v>
+        <v>101.1</v>
       </c>
       <c r="P22" t="n">
-        <v>1.7</v>
+        <v>1.1</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.4</v>
+        <v>1.1</v>
       </c>
       <c r="R22" t="n">
-        <v>2343465</v>
+        <v>2310060</v>
       </c>
       <c r="S22" t="n">
-        <v>2735246</v>
+        <v>453361</v>
       </c>
       <c r="T22" t="n">
         <v>2</v>
       </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+      <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="D23" t="n">
-        <v>67.5</v>
+        <v>68.8</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -6019,16 +6267,16 @@
         <v>93</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="J23" t="n">
         <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L23" t="n">
         <v>0</v>
@@ -6037,25 +6285,25 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="O23" t="n">
-        <v>101.9</v>
+        <v>101.7</v>
       </c>
       <c r="P23" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="R23" t="n">
-        <v>2778338</v>
+        <v>2382041</v>
       </c>
       <c r="S23" t="n">
-        <v>2489160</v>
+        <v>2735246</v>
       </c>
       <c r="T23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U23" t="inlineStr">
         <is>
@@ -6066,37 +6314,37 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="D24" t="n">
         <v>67.5</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G24" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K24" t="n">
         <v>3</v>
@@ -6108,27 +6356,31 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="O24" t="n">
-        <v>101.1</v>
+        <v>101.9</v>
       </c>
       <c r="P24" t="n">
-        <v>1.1</v>
+        <v>1.9</v>
       </c>
       <c r="Q24" t="n">
-        <v>1.1</v>
+        <v>0.6</v>
       </c>
       <c r="R24" t="n">
-        <v>2778338</v>
+        <v>2653085</v>
       </c>
       <c r="S24" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T24" t="n">
-        <v>2</v>
-      </c>
-      <c r="U24" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6142,7 +6394,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="D25" t="n">
         <v>67.2</v>
@@ -6187,7 +6439,7 @@
         <v>1.8</v>
       </c>
       <c r="R25" t="n">
-        <v>2868689</v>
+        <v>2920575</v>
       </c>
       <c r="S25" t="n">
         <v>1595922</v>
@@ -6204,209 +6456,209 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D26" t="n">
-        <v>66.8</v>
+        <v>66.5</v>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="G26" t="n">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="H26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I26" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="J26" t="n">
+        <v>1</v>
+      </c>
+      <c r="K26" t="n">
+        <v>4</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" t="n">
+        <v>33</v>
+      </c>
+      <c r="O26" t="n">
+        <v>100.8</v>
+      </c>
+      <c r="P26" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" t="n">
+        <v>3408814</v>
+      </c>
+      <c r="S26" t="n">
+        <v>3395267</v>
+      </c>
+      <c r="T26" t="n">
         <v>3</v>
       </c>
-      <c r="K26" t="n">
-        <v>5</v>
-      </c>
-      <c r="L26" t="n">
-        <v>2</v>
-      </c>
-      <c r="M26" t="n">
-        <v>-8</v>
-      </c>
-      <c r="N26" t="n">
-        <v>55</v>
-      </c>
-      <c r="O26" t="n">
-        <v>101.1</v>
-      </c>
-      <c r="P26" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="R26" t="n">
-        <v>3077476</v>
-      </c>
-      <c r="S26" t="n">
-        <v>1948104</v>
-      </c>
-      <c r="T26" t="n">
-        <v>2</v>
-      </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>3xc</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D27" t="n">
-        <v>66.5</v>
+        <v>65.8</v>
       </c>
       <c r="E27" t="n">
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="G27" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H27" t="n">
+        <v>2</v>
+      </c>
+      <c r="I27" t="n">
+        <v>47</v>
+      </c>
+      <c r="J27" t="n">
         <v>3</v>
       </c>
-      <c r="I27" t="n">
-        <v>41</v>
-      </c>
-      <c r="J27" t="n">
-        <v>1</v>
-      </c>
       <c r="K27" t="n">
+        <v>2</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="n">
+        <v>60</v>
+      </c>
+      <c r="O27" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="P27" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="R27" t="n">
+        <v>3467701</v>
+      </c>
+      <c r="S27" t="n">
+        <v>614528</v>
+      </c>
+      <c r="T27" t="n">
         <v>4</v>
       </c>
-      <c r="L27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" t="n">
-        <v>33</v>
-      </c>
-      <c r="O27" t="n">
-        <v>100.8</v>
-      </c>
-      <c r="P27" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" t="n">
-        <v>3170793</v>
-      </c>
-      <c r="S27" t="n">
-        <v>3395267</v>
-      </c>
-      <c r="T27" t="n">
-        <v>3</v>
-      </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>3xc</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D28" t="n">
-        <v>65.8</v>
+        <v>66.8</v>
       </c>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F28" t="n">
         <v>58</v>
       </c>
       <c r="G28" t="n">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="H28" t="n">
         <v>2</v>
       </c>
       <c r="I28" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J28" t="n">
         <v>3</v>
       </c>
       <c r="K28" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M28" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="N28" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="O28" t="n">
-        <v>101.7</v>
+        <v>101.1</v>
       </c>
       <c r="P28" t="n">
-        <v>1.7</v>
+        <v>1.1</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="R28" t="n">
-        <v>3430081</v>
+        <v>3529338</v>
       </c>
       <c r="S28" t="n">
-        <v>614528</v>
+        <v>1948104</v>
       </c>
       <c r="T28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U28" t="inlineStr">
         <is>
@@ -6426,7 +6678,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D29" t="n">
         <v>61.8</v>
@@ -6471,7 +6723,7 @@
         <v>0</v>
       </c>
       <c r="R29" t="n">
-        <v>4982912</v>
+        <v>5014901</v>
       </c>
       <c r="S29" t="n">
         <v>3963132</v>
@@ -6497,7 +6749,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D30" t="n">
         <v>58</v>
@@ -6530,7 +6782,7 @@
         <v>-8</v>
       </c>
       <c r="N30" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="O30" t="n">
         <v>101.4</v>
@@ -6542,7 +6794,7 @@
         <v>1</v>
       </c>
       <c r="R30" t="n">
-        <v>6376870</v>
+        <v>6407277</v>
       </c>
       <c r="S30" t="n">
         <v>1952243</v>
@@ -6568,13 +6820,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="D31" t="n">
         <v>56.8</v>
       </c>
       <c r="E31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F31" t="n">
         <v>62</v>
@@ -6613,7 +6865,7 @@
         <v>1.2</v>
       </c>
       <c r="R31" t="n">
-        <v>6761783</v>
+        <v>6473731</v>
       </c>
       <c r="S31" t="n">
         <v>553038</v>
@@ -6684,7 +6936,7 @@
         <v>2.2</v>
       </c>
       <c r="R32" t="n">
-        <v>8951568</v>
+        <v>9014751</v>
       </c>
       <c r="S32" t="n">
         <v>216389</v>

</xml_diff>

<commit_message>
Update standings 2026-09-19 03:26 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -4889,7 +4889,7 @@
         <v>0.2</v>
       </c>
       <c r="R3" t="n">
-        <v>125991</v>
+        <v>125992</v>
       </c>
       <c r="S3" t="n">
         <v>1461471</v>
@@ -5240,7 +5240,7 @@
         <v>0.2</v>
       </c>
       <c r="R8" t="n">
-        <v>572309</v>
+        <v>572310</v>
       </c>
       <c r="S8" t="n">
         <v>466127</v>
@@ -5311,7 +5311,7 @@
         <v>0.5</v>
       </c>
       <c r="R9" t="n">
-        <v>590502</v>
+        <v>590503</v>
       </c>
       <c r="S9" t="n">
         <v>617418</v>
@@ -5382,7 +5382,7 @@
         <v>0.6</v>
       </c>
       <c r="R10" t="n">
-        <v>692220</v>
+        <v>692223</v>
       </c>
       <c r="S10" t="n">
         <v>637992</v>
@@ -5453,7 +5453,7 @@
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>812371</v>
+        <v>812374</v>
       </c>
       <c r="S11" t="n">
         <v>3039834</v>
@@ -5524,7 +5524,7 @@
         <v>1.1</v>
       </c>
       <c r="R12" t="n">
-        <v>954058</v>
+        <v>954063</v>
       </c>
       <c r="S12" t="n">
         <v>101935</v>
@@ -5595,7 +5595,7 @@
         <v>1</v>
       </c>
       <c r="R13" t="n">
-        <v>954058</v>
+        <v>954063</v>
       </c>
       <c r="S13" t="n">
         <v>3046343</v>
@@ -5666,7 +5666,7 @@
         <v>2.7</v>
       </c>
       <c r="R14" t="n">
-        <v>1029186</v>
+        <v>1029192</v>
       </c>
       <c r="S14" t="n">
         <v>4399137</v>
@@ -5733,7 +5733,7 @@
         <v>0.2</v>
       </c>
       <c r="R15" t="n">
-        <v>1225258</v>
+        <v>1225264</v>
       </c>
       <c r="S15" t="n">
         <v>878473</v>
@@ -5804,7 +5804,7 @@
         <v>0</v>
       </c>
       <c r="R16" t="n">
-        <v>1474436</v>
+        <v>1474444</v>
       </c>
       <c r="S16" t="n">
         <v>1066412</v>
@@ -5875,7 +5875,7 @@
         <v>0.6</v>
       </c>
       <c r="R17" t="n">
-        <v>1531344</v>
+        <v>1531354</v>
       </c>
       <c r="S17" t="n">
         <v>5881370</v>
@@ -5946,7 +5946,7 @@
         <v>1.3</v>
       </c>
       <c r="R18" t="n">
-        <v>1540621</v>
+        <v>1540631</v>
       </c>
       <c r="S18" t="n">
         <v>3009015</v>
@@ -6017,7 +6017,7 @@
         <v>0.5</v>
       </c>
       <c r="R19" t="n">
-        <v>1750901</v>
+        <v>1750909</v>
       </c>
       <c r="S19" t="n">
         <v>5250200</v>
@@ -6088,7 +6088,7 @@
         <v>0.7</v>
       </c>
       <c r="R20" t="n">
-        <v>1804176</v>
+        <v>1804185</v>
       </c>
       <c r="S20" t="n">
         <v>3048395</v>
@@ -6159,7 +6159,7 @@
         <v>0.4</v>
       </c>
       <c r="R21" t="n">
-        <v>1824720</v>
+        <v>1824730</v>
       </c>
       <c r="S21" t="n">
         <v>4185865</v>
@@ -6230,7 +6230,7 @@
         <v>1.1</v>
       </c>
       <c r="R22" t="n">
-        <v>2310060</v>
+        <v>2310073</v>
       </c>
       <c r="S22" t="n">
         <v>453361</v>
@@ -6297,7 +6297,7 @@
         <v>0.4</v>
       </c>
       <c r="R23" t="n">
-        <v>2382041</v>
+        <v>2382054</v>
       </c>
       <c r="S23" t="n">
         <v>2735246</v>
@@ -6368,7 +6368,7 @@
         <v>0.6</v>
       </c>
       <c r="R24" t="n">
-        <v>2653085</v>
+        <v>2653099</v>
       </c>
       <c r="S24" t="n">
         <v>2489160</v>
@@ -6439,7 +6439,7 @@
         <v>1.8</v>
       </c>
       <c r="R25" t="n">
-        <v>2920575</v>
+        <v>2920591</v>
       </c>
       <c r="S25" t="n">
         <v>1595922</v>
@@ -6510,7 +6510,7 @@
         <v>0</v>
       </c>
       <c r="R26" t="n">
-        <v>3408814</v>
+        <v>3408831</v>
       </c>
       <c r="S26" t="n">
         <v>3395267</v>
@@ -6581,7 +6581,7 @@
         <v>0.7</v>
       </c>
       <c r="R27" t="n">
-        <v>3467701</v>
+        <v>3467718</v>
       </c>
       <c r="S27" t="n">
         <v>614528</v>
@@ -6652,7 +6652,7 @@
         <v>0.1</v>
       </c>
       <c r="R28" t="n">
-        <v>3529338</v>
+        <v>3529354</v>
       </c>
       <c r="S28" t="n">
         <v>1948104</v>
@@ -6723,7 +6723,7 @@
         <v>0</v>
       </c>
       <c r="R29" t="n">
-        <v>5014901</v>
+        <v>5014924</v>
       </c>
       <c r="S29" t="n">
         <v>3963132</v>
@@ -6794,7 +6794,7 @@
         <v>1</v>
       </c>
       <c r="R30" t="n">
-        <v>6407277</v>
+        <v>6407301</v>
       </c>
       <c r="S30" t="n">
         <v>1952243</v>
@@ -6865,7 +6865,7 @@
         <v>1.2</v>
       </c>
       <c r="R31" t="n">
-        <v>6473731</v>
+        <v>6473757</v>
       </c>
       <c r="S31" t="n">
         <v>553038</v>
@@ -6936,7 +6936,7 @@
         <v>2.2</v>
       </c>
       <c r="R32" t="n">
-        <v>9014751</v>
+        <v>9014775</v>
       </c>
       <c r="S32" t="n">
         <v>216389</v>

</xml_diff>

<commit_message>
Update standings 2026-09-19 08:35 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -715,12 +715,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -739,12 +739,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1781,39 +1781,39 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="C12" t="n">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="D12" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="E12" t="n">
-        <v>69</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="C13" t="n">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="D13" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="E13" t="n">
-        <v>77</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14">
@@ -2962,7 +2962,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2973,7 +2973,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -3888,30 +3888,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E12" t="n">
-        <v>37120</v>
+        <v>189374</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1571193</v>
+        <v>1757289</v>
       </c>
       <c r="H12" t="n">
-        <v>3349378</v>
+        <v>250879</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -3925,30 +3925,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E13" t="n">
-        <v>189374</v>
+        <v>37120</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>1757289</v>
+        <v>1571193</v>
       </c>
       <c r="H13" t="n">
-        <v>250879</v>
+        <v>3349378</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -5470,12 +5470,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -5485,19 +5485,19 @@
         <v>71.8</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="G12" t="n">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="H12" t="n">
         <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="J12" t="n">
         <v>3</v>
@@ -5512,41 +5512,41 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="O12" t="n">
-        <v>101.2</v>
+        <v>100.8</v>
       </c>
       <c r="P12" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="Q12" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="R12" t="n">
         <v>954063</v>
       </c>
       <c r="S12" t="n">
-        <v>101935</v>
+        <v>3046343</v>
       </c>
       <c r="T12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -5556,19 +5556,19 @@
         <v>71.8</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="G13" t="n">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="H13" t="n">
         <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="J13" t="n">
         <v>3</v>
@@ -5583,29 +5583,29 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="O13" t="n">
-        <v>100.8</v>
+        <v>101.2</v>
       </c>
       <c r="P13" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="Q13" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="R13" t="n">
         <v>954063</v>
       </c>
       <c r="S13" t="n">
-        <v>3046343</v>
+        <v>101935</v>
       </c>
       <c r="T13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-19 13:42 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -484,13 +484,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="3">
@@ -556,13 +556,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
         <v>-4</v>
       </c>
       <c r="F5" t="n">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="6">
@@ -580,13 +580,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="7">
@@ -619,22 +619,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="9">
@@ -643,12 +643,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -715,36 +715,36 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -759,26 +759,26 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="15">
@@ -796,13 +796,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="16">
@@ -811,22 +811,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="17">
@@ -835,12 +835,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -850,7 +850,7 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="18">
@@ -883,22 +883,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="F19" t="n">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="20">
@@ -907,19 +907,19 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D20" t="n">
         <v>2</v>
       </c>
       <c r="E20" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
         <v>285</v>
@@ -964,13 +964,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="23">
@@ -1012,13 +1012,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="25">
@@ -1036,13 +1036,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="26">
@@ -1060,13 +1060,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="27">
@@ -1084,13 +1084,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="28">
@@ -1108,13 +1108,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E28" t="n">
         <v>-8</v>
       </c>
       <c r="F28" t="n">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="29">
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="30">
@@ -1705,39 +1705,39 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="C8" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D8" t="n">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="E8" t="n">
-        <v>91</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="C9" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D9" t="n">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="E9" t="n">
-        <v>76</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10">
@@ -1781,58 +1781,58 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C12" t="n">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="D12" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E12" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="C13" t="n">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="D13" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="E13" t="n">
-        <v>69</v>
+        <v>77</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>48</v>
+        <v>73</v>
       </c>
       <c r="C14" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="D14" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E14" t="n">
-        <v>76</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15">
@@ -1857,39 +1857,39 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="C16" t="n">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D16" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>58</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="C17" t="n">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="D17" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E17" t="n">
-        <v>71</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18">
@@ -1914,39 +1914,39 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C19" t="n">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="D19" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="E19" t="n">
-        <v>75</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C20" t="n">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="D20" t="n">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="E20" t="n">
-        <v>87</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21">
@@ -2448,7 +2448,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2459,7 +2459,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2808,7 +2808,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -2819,7 +2819,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -2962,7 +2962,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2973,7 +2973,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2984,7 +2984,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -3740,30 +3740,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E8" t="n">
-        <v>28582</v>
+        <v>6474</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>881388</v>
+        <v>1177681</v>
       </c>
       <c r="H8" t="n">
-        <v>239490</v>
+        <v>6474</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -3777,30 +3777,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E9" t="n">
-        <v>6474</v>
+        <v>28582</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>1177681</v>
+        <v>881388</v>
       </c>
       <c r="H9" t="n">
-        <v>6474</v>
+        <v>239490</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -3888,30 +3888,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E12" t="n">
-        <v>189374</v>
+        <v>60517</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2015/16</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1757289</v>
+        <v>1414622</v>
       </c>
       <c r="H12" t="n">
-        <v>250879</v>
+        <v>339763</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -3921,34 +3921,34 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E13" t="n">
-        <v>37120</v>
+        <v>189374</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>1571193</v>
+        <v>1757289</v>
       </c>
       <c r="H13" t="n">
-        <v>3349378</v>
+        <v>250879</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -3958,34 +3958,34 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E14" t="n">
-        <v>60517</v>
+        <v>37120</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2015/16</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>1414622</v>
+        <v>1571193</v>
       </c>
       <c r="H14" t="n">
-        <v>339763</v>
+        <v>3349378</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -4036,30 +4036,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E16" t="n">
-        <v>31543</v>
+        <v>273503</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>820692</v>
+        <v>1994005</v>
       </c>
       <c r="H16" t="n">
-        <v>1637750</v>
+        <v>1917309</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -4073,30 +4073,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E17" t="n">
-        <v>273503</v>
+        <v>31543</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>1994005</v>
+        <v>820692</v>
       </c>
       <c r="H17" t="n">
-        <v>1917309</v>
+        <v>1637750</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4147,30 +4147,30 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E19" t="n">
-        <v>486041</v>
+        <v>1128645</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>2415786</v>
+        <v>3434302</v>
       </c>
       <c r="H19" t="n">
-        <v>1206623</v>
+        <v>1128645</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -4184,30 +4184,30 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>1128645</v>
+        <v>486041</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>3434302</v>
+        <v>2415786</v>
       </c>
       <c r="H20" t="n">
-        <v>1128645</v>
+        <v>1206623</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="D2" t="n">
         <v>86</v>
@@ -4982,7 +4982,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D5" t="n">
         <v>78.8</v>
@@ -5053,7 +5053,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="D6" t="n">
         <v>78.5</v>
@@ -5186,16 +5186,16 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="D8" t="n">
         <v>76.2</v>
@@ -5204,22 +5204,22 @@
         <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="G8" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H8" t="n">
         <v>2</v>
       </c>
       <c r="I8" t="n">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="J8" t="n">
         <v>3</v>
       </c>
       <c r="K8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -5228,41 +5228,41 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="O8" t="n">
-        <v>101.8</v>
+        <v>101</v>
       </c>
       <c r="P8" t="n">
-        <v>1.8</v>
+        <v>1</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="R8" t="n">
-        <v>572310</v>
+        <v>590503</v>
       </c>
       <c r="S8" t="n">
-        <v>466127</v>
+        <v>617418</v>
       </c>
       <c r="T8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -5275,53 +5275,53 @@
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="G9" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H9" t="n">
         <v>2</v>
       </c>
       <c r="I9" t="n">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="J9" t="n">
         <v>3</v>
       </c>
       <c r="K9" t="n">
+        <v>2</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>21</v>
+      </c>
+      <c r="O9" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="P9" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="R9" t="n">
+        <v>572310</v>
+      </c>
+      <c r="S9" t="n">
+        <v>466127</v>
+      </c>
+      <c r="T9" t="n">
         <v>4</v>
       </c>
-      <c r="L9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" t="n">
-        <v>57</v>
-      </c>
-      <c r="O9" t="n">
-        <v>101</v>
-      </c>
-      <c r="P9" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="R9" t="n">
-        <v>590503</v>
-      </c>
-      <c r="S9" t="n">
-        <v>617418</v>
-      </c>
-      <c r="T9" t="n">
-        <v>2</v>
-      </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
@@ -5470,19 +5470,19 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D12" t="n">
-        <v>71.8</v>
+        <v>73.2</v>
       </c>
       <c r="E12" t="n">
         <v>1</v>
@@ -5491,19 +5491,19 @@
         <v>78</v>
       </c>
       <c r="G12" t="n">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="H12" t="n">
         <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -5512,41 +5512,37 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="O12" t="n">
-        <v>100.8</v>
+        <v>100.3</v>
       </c>
       <c r="P12" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="Q12" t="n">
-        <v>1</v>
+        <v>2.7</v>
       </c>
       <c r="R12" t="n">
-        <v>954063</v>
+        <v>1029192</v>
       </c>
       <c r="S12" t="n">
-        <v>3046343</v>
+        <v>4399137</v>
       </c>
       <c r="T12" t="n">
         <v>2</v>
       </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+      <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -5556,19 +5552,19 @@
         <v>71.8</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="G13" t="n">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="H13" t="n">
         <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="J13" t="n">
         <v>3</v>
@@ -5583,69 +5579,69 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="O13" t="n">
-        <v>101.2</v>
+        <v>100.8</v>
       </c>
       <c r="P13" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="Q13" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="R13" t="n">
         <v>954063</v>
       </c>
       <c r="S13" t="n">
-        <v>101935</v>
+        <v>3046343</v>
       </c>
       <c r="T13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D14" t="n">
-        <v>73.2</v>
+        <v>71.8</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="G14" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="H14" t="n">
         <v>2</v>
       </c>
       <c r="I14" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -5654,27 +5650,31 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="O14" t="n">
-        <v>100.3</v>
+        <v>101.2</v>
       </c>
       <c r="P14" t="n">
-        <v>0.3</v>
+        <v>1.2</v>
       </c>
       <c r="Q14" t="n">
-        <v>2.7</v>
+        <v>1.1</v>
       </c>
       <c r="R14" t="n">
-        <v>1029192</v>
+        <v>954063</v>
       </c>
       <c r="S14" t="n">
-        <v>4399137</v>
+        <v>101935</v>
       </c>
       <c r="T14" t="n">
-        <v>2</v>
-      </c>
-      <c r="U14" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>bboost</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5688,7 +5688,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D15" t="n">
         <v>72.2</v>
@@ -5750,40 +5750,40 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D16" t="n">
-        <v>71.2</v>
+        <v>71</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" t="n">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="G16" t="n">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="J16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
@@ -5792,7 +5792,7 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="O16" t="n">
         <v>100.9</v>
@@ -5801,13 +5801,13 @@
         <v>0.9</v>
       </c>
       <c r="Q16" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="R16" t="n">
-        <v>1474444</v>
+        <v>1531354</v>
       </c>
       <c r="S16" t="n">
-        <v>1066412</v>
+        <v>5881370</v>
       </c>
       <c r="T16" t="n">
         <v>2</v>
@@ -5821,40 +5821,40 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D17" t="n">
-        <v>71</v>
+        <v>71.2</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="G17" t="n">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="H17" t="n">
         <v>2</v>
       </c>
       <c r="I17" t="n">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="J17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
@@ -5863,7 +5863,7 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="O17" t="n">
         <v>100.9</v>
@@ -5872,13 +5872,13 @@
         <v>0.9</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>1531354</v>
+        <v>1474444</v>
       </c>
       <c r="S17" t="n">
-        <v>5881370</v>
+        <v>1066412</v>
       </c>
       <c r="T17" t="n">
         <v>2</v>
@@ -5963,64 +5963,64 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="D19" t="n">
-        <v>70.8</v>
+        <v>71.8</v>
       </c>
       <c r="E19" t="n">
         <v>2</v>
       </c>
       <c r="F19" t="n">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="G19" t="n">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="H19" t="n">
         <v>2</v>
       </c>
       <c r="I19" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J19" t="n">
         <v>1</v>
       </c>
       <c r="K19" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="N19" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="O19" t="n">
-        <v>101.1</v>
+        <v>100.6</v>
       </c>
       <c r="P19" t="n">
-        <v>1.1</v>
+        <v>0.6</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="R19" t="n">
-        <v>1750909</v>
+        <v>1804185</v>
       </c>
       <c r="S19" t="n">
-        <v>5250200</v>
+        <v>3048395</v>
       </c>
       <c r="T19" t="n">
         <v>2</v>
@@ -6034,64 +6034,64 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="C20" t="n">
         <v>285</v>
       </c>
       <c r="D20" t="n">
-        <v>71.8</v>
+        <v>70.8</v>
       </c>
       <c r="E20" t="n">
         <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="G20" t="n">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="H20" t="n">
         <v>2</v>
       </c>
       <c r="I20" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J20" t="n">
         <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="O20" t="n">
-        <v>100.6</v>
+        <v>101.1</v>
       </c>
       <c r="P20" t="n">
-        <v>0.6</v>
+        <v>1.1</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="R20" t="n">
-        <v>1804185</v>
+        <v>1750909</v>
       </c>
       <c r="S20" t="n">
-        <v>3048395</v>
+        <v>5250200</v>
       </c>
       <c r="T20" t="n">
         <v>2</v>
@@ -6185,7 +6185,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D22" t="n">
         <v>67.5</v>
@@ -6323,7 +6323,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="D24" t="n">
         <v>67.5</v>
@@ -6394,7 +6394,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D25" t="n">
         <v>67.2</v>
@@ -6465,7 +6465,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D26" t="n">
         <v>66.5</v>
@@ -6536,7 +6536,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D27" t="n">
         <v>65.8</v>
@@ -6607,7 +6607,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D28" t="n">
         <v>66.8</v>
@@ -6678,7 +6678,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D29" t="n">
         <v>61.8</v>

</xml_diff>

<commit_message>
Update standings 2026-09-19 17:01 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -484,13 +484,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>350</v>
+        <v>383</v>
       </c>
     </row>
     <row r="3">
@@ -508,13 +508,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>327</v>
+        <v>345</v>
       </c>
     </row>
     <row r="4">
@@ -523,22 +523,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>9</v>
+        <v>52</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>322</v>
+        <v>339</v>
       </c>
     </row>
     <row r="5">
@@ -556,13 +556,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="E5" t="n">
         <v>-4</v>
       </c>
       <c r="F5" t="n">
-        <v>319</v>
+        <v>335</v>
       </c>
     </row>
     <row r="6">
@@ -571,22 +571,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>318</v>
+        <v>331</v>
       </c>
     </row>
     <row r="7">
@@ -595,22 +595,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>310</v>
+        <v>328</v>
       </c>
     </row>
     <row r="8">
@@ -628,13 +628,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>309</v>
+        <v>325</v>
       </c>
     </row>
     <row r="9">
@@ -643,22 +643,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>307</v>
+        <v>324</v>
       </c>
     </row>
     <row r="10">
@@ -667,22 +667,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>304</v>
+        <v>322</v>
       </c>
     </row>
     <row r="11">
@@ -691,22 +691,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>301</v>
+        <v>321</v>
       </c>
     </row>
     <row r="12">
@@ -715,22 +715,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>299</v>
+        <v>315</v>
       </c>
     </row>
     <row r="13">
@@ -739,46 +739,46 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>298</v>
+        <v>315</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>298</v>
+        <v>312</v>
       </c>
     </row>
     <row r="15">
@@ -787,22 +787,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>295</v>
+        <v>310</v>
       </c>
     </row>
     <row r="16">
@@ -811,22 +811,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>290</v>
+        <v>310</v>
       </c>
     </row>
     <row r="17">
@@ -835,22 +835,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>289</v>
+        <v>309</v>
       </c>
     </row>
     <row r="18">
@@ -859,22 +859,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>288</v>
+        <v>308</v>
       </c>
     </row>
     <row r="19">
@@ -883,22 +883,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="E19" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>287</v>
+        <v>307</v>
       </c>
     </row>
     <row r="20">
@@ -907,22 +907,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>285</v>
+        <v>301</v>
       </c>
     </row>
     <row r="21">
@@ -931,22 +931,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>284</v>
+        <v>299</v>
       </c>
     </row>
     <row r="22">
@@ -955,22 +955,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="F22" t="n">
-        <v>280</v>
+        <v>297</v>
       </c>
     </row>
     <row r="23">
@@ -979,22 +979,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>277</v>
+        <v>296</v>
       </c>
     </row>
     <row r="24">
@@ -1003,22 +1003,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>276</v>
+        <v>293</v>
       </c>
     </row>
     <row r="25">
@@ -1027,22 +1027,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>273</v>
+        <v>290</v>
       </c>
     </row>
     <row r="26">
@@ -1051,22 +1051,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="F26" t="n">
-        <v>268</v>
+        <v>290</v>
       </c>
     </row>
     <row r="27">
@@ -1084,13 +1084,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>267</v>
+        <v>284</v>
       </c>
     </row>
     <row r="28">
@@ -1099,22 +1099,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="E28" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>267</v>
+        <v>281</v>
       </c>
     </row>
     <row r="29">
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>251</v>
+        <v>272</v>
       </c>
     </row>
     <row r="30">
@@ -1156,13 +1156,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="E30" t="n">
         <v>-8</v>
       </c>
       <c r="F30" t="n">
-        <v>234</v>
+        <v>258</v>
       </c>
     </row>
     <row r="31">
@@ -1180,13 +1180,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E31" t="n">
         <v>-4</v>
       </c>
       <c r="F31" t="n">
-        <v>233</v>
+        <v>237</v>
       </c>
     </row>
     <row r="32">
@@ -1204,13 +1204,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>187</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -1629,20 +1629,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>72</v>
+        <v>52</v>
       </c>
       <c r="C4" t="n">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="D4" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="E4" t="n">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5">
@@ -1667,39 +1667,39 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="C6" t="n">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="D6" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="E6" t="n">
-        <v>92</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="C7" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D7" t="n">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="E7" t="n">
-        <v>91</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8">
@@ -1724,343 +1724,343 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C9" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D9" t="n">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="E9" t="n">
-        <v>91</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="C10" t="n">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="D10" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="E10" t="n">
-        <v>62</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="C11" t="n">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="D11" t="n">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="E11" t="n">
-        <v>71</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C12" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D12" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E12" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C13" t="n">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="D13" t="n">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="E13" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>73</v>
       </c>
       <c r="C14" t="n">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="D14" t="n">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="E14" t="n">
-        <v>69</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="C15" t="n">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D15" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="E15" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>40</v>
+        <v>66</v>
       </c>
       <c r="C16" t="n">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C17" t="n">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D17" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="E17" t="n">
-        <v>58</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="C18" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="D18" t="n">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="E18" t="n">
-        <v>71</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C19" t="n">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="D19" t="n">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="E19" t="n">
-        <v>87</v>
+        <v>76</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="C20" t="n">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="D20" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E20" t="n">
-        <v>75</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C21" t="n">
-        <v>107</v>
+        <v>86</v>
       </c>
       <c r="D21" t="n">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="E21" t="n">
-        <v>73</v>
+        <v>93</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="C22" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D22" t="n">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="E22" t="n">
-        <v>77</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C23" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="D23" t="n">
         <v>50</v>
       </c>
       <c r="E23" t="n">
-        <v>90</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C24" t="n">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E24" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="C25" t="n">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="D25" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="E25" t="n">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="C26" t="n">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="D26" t="n">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="E26" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27">
@@ -2085,20 +2085,20 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="C28" t="n">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="D28" t="n">
-        <v>46</v>
+        <v>78</v>
       </c>
       <c r="E28" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="29">
@@ -2221,7 +2221,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -2369,7 +2369,11 @@
       <c r="B6" t="n">
         <v>87</v>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2411,7 +2415,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -2426,7 +2430,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -2437,7 +2441,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2448,7 +2452,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2459,7 +2463,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2470,7 +2474,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2498,11 +2502,7 @@
       <c r="B17" t="n">
         <v>77</v>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2614,7 +2614,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2625,7 +2625,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2636,7 +2636,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2647,7 +2647,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -2752,7 +2752,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -2767,7 +2767,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -2782,22 +2782,18 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>2</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -2808,7 +2804,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -2819,7 +2815,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -2830,7 +2826,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -2841,7 +2837,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2852,7 +2848,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2863,7 +2859,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2874,7 +2870,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2885,7 +2881,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2896,7 +2892,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2907,7 +2903,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -2918,7 +2914,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -2962,18 +2958,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>1</v>
       </c>
-      <c r="C23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2984,7 +2984,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2995,7 +2995,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -3006,7 +3006,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -3017,7 +3017,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -3028,7 +3028,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -3039,7 +3039,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -3412,7 +3412,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3433,7 +3433,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3592,30 +3592,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E4" t="n">
-        <v>27153</v>
+        <v>189374</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>606381</v>
+        <v>1757289</v>
       </c>
       <c r="H4" t="n">
-        <v>240451</v>
+        <v>250879</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -3666,30 +3666,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E6" t="n">
-        <v>71857</v>
+        <v>182900</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1929309</v>
+        <v>2098988</v>
       </c>
       <c r="H6" t="n">
-        <v>297407</v>
+        <v>182900</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -3703,30 +3703,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E7" t="n">
-        <v>30971</v>
+        <v>27153</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>820221</v>
+        <v>606381</v>
       </c>
       <c r="H7" t="n">
-        <v>58227</v>
+        <v>240451</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -3777,30 +3777,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E9" t="n">
-        <v>28582</v>
+        <v>453230</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>881388</v>
+        <v>5483351</v>
       </c>
       <c r="H9" t="n">
-        <v>239490</v>
+        <v>8188106</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -3814,30 +3814,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E10" t="n">
-        <v>15136</v>
+        <v>71857</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>983840</v>
+        <v>1929309</v>
       </c>
       <c r="H10" t="n">
-        <v>45077</v>
+        <v>297407</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -3851,30 +3851,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E11" t="n">
-        <v>182900</v>
+        <v>30971</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2098988</v>
+        <v>820221</v>
       </c>
       <c r="H11" t="n">
-        <v>182900</v>
+        <v>58227</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -3888,30 +3888,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E12" t="n">
-        <v>60517</v>
+        <v>273503</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2015/16</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1414622</v>
+        <v>1994005</v>
       </c>
       <c r="H12" t="n">
-        <v>339763</v>
+        <v>1917309</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -3925,30 +3925,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E13" t="n">
-        <v>189374</v>
+        <v>410102</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>1757289</v>
+        <v>2088802</v>
       </c>
       <c r="H13" t="n">
-        <v>250879</v>
+        <v>5360778</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -3958,34 +3958,34 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E14" t="n">
-        <v>37120</v>
+        <v>28582</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>1571193</v>
+        <v>881388</v>
       </c>
       <c r="H14" t="n">
-        <v>3349378</v>
+        <v>239490</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -3999,30 +3999,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E15" t="n">
-        <v>8917</v>
+        <v>486041</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>2118382</v>
+        <v>2415786</v>
       </c>
       <c r="H15" t="n">
-        <v>9146930</v>
+        <v>1206623</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4036,30 +4036,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E16" t="n">
-        <v>273503</v>
+        <v>15136</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1994005</v>
+        <v>983840</v>
       </c>
       <c r="H16" t="n">
-        <v>1917309</v>
+        <v>45077</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -4073,30 +4073,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D17" t="n">
         <v>7</v>
       </c>
       <c r="E17" t="n">
-        <v>31543</v>
+        <v>8917</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>820692</v>
+        <v>2118382</v>
       </c>
       <c r="H17" t="n">
-        <v>1637750</v>
+        <v>9146930</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4110,30 +4110,30 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E18" t="n">
-        <v>453230</v>
+        <v>31543</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>5483351</v>
+        <v>820692</v>
       </c>
       <c r="H18" t="n">
-        <v>8188106</v>
+        <v>1637750</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -4147,30 +4147,30 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="E19" t="n">
-        <v>1128645</v>
+        <v>60517</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2015/16</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>3434302</v>
+        <v>1414622</v>
       </c>
       <c r="H19" t="n">
-        <v>1128645</v>
+        <v>339763</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -4184,30 +4184,30 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E20" t="n">
-        <v>486041</v>
+        <v>37120</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>2415786</v>
+        <v>1571193</v>
       </c>
       <c r="H20" t="n">
-        <v>1206623</v>
+        <v>3349378</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -4221,30 +4221,30 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E21" t="n">
-        <v>410102</v>
+        <v>95791</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>2088802</v>
+        <v>2404119</v>
       </c>
       <c r="H21" t="n">
-        <v>5360778</v>
+        <v>5124417</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -4258,30 +4258,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E22" t="n">
-        <v>334016</v>
+        <v>1128645</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>2156629</v>
+        <v>3434302</v>
       </c>
       <c r="H22" t="n">
-        <v>2691725</v>
+        <v>1128645</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E23" t="n">
-        <v>14603</v>
+        <v>1615102</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2016/17</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>949628</v>
+        <v>4234674</v>
       </c>
       <c r="H23" t="n">
-        <v>515830</v>
+        <v>6092784</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E24" t="n">
-        <v>95791</v>
+        <v>14603</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2016/17</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2404119</v>
+        <v>949628</v>
       </c>
       <c r="H24" t="n">
-        <v>5124417</v>
+        <v>515830</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -4369,30 +4369,30 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E25" t="n">
-        <v>1615102</v>
+        <v>334016</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>4234674</v>
+        <v>2156629</v>
       </c>
       <c r="H25" t="n">
-        <v>6092784</v>
+        <v>2691725</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -4406,19 +4406,19 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E26" t="n">
-        <v>15288</v>
+        <v>1320699</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -4426,14 +4426,14 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>329510</v>
+        <v>2490743</v>
       </c>
       <c r="H26" t="n">
-        <v>538046</v>
+        <v>1861933</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2024/25</t>
         </is>
       </c>
     </row>
@@ -4480,19 +4480,19 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E28" t="n">
-        <v>1320699</v>
+        <v>15288</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -4500,14 +4500,14 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>2490743</v>
+        <v>329510</v>
       </c>
       <c r="H28" t="n">
-        <v>1861933</v>
+        <v>538046</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
     </row>
@@ -4773,7 +4773,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>350</v>
+        <v>383</v>
       </c>
       <c r="D2" t="n">
         <v>86</v>
@@ -4844,7 +4844,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>327</v>
+        <v>345</v>
       </c>
       <c r="D3" t="n">
         <v>81.2</v>
@@ -4902,40 +4902,40 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>322</v>
+        <v>339</v>
       </c>
       <c r="D4" t="n">
-        <v>78.2</v>
+        <v>71.8</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G4" t="n">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="H4" t="n">
         <v>2</v>
       </c>
       <c r="I4" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="J4" t="n">
         <v>3</v>
       </c>
       <c r="K4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -4944,29 +4944,29 @@
         <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="O4" t="n">
-        <v>100.5</v>
+        <v>100.8</v>
       </c>
       <c r="P4" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="Q4" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="R4" t="n">
-        <v>202778</v>
+        <v>954063</v>
       </c>
       <c r="S4" t="n">
-        <v>166751</v>
+        <v>3046343</v>
       </c>
       <c r="T4" t="n">
         <v>2</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
@@ -4982,7 +4982,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>319</v>
+        <v>335</v>
       </c>
       <c r="D5" t="n">
         <v>78.8</v>
@@ -5044,111 +5044,111 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>318</v>
+        <v>331</v>
       </c>
       <c r="D6" t="n">
-        <v>78.5</v>
+        <v>74.2</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="G6" t="n">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="H6" t="n">
         <v>2</v>
       </c>
       <c r="I6" t="n">
+        <v>53</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
         <v>45</v>
       </c>
-      <c r="J6" t="n">
-        <v>3</v>
-      </c>
-      <c r="K6" t="n">
+      <c r="O6" t="n">
+        <v>101</v>
+      </c>
+      <c r="P6" t="n">
         <v>1</v>
       </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="n">
-        <v>66</v>
-      </c>
-      <c r="O6" t="n">
-        <v>101.6</v>
-      </c>
-      <c r="P6" t="n">
-        <v>1.6</v>
-      </c>
       <c r="Q6" t="n">
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>307625</v>
+        <v>812374</v>
       </c>
       <c r="S6" t="n">
-        <v>266328</v>
+        <v>3039834</v>
       </c>
       <c r="T6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>310</v>
+        <v>328</v>
       </c>
       <c r="D7" t="n">
-        <v>74.8</v>
+        <v>78.2</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F7" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G7" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H7" t="n">
         <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="J7" t="n">
         <v>3</v>
       </c>
       <c r="K7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -5157,29 +5157,29 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="O7" t="n">
-        <v>101.3</v>
+        <v>100.5</v>
       </c>
       <c r="P7" t="n">
-        <v>1.3</v>
+        <v>0.5</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.2</v>
+        <v>2.5</v>
       </c>
       <c r="R7" t="n">
-        <v>473776</v>
+        <v>202778</v>
       </c>
       <c r="S7" t="n">
-        <v>1034411</v>
+        <v>166751</v>
       </c>
       <c r="T7" t="n">
         <v>2</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>
@@ -5195,7 +5195,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>309</v>
+        <v>325</v>
       </c>
       <c r="D8" t="n">
         <v>76.2</v>
@@ -5257,37 +5257,37 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>307</v>
+        <v>324</v>
       </c>
       <c r="D9" t="n">
-        <v>76.2</v>
+        <v>71.5</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
-        <v>78</v>
+        <v>99</v>
       </c>
       <c r="G9" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="H9" t="n">
         <v>2</v>
       </c>
       <c r="I9" t="n">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="J9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
         <v>2</v>
@@ -5299,69 +5299,69 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="O9" t="n">
-        <v>101.8</v>
+        <v>100.4</v>
       </c>
       <c r="P9" t="n">
-        <v>1.8</v>
+        <v>0.4</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.2</v>
+        <v>1.3</v>
       </c>
       <c r="R9" t="n">
-        <v>572310</v>
+        <v>1540631</v>
       </c>
       <c r="S9" t="n">
-        <v>466127</v>
+        <v>3009015</v>
       </c>
       <c r="T9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>304</v>
+        <v>322</v>
       </c>
       <c r="D10" t="n">
-        <v>75</v>
+        <v>78.5</v>
       </c>
       <c r="E10" t="n">
         <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="G10" t="n">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="H10" t="n">
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="J10" t="n">
         <v>3</v>
       </c>
       <c r="K10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -5370,66 +5370,66 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="O10" t="n">
-        <v>100.4</v>
+        <v>101.6</v>
       </c>
       <c r="P10" t="n">
-        <v>0.4</v>
+        <v>1.6</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>692223</v>
+        <v>307625</v>
       </c>
       <c r="S10" t="n">
-        <v>637992</v>
+        <v>266328</v>
       </c>
       <c r="T10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>301</v>
+        <v>321</v>
       </c>
       <c r="D11" t="n">
-        <v>74.2</v>
+        <v>74.8</v>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="G11" t="n">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="H11" t="n">
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K11" t="n">
         <v>2</v>
@@ -5441,69 +5441,69 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="O11" t="n">
-        <v>101</v>
+        <v>101.3</v>
       </c>
       <c r="P11" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="Q11" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="R11" t="n">
-        <v>812374</v>
+        <v>473776</v>
       </c>
       <c r="S11" t="n">
-        <v>3039834</v>
+        <v>1034411</v>
       </c>
       <c r="T11" t="n">
         <v>2</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>299</v>
+        <v>315</v>
       </c>
       <c r="D12" t="n">
-        <v>73.2</v>
+        <v>71</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="G12" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H12" t="n">
         <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="J12" t="n">
         <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -5512,130 +5512,134 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="O12" t="n">
-        <v>100.3</v>
+        <v>100.9</v>
       </c>
       <c r="P12" t="n">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
       <c r="Q12" t="n">
-        <v>2.7</v>
+        <v>0.6</v>
       </c>
       <c r="R12" t="n">
-        <v>1029192</v>
+        <v>1531354</v>
       </c>
       <c r="S12" t="n">
-        <v>4399137</v>
+        <v>5881370</v>
       </c>
       <c r="T12" t="n">
         <v>2</v>
       </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>3xc, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>298</v>
+        <v>315</v>
       </c>
       <c r="D13" t="n">
-        <v>71.8</v>
+        <v>70</v>
       </c>
       <c r="E13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" t="n">
+        <v>81</v>
+      </c>
+      <c r="G13" t="n">
+        <v>107</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" t="n">
+        <v>44</v>
+      </c>
+      <c r="J13" t="n">
         <v>1</v>
       </c>
-      <c r="F13" t="n">
-        <v>78</v>
-      </c>
-      <c r="G13" t="n">
-        <v>113</v>
-      </c>
-      <c r="H13" t="n">
-        <v>2</v>
-      </c>
-      <c r="I13" t="n">
+      <c r="K13" t="n">
+        <v>2</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="n">
         <v>45</v>
       </c>
-      <c r="J13" t="n">
-        <v>3</v>
-      </c>
-      <c r="K13" t="n">
-        <v>2</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" t="n">
-        <v>40</v>
-      </c>
       <c r="O13" t="n">
-        <v>100.8</v>
+        <v>100.6</v>
       </c>
       <c r="P13" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="Q13" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="R13" t="n">
-        <v>954063</v>
+        <v>1824730</v>
       </c>
       <c r="S13" t="n">
-        <v>3046343</v>
+        <v>4185865</v>
       </c>
       <c r="T13" t="n">
         <v>2</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>298</v>
+        <v>312</v>
       </c>
       <c r="D14" t="n">
-        <v>71.8</v>
+        <v>76.2</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="G14" t="n">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="H14" t="n">
         <v>2</v>
       </c>
       <c r="I14" t="n">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="J14" t="n">
         <v>3</v>
@@ -5650,66 +5654,66 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="O14" t="n">
-        <v>101.2</v>
+        <v>101.8</v>
       </c>
       <c r="P14" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="Q14" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
       <c r="R14" t="n">
-        <v>954063</v>
+        <v>572310</v>
       </c>
       <c r="S14" t="n">
-        <v>101935</v>
+        <v>466127</v>
       </c>
       <c r="T14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>295</v>
+        <v>310</v>
       </c>
       <c r="D15" t="n">
-        <v>72.2</v>
+        <v>70.8</v>
       </c>
       <c r="E15" t="n">
         <v>2</v>
       </c>
       <c r="F15" t="n">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="G15" t="n">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="J15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5721,69 +5725,69 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="O15" t="n">
-        <v>101.4</v>
+        <v>101.1</v>
       </c>
       <c r="P15" t="n">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="R15" t="n">
-        <v>1225264</v>
+        <v>1750909</v>
       </c>
       <c r="S15" t="n">
-        <v>878473</v>
+        <v>5250200</v>
       </c>
       <c r="T15" t="n">
         <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>290</v>
+        <v>310</v>
       </c>
       <c r="D16" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="G16" t="n">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
@@ -5792,63 +5796,63 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="O16" t="n">
-        <v>100.9</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
         <v>0.6</v>
       </c>
       <c r="R16" t="n">
-        <v>1531354</v>
+        <v>692223</v>
       </c>
       <c r="S16" t="n">
-        <v>5881370</v>
+        <v>637992</v>
       </c>
       <c r="T16" t="n">
         <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>289</v>
+        <v>309</v>
       </c>
       <c r="D17" t="n">
-        <v>71.2</v>
+        <v>72.2</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
-        <v>105</v>
+        <v>78</v>
       </c>
       <c r="G17" t="n">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H17" t="n">
         <v>2</v>
       </c>
       <c r="I17" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="J17" t="n">
         <v>3</v>
@@ -5863,66 +5867,66 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="O17" t="n">
-        <v>100.9</v>
+        <v>101.4</v>
       </c>
       <c r="P17" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="Q17" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="R17" t="n">
-        <v>1474444</v>
+        <v>1225264</v>
       </c>
       <c r="S17" t="n">
-        <v>1066412</v>
+        <v>878473</v>
       </c>
       <c r="T17" t="n">
         <v>2</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>288</v>
+        <v>308</v>
       </c>
       <c r="D18" t="n">
-        <v>71.5</v>
+        <v>71.2</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G18" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="H18" t="n">
         <v>2</v>
       </c>
       <c r="I18" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K18" t="n">
         <v>2</v>
@@ -5934,137 +5938,133 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="O18" t="n">
-        <v>100.4</v>
+        <v>100.9</v>
       </c>
       <c r="P18" t="n">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
       <c r="Q18" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="R18" t="n">
-        <v>1540631</v>
+        <v>1474444</v>
       </c>
       <c r="S18" t="n">
-        <v>3009015</v>
+        <v>1066412</v>
       </c>
       <c r="T18" t="n">
         <v>2</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>287</v>
+        <v>307</v>
       </c>
       <c r="D19" t="n">
-        <v>71.8</v>
+        <v>73.2</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="G19" t="n">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="H19" t="n">
         <v>2</v>
       </c>
       <c r="I19" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="J19" t="n">
         <v>1</v>
       </c>
       <c r="K19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="O19" t="n">
-        <v>100.6</v>
+        <v>100.3</v>
       </c>
       <c r="P19" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.7</v>
+        <v>2.7</v>
       </c>
       <c r="R19" t="n">
-        <v>1804185</v>
+        <v>1029192</v>
       </c>
       <c r="S19" t="n">
-        <v>3048395</v>
+        <v>4399137</v>
       </c>
       <c r="T19" t="n">
         <v>2</v>
       </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>3xc, wildcard</t>
-        </is>
-      </c>
+      <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>285</v>
+        <v>301</v>
       </c>
       <c r="D20" t="n">
-        <v>70.8</v>
+        <v>71.8</v>
       </c>
       <c r="E20" t="n">
         <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="G20" t="n">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="H20" t="n">
         <v>2</v>
       </c>
       <c r="I20" t="n">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K20" t="n">
         <v>2</v>
@@ -6076,69 +6076,69 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="O20" t="n">
-        <v>101.1</v>
+        <v>101.2</v>
       </c>
       <c r="P20" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="Q20" t="n">
         <v>1.1</v>
       </c>
-      <c r="Q20" t="n">
-        <v>0.5</v>
-      </c>
       <c r="R20" t="n">
-        <v>1750909</v>
+        <v>954063</v>
       </c>
       <c r="S20" t="n">
-        <v>5250200</v>
+        <v>101935</v>
       </c>
       <c r="T20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>284</v>
+        <v>299</v>
       </c>
       <c r="D21" t="n">
-        <v>70</v>
+        <v>67.5</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="G21" t="n">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="H21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I21" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J21" t="n">
         <v>1</v>
       </c>
       <c r="K21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L21" t="n">
         <v>0</v>
@@ -6147,136 +6147,140 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="O21" t="n">
-        <v>100.6</v>
+        <v>101.9</v>
       </c>
       <c r="P21" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="Q21" t="n">
         <v>0.6</v>
       </c>
-      <c r="Q21" t="n">
-        <v>0.4</v>
-      </c>
       <c r="R21" t="n">
-        <v>1824730</v>
+        <v>2653099</v>
       </c>
       <c r="S21" t="n">
-        <v>4185865</v>
+        <v>2489160</v>
       </c>
       <c r="T21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>280</v>
+        <v>297</v>
       </c>
       <c r="D22" t="n">
-        <v>67.5</v>
+        <v>71.8</v>
       </c>
       <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="n">
+        <v>67</v>
+      </c>
+      <c r="G22" t="n">
+        <v>97</v>
+      </c>
+      <c r="H22" t="n">
+        <v>2</v>
+      </c>
+      <c r="I22" t="n">
+        <v>43</v>
+      </c>
+      <c r="J22" t="n">
         <v>1</v>
       </c>
-      <c r="F22" t="n">
-        <v>72</v>
-      </c>
-      <c r="G22" t="n">
-        <v>96</v>
-      </c>
-      <c r="H22" t="n">
-        <v>2</v>
-      </c>
-      <c r="I22" t="n">
-        <v>38</v>
-      </c>
-      <c r="J22" t="n">
-        <v>3</v>
-      </c>
       <c r="K22" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M22" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="N22" t="n">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="O22" t="n">
-        <v>101.1</v>
+        <v>100.6</v>
       </c>
       <c r="P22" t="n">
-        <v>1.1</v>
+        <v>0.6</v>
       </c>
       <c r="Q22" t="n">
-        <v>1.1</v>
+        <v>0.7</v>
       </c>
       <c r="R22" t="n">
-        <v>2310073</v>
+        <v>1804185</v>
       </c>
       <c r="S22" t="n">
-        <v>453361</v>
+        <v>3048395</v>
       </c>
       <c r="T22" t="n">
         <v>2</v>
       </c>
-      <c r="U22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>3xc, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>277</v>
+        <v>296</v>
       </c>
       <c r="D23" t="n">
-        <v>68.8</v>
+        <v>67.2</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="G23" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="H23" t="n">
         <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="J23" t="n">
         <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L23" t="n">
         <v>0</v>
@@ -6285,48 +6289,48 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="O23" t="n">
-        <v>101.7</v>
+        <v>100.2</v>
       </c>
       <c r="P23" t="n">
-        <v>1.7</v>
+        <v>0.2</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.4</v>
+        <v>1.8</v>
       </c>
       <c r="R23" t="n">
-        <v>2382054</v>
+        <v>2920591</v>
       </c>
       <c r="S23" t="n">
-        <v>2735246</v>
+        <v>1595922</v>
       </c>
       <c r="T23" t="n">
         <v>2</v>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>bboost, 3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>276</v>
+        <v>293</v>
       </c>
       <c r="D24" t="n">
-        <v>67.5</v>
+        <v>68.8</v>
       </c>
       <c r="E24" t="n">
         <v>1</v>
@@ -6338,16 +6342,16 @@
         <v>93</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="J24" t="n">
         <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
@@ -6356,25 +6360,25 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="O24" t="n">
-        <v>101.9</v>
+        <v>101.7</v>
       </c>
       <c r="P24" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="R24" t="n">
-        <v>2653099</v>
+        <v>2382054</v>
       </c>
       <c r="S24" t="n">
-        <v>2489160</v>
+        <v>2735246</v>
       </c>
       <c r="T24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U24" t="inlineStr">
         <is>
@@ -6385,37 +6389,37 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>273</v>
+        <v>290</v>
       </c>
       <c r="D25" t="n">
-        <v>67.2</v>
+        <v>67.5</v>
       </c>
       <c r="E25" t="n">
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="G25" t="n">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="H25" t="n">
         <v>2</v>
       </c>
       <c r="I25" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="J25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K25" t="n">
         <v>3</v>
@@ -6427,100 +6431,96 @@
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="O25" t="n">
-        <v>100.2</v>
+        <v>101.1</v>
       </c>
       <c r="P25" t="n">
-        <v>0.2</v>
+        <v>1.1</v>
       </c>
       <c r="Q25" t="n">
-        <v>1.8</v>
+        <v>1.1</v>
       </c>
       <c r="R25" t="n">
-        <v>2920591</v>
+        <v>2310073</v>
       </c>
       <c r="S25" t="n">
-        <v>1595922</v>
+        <v>453361</v>
       </c>
       <c r="T25" t="n">
         <v>2</v>
       </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>bboost, 3xc, wildcard</t>
-        </is>
-      </c>
+      <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>268</v>
+        <v>290</v>
       </c>
       <c r="D26" t="n">
-        <v>66.5</v>
+        <v>66.8</v>
       </c>
       <c r="E26" t="n">
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="G26" t="n">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="H26" t="n">
+        <v>2</v>
+      </c>
+      <c r="I26" t="n">
+        <v>46</v>
+      </c>
+      <c r="J26" t="n">
         <v>3</v>
       </c>
-      <c r="I26" t="n">
-        <v>41</v>
-      </c>
-      <c r="J26" t="n">
-        <v>1</v>
-      </c>
       <c r="K26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M26" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="N26" t="n">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="O26" t="n">
-        <v>100.8</v>
+        <v>101.1</v>
       </c>
       <c r="P26" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="Q26" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="R26" t="n">
-        <v>3408831</v>
+        <v>3529354</v>
       </c>
       <c r="S26" t="n">
-        <v>3395267</v>
+        <v>1948104</v>
       </c>
       <c r="T26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>3xc</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
@@ -6536,7 +6536,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>267</v>
+        <v>284</v>
       </c>
       <c r="D27" t="n">
         <v>65.8</v>
@@ -6598,71 +6598,71 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>267</v>
+        <v>281</v>
       </c>
       <c r="D28" t="n">
-        <v>66.8</v>
+        <v>66.5</v>
       </c>
       <c r="E28" t="n">
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="G28" t="n">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="H28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I28" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="J28" t="n">
+        <v>1</v>
+      </c>
+      <c r="K28" t="n">
+        <v>4</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" t="n">
+        <v>33</v>
+      </c>
+      <c r="O28" t="n">
+        <v>100.8</v>
+      </c>
+      <c r="P28" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" t="n">
+        <v>3408831</v>
+      </c>
+      <c r="S28" t="n">
+        <v>3395267</v>
+      </c>
+      <c r="T28" t="n">
         <v>3</v>
       </c>
-      <c r="K28" t="n">
-        <v>5</v>
-      </c>
-      <c r="L28" t="n">
-        <v>2</v>
-      </c>
-      <c r="M28" t="n">
-        <v>-8</v>
-      </c>
-      <c r="N28" t="n">
-        <v>55</v>
-      </c>
-      <c r="O28" t="n">
-        <v>101.1</v>
-      </c>
-      <c r="P28" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="R28" t="n">
-        <v>3529354</v>
-      </c>
-      <c r="S28" t="n">
-        <v>1948104</v>
-      </c>
-      <c r="T28" t="n">
-        <v>2</v>
-      </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>3xc</t>
         </is>
       </c>
     </row>
@@ -6678,7 +6678,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>251</v>
+        <v>272</v>
       </c>
       <c r="D29" t="n">
         <v>61.8</v>
@@ -6749,7 +6749,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>234</v>
+        <v>258</v>
       </c>
       <c r="D30" t="n">
         <v>58</v>
@@ -6820,7 +6820,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="D31" t="n">
         <v>56.8</v>
@@ -6891,7 +6891,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D32" t="n">
         <v>46.8</v>

</xml_diff>

<commit_message>
Update standings 2026-09-19 20:07 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -508,13 +508,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="4">
@@ -556,13 +556,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E5" t="n">
         <v>-4</v>
       </c>
       <c r="F5" t="n">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="6">
@@ -580,13 +580,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="7">
@@ -595,22 +595,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="8">
@@ -619,22 +619,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="9">
@@ -652,13 +652,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="10">
@@ -700,13 +700,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="12">
@@ -715,22 +715,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>315</v>
+        <v>318</v>
       </c>
     </row>
     <row r="13">
@@ -739,22 +739,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="14">
@@ -763,22 +763,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>312</v>
+        <v>316</v>
       </c>
     </row>
     <row r="15">
@@ -787,22 +787,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>310</v>
+        <v>314</v>
       </c>
     </row>
     <row r="16">
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -835,16 +835,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -855,26 +855,26 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="19">
@@ -883,22 +883,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="20">
@@ -907,22 +907,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
     <row r="21">
@@ -940,13 +940,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="22">
@@ -1012,13 +1012,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="25">
@@ -1027,22 +1027,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="F25" t="n">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="26">
@@ -1051,19 +1051,19 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E26" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
         <v>290</v>
@@ -1084,13 +1084,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="28">
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="30">
@@ -1156,13 +1156,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E30" t="n">
         <v>-8</v>
       </c>
       <c r="F30" t="n">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="31">
@@ -1686,39 +1686,39 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="C7" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D7" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="E7" t="n">
-        <v>84</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="C8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D8" t="n">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="E8" t="n">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9">
@@ -1781,172 +1781,172 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C12" t="n">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D12" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E12" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C13" t="n">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="D13" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E13" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B14" t="n">
+        <v>44</v>
+      </c>
+      <c r="C14" t="n">
+        <v>107</v>
+      </c>
+      <c r="D14" t="n">
+        <v>56</v>
+      </c>
+      <c r="E14" t="n">
         <v>73</v>
-      </c>
-      <c r="C14" t="n">
-        <v>104</v>
-      </c>
-      <c r="D14" t="n">
-        <v>37</v>
-      </c>
-      <c r="E14" t="n">
-        <v>91</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="D15" t="n">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="E15" t="n">
-        <v>75</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C16" t="n">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D16" t="n">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="E16" t="n">
-        <v>62</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C17" t="n">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D17" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="E17" t="n">
-        <v>70</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="C18" t="n">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="D18" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E18" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="C19" t="n">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="D19" t="n">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="E19" t="n">
-        <v>76</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>73</v>
+        <v>48</v>
       </c>
       <c r="C20" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="D20" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="E20" t="n">
-        <v>69</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21">
@@ -2028,39 +2028,39 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C25" t="n">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D25" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E25" t="n">
-        <v>77</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C26" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D26" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E26" t="n">
-        <v>66</v>
+        <v>77</v>
       </c>
     </row>
     <row r="27">
@@ -2782,7 +2782,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -2793,7 +2793,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -3006,7 +3006,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -3017,7 +3017,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -3286,7 +3286,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3307,7 +3307,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -3412,7 +3412,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3433,7 +3433,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3703,30 +3703,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E7" t="n">
-        <v>27153</v>
+        <v>6474</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>606381</v>
+        <v>1177681</v>
       </c>
       <c r="H7" t="n">
-        <v>240451</v>
+        <v>6474</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -3740,30 +3740,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E8" t="n">
-        <v>6474</v>
+        <v>27153</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>1177681</v>
+        <v>606381</v>
       </c>
       <c r="H8" t="n">
-        <v>6474</v>
+        <v>240451</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -3888,19 +3888,19 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>273503</v>
+        <v>486041</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -3908,10 +3908,10 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1994005</v>
+        <v>2415786</v>
       </c>
       <c r="H12" t="n">
-        <v>1917309</v>
+        <v>1206623</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -3925,30 +3925,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E13" t="n">
-        <v>410102</v>
+        <v>273503</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>2088802</v>
+        <v>1994005</v>
       </c>
       <c r="H13" t="n">
-        <v>5360778</v>
+        <v>1917309</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -3962,30 +3962,30 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E14" t="n">
-        <v>28582</v>
+        <v>410102</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>881388</v>
+        <v>2088802</v>
       </c>
       <c r="H14" t="n">
-        <v>239490</v>
+        <v>5360778</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -3999,30 +3999,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E15" t="n">
-        <v>486041</v>
+        <v>28582</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>2415786</v>
+        <v>881388</v>
       </c>
       <c r="H15" t="n">
-        <v>1206623</v>
+        <v>239490</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4036,19 +4036,19 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E16" t="n">
-        <v>15136</v>
+        <v>8917</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -4056,10 +4056,10 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>983840</v>
+        <v>2118382</v>
       </c>
       <c r="H16" t="n">
-        <v>45077</v>
+        <v>9146930</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -4073,30 +4073,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D17" t="n">
         <v>7</v>
       </c>
       <c r="E17" t="n">
-        <v>8917</v>
+        <v>31543</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>2118382</v>
+        <v>820692</v>
       </c>
       <c r="H17" t="n">
-        <v>9146930</v>
+        <v>1637750</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4106,34 +4106,34 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E18" t="n">
-        <v>31543</v>
+        <v>37120</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>820692</v>
+        <v>1571193</v>
       </c>
       <c r="H18" t="n">
-        <v>1637750</v>
+        <v>3349378</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -4147,30 +4147,30 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E19" t="n">
-        <v>60517</v>
+        <v>15136</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2015/16</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>1414622</v>
+        <v>983840</v>
       </c>
       <c r="H19" t="n">
-        <v>339763</v>
+        <v>45077</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -4184,30 +4184,30 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E20" t="n">
-        <v>37120</v>
+        <v>60517</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2015/16</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>1571193</v>
+        <v>1414622</v>
       </c>
       <c r="H20" t="n">
-        <v>3349378</v>
+        <v>339763</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -4369,19 +4369,19 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E25" t="n">
-        <v>334016</v>
+        <v>1320699</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -4389,14 +4389,14 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>2156629</v>
+        <v>2490743</v>
       </c>
       <c r="H25" t="n">
-        <v>2691725</v>
+        <v>1861933</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2024/25</t>
         </is>
       </c>
     </row>
@@ -4406,19 +4406,19 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E26" t="n">
-        <v>1320699</v>
+        <v>334016</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -4426,14 +4426,14 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>2490743</v>
+        <v>2156629</v>
       </c>
       <c r="H26" t="n">
-        <v>1861933</v>
+        <v>2691725</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
     </row>
@@ -4844,7 +4844,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D3" t="n">
         <v>81.2</v>
@@ -4982,7 +4982,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D5" t="n">
         <v>78.8</v>
@@ -5053,7 +5053,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="D6" t="n">
         <v>74.2</v>
@@ -5115,34 +5115,34 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D7" t="n">
-        <v>78.2</v>
+        <v>76.2</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="G7" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H7" t="n">
         <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="J7" t="n">
         <v>3</v>
@@ -5157,22 +5157,22 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>35</v>
+        <v>57</v>
       </c>
       <c r="O7" t="n">
-        <v>100.5</v>
+        <v>101</v>
       </c>
       <c r="P7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" t="n">
         <v>0.5</v>
       </c>
-      <c r="Q7" t="n">
-        <v>2.5</v>
-      </c>
       <c r="R7" t="n">
-        <v>202778</v>
+        <v>590503</v>
       </c>
       <c r="S7" t="n">
-        <v>166751</v>
+        <v>617418</v>
       </c>
       <c r="T7" t="n">
         <v>2</v>
@@ -5186,34 +5186,34 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D8" t="n">
-        <v>76.2</v>
+        <v>78.2</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F8" t="n">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="G8" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H8" t="n">
         <v>2</v>
       </c>
       <c r="I8" t="n">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="J8" t="n">
         <v>3</v>
@@ -5228,22 +5228,22 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="O8" t="n">
-        <v>101</v>
+        <v>100.5</v>
       </c>
       <c r="P8" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="R8" t="n">
-        <v>590503</v>
+        <v>202778</v>
       </c>
       <c r="S8" t="n">
-        <v>617418</v>
+        <v>166751</v>
       </c>
       <c r="T8" t="n">
         <v>2</v>
@@ -5266,7 +5266,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D9" t="n">
         <v>71.5</v>
@@ -5408,7 +5408,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D11" t="n">
         <v>74.8</v>
@@ -5470,40 +5470,40 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="D12" t="n">
-        <v>71</v>
+        <v>70.8</v>
       </c>
       <c r="E12" t="n">
         <v>2</v>
       </c>
       <c r="F12" t="n">
-        <v>95</v>
+        <v>57</v>
       </c>
       <c r="G12" t="n">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="H12" t="n">
         <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J12" t="n">
         <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -5512,22 +5512,22 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="O12" t="n">
-        <v>100.9</v>
+        <v>101.1</v>
       </c>
       <c r="P12" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="R12" t="n">
-        <v>1531354</v>
+        <v>1750909</v>
       </c>
       <c r="S12" t="n">
-        <v>5881370</v>
+        <v>5250200</v>
       </c>
       <c r="T12" t="n">
         <v>2</v>
@@ -5541,40 +5541,40 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D13" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E13" t="n">
         <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="G13" t="n">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="H13" t="n">
         <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J13" t="n">
         <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -5583,66 +5583,66 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="O13" t="n">
-        <v>100.6</v>
+        <v>100.9</v>
       </c>
       <c r="P13" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q13" t="n">
         <v>0.6</v>
       </c>
-      <c r="Q13" t="n">
-        <v>0.4</v>
-      </c>
       <c r="R13" t="n">
-        <v>1824730</v>
+        <v>1531354</v>
       </c>
       <c r="S13" t="n">
-        <v>4185865</v>
+        <v>5881370</v>
       </c>
       <c r="T13" t="n">
         <v>2</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="D14" t="n">
-        <v>76.2</v>
+        <v>70</v>
       </c>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F14" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="G14" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="H14" t="n">
         <v>2</v>
       </c>
       <c r="I14" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="J14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
         <v>2</v>
@@ -5654,66 +5654,66 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="O14" t="n">
-        <v>101.8</v>
+        <v>100.6</v>
       </c>
       <c r="P14" t="n">
-        <v>1.8</v>
+        <v>0.6</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="R14" t="n">
-        <v>572310</v>
+        <v>1824730</v>
       </c>
       <c r="S14" t="n">
-        <v>466127</v>
+        <v>4185865</v>
       </c>
       <c r="T14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="D15" t="n">
-        <v>70.8</v>
+        <v>76.2</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="G15" t="n">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5725,69 +5725,69 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="O15" t="n">
-        <v>101.1</v>
+        <v>101.8</v>
       </c>
       <c r="P15" t="n">
-        <v>1.1</v>
+        <v>1.8</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="R15" t="n">
-        <v>1750909</v>
+        <v>572310</v>
       </c>
       <c r="S15" t="n">
-        <v>5250200</v>
+        <v>466127</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="C16" t="n">
         <v>310</v>
       </c>
       <c r="D16" t="n">
-        <v>75</v>
+        <v>72.2</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" t="n">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="G16" t="n">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
         <v>3</v>
       </c>
       <c r="K16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
@@ -5796,63 +5796,63 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.4</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="R16" t="n">
-        <v>692223</v>
+        <v>1225264</v>
       </c>
       <c r="S16" t="n">
-        <v>637992</v>
+        <v>878473</v>
       </c>
       <c r="T16" t="n">
         <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C17" t="n">
         <v>309</v>
       </c>
       <c r="D17" t="n">
-        <v>72.2</v>
+        <v>71.2</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>78</v>
+        <v>105</v>
       </c>
       <c r="G17" t="n">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H17" t="n">
         <v>2</v>
       </c>
       <c r="I17" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="J17" t="n">
         <v>3</v>
@@ -5867,63 +5867,63 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="O17" t="n">
-        <v>101.4</v>
+        <v>100.9</v>
       </c>
       <c r="P17" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>1225264</v>
+        <v>1474444</v>
       </c>
       <c r="S17" t="n">
-        <v>878473</v>
+        <v>1066412</v>
       </c>
       <c r="T17" t="n">
         <v>2</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D18" t="n">
-        <v>71.2</v>
+        <v>71.8</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
-        <v>105</v>
+        <v>62</v>
       </c>
       <c r="G18" t="n">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="H18" t="n">
         <v>2</v>
       </c>
       <c r="I18" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J18" t="n">
         <v>3</v>
@@ -5938,136 +5938,140 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="O18" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P18" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q18" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="R18" t="n">
-        <v>1474444</v>
+        <v>954063</v>
       </c>
       <c r="S18" t="n">
-        <v>1066412</v>
+        <v>101935</v>
       </c>
       <c r="T18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="D19" t="n">
-        <v>73.2</v>
+        <v>75</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F19" t="n">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="G19" t="n">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="H19" t="n">
         <v>2</v>
       </c>
       <c r="I19" t="n">
+        <v>61</v>
+      </c>
+      <c r="J19" t="n">
+        <v>3</v>
+      </c>
+      <c r="K19" t="n">
+        <v>3</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="n">
         <v>48</v>
       </c>
-      <c r="J19" t="n">
-        <v>1</v>
-      </c>
-      <c r="K19" t="n">
-        <v>4</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" t="n">
-        <v>56</v>
-      </c>
       <c r="O19" t="n">
-        <v>100.3</v>
+        <v>100.4</v>
       </c>
       <c r="P19" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="Q19" t="n">
-        <v>2.7</v>
+        <v>0.6</v>
       </c>
       <c r="R19" t="n">
-        <v>1029192</v>
+        <v>692223</v>
       </c>
       <c r="S19" t="n">
-        <v>4399137</v>
+        <v>637992</v>
       </c>
       <c r="T19" t="n">
         <v>2</v>
       </c>
-      <c r="U19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>bboost, 3xc</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="D20" t="n">
-        <v>71.8</v>
+        <v>73.2</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="G20" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="H20" t="n">
         <v>2</v>
       </c>
       <c r="I20" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="J20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L20" t="n">
         <v>0</v>
@@ -6076,31 +6080,27 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="O20" t="n">
-        <v>101.2</v>
+        <v>100.3</v>
       </c>
       <c r="P20" t="n">
-        <v>1.2</v>
+        <v>0.3</v>
       </c>
       <c r="Q20" t="n">
-        <v>1.1</v>
+        <v>2.7</v>
       </c>
       <c r="R20" t="n">
-        <v>954063</v>
+        <v>1029192</v>
       </c>
       <c r="S20" t="n">
-        <v>101935</v>
+        <v>4399137</v>
       </c>
       <c r="T20" t="n">
-        <v>3</v>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>bboost</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6114,7 +6114,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D21" t="n">
         <v>67.5</v>
@@ -6327,7 +6327,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D24" t="n">
         <v>68.8</v>
@@ -6389,49 +6389,49 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D25" t="n">
-        <v>67.5</v>
+        <v>66.8</v>
       </c>
       <c r="E25" t="n">
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="G25" t="n">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="H25" t="n">
         <v>2</v>
       </c>
       <c r="I25" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="J25" t="n">
         <v>3</v>
       </c>
       <c r="K25" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M25" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="N25" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="O25" t="n">
         <v>101.1</v>
@@ -6440,65 +6440,69 @@
         <v>1.1</v>
       </c>
       <c r="Q25" t="n">
-        <v>1.1</v>
+        <v>0.1</v>
       </c>
       <c r="R25" t="n">
-        <v>2310073</v>
+        <v>3529354</v>
       </c>
       <c r="S25" t="n">
-        <v>453361</v>
+        <v>1948104</v>
       </c>
       <c r="T25" t="n">
         <v>2</v>
       </c>
-      <c r="U25" t="inlineStr"/>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C26" t="n">
         <v>290</v>
       </c>
       <c r="D26" t="n">
-        <v>66.8</v>
+        <v>67.5</v>
       </c>
       <c r="E26" t="n">
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G26" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="H26" t="n">
         <v>2</v>
       </c>
       <c r="I26" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="J26" t="n">
         <v>3</v>
       </c>
       <c r="K26" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="O26" t="n">
         <v>101.1</v>
@@ -6507,22 +6511,18 @@
         <v>1.1</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.1</v>
+        <v>1.1</v>
       </c>
       <c r="R26" t="n">
-        <v>3529354</v>
+        <v>2310073</v>
       </c>
       <c r="S26" t="n">
-        <v>1948104</v>
+        <v>453361</v>
       </c>
       <c r="T26" t="n">
         <v>2</v>
       </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+      <c r="U26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6536,7 +6536,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D27" t="n">
         <v>65.8</v>
@@ -6678,7 +6678,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D29" t="n">
         <v>61.8</v>
@@ -6749,7 +6749,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D30" t="n">
         <v>58</v>

</xml_diff>

<commit_message>
Update standings 2026-09-19 23:55 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -4806,7 +4806,7 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="O2" t="n">
         <v>101.5</v>
@@ -4818,7 +4818,7 @@
         <v>2.4</v>
       </c>
       <c r="R2" t="n">
-        <v>10970</v>
+        <v>2278</v>
       </c>
       <c r="S2" t="n">
         <v>270274</v>
@@ -4877,7 +4877,7 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="O3" t="n">
         <v>100.8</v>
@@ -4889,7 +4889,7 @@
         <v>0.2</v>
       </c>
       <c r="R3" t="n">
-        <v>125992</v>
+        <v>152850</v>
       </c>
       <c r="S3" t="n">
         <v>1461471</v>
@@ -4944,7 +4944,7 @@
         <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="O4" t="n">
         <v>100.8</v>
@@ -4956,7 +4956,7 @@
         <v>1</v>
       </c>
       <c r="R4" t="n">
-        <v>954063</v>
+        <v>241342</v>
       </c>
       <c r="S4" t="n">
         <v>3046343</v>
@@ -5015,7 +5015,7 @@
         <v>-4</v>
       </c>
       <c r="N5" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="O5" t="n">
         <v>101.6</v>
@@ -5027,7 +5027,7 @@
         <v>0.7</v>
       </c>
       <c r="R5" t="n">
-        <v>298748</v>
+        <v>330274</v>
       </c>
       <c r="S5" t="n">
         <v>1229264</v>
@@ -5086,7 +5086,7 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="O6" t="n">
         <v>101</v>
@@ -5098,7 +5098,7 @@
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>812374</v>
+        <v>387912</v>
       </c>
       <c r="S6" t="n">
         <v>3039834</v>
@@ -5157,7 +5157,7 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="O7" t="n">
         <v>101</v>
@@ -5169,7 +5169,7 @@
         <v>0.5</v>
       </c>
       <c r="R7" t="n">
-        <v>590503</v>
+        <v>573851</v>
       </c>
       <c r="S7" t="n">
         <v>617418</v>
@@ -5228,7 +5228,7 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="O8" t="n">
         <v>100.5</v>
@@ -5240,7 +5240,7 @@
         <v>2.5</v>
       </c>
       <c r="R8" t="n">
-        <v>202778</v>
+        <v>607290</v>
       </c>
       <c r="S8" t="n">
         <v>166751</v>
@@ -5299,7 +5299,7 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="O9" t="n">
         <v>100.4</v>
@@ -5311,7 +5311,7 @@
         <v>1.3</v>
       </c>
       <c r="R9" t="n">
-        <v>1540631</v>
+        <v>660299</v>
       </c>
       <c r="S9" t="n">
         <v>3009015</v>
@@ -5370,7 +5370,7 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="O10" t="n">
         <v>101.6</v>
@@ -5382,7 +5382,7 @@
         <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>307625</v>
+        <v>732747</v>
       </c>
       <c r="S10" t="n">
         <v>266328</v>
@@ -5441,7 +5441,7 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="O11" t="n">
         <v>101.3</v>
@@ -5453,7 +5453,7 @@
         <v>0.2</v>
       </c>
       <c r="R11" t="n">
-        <v>473776</v>
+        <v>774708</v>
       </c>
       <c r="S11" t="n">
         <v>1034411</v>
@@ -5512,7 +5512,7 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="O12" t="n">
         <v>101.1</v>
@@ -5524,7 +5524,7 @@
         <v>0.5</v>
       </c>
       <c r="R12" t="n">
-        <v>1750909</v>
+        <v>901537</v>
       </c>
       <c r="S12" t="n">
         <v>5250200</v>
@@ -5583,7 +5583,7 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="O13" t="n">
         <v>100.9</v>
@@ -5595,7 +5595,7 @@
         <v>0.6</v>
       </c>
       <c r="R13" t="n">
-        <v>1531354</v>
+        <v>989440</v>
       </c>
       <c r="S13" t="n">
         <v>5881370</v>
@@ -5654,7 +5654,7 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="O14" t="n">
         <v>100.6</v>
@@ -5666,7 +5666,7 @@
         <v>0.4</v>
       </c>
       <c r="R14" t="n">
-        <v>1824730</v>
+        <v>995232</v>
       </c>
       <c r="S14" t="n">
         <v>4185865</v>
@@ -5725,7 +5725,7 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="O15" t="n">
         <v>101.8</v>
@@ -5737,7 +5737,7 @@
         <v>0.2</v>
       </c>
       <c r="R15" t="n">
-        <v>572310</v>
+        <v>1091532</v>
       </c>
       <c r="S15" t="n">
         <v>466127</v>
@@ -5796,7 +5796,7 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="O16" t="n">
         <v>101.4</v>
@@ -5808,7 +5808,7 @@
         <v>0.2</v>
       </c>
       <c r="R16" t="n">
-        <v>1225264</v>
+        <v>1300624</v>
       </c>
       <c r="S16" t="n">
         <v>878473</v>
@@ -5867,7 +5867,7 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="O17" t="n">
         <v>100.9</v>
@@ -5879,7 +5879,7 @@
         <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>1474444</v>
+        <v>1356982</v>
       </c>
       <c r="S17" t="n">
         <v>1066412</v>
@@ -5938,7 +5938,7 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="O18" t="n">
         <v>101.2</v>
@@ -5950,7 +5950,7 @@
         <v>1.1</v>
       </c>
       <c r="R18" t="n">
-        <v>954063</v>
+        <v>1356982</v>
       </c>
       <c r="S18" t="n">
         <v>101935</v>
@@ -6009,7 +6009,7 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="O19" t="n">
         <v>100.4</v>
@@ -6021,7 +6021,7 @@
         <v>0.6</v>
       </c>
       <c r="R19" t="n">
-        <v>692223</v>
+        <v>1366400</v>
       </c>
       <c r="S19" t="n">
         <v>637992</v>
@@ -6080,7 +6080,7 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="O20" t="n">
         <v>100.3</v>
@@ -6092,7 +6092,7 @@
         <v>2.7</v>
       </c>
       <c r="R20" t="n">
-        <v>1029192</v>
+        <v>1683534</v>
       </c>
       <c r="S20" t="n">
         <v>4399137</v>
@@ -6147,7 +6147,7 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>61</v>
+        <v>87</v>
       </c>
       <c r="O21" t="n">
         <v>101.9</v>
@@ -6159,7 +6159,7 @@
         <v>0.6</v>
       </c>
       <c r="R21" t="n">
-        <v>2653099</v>
+        <v>1861457</v>
       </c>
       <c r="S21" t="n">
         <v>2489160</v>
@@ -6218,7 +6218,7 @@
         <v>-8</v>
       </c>
       <c r="N22" t="n">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="O22" t="n">
         <v>100.6</v>
@@ -6230,7 +6230,7 @@
         <v>0.7</v>
       </c>
       <c r="R22" t="n">
-        <v>1804185</v>
+        <v>2179604</v>
       </c>
       <c r="S22" t="n">
         <v>3048395</v>
@@ -6289,7 +6289,7 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="O23" t="n">
         <v>100.2</v>
@@ -6301,7 +6301,7 @@
         <v>1.8</v>
       </c>
       <c r="R23" t="n">
-        <v>2920591</v>
+        <v>2211172</v>
       </c>
       <c r="S23" t="n">
         <v>1595922</v>
@@ -6360,7 +6360,7 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="O24" t="n">
         <v>101.7</v>
@@ -6372,7 +6372,7 @@
         <v>0.4</v>
       </c>
       <c r="R24" t="n">
-        <v>2382054</v>
+        <v>2348198</v>
       </c>
       <c r="S24" t="n">
         <v>2735246</v>
@@ -6431,7 +6431,7 @@
         <v>-8</v>
       </c>
       <c r="N25" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="O25" t="n">
         <v>101.1</v>
@@ -6443,7 +6443,7 @@
         <v>0.1</v>
       </c>
       <c r="R25" t="n">
-        <v>3529354</v>
+        <v>2633084</v>
       </c>
       <c r="S25" t="n">
         <v>1948104</v>
@@ -6502,7 +6502,7 @@
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>51</v>
+        <v>79</v>
       </c>
       <c r="O26" t="n">
         <v>101.1</v>
@@ -6514,7 +6514,7 @@
         <v>1.1</v>
       </c>
       <c r="R26" t="n">
-        <v>2310073</v>
+        <v>2669248</v>
       </c>
       <c r="S26" t="n">
         <v>453361</v>
@@ -6569,7 +6569,7 @@
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="O27" t="n">
         <v>101.7</v>
@@ -6581,7 +6581,7 @@
         <v>0.7</v>
       </c>
       <c r="R27" t="n">
-        <v>3467718</v>
+        <v>3150671</v>
       </c>
       <c r="S27" t="n">
         <v>614528</v>
@@ -6640,7 +6640,7 @@
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="O28" t="n">
         <v>100.8</v>
@@ -6652,7 +6652,7 @@
         <v>0</v>
       </c>
       <c r="R28" t="n">
-        <v>3408831</v>
+        <v>3441670</v>
       </c>
       <c r="S28" t="n">
         <v>3395267</v>
@@ -6711,7 +6711,7 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="O29" t="n">
         <v>100.7</v>
@@ -6723,7 +6723,7 @@
         <v>0</v>
       </c>
       <c r="R29" t="n">
-        <v>5014924</v>
+        <v>4297158</v>
       </c>
       <c r="S29" t="n">
         <v>3963132</v>
@@ -6782,7 +6782,7 @@
         <v>-8</v>
       </c>
       <c r="N30" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="O30" t="n">
         <v>101.4</v>
@@ -6794,7 +6794,7 @@
         <v>1</v>
       </c>
       <c r="R30" t="n">
-        <v>6407301</v>
+        <v>5509780</v>
       </c>
       <c r="S30" t="n">
         <v>1952243</v>
@@ -6853,7 +6853,7 @@
         <v>-4</v>
       </c>
       <c r="N31" t="n">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="O31" t="n">
         <v>100.7</v>
@@ -6865,7 +6865,7 @@
         <v>1.2</v>
       </c>
       <c r="R31" t="n">
-        <v>6473757</v>
+        <v>7139131</v>
       </c>
       <c r="S31" t="n">
         <v>553038</v>
@@ -6924,7 +6924,7 @@
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="O32" t="n">
         <v>99.2</v>
@@ -6936,7 +6936,7 @@
         <v>2.2</v>
       </c>
       <c r="R32" t="n">
-        <v>9014775</v>
+        <v>9241407</v>
       </c>
       <c r="S32" t="n">
         <v>216389</v>

</xml_diff>

<commit_message>
Update standings 2026-09-20 09:06 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -835,16 +835,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -859,16 +859,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -1876,39 +1876,39 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="C17" t="n">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="D17" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E17" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="C18" t="n">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="D18" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E18" t="n">
-        <v>69</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19">
@@ -2995,7 +2995,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -3006,7 +3006,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -4073,30 +4073,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E17" t="n">
-        <v>31543</v>
+        <v>37120</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>820692</v>
+        <v>1571193</v>
       </c>
       <c r="H17" t="n">
-        <v>1637750</v>
+        <v>3349378</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4110,30 +4110,30 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E18" t="n">
-        <v>37120</v>
+        <v>31543</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>1571193</v>
+        <v>820692</v>
       </c>
       <c r="H18" t="n">
-        <v>3349378</v>
+        <v>1637750</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -5825,34 +5825,34 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C17" t="n">
         <v>309</v>
       </c>
       <c r="D17" t="n">
-        <v>71.2</v>
+        <v>71.8</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
-        <v>105</v>
+        <v>62</v>
       </c>
       <c r="G17" t="n">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="H17" t="n">
         <v>2</v>
       </c>
       <c r="I17" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J17" t="n">
         <v>3</v>
@@ -5867,63 +5867,63 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="O17" t="n">
-        <v>100.9</v>
+        <v>101.2</v>
       </c>
       <c r="P17" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q17" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="R17" t="n">
         <v>1356982</v>
       </c>
       <c r="S17" t="n">
-        <v>1066412</v>
+        <v>101935</v>
       </c>
       <c r="T17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C18" t="n">
         <v>309</v>
       </c>
       <c r="D18" t="n">
-        <v>71.8</v>
+        <v>71.2</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
-        <v>62</v>
+        <v>105</v>
       </c>
       <c r="G18" t="n">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="H18" t="n">
         <v>2</v>
       </c>
       <c r="I18" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J18" t="n">
         <v>3</v>
@@ -5938,29 +5938,29 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="O18" t="n">
-        <v>101.2</v>
+        <v>100.9</v>
       </c>
       <c r="P18" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="Q18" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="R18" t="n">
         <v>1356982</v>
       </c>
       <c r="S18" t="n">
-        <v>101935</v>
+        <v>1066412</v>
       </c>
       <c r="T18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-20 13:58 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -484,13 +484,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="3">
@@ -508,13 +508,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>346</v>
+        <v>360</v>
       </c>
     </row>
     <row r="4">
@@ -523,22 +523,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F4" t="n">
-        <v>339</v>
+        <v>346</v>
       </c>
     </row>
     <row r="5">
@@ -547,22 +547,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="E5" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>336</v>
+        <v>341</v>
       </c>
     </row>
     <row r="6">
@@ -580,13 +580,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="7">
@@ -604,13 +604,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>327</v>
+        <v>333</v>
       </c>
     </row>
     <row r="8">
@@ -628,13 +628,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="9">
@@ -643,22 +643,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="10">
@@ -667,22 +667,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>322</v>
+        <v>326</v>
       </c>
     </row>
     <row r="11">
@@ -691,22 +691,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
     <row r="12">
@@ -724,13 +724,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>318</v>
+        <v>325</v>
       </c>
     </row>
     <row r="13">
@@ -739,22 +739,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>316</v>
+        <v>323</v>
       </c>
     </row>
     <row r="14">
@@ -763,22 +763,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="15">
@@ -787,46 +787,46 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>314</v>
+        <v>318</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>310</v>
+        <v>318</v>
       </c>
     </row>
     <row r="17">
@@ -835,27 +835,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -868,13 +868,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>309</v>
+        <v>312</v>
       </c>
     </row>
     <row r="19">
@@ -892,13 +892,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>309</v>
+        <v>312</v>
       </c>
     </row>
     <row r="20">
@@ -916,13 +916,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>304</v>
+        <v>308</v>
       </c>
     </row>
     <row r="21">
@@ -940,13 +940,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>301</v>
+        <v>305</v>
       </c>
     </row>
     <row r="22">
@@ -955,22 +955,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="E22" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>297</v>
+        <v>303</v>
       </c>
     </row>
     <row r="23">
@@ -979,22 +979,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="F23" t="n">
-        <v>296</v>
+        <v>301</v>
       </c>
     </row>
     <row r="24">
@@ -1003,22 +1003,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>294</v>
+        <v>300</v>
       </c>
     </row>
     <row r="25">
@@ -1036,13 +1036,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E25" t="n">
         <v>-8</v>
       </c>
       <c r="F25" t="n">
-        <v>291</v>
+        <v>296</v>
       </c>
     </row>
     <row r="26">
@@ -1060,13 +1060,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>290</v>
+        <v>295</v>
       </c>
     </row>
     <row r="27">
@@ -1084,13 +1084,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>285</v>
+        <v>294</v>
       </c>
     </row>
     <row r="28">
@@ -1108,13 +1108,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>281</v>
+        <v>292</v>
       </c>
     </row>
     <row r="29">
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>271</v>
+        <v>280</v>
       </c>
     </row>
     <row r="30">
@@ -1156,13 +1156,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E30" t="n">
         <v>-8</v>
       </c>
       <c r="F30" t="n">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="31">
@@ -1180,13 +1180,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="E31" t="n">
         <v>-4</v>
       </c>
       <c r="F31" t="n">
-        <v>237</v>
+        <v>251</v>
       </c>
     </row>
     <row r="32">
@@ -1204,13 +1204,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>190</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -1629,39 +1629,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C4" t="n">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="D4" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E4" t="n">
-        <v>77</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="C5" t="n">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="D5" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E5" t="n">
-        <v>107</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6">
@@ -1724,58 +1724,58 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="C9" t="n">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D9" t="n">
-        <v>67</v>
+        <v>40</v>
       </c>
       <c r="E9" t="n">
-        <v>71</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="C10" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D10" t="n">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="E10" t="n">
-        <v>92</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="C11" t="n">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D11" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="E11" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12">
@@ -1800,96 +1800,96 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="C13" t="n">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="D13" t="n">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="E13" t="n">
-        <v>71</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C14" t="n">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="D14" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E14" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B15" t="n">
+        <v>44</v>
+      </c>
+      <c r="C15" t="n">
+        <v>107</v>
+      </c>
+      <c r="D15" t="n">
+        <v>56</v>
+      </c>
+      <c r="E15" t="n">
         <v>73</v>
-      </c>
-      <c r="C15" t="n">
-        <v>104</v>
-      </c>
-      <c r="D15" t="n">
-        <v>37</v>
-      </c>
-      <c r="E15" t="n">
-        <v>91</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="C17" t="n">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="D17" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E17" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18">
@@ -1971,58 +1971,58 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C22" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D22" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E22" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C23" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="D23" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="E23" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C24" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="D24" t="n">
         <v>50</v>
       </c>
       <c r="E24" t="n">
-        <v>90</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25">
@@ -2430,7 +2430,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -2441,7 +2441,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2804,7 +2804,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -2815,7 +2815,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -2826,7 +2826,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -2837,7 +2837,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2848,7 +2848,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2859,7 +2859,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2892,7 +2892,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2903,7 +2903,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -2984,7 +2984,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2995,7 +2995,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -3592,30 +3592,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E4" t="n">
-        <v>189374</v>
+        <v>281617</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1757289</v>
+        <v>1051323</v>
       </c>
       <c r="H4" t="n">
-        <v>250879</v>
+        <v>1076546</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -3629,30 +3629,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E5" t="n">
-        <v>281617</v>
+        <v>189374</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>1051323</v>
+        <v>1757289</v>
       </c>
       <c r="H5" t="n">
-        <v>1076546</v>
+        <v>250879</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -3777,30 +3777,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>453230</v>
+        <v>30971</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>5483351</v>
+        <v>820221</v>
       </c>
       <c r="H9" t="n">
-        <v>8188106</v>
+        <v>58227</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -3814,30 +3814,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E10" t="n">
-        <v>71857</v>
+        <v>453230</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>1929309</v>
+        <v>5483351</v>
       </c>
       <c r="H10" t="n">
-        <v>297407</v>
+        <v>8188106</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -3851,30 +3851,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>30971</v>
+        <v>71857</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>820221</v>
+        <v>1929309</v>
       </c>
       <c r="H11" t="n">
-        <v>58227</v>
+        <v>297407</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -3925,30 +3925,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E13" t="n">
-        <v>273503</v>
+        <v>28582</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>1994005</v>
+        <v>881388</v>
       </c>
       <c r="H13" t="n">
-        <v>1917309</v>
+        <v>239490</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -3962,30 +3962,30 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E14" t="n">
-        <v>410102</v>
+        <v>273503</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>2088802</v>
+        <v>1994005</v>
       </c>
       <c r="H14" t="n">
-        <v>5360778</v>
+        <v>1917309</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -3999,30 +3999,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E15" t="n">
-        <v>28582</v>
+        <v>410102</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>881388</v>
+        <v>2088802</v>
       </c>
       <c r="H15" t="n">
-        <v>239490</v>
+        <v>5360778</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4032,34 +4032,34 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>8917</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>2118382</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>9146930</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -4073,30 +4073,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E17" t="n">
-        <v>37120</v>
+        <v>8917</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>1571193</v>
+        <v>2118382</v>
       </c>
       <c r="H17" t="n">
-        <v>3349378</v>
+        <v>9146930</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4106,7 +4106,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -4258,30 +4258,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="E22" t="n">
-        <v>1128645</v>
+        <v>14603</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2016/17</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>3434302</v>
+        <v>949628</v>
       </c>
       <c r="H22" t="n">
-        <v>1128645</v>
+        <v>515830</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E23" t="n">
-        <v>1615102</v>
+        <v>1128645</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>4234674</v>
+        <v>3434302</v>
       </c>
       <c r="H23" t="n">
-        <v>6092784</v>
+        <v>1128645</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E24" t="n">
-        <v>14603</v>
+        <v>1615102</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2016/17</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>949628</v>
+        <v>4234674</v>
       </c>
       <c r="H24" t="n">
-        <v>515830</v>
+        <v>6092784</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="D2" t="n">
         <v>86</v>
@@ -4844,7 +4844,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>346</v>
+        <v>360</v>
       </c>
       <c r="D3" t="n">
         <v>81.2</v>
@@ -4902,142 +4902,142 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="D4" t="n">
-        <v>71.8</v>
+        <v>78.8</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="G4" t="n">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="J4" t="n">
         <v>3</v>
       </c>
       <c r="K4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N4" t="n">
-        <v>46</v>
+        <v>73</v>
       </c>
       <c r="O4" t="n">
-        <v>100.8</v>
+        <v>101.6</v>
       </c>
       <c r="P4" t="n">
-        <v>0.8</v>
+        <v>1.6</v>
       </c>
       <c r="Q4" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="R4" t="n">
-        <v>241342</v>
+        <v>330274</v>
       </c>
       <c r="S4" t="n">
-        <v>3046343</v>
+        <v>1229264</v>
       </c>
       <c r="T4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="D5" t="n">
-        <v>78.8</v>
+        <v>71.8</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="G5" t="n">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="H5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I5" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="J5" t="n">
         <v>3</v>
       </c>
       <c r="K5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>46</v>
+      </c>
+      <c r="O5" t="n">
+        <v>100.8</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="Q5" t="n">
         <v>1</v>
       </c>
-      <c r="M5" t="n">
-        <v>-4</v>
-      </c>
-      <c r="N5" t="n">
-        <v>73</v>
-      </c>
-      <c r="O5" t="n">
-        <v>101.6</v>
-      </c>
-      <c r="P5" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0.7</v>
-      </c>
       <c r="R5" t="n">
-        <v>330274</v>
+        <v>241342</v>
       </c>
       <c r="S5" t="n">
-        <v>1229264</v>
+        <v>3046343</v>
       </c>
       <c r="T5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
@@ -5053,7 +5053,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="D6" t="n">
         <v>74.2</v>
@@ -5124,7 +5124,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="D7" t="n">
         <v>76.2</v>
@@ -5195,7 +5195,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="D8" t="n">
         <v>78.2</v>
@@ -5257,37 +5257,37 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="D9" t="n">
-        <v>71.5</v>
+        <v>74.8</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="G9" t="n">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H9" t="n">
         <v>2</v>
       </c>
       <c r="I9" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K9" t="n">
         <v>2</v>
@@ -5299,69 +5299,69 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="O9" t="n">
-        <v>100.4</v>
+        <v>101.3</v>
       </c>
       <c r="P9" t="n">
-        <v>0.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q9" t="n">
-        <v>1.3</v>
+        <v>0.2</v>
       </c>
       <c r="R9" t="n">
-        <v>660299</v>
+        <v>774708</v>
       </c>
       <c r="S9" t="n">
-        <v>3009015</v>
+        <v>1034411</v>
       </c>
       <c r="T9" t="n">
         <v>2</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="D10" t="n">
-        <v>78.5</v>
+        <v>71.5</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
-        <v>78</v>
+        <v>99</v>
       </c>
       <c r="G10" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H10" t="n">
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -5370,48 +5370,48 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>92</v>
+        <v>42</v>
       </c>
       <c r="O10" t="n">
-        <v>101.6</v>
+        <v>100.4</v>
       </c>
       <c r="P10" t="n">
-        <v>1.6</v>
+        <v>0.4</v>
       </c>
       <c r="Q10" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="R10" t="n">
-        <v>732747</v>
+        <v>660299</v>
       </c>
       <c r="S10" t="n">
-        <v>266328</v>
+        <v>3009015</v>
       </c>
       <c r="T10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="D11" t="n">
-        <v>74.8</v>
+        <v>78.5</v>
       </c>
       <c r="E11" t="n">
         <v>3</v>
@@ -5420,19 +5420,19 @@
         <v>78</v>
       </c>
       <c r="G11" t="n">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="H11" t="n">
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="J11" t="n">
         <v>3</v>
       </c>
       <c r="K11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -5441,25 +5441,25 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="O11" t="n">
-        <v>101.3</v>
+        <v>101.6</v>
       </c>
       <c r="P11" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>774708</v>
+        <v>732747</v>
       </c>
       <c r="S11" t="n">
-        <v>1034411</v>
+        <v>266328</v>
       </c>
       <c r="T11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
@@ -5479,7 +5479,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="D12" t="n">
         <v>70.8</v>
@@ -5541,111 +5541,111 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="D13" t="n">
-        <v>71</v>
+        <v>76.2</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="G13" t="n">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="H13" t="n">
         <v>2</v>
       </c>
       <c r="I13" t="n">
+        <v>37</v>
+      </c>
+      <c r="J13" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" t="n">
+        <v>2</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="n">
         <v>40</v>
       </c>
-      <c r="J13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" t="n">
-        <v>74</v>
-      </c>
       <c r="O13" t="n">
-        <v>100.9</v>
+        <v>101.8</v>
       </c>
       <c r="P13" t="n">
-        <v>0.9</v>
+        <v>1.8</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="R13" t="n">
-        <v>989440</v>
+        <v>1091532</v>
       </c>
       <c r="S13" t="n">
-        <v>5881370</v>
+        <v>466127</v>
       </c>
       <c r="T13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D14" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E14" t="n">
         <v>2</v>
       </c>
       <c r="F14" t="n">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="G14" t="n">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="H14" t="n">
         <v>2</v>
       </c>
       <c r="I14" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J14" t="n">
         <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -5654,66 +5654,66 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>53</v>
+        <v>74</v>
       </c>
       <c r="O14" t="n">
-        <v>100.6</v>
+        <v>100.9</v>
       </c>
       <c r="P14" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q14" t="n">
         <v>0.6</v>
       </c>
-      <c r="Q14" t="n">
-        <v>0.4</v>
-      </c>
       <c r="R14" t="n">
-        <v>995232</v>
+        <v>989440</v>
       </c>
       <c r="S14" t="n">
-        <v>4185865</v>
+        <v>5881370</v>
       </c>
       <c r="T14" t="n">
         <v>2</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="D15" t="n">
-        <v>76.2</v>
+        <v>70</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F15" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="G15" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="J15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5725,63 +5725,63 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="O15" t="n">
-        <v>101.8</v>
+        <v>100.6</v>
       </c>
       <c r="P15" t="n">
-        <v>1.8</v>
+        <v>0.6</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="R15" t="n">
-        <v>1091532</v>
+        <v>995232</v>
       </c>
       <c r="S15" t="n">
-        <v>466127</v>
+        <v>4185865</v>
       </c>
       <c r="T15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="D16" t="n">
-        <v>72.2</v>
+        <v>71.8</v>
       </c>
       <c r="E16" t="n">
         <v>2</v>
       </c>
       <c r="F16" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="G16" t="n">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="J16" t="n">
         <v>3</v>
@@ -5796,63 +5796,63 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>78</v>
+        <v>44</v>
       </c>
       <c r="O16" t="n">
-        <v>101.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.2</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
-        <v>1300624</v>
+        <v>1356982</v>
       </c>
       <c r="S16" t="n">
-        <v>878473</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="D17" t="n">
-        <v>71.8</v>
+        <v>72.2</v>
       </c>
       <c r="E17" t="n">
         <v>2</v>
       </c>
       <c r="F17" t="n">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="G17" t="n">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="H17" t="n">
         <v>2</v>
       </c>
       <c r="I17" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="J17" t="n">
         <v>3</v>
@@ -5867,29 +5867,29 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>44</v>
+        <v>78</v>
       </c>
       <c r="O17" t="n">
-        <v>101.2</v>
+        <v>101.4</v>
       </c>
       <c r="P17" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="Q17" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
       <c r="R17" t="n">
-        <v>1356982</v>
+        <v>1300624</v>
       </c>
       <c r="S17" t="n">
-        <v>101935</v>
+        <v>878473</v>
       </c>
       <c r="T17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
@@ -5905,7 +5905,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D18" t="n">
         <v>71.2</v>
@@ -5976,7 +5976,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D19" t="n">
         <v>75</v>
@@ -6047,7 +6047,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="D20" t="n">
         <v>73.2</v>
@@ -6114,7 +6114,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="D21" t="n">
         <v>67.5</v>
@@ -6176,182 +6176,182 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>297</v>
+        <v>303</v>
       </c>
       <c r="D22" t="n">
-        <v>71.8</v>
+        <v>68.8</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="G22" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="H22" t="n">
         <v>2</v>
       </c>
       <c r="I22" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J22" t="n">
         <v>1</v>
       </c>
       <c r="K22" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M22" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="O22" t="n">
-        <v>100.6</v>
+        <v>101.7</v>
       </c>
       <c r="P22" t="n">
-        <v>0.6</v>
+        <v>1.7</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
       <c r="R22" t="n">
-        <v>2179604</v>
+        <v>2348198</v>
       </c>
       <c r="S22" t="n">
-        <v>3048395</v>
+        <v>2735246</v>
       </c>
       <c r="T22" t="n">
         <v>2</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="D23" t="n">
-        <v>67.2</v>
+        <v>71.8</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
         <v>67</v>
       </c>
       <c r="G23" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="H23" t="n">
         <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="J23" t="n">
         <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M23" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="N23" t="n">
-        <v>81</v>
+        <v>55</v>
       </c>
       <c r="O23" t="n">
-        <v>100.2</v>
+        <v>100.6</v>
       </c>
       <c r="P23" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="Q23" t="n">
-        <v>1.8</v>
+        <v>0.7</v>
       </c>
       <c r="R23" t="n">
-        <v>2211172</v>
+        <v>2179604</v>
       </c>
       <c r="S23" t="n">
-        <v>1595922</v>
+        <v>3048395</v>
       </c>
       <c r="T23" t="n">
         <v>2</v>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>bboost, 3xc, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="D24" t="n">
-        <v>68.8</v>
+        <v>67.2</v>
       </c>
       <c r="E24" t="n">
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="G24" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="H24" t="n">
         <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="J24" t="n">
         <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
@@ -6360,29 +6360,29 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="O24" t="n">
-        <v>101.7</v>
+        <v>100.2</v>
       </c>
       <c r="P24" t="n">
-        <v>1.7</v>
+        <v>0.2</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.4</v>
+        <v>1.8</v>
       </c>
       <c r="R24" t="n">
-        <v>2348198</v>
+        <v>2211172</v>
       </c>
       <c r="S24" t="n">
-        <v>2735246</v>
+        <v>1595922</v>
       </c>
       <c r="T24" t="n">
         <v>2</v>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>bboost, 3xc, wildcard</t>
         </is>
       </c>
     </row>
@@ -6398,7 +6398,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="D25" t="n">
         <v>66.8</v>
@@ -6469,7 +6469,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="D26" t="n">
         <v>67.5</v>
@@ -6536,7 +6536,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>285</v>
+        <v>294</v>
       </c>
       <c r="D27" t="n">
         <v>65.8</v>
@@ -6607,7 +6607,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>281</v>
+        <v>292</v>
       </c>
       <c r="D28" t="n">
         <v>66.5</v>
@@ -6678,7 +6678,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="D29" t="n">
         <v>61.8</v>
@@ -6749,7 +6749,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D30" t="n">
         <v>58</v>
@@ -6820,7 +6820,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>237</v>
+        <v>251</v>
       </c>
       <c r="D31" t="n">
         <v>56.8</v>
@@ -6891,7 +6891,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>190</v>
+        <v>207</v>
       </c>
       <c r="D32" t="n">
         <v>46.8</v>

</xml_diff>

<commit_message>
Update standings 2026-09-20 17:23 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -484,13 +484,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>385</v>
+        <v>395</v>
       </c>
     </row>
     <row r="3">
@@ -508,13 +508,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>360</v>
+        <v>381</v>
       </c>
     </row>
     <row r="4">
@@ -532,13 +532,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="E4" t="n">
         <v>-4</v>
       </c>
       <c r="F4" t="n">
-        <v>346</v>
+        <v>362</v>
       </c>
     </row>
     <row r="5">
@@ -556,13 +556,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>341</v>
+        <v>351</v>
       </c>
     </row>
     <row r="6">
@@ -571,22 +571,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>335</v>
+        <v>349</v>
       </c>
     </row>
     <row r="7">
@@ -595,22 +595,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>333</v>
+        <v>345</v>
       </c>
     </row>
     <row r="8">
@@ -628,13 +628,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>331</v>
+        <v>345</v>
       </c>
     </row>
     <row r="9">
@@ -643,22 +643,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>329</v>
+        <v>344</v>
       </c>
     </row>
     <row r="10">
@@ -667,22 +667,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>326</v>
+        <v>342</v>
       </c>
     </row>
     <row r="11">
@@ -700,13 +700,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>325</v>
+        <v>340</v>
       </c>
     </row>
     <row r="12">
@@ -715,22 +715,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>325</v>
+        <v>338</v>
       </c>
     </row>
     <row r="13">
@@ -739,22 +739,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>323</v>
+        <v>337</v>
       </c>
     </row>
     <row r="14">
@@ -772,13 +772,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>319</v>
+        <v>336</v>
       </c>
     </row>
     <row r="15">
@@ -787,46 +787,46 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>318</v>
+        <v>335</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>318</v>
+        <v>334</v>
       </c>
     </row>
     <row r="17">
@@ -835,22 +835,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>316</v>
+        <v>332</v>
       </c>
     </row>
     <row r="18">
@@ -868,13 +868,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>312</v>
+        <v>331</v>
       </c>
     </row>
     <row r="19">
@@ -892,13 +892,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>312</v>
+        <v>327</v>
       </c>
     </row>
     <row r="20">
@@ -907,22 +907,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>15</v>
+        <v>42</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="F20" t="n">
-        <v>308</v>
+        <v>325</v>
       </c>
     </row>
     <row r="21">
@@ -931,22 +931,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>305</v>
+        <v>322</v>
       </c>
     </row>
     <row r="22">
@@ -955,22 +955,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>303</v>
+        <v>321</v>
       </c>
     </row>
     <row r="23">
@@ -979,22 +979,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="E23" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>301</v>
+        <v>319</v>
       </c>
     </row>
     <row r="24">
@@ -1003,22 +1003,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>300</v>
+        <v>319</v>
       </c>
     </row>
     <row r="25">
@@ -1036,13 +1036,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="E25" t="n">
         <v>-8</v>
       </c>
       <c r="F25" t="n">
-        <v>296</v>
+        <v>317</v>
       </c>
     </row>
     <row r="26">
@@ -1051,22 +1051,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>295</v>
+        <v>314</v>
       </c>
     </row>
     <row r="27">
@@ -1075,22 +1075,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>294</v>
+        <v>310</v>
       </c>
     </row>
     <row r="28">
@@ -1099,22 +1099,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>292</v>
+        <v>309</v>
       </c>
     </row>
     <row r="29">
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>280</v>
+        <v>293</v>
       </c>
     </row>
     <row r="30">
@@ -1156,13 +1156,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="E30" t="n">
         <v>-8</v>
       </c>
       <c r="F30" t="n">
-        <v>261</v>
+        <v>278</v>
       </c>
     </row>
     <row r="31">
@@ -1180,13 +1180,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="E31" t="n">
         <v>-4</v>
       </c>
       <c r="F31" t="n">
-        <v>251</v>
+        <v>271</v>
       </c>
     </row>
     <row r="32">
@@ -1204,13 +1204,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>207</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -1667,39 +1667,39 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="C6" t="n">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="D6" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E6" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="C7" t="n">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="D7" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E7" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8">
@@ -1724,39 +1724,39 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="C9" t="n">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="D9" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="E9" t="n">
-        <v>91</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="C10" t="n">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D10" t="n">
-        <v>67</v>
+        <v>40</v>
       </c>
       <c r="E10" t="n">
-        <v>71</v>
+        <v>91</v>
       </c>
     </row>
     <row r="11">
@@ -1781,39 +1781,39 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="C12" t="n">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="D12" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E12" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C13" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D13" t="n">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="E13" t="n">
-        <v>91</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14">
@@ -1838,58 +1838,58 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>44</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>91</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="C17" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D17" t="n">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="E17" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18">
@@ -1933,96 +1933,96 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C20" t="n">
-        <v>120</v>
+        <v>97</v>
       </c>
       <c r="D20" t="n">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="E20" t="n">
-        <v>76</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C21" t="n">
-        <v>86</v>
+        <v>120</v>
       </c>
       <c r="D21" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E21" t="n">
-        <v>93</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C22" t="n">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="D22" t="n">
-        <v>50</v>
+        <v>78</v>
       </c>
       <c r="E22" t="n">
-        <v>90</v>
+        <v>69</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C23" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D23" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E23" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="n">
+        <v>45</v>
+      </c>
+      <c r="C24" t="n">
+        <v>86</v>
+      </c>
+      <c r="D24" t="n">
         <v>46</v>
       </c>
-      <c r="C24" t="n">
-        <v>89</v>
-      </c>
-      <c r="D24" t="n">
-        <v>50</v>
-      </c>
       <c r="E24" t="n">
-        <v>84</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25">
@@ -2047,36 +2047,36 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="C26" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="D26" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E26" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>59</v>
       </c>
       <c r="C27" t="n">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D27" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="E27" t="n">
         <v>77</v>
@@ -2085,20 +2085,20 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="C28" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D28" t="n">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="E28" t="n">
-        <v>69</v>
+        <v>77</v>
       </c>
     </row>
     <row r="29">
@@ -2221,7 +2221,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -2369,11 +2369,7 @@
       <c r="B6" t="n">
         <v>87</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2452,7 +2448,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2463,7 +2459,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2554,7 +2550,11 @@
       <c r="B21" t="n">
         <v>67</v>
       </c>
-      <c r="C21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2614,7 +2614,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2625,7 +2625,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2767,7 +2767,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -2782,7 +2782,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -2815,7 +2815,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -2826,7 +2826,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -2837,7 +2837,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2848,7 +2848,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2881,7 +2881,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2903,7 +2903,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -2914,7 +2914,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -2925,7 +2925,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -2984,7 +2984,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2995,7 +2995,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -3666,19 +3666,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E6" t="n">
-        <v>182900</v>
+        <v>6474</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -3686,10 +3686,10 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>2098988</v>
+        <v>1177681</v>
       </c>
       <c r="H6" t="n">
-        <v>182900</v>
+        <v>6474</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -3703,19 +3703,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>6474</v>
+        <v>182900</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -3723,10 +3723,10 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1177681</v>
+        <v>2098988</v>
       </c>
       <c r="H7" t="n">
-        <v>6474</v>
+        <v>182900</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -3777,30 +3777,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D9" t="n">
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>30971</v>
+        <v>486041</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>820221</v>
+        <v>2415786</v>
       </c>
       <c r="H9" t="n">
-        <v>58227</v>
+        <v>1206623</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -3814,30 +3814,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E10" t="n">
-        <v>453230</v>
+        <v>30971</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>5483351</v>
+        <v>820221</v>
       </c>
       <c r="H10" t="n">
-        <v>8188106</v>
+        <v>58227</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -3888,30 +3888,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E12" t="n">
-        <v>486041</v>
+        <v>8917</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>2415786</v>
+        <v>2118382</v>
       </c>
       <c r="H12" t="n">
-        <v>1206623</v>
+        <v>9146930</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -3925,30 +3925,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E13" t="n">
-        <v>28582</v>
+        <v>453230</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>881388</v>
+        <v>5483351</v>
       </c>
       <c r="H13" t="n">
-        <v>239490</v>
+        <v>8188106</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -3999,30 +3999,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>410102</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>2088802</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>5360778</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4032,34 +4032,34 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>28582</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>881388</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>239490</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -4073,30 +4073,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E17" t="n">
-        <v>8917</v>
+        <v>410102</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>2118382</v>
+        <v>2088802</v>
       </c>
       <c r="H17" t="n">
-        <v>9146930</v>
+        <v>5360778</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4184,30 +4184,30 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="E20" t="n">
-        <v>60517</v>
+        <v>1128645</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2015/16</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>1414622</v>
+        <v>3434302</v>
       </c>
       <c r="H20" t="n">
-        <v>339763</v>
+        <v>1128645</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -4221,30 +4221,30 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E21" t="n">
-        <v>95791</v>
+        <v>60517</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2015/16</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>2404119</v>
+        <v>1414622</v>
       </c>
       <c r="H21" t="n">
-        <v>5124417</v>
+        <v>339763</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -4258,30 +4258,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E22" t="n">
-        <v>14603</v>
+        <v>15288</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2016/17</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>949628</v>
+        <v>329510</v>
       </c>
       <c r="H22" t="n">
-        <v>515830</v>
+        <v>538046</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -4295,30 +4295,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="E23" t="n">
-        <v>1128645</v>
+        <v>14603</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2016/17</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>3434302</v>
+        <v>949628</v>
       </c>
       <c r="H23" t="n">
-        <v>1128645</v>
+        <v>515830</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4332,30 +4332,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>1615102</v>
+        <v>95791</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>4234674</v>
+        <v>2404119</v>
       </c>
       <c r="H24" t="n">
-        <v>6092784</v>
+        <v>5124417</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -4406,30 +4406,30 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E26" t="n">
-        <v>334016</v>
+        <v>1615102</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>2156629</v>
+        <v>4234674</v>
       </c>
       <c r="H26" t="n">
-        <v>2691725</v>
+        <v>6092784</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -4443,19 +4443,19 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E27" t="n">
-        <v>81907</v>
+        <v>334016</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -4463,10 +4463,10 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>3252487</v>
+        <v>2156629</v>
       </c>
       <c r="H27" t="n">
-        <v>11118394</v>
+        <v>2691725</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -4480,19 +4480,19 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="D28" t="n">
         <v>12</v>
       </c>
       <c r="E28" t="n">
-        <v>15288</v>
+        <v>81907</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -4500,10 +4500,10 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>329510</v>
+        <v>3252487</v>
       </c>
       <c r="H28" t="n">
-        <v>538046</v>
+        <v>11118394</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>385</v>
+        <v>395</v>
       </c>
       <c r="D2" t="n">
         <v>86</v>
@@ -4844,7 +4844,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>360</v>
+        <v>381</v>
       </c>
       <c r="D3" t="n">
         <v>81.2</v>
@@ -4911,7 +4911,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>346</v>
+        <v>362</v>
       </c>
       <c r="D4" t="n">
         <v>78.8</v>
@@ -4982,7 +4982,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>341</v>
+        <v>351</v>
       </c>
       <c r="D5" t="n">
         <v>71.8</v>
@@ -5044,40 +5044,40 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>335</v>
+        <v>349</v>
       </c>
       <c r="D6" t="n">
-        <v>74.2</v>
+        <v>76.2</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="G6" t="n">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="H6" t="n">
         <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="J6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
@@ -5086,7 +5086,7 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="O6" t="n">
         <v>101</v>
@@ -5095,60 +5095,60 @@
         <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="R6" t="n">
-        <v>387912</v>
+        <v>573851</v>
       </c>
       <c r="S6" t="n">
-        <v>3039834</v>
+        <v>617418</v>
       </c>
       <c r="T6" t="n">
         <v>2</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="D7" t="n">
-        <v>76.2</v>
+        <v>74.2</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>67</v>
+        <v>87</v>
       </c>
       <c r="G7" t="n">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="H7" t="n">
         <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="J7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -5157,7 +5157,7 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="O7" t="n">
         <v>101</v>
@@ -5166,20 +5166,20 @@
         <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>573851</v>
+        <v>387912</v>
       </c>
       <c r="S7" t="n">
-        <v>617418</v>
+        <v>3039834</v>
       </c>
       <c r="T7" t="n">
         <v>2</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
@@ -5195,7 +5195,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>331</v>
+        <v>345</v>
       </c>
       <c r="D8" t="n">
         <v>78.2</v>
@@ -5257,37 +5257,37 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>329</v>
+        <v>344</v>
       </c>
       <c r="D9" t="n">
-        <v>74.8</v>
+        <v>70.8</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="G9" t="n">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="H9" t="n">
         <v>2</v>
       </c>
       <c r="I9" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
         <v>2</v>
@@ -5299,66 +5299,66 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="O9" t="n">
-        <v>101.3</v>
+        <v>101.1</v>
       </c>
       <c r="P9" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="R9" t="n">
-        <v>774708</v>
+        <v>901537</v>
       </c>
       <c r="S9" t="n">
-        <v>1034411</v>
+        <v>5250200</v>
       </c>
       <c r="T9" t="n">
         <v>2</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>326</v>
+        <v>342</v>
       </c>
       <c r="D10" t="n">
-        <v>71.5</v>
+        <v>74.8</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="G10" t="n">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H10" t="n">
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
@@ -5370,29 +5370,29 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="O10" t="n">
-        <v>100.4</v>
+        <v>101.3</v>
       </c>
       <c r="P10" t="n">
-        <v>0.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q10" t="n">
-        <v>1.3</v>
+        <v>0.2</v>
       </c>
       <c r="R10" t="n">
-        <v>660299</v>
+        <v>774708</v>
       </c>
       <c r="S10" t="n">
-        <v>3009015</v>
+        <v>1034411</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
@@ -5408,7 +5408,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>325</v>
+        <v>340</v>
       </c>
       <c r="D11" t="n">
         <v>78.5</v>
@@ -5470,37 +5470,37 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>325</v>
+        <v>338</v>
       </c>
       <c r="D12" t="n">
-        <v>70.8</v>
+        <v>72.2</v>
       </c>
       <c r="E12" t="n">
         <v>2</v>
       </c>
       <c r="F12" t="n">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="G12" t="n">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="H12" t="n">
         <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="J12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K12" t="n">
         <v>2</v>
@@ -5512,66 +5512,66 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>46</v>
+        <v>78</v>
       </c>
       <c r="O12" t="n">
-        <v>101.1</v>
+        <v>101.4</v>
       </c>
       <c r="P12" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="R12" t="n">
-        <v>901537</v>
+        <v>1300624</v>
       </c>
       <c r="S12" t="n">
-        <v>5250200</v>
+        <v>878473</v>
       </c>
       <c r="T12" t="n">
         <v>2</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>323</v>
+        <v>337</v>
       </c>
       <c r="D13" t="n">
-        <v>76.2</v>
+        <v>71.5</v>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>78</v>
+        <v>99</v>
       </c>
       <c r="G13" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="H13" t="n">
         <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="J13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K13" t="n">
         <v>2</v>
@@ -5583,29 +5583,29 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="O13" t="n">
-        <v>101.8</v>
+        <v>100.4</v>
       </c>
       <c r="P13" t="n">
-        <v>1.8</v>
+        <v>0.4</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.2</v>
+        <v>1.3</v>
       </c>
       <c r="R13" t="n">
-        <v>1091532</v>
+        <v>660299</v>
       </c>
       <c r="S13" t="n">
-        <v>466127</v>
+        <v>3009015</v>
       </c>
       <c r="T13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
@@ -5621,7 +5621,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>319</v>
+        <v>336</v>
       </c>
       <c r="D14" t="n">
         <v>71</v>
@@ -5683,105 +5683,105 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>318</v>
+        <v>335</v>
       </c>
       <c r="D15" t="n">
-        <v>70</v>
+        <v>71.8</v>
       </c>
       <c r="E15" t="n">
         <v>2</v>
       </c>
       <c r="F15" t="n">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="G15" t="n">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
+        <v>55</v>
+      </c>
+      <c r="J15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
         <v>44</v>
       </c>
-      <c r="J15" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" t="n">
-        <v>2</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" t="n">
-        <v>53</v>
-      </c>
       <c r="O15" t="n">
-        <v>100.6</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.4</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
-        <v>995232</v>
+        <v>1356982</v>
       </c>
       <c r="S15" t="n">
-        <v>4185865</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>318</v>
+        <v>334</v>
       </c>
       <c r="D16" t="n">
-        <v>71.8</v>
+        <v>76.2</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="J16" t="n">
         <v>3</v>
@@ -5796,66 +5796,66 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>101.8</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
       <c r="R16" t="n">
-        <v>1356982</v>
+        <v>1091532</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>466127</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="D17" t="n">
-        <v>72.2</v>
+        <v>70</v>
       </c>
       <c r="E17" t="n">
         <v>2</v>
       </c>
       <c r="F17" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="G17" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H17" t="n">
         <v>2</v>
       </c>
       <c r="I17" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="J17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K17" t="n">
         <v>2</v>
@@ -5867,29 +5867,29 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>78</v>
+        <v>53</v>
       </c>
       <c r="O17" t="n">
-        <v>101.4</v>
+        <v>100.6</v>
       </c>
       <c r="P17" t="n">
-        <v>1.4</v>
+        <v>0.6</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="R17" t="n">
-        <v>1300624</v>
+        <v>995232</v>
       </c>
       <c r="S17" t="n">
-        <v>878473</v>
+        <v>4185865</v>
       </c>
       <c r="T17" t="n">
         <v>2</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
@@ -5905,7 +5905,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>312</v>
+        <v>331</v>
       </c>
       <c r="D18" t="n">
         <v>71.2</v>
@@ -5976,7 +5976,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="D19" t="n">
         <v>75</v>
@@ -6038,107 +6038,111 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>308</v>
+        <v>325</v>
       </c>
       <c r="D20" t="n">
-        <v>73.2</v>
+        <v>71.8</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="G20" t="n">
-        <v>120</v>
+        <v>97</v>
       </c>
       <c r="H20" t="n">
         <v>2</v>
       </c>
       <c r="I20" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="J20" t="n">
         <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M20" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="N20" t="n">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="O20" t="n">
-        <v>100.3</v>
+        <v>100.6</v>
       </c>
       <c r="P20" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="Q20" t="n">
-        <v>2.7</v>
+        <v>0.7</v>
       </c>
       <c r="R20" t="n">
-        <v>1683534</v>
+        <v>2179604</v>
       </c>
       <c r="S20" t="n">
-        <v>4399137</v>
+        <v>3048395</v>
       </c>
       <c r="T20" t="n">
         <v>2</v>
       </c>
-      <c r="U20" t="inlineStr"/>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>3xc, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>305</v>
+        <v>322</v>
       </c>
       <c r="D21" t="n">
-        <v>67.5</v>
+        <v>73.2</v>
       </c>
       <c r="E21" t="n">
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="G21" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="H21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I21" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J21" t="n">
         <v>1</v>
       </c>
       <c r="K21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L21" t="n">
         <v>0</v>
@@ -6147,69 +6151,65 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="O21" t="n">
-        <v>101.9</v>
+        <v>100.3</v>
       </c>
       <c r="P21" t="n">
-        <v>1.9</v>
+        <v>0.3</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.6</v>
+        <v>2.7</v>
       </c>
       <c r="R21" t="n">
-        <v>1861457</v>
+        <v>1683534</v>
       </c>
       <c r="S21" t="n">
-        <v>2489160</v>
+        <v>4399137</v>
       </c>
       <c r="T21" t="n">
-        <v>4</v>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>303</v>
+        <v>321</v>
       </c>
       <c r="D22" t="n">
-        <v>68.8</v>
+        <v>66.5</v>
       </c>
       <c r="E22" t="n">
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="G22" t="n">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="H22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I22" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J22" t="n">
         <v>1</v>
       </c>
       <c r="K22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
@@ -6218,134 +6218,134 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="O22" t="n">
-        <v>101.7</v>
+        <v>100.8</v>
       </c>
       <c r="P22" t="n">
-        <v>1.7</v>
+        <v>0.8</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="R22" t="n">
-        <v>2348198</v>
+        <v>3441670</v>
       </c>
       <c r="S22" t="n">
-        <v>2735246</v>
+        <v>3395267</v>
       </c>
       <c r="T22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>3xc</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>301</v>
+        <v>319</v>
       </c>
       <c r="D23" t="n">
-        <v>71.8</v>
+        <v>68.8</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="G23" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="H23" t="n">
         <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J23" t="n">
         <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M23" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="O23" t="n">
-        <v>100.6</v>
+        <v>101.7</v>
       </c>
       <c r="P23" t="n">
-        <v>0.6</v>
+        <v>1.7</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
       <c r="R23" t="n">
-        <v>2179604</v>
+        <v>2348198</v>
       </c>
       <c r="S23" t="n">
-        <v>3048395</v>
+        <v>2735246</v>
       </c>
       <c r="T23" t="n">
         <v>2</v>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>300</v>
+        <v>319</v>
       </c>
       <c r="D24" t="n">
-        <v>67.2</v>
+        <v>67.5</v>
       </c>
       <c r="E24" t="n">
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="G24" t="n">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J24" t="n">
         <v>1</v>
@@ -6360,29 +6360,29 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="O24" t="n">
-        <v>100.2</v>
+        <v>101.9</v>
       </c>
       <c r="P24" t="n">
-        <v>0.2</v>
+        <v>1.9</v>
       </c>
       <c r="Q24" t="n">
-        <v>1.8</v>
+        <v>0.6</v>
       </c>
       <c r="R24" t="n">
-        <v>2211172</v>
+        <v>1861457</v>
       </c>
       <c r="S24" t="n">
-        <v>1595922</v>
+        <v>2489160</v>
       </c>
       <c r="T24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>bboost, 3xc, wildcard</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
@@ -6398,7 +6398,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>296</v>
+        <v>317</v>
       </c>
       <c r="D25" t="n">
         <v>66.8</v>
@@ -6460,37 +6460,37 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>295</v>
+        <v>314</v>
       </c>
       <c r="D26" t="n">
-        <v>67.5</v>
+        <v>67.2</v>
       </c>
       <c r="E26" t="n">
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="G26" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="H26" t="n">
         <v>2</v>
       </c>
       <c r="I26" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="J26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K26" t="n">
         <v>3</v>
@@ -6502,65 +6502,69 @@
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="O26" t="n">
-        <v>101.1</v>
+        <v>100.2</v>
       </c>
       <c r="P26" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
       <c r="Q26" t="n">
-        <v>1.1</v>
+        <v>1.8</v>
       </c>
       <c r="R26" t="n">
-        <v>2669248</v>
+        <v>2211172</v>
       </c>
       <c r="S26" t="n">
-        <v>453361</v>
+        <v>1595922</v>
       </c>
       <c r="T26" t="n">
         <v>2</v>
       </c>
-      <c r="U26" t="inlineStr"/>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>bboost, 3xc, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>294</v>
+        <v>310</v>
       </c>
       <c r="D27" t="n">
-        <v>65.8</v>
+        <v>67.5</v>
       </c>
       <c r="E27" t="n">
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="G27" t="n">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="H27" t="n">
         <v>2</v>
       </c>
       <c r="I27" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="J27" t="n">
         <v>3</v>
       </c>
       <c r="K27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
@@ -6569,100 +6573,96 @@
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="O27" t="n">
-        <v>101.7</v>
+        <v>101.1</v>
       </c>
       <c r="P27" t="n">
-        <v>1.7</v>
+        <v>1.1</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.7</v>
+        <v>1.1</v>
       </c>
       <c r="R27" t="n">
-        <v>3150671</v>
+        <v>2669248</v>
       </c>
       <c r="S27" t="n">
-        <v>614528</v>
+        <v>453361</v>
       </c>
       <c r="T27" t="n">
-        <v>4</v>
-      </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>292</v>
+        <v>309</v>
       </c>
       <c r="D28" t="n">
-        <v>66.5</v>
+        <v>65.8</v>
       </c>
       <c r="E28" t="n">
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="G28" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H28" t="n">
+        <v>2</v>
+      </c>
+      <c r="I28" t="n">
+        <v>47</v>
+      </c>
+      <c r="J28" t="n">
         <v>3</v>
       </c>
-      <c r="I28" t="n">
-        <v>41</v>
-      </c>
-      <c r="J28" t="n">
-        <v>1</v>
-      </c>
       <c r="K28" t="n">
+        <v>2</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" t="n">
+        <v>69</v>
+      </c>
+      <c r="O28" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="P28" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="R28" t="n">
+        <v>3150671</v>
+      </c>
+      <c r="S28" t="n">
+        <v>614528</v>
+      </c>
+      <c r="T28" t="n">
         <v>4</v>
       </c>
-      <c r="L28" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" t="n">
-        <v>38</v>
-      </c>
-      <c r="O28" t="n">
-        <v>100.8</v>
-      </c>
-      <c r="P28" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>0</v>
-      </c>
-      <c r="R28" t="n">
-        <v>3441670</v>
-      </c>
-      <c r="S28" t="n">
-        <v>3395267</v>
-      </c>
-      <c r="T28" t="n">
-        <v>3</v>
-      </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>3xc</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
@@ -6678,7 +6678,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="D29" t="n">
         <v>61.8</v>
@@ -6749,7 +6749,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>261</v>
+        <v>278</v>
       </c>
       <c r="D30" t="n">
         <v>58</v>
@@ -6820,7 +6820,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>251</v>
+        <v>271</v>
       </c>
       <c r="D31" t="n">
         <v>56.8</v>
@@ -6891,7 +6891,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>207</v>
+        <v>225</v>
       </c>
       <c r="D32" t="n">
         <v>46.8</v>

</xml_diff>

<commit_message>
Update standings 2026-09-20 20:24 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -4818,7 +4818,7 @@
         <v>2.4</v>
       </c>
       <c r="R2" t="n">
-        <v>2278</v>
+        <v>8887</v>
       </c>
       <c r="S2" t="n">
         <v>270274</v>
@@ -4877,7 +4877,7 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="O3" t="n">
         <v>100.8</v>
@@ -4889,7 +4889,7 @@
         <v>0.2</v>
       </c>
       <c r="R3" t="n">
-        <v>152850</v>
+        <v>46691</v>
       </c>
       <c r="S3" t="n">
         <v>1461471</v>
@@ -4956,7 +4956,7 @@
         <v>0.7</v>
       </c>
       <c r="R4" t="n">
-        <v>330274</v>
+        <v>270586</v>
       </c>
       <c r="S4" t="n">
         <v>1229264</v>
@@ -5015,7 +5015,7 @@
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="O5" t="n">
         <v>100.8</v>
@@ -5027,7 +5027,7 @@
         <v>1</v>
       </c>
       <c r="R5" t="n">
-        <v>241342</v>
+        <v>552259</v>
       </c>
       <c r="S5" t="n">
         <v>3046343</v>
@@ -5086,7 +5086,7 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O6" t="n">
         <v>101</v>
@@ -5098,7 +5098,7 @@
         <v>0.5</v>
       </c>
       <c r="R6" t="n">
-        <v>573851</v>
+        <v>641704</v>
       </c>
       <c r="S6" t="n">
         <v>617418</v>
@@ -5157,7 +5157,7 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="O7" t="n">
         <v>101</v>
@@ -5169,7 +5169,7 @@
         <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>387912</v>
+        <v>784753</v>
       </c>
       <c r="S7" t="n">
         <v>3039834</v>
@@ -5228,7 +5228,7 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O8" t="n">
         <v>100.5</v>
@@ -5240,7 +5240,7 @@
         <v>2.5</v>
       </c>
       <c r="R8" t="n">
-        <v>607290</v>
+        <v>805575</v>
       </c>
       <c r="S8" t="n">
         <v>166751</v>
@@ -5299,7 +5299,7 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="O9" t="n">
         <v>101.1</v>
@@ -5311,7 +5311,7 @@
         <v>0.5</v>
       </c>
       <c r="R9" t="n">
-        <v>901537</v>
+        <v>828955</v>
       </c>
       <c r="S9" t="n">
         <v>5250200</v>
@@ -5382,7 +5382,7 @@
         <v>0.2</v>
       </c>
       <c r="R10" t="n">
-        <v>774708</v>
+        <v>923810</v>
       </c>
       <c r="S10" t="n">
         <v>1034411</v>
@@ -5453,7 +5453,7 @@
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>732747</v>
+        <v>1019924</v>
       </c>
       <c r="S11" t="n">
         <v>266328</v>
@@ -5512,7 +5512,7 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O12" t="n">
         <v>101.4</v>
@@ -5524,7 +5524,7 @@
         <v>0.2</v>
       </c>
       <c r="R12" t="n">
-        <v>1300624</v>
+        <v>1129549</v>
       </c>
       <c r="S12" t="n">
         <v>878473</v>
@@ -5583,7 +5583,7 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="O13" t="n">
         <v>100.4</v>
@@ -5595,7 +5595,7 @@
         <v>1.3</v>
       </c>
       <c r="R13" t="n">
-        <v>660299</v>
+        <v>1185799</v>
       </c>
       <c r="S13" t="n">
         <v>3009015</v>
@@ -5654,7 +5654,7 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O14" t="n">
         <v>100.9</v>
@@ -5666,7 +5666,7 @@
         <v>0.6</v>
       </c>
       <c r="R14" t="n">
-        <v>989440</v>
+        <v>1236521</v>
       </c>
       <c r="S14" t="n">
         <v>5881370</v>
@@ -5725,7 +5725,7 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="O15" t="n">
         <v>101.2</v>
@@ -5737,7 +5737,7 @@
         <v>1.1</v>
       </c>
       <c r="R15" t="n">
-        <v>1356982</v>
+        <v>1302824</v>
       </c>
       <c r="S15" t="n">
         <v>101935</v>
@@ -5796,7 +5796,7 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
         <v>101.8</v>
@@ -5808,7 +5808,7 @@
         <v>0.2</v>
       </c>
       <c r="R16" t="n">
-        <v>1091532</v>
+        <v>1363053</v>
       </c>
       <c r="S16" t="n">
         <v>466127</v>
@@ -5867,7 +5867,7 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="O17" t="n">
         <v>100.6</v>
@@ -5879,7 +5879,7 @@
         <v>0.4</v>
       </c>
       <c r="R17" t="n">
-        <v>995232</v>
+        <v>1488285</v>
       </c>
       <c r="S17" t="n">
         <v>4185865</v>
@@ -5938,7 +5938,7 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="O18" t="n">
         <v>100.9</v>
@@ -5950,7 +5950,7 @@
         <v>0</v>
       </c>
       <c r="R18" t="n">
-        <v>1356982</v>
+        <v>1553590</v>
       </c>
       <c r="S18" t="n">
         <v>1066412</v>
@@ -6009,7 +6009,7 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="O19" t="n">
         <v>100.4</v>
@@ -6021,7 +6021,7 @@
         <v>0.6</v>
       </c>
       <c r="R19" t="n">
-        <v>1366400</v>
+        <v>1838986</v>
       </c>
       <c r="S19" t="n">
         <v>637992</v>
@@ -6080,7 +6080,7 @@
         <v>-8</v>
       </c>
       <c r="N20" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O20" t="n">
         <v>100.6</v>
@@ -6092,7 +6092,7 @@
         <v>0.7</v>
       </c>
       <c r="R20" t="n">
-        <v>2179604</v>
+        <v>2026614</v>
       </c>
       <c r="S20" t="n">
         <v>3048395</v>
@@ -6151,7 +6151,7 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O21" t="n">
         <v>100.3</v>
@@ -6163,7 +6163,7 @@
         <v>2.7</v>
       </c>
       <c r="R21" t="n">
-        <v>1683534</v>
+        <v>2234745</v>
       </c>
       <c r="S21" t="n">
         <v>4399137</v>
@@ -6230,7 +6230,7 @@
         <v>0</v>
       </c>
       <c r="R22" t="n">
-        <v>3441670</v>
+        <v>2313816</v>
       </c>
       <c r="S22" t="n">
         <v>3395267</v>
@@ -6301,7 +6301,7 @@
         <v>0.4</v>
       </c>
       <c r="R23" t="n">
-        <v>2348198</v>
+        <v>2441235</v>
       </c>
       <c r="S23" t="n">
         <v>2735246</v>
@@ -6372,7 +6372,7 @@
         <v>0.6</v>
       </c>
       <c r="R24" t="n">
-        <v>1861457</v>
+        <v>2453794</v>
       </c>
       <c r="S24" t="n">
         <v>2489160</v>
@@ -6443,7 +6443,7 @@
         <v>0.1</v>
       </c>
       <c r="R25" t="n">
-        <v>2633084</v>
+        <v>2664369</v>
       </c>
       <c r="S25" t="n">
         <v>1948104</v>
@@ -6514,7 +6514,7 @@
         <v>1.8</v>
       </c>
       <c r="R26" t="n">
-        <v>2211172</v>
+        <v>2874375</v>
       </c>
       <c r="S26" t="n">
         <v>1595922</v>
@@ -6573,7 +6573,7 @@
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O27" t="n">
         <v>101.1</v>
@@ -6585,7 +6585,7 @@
         <v>1.1</v>
       </c>
       <c r="R27" t="n">
-        <v>2669248</v>
+        <v>3227559</v>
       </c>
       <c r="S27" t="n">
         <v>453361</v>
@@ -6640,7 +6640,7 @@
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="O28" t="n">
         <v>101.7</v>
@@ -6652,7 +6652,7 @@
         <v>0.7</v>
       </c>
       <c r="R28" t="n">
-        <v>3150671</v>
+        <v>3304136</v>
       </c>
       <c r="S28" t="n">
         <v>614528</v>
@@ -6723,7 +6723,7 @@
         <v>0</v>
       </c>
       <c r="R29" t="n">
-        <v>4297158</v>
+        <v>4785874</v>
       </c>
       <c r="S29" t="n">
         <v>3963132</v>
@@ -6794,7 +6794,7 @@
         <v>1</v>
       </c>
       <c r="R30" t="n">
-        <v>5509780</v>
+        <v>6152689</v>
       </c>
       <c r="S30" t="n">
         <v>1952243</v>
@@ -6853,7 +6853,7 @@
         <v>-4</v>
       </c>
       <c r="N31" t="n">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="O31" t="n">
         <v>100.7</v>
@@ -6865,7 +6865,7 @@
         <v>1.2</v>
       </c>
       <c r="R31" t="n">
-        <v>7139131</v>
+        <v>6685768</v>
       </c>
       <c r="S31" t="n">
         <v>553038</v>
@@ -6936,7 +6936,7 @@
         <v>2.2</v>
       </c>
       <c r="R32" t="n">
-        <v>9241407</v>
+        <v>8999562</v>
       </c>
       <c r="S32" t="n">
         <v>216389</v>

</xml_diff>

<commit_message>
Update standings 2026-09-21 15:38 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -508,13 +508,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="4">
@@ -547,22 +547,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="6">
@@ -571,22 +571,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="7">
@@ -595,22 +595,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>345</v>
+        <v>351</v>
       </c>
     </row>
     <row r="8">
@@ -619,22 +619,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>345</v>
+        <v>348</v>
       </c>
     </row>
     <row r="9">
@@ -643,22 +643,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="10">
@@ -667,22 +667,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>342</v>
+        <v>345</v>
       </c>
     </row>
     <row r="11">
@@ -691,22 +691,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>26</v>
+        <v>60</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>340</v>
+        <v>344</v>
       </c>
     </row>
     <row r="12">
@@ -715,22 +715,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>338</v>
+        <v>344</v>
       </c>
     </row>
     <row r="13">
@@ -739,22 +739,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>337</v>
+        <v>343</v>
       </c>
     </row>
     <row r="14">
@@ -763,22 +763,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>336</v>
+        <v>340</v>
       </c>
     </row>
     <row r="15">
@@ -796,37 +796,37 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>334</v>
+        <v>337</v>
       </c>
     </row>
     <row r="17">
@@ -835,22 +835,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="18">
@@ -859,22 +859,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="19">
@@ -988,13 +988,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="24">
@@ -1027,22 +1027,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="E25" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="26">
@@ -1051,22 +1051,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="F26" t="n">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="27">
@@ -1075,22 +1075,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>310</v>
+        <v>314</v>
       </c>
     </row>
     <row r="28">
@@ -1108,13 +1108,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="29">
@@ -1156,13 +1156,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="E30" t="n">
         <v>-8</v>
       </c>
       <c r="F30" t="n">
-        <v>278</v>
+        <v>284</v>
       </c>
     </row>
     <row r="31">
@@ -1180,13 +1180,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E31" t="n">
         <v>-4</v>
       </c>
       <c r="F31" t="n">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="32">
@@ -1204,13 +1204,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>225</v>
+        <v>233</v>
       </c>
     </row>
   </sheetData>
@@ -1262,14 +1262,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -1286,17 +1286,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C3" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D3" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -1310,14 +1310,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pranav Thomas</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -1334,14 +1334,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C5" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -1358,17 +1358,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -1382,17 +1382,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Pranav Thomas</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D7" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -1406,14 +1406,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>3</v>
       </c>
       <c r="C8" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -1430,14 +1430,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C9" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -1454,17 +1454,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -1478,17 +1478,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C11" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -1502,14 +1502,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C12" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
@@ -1526,14 +1526,14 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C13" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -1558,7 +1558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1587,6 +1587,11 @@
           <t>GW4</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>GW5</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1606,6 +1611,9 @@
       <c r="E2" t="n">
         <v>81</v>
       </c>
+      <c r="F2" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1625,6 +1633,9 @@
       <c r="E3" t="n">
         <v>116</v>
       </c>
+      <c r="F3" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1644,195 +1655,228 @@
       <c r="E4" t="n">
         <v>107</v>
       </c>
+      <c r="F4" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C5" t="n">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="D5" t="n">
         <v>45</v>
       </c>
       <c r="E5" t="n">
-        <v>77</v>
+        <v>92</v>
+      </c>
+      <c r="F5" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B6" t="n">
+        <v>52</v>
+      </c>
+      <c r="C6" t="n">
+        <v>113</v>
+      </c>
+      <c r="D6" t="n">
+        <v>45</v>
+      </c>
+      <c r="E6" t="n">
+        <v>77</v>
+      </c>
+      <c r="F6" t="n">
         <v>64</v>
-      </c>
-      <c r="C6" t="n">
-        <v>105</v>
-      </c>
-      <c r="D6" t="n">
-        <v>60</v>
-      </c>
-      <c r="E6" t="n">
-        <v>76</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="C7" t="n">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="D7" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E7" t="n">
-        <v>71</v>
+        <v>76</v>
+      </c>
+      <c r="F7" t="n">
+        <v>46</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D8" t="n">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="E8" t="n">
-        <v>84</v>
+        <v>91</v>
+      </c>
+      <c r="F8" t="n">
+        <v>43</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="C9" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D9" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E9" t="n">
-        <v>75</v>
+        <v>71</v>
+      </c>
+      <c r="F9" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="C10" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D10" t="n">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="E10" t="n">
-        <v>91</v>
+        <v>84</v>
+      </c>
+      <c r="F10" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>74</v>
+        <v>40</v>
       </c>
       <c r="C11" t="n">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="D11" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="E11" t="n">
-        <v>92</v>
+        <v>71</v>
+      </c>
+      <c r="F11" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="C12" t="n">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D12" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="E12" t="n">
-        <v>70</v>
+        <v>75</v>
+      </c>
+      <c r="F12" t="n">
+        <v>61</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="C13" t="n">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D13" t="n">
-        <v>67</v>
+        <v>40</v>
       </c>
       <c r="E13" t="n">
-        <v>71</v>
+        <v>91</v>
+      </c>
+      <c r="F13" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="C14" t="n">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="D14" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E14" t="n">
-        <v>71</v>
+        <v>70</v>
+      </c>
+      <c r="F14" t="n">
+        <v>51</v>
       </c>
     </row>
     <row r="15">
@@ -1853,62 +1897,74 @@
       <c r="E15" t="n">
         <v>69</v>
       </c>
+      <c r="F15" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>91</v>
+        <v>71</v>
+      </c>
+      <c r="F16" t="n">
+        <v>51</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="C17" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D17" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E17" t="n">
-        <v>73</v>
+        <v>58</v>
+      </c>
+      <c r="F17" t="n">
+        <v>49</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="C18" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D18" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E18" t="n">
-        <v>58</v>
+        <v>73</v>
+      </c>
+      <c r="F18" t="n">
+        <v>52</v>
       </c>
     </row>
     <row r="19">
@@ -1929,6 +1985,9 @@
       <c r="E19" t="n">
         <v>62</v>
       </c>
+      <c r="F19" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1948,6 +2007,9 @@
       <c r="E20" t="n">
         <v>87</v>
       </c>
+      <c r="F20" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1967,6 +2029,9 @@
       <c r="E21" t="n">
         <v>76</v>
       </c>
+      <c r="F21" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1986,6 +2051,9 @@
       <c r="E22" t="n">
         <v>69</v>
       </c>
+      <c r="F22" t="n">
+        <v>55</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2005,6 +2073,9 @@
       <c r="E23" t="n">
         <v>90</v>
       </c>
+      <c r="F23" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2024,62 +2095,74 @@
       <c r="E24" t="n">
         <v>93</v>
       </c>
+      <c r="F24" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C25" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D25" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E25" t="n">
-        <v>66</v>
+        <v>77</v>
+      </c>
+      <c r="F25" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B26" t="n">
+        <v>53</v>
+      </c>
+      <c r="C26" t="n">
+        <v>102</v>
+      </c>
+      <c r="D26" t="n">
         <v>46</v>
       </c>
-      <c r="C26" t="n">
-        <v>89</v>
-      </c>
-      <c r="D26" t="n">
+      <c r="E26" t="n">
+        <v>66</v>
+      </c>
+      <c r="F26" t="n">
         <v>50</v>
-      </c>
-      <c r="E26" t="n">
-        <v>84</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="C27" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="D27" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E27" t="n">
-        <v>77</v>
+        <v>84</v>
+      </c>
+      <c r="F27" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="28">
@@ -2100,6 +2183,9 @@
       <c r="E28" t="n">
         <v>77</v>
       </c>
+      <c r="F28" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2119,6 +2205,9 @@
       <c r="E29" t="n">
         <v>69</v>
       </c>
+      <c r="F29" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2138,6 +2227,9 @@
       <c r="E30" t="n">
         <v>89</v>
       </c>
+      <c r="F30" t="n">
+        <v>52</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2157,6 +2249,9 @@
       <c r="E31" t="n">
         <v>69</v>
       </c>
+      <c r="F31" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2175,6 +2270,9 @@
       </c>
       <c r="E32" t="n">
         <v>55</v>
+      </c>
+      <c r="F32" t="n">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -2323,51 +2421,51 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="C6" t="inlineStr"/>
     </row>
@@ -2378,7 +2476,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="C7" t="inlineStr"/>
     </row>
@@ -2389,7 +2487,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="C8" t="inlineStr"/>
     </row>
@@ -2400,7 +2498,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -2411,11 +2509,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -2426,44 +2524,48 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>78</v>
-      </c>
-      <c r="C11" t="inlineStr"/>
+        <v>90</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="C14" t="inlineStr"/>
     </row>
@@ -2474,7 +2576,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="C15" t="inlineStr"/>
     </row>
@@ -2485,29 +2587,33 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>77</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
+        <v>84</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2518,26 +2624,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>72</v>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="C20" t="inlineStr"/>
     </row>
@@ -2548,13 +2650,9 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>67</v>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="C21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2563,7 +2661,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="C22" t="inlineStr"/>
     </row>
@@ -2574,95 +2672,95 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="C23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="C24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="C25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="C26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="C27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="C28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="C29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="C31" t="inlineStr"/>
     </row>
@@ -2673,7 +2771,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C32" t="inlineStr"/>
     </row>
@@ -2715,7 +2813,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -2726,7 +2824,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -2737,129 +2835,133 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Abhay Rawat</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Abhay Rawat</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>2</v>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>2</v>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>2</v>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>2</v>
       </c>
-      <c r="C13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2870,7 +2972,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2881,7 +2983,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2892,7 +2994,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2903,7 +3005,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -2914,7 +3016,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -2925,7 +3027,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -2936,7 +3038,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -2947,7 +3049,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -2958,77 +3060,73 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Pranav Thomas</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -3039,7 +3137,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -3050,7 +3148,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -3061,7 +3159,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Pranav Thomas</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -3370,85 +3468,85 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Jacquet</t>
+          <t>Trafford</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D13" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E13" t="n">
-        <v>2.7</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Abhay Rawat</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Ballard</t>
+          <t>Jacquet</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E14" t="n">
-        <v>4.9</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Abhay Rawat</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ballard</t>
+          <t>Barnes</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E15" t="n">
-        <v>4.9</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Ballard</t>
+          <t>Barnes</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E16" t="n">
-        <v>4.9</v>
+        <v>4.4</v>
       </c>
     </row>
   </sheetData>
@@ -3629,30 +3727,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E5" t="n">
-        <v>189374</v>
+        <v>71857</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>1757289</v>
+        <v>1929309</v>
       </c>
       <c r="H5" t="n">
-        <v>250879</v>
+        <v>297407</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -3666,30 +3764,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E6" t="n">
-        <v>6474</v>
+        <v>189374</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1177681</v>
+        <v>1757289</v>
       </c>
       <c r="H6" t="n">
-        <v>6474</v>
+        <v>250879</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -3703,19 +3801,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E7" t="n">
-        <v>182900</v>
+        <v>6474</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -3723,10 +3821,10 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>2098988</v>
+        <v>1177681</v>
       </c>
       <c r="H7" t="n">
-        <v>182900</v>
+        <v>6474</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -3740,30 +3838,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E8" t="n">
-        <v>27153</v>
+        <v>28582</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>606381</v>
+        <v>881388</v>
       </c>
       <c r="H8" t="n">
-        <v>240451</v>
+        <v>239490</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -3777,30 +3875,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E9" t="n">
-        <v>486041</v>
+        <v>182900</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>2415786</v>
+        <v>2098988</v>
       </c>
       <c r="H9" t="n">
-        <v>1206623</v>
+        <v>182900</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -3814,30 +3912,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E10" t="n">
-        <v>30971</v>
+        <v>27153</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>820221</v>
+        <v>606381</v>
       </c>
       <c r="H10" t="n">
-        <v>58227</v>
+        <v>240451</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -3851,30 +3949,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E11" t="n">
-        <v>71857</v>
+        <v>273503</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>1929309</v>
+        <v>1994005</v>
       </c>
       <c r="H11" t="n">
-        <v>297407</v>
+        <v>1917309</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -3888,30 +3986,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>8917</v>
+        <v>486041</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>2118382</v>
+        <v>2415786</v>
       </c>
       <c r="H12" t="n">
-        <v>9146930</v>
+        <v>1206623</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -3925,30 +4023,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E13" t="n">
-        <v>453230</v>
+        <v>30971</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>5483351</v>
+        <v>820221</v>
       </c>
       <c r="H13" t="n">
-        <v>8188106</v>
+        <v>58227</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -3962,30 +4060,30 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E14" t="n">
-        <v>273503</v>
+        <v>8917</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>1994005</v>
+        <v>2118382</v>
       </c>
       <c r="H14" t="n">
-        <v>1917309</v>
+        <v>9146930</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -4032,34 +4130,34 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>28582</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>881388</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>239490</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -4073,30 +4171,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="E17" t="n">
-        <v>410102</v>
+        <v>31543</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>2088802</v>
+        <v>820692</v>
       </c>
       <c r="H17" t="n">
-        <v>5360778</v>
+        <v>1637750</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4110,30 +4208,30 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E18" t="n">
-        <v>31543</v>
+        <v>410102</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>820692</v>
+        <v>2088802</v>
       </c>
       <c r="H18" t="n">
-        <v>1637750</v>
+        <v>5360778</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -4369,19 +4467,19 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E25" t="n">
-        <v>1320699</v>
+        <v>334016</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -4389,14 +4487,14 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>2490743</v>
+        <v>2156629</v>
       </c>
       <c r="H25" t="n">
-        <v>1861933</v>
+        <v>2691725</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
     </row>
@@ -4406,34 +4504,34 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E26" t="n">
-        <v>1615102</v>
+        <v>1320699</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
+          <t>2020/21</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>2490743</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1861933</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
           <t>2024/25</t>
-        </is>
-      </c>
-      <c r="G26" t="n">
-        <v>4234674</v>
-      </c>
-      <c r="H26" t="n">
-        <v>6092784</v>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>2025/26</t>
         </is>
       </c>
     </row>
@@ -4443,30 +4541,30 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>334016</v>
+        <v>1615102</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>2156629</v>
+        <v>4234674</v>
       </c>
       <c r="H27" t="n">
-        <v>2691725</v>
+        <v>6092784</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -4776,13 +4874,13 @@
         <v>395</v>
       </c>
       <c r="D2" t="n">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F2" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="G2" t="n">
         <v>126</v>
@@ -4791,10 +4889,10 @@
         <v>2</v>
       </c>
       <c r="I2" t="n">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="J2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K2" t="n">
         <v>2</v>
@@ -4818,7 +4916,7 @@
         <v>2.4</v>
       </c>
       <c r="R2" t="n">
-        <v>8887</v>
+        <v>14101</v>
       </c>
       <c r="S2" t="n">
         <v>270274</v>
@@ -4844,16 +4942,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="D3" t="n">
-        <v>81.2</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="G3" t="n">
         <v>116</v>
@@ -4877,7 +4975,7 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="O3" t="n">
         <v>100.8</v>
@@ -4889,7 +4987,7 @@
         <v>0.2</v>
       </c>
       <c r="R3" t="n">
-        <v>46691</v>
+        <v>56391</v>
       </c>
       <c r="S3" t="n">
         <v>1461471</v>
@@ -4914,13 +5012,13 @@
         <v>362</v>
       </c>
       <c r="D4" t="n">
-        <v>78.8</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
       </c>
       <c r="F4" t="n">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="G4" t="n">
         <v>107</v>
@@ -4956,7 +5054,7 @@
         <v>0.7</v>
       </c>
       <c r="R4" t="n">
-        <v>270586</v>
+        <v>352905</v>
       </c>
       <c r="S4" t="n">
         <v>1229264</v>
@@ -4973,111 +5071,111 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="D5" t="n">
-        <v>71.8</v>
+        <v>70.8</v>
       </c>
       <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>90</v>
+      </c>
+      <c r="G5" t="n">
+        <v>103</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>40</v>
+      </c>
+      <c r="J5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K5" t="n">
         <v>1</v>
       </c>
-      <c r="F5" t="n">
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
         <v>78</v>
       </c>
-      <c r="G5" t="n">
-        <v>113</v>
-      </c>
-      <c r="H5" t="n">
-        <v>2</v>
-      </c>
-      <c r="I5" t="n">
-        <v>45</v>
-      </c>
-      <c r="J5" t="n">
-        <v>3</v>
-      </c>
-      <c r="K5" t="n">
-        <v>2</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" t="n">
-        <v>47</v>
-      </c>
       <c r="O5" t="n">
-        <v>100.8</v>
+        <v>101.6</v>
       </c>
       <c r="P5" t="n">
-        <v>0.8</v>
+        <v>1.6</v>
       </c>
       <c r="Q5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>552259</v>
+        <v>572645</v>
       </c>
       <c r="S5" t="n">
-        <v>3046343</v>
+        <v>266328</v>
       </c>
       <c r="T5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="D6" t="n">
-        <v>76.2</v>
+        <v>70.2</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="G6" t="n">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="H6" t="n">
         <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="J6" t="n">
         <v>3</v>
       </c>
       <c r="K6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
@@ -5086,69 +5184,69 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>79</v>
+        <v>47</v>
       </c>
       <c r="O6" t="n">
-        <v>101</v>
+        <v>100.8</v>
       </c>
       <c r="P6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="Q6" t="n">
         <v>1</v>
       </c>
-      <c r="Q6" t="n">
-        <v>0.5</v>
-      </c>
       <c r="R6" t="n">
-        <v>641704</v>
+        <v>686560</v>
       </c>
       <c r="S6" t="n">
-        <v>617418</v>
+        <v>3046343</v>
       </c>
       <c r="T6" t="n">
         <v>2</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="D7" t="n">
-        <v>74.2</v>
+        <v>70.2</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="G7" t="n">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="H7" t="n">
         <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="J7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -5157,7 +5255,7 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="O7" t="n">
         <v>101</v>
@@ -5166,155 +5264,155 @@
         <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="R7" t="n">
-        <v>784753</v>
+        <v>706165</v>
       </c>
       <c r="S7" t="n">
-        <v>3039834</v>
+        <v>617418</v>
       </c>
       <c r="T7" t="n">
         <v>2</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="D8" t="n">
-        <v>78.2</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="G8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="H8" t="n">
         <v>2</v>
       </c>
       <c r="I8" t="n">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="J8" t="n">
         <v>3</v>
       </c>
       <c r="K8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>27</v>
+      </c>
+      <c r="O8" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="P8" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="R8" t="n">
+        <v>812352</v>
+      </c>
+      <c r="S8" t="n">
+        <v>466127</v>
+      </c>
+      <c r="T8" t="n">
         <v>4</v>
       </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" t="n">
-        <v>54</v>
-      </c>
-      <c r="O8" t="n">
-        <v>100.5</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="R8" t="n">
-        <v>805575</v>
-      </c>
-      <c r="S8" t="n">
-        <v>166751</v>
-      </c>
-      <c r="T8" t="n">
-        <v>2</v>
-      </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D9" t="n">
-        <v>70.8</v>
+        <v>69</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>57</v>
+        <v>99</v>
       </c>
       <c r="G9" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="H9" t="n">
         <v>2</v>
       </c>
       <c r="I9" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="J9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>61</v>
+      </c>
+      <c r="O9" t="n">
+        <v>101</v>
+      </c>
+      <c r="P9" t="n">
         <v>1</v>
       </c>
-      <c r="K9" t="n">
-        <v>2</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" t="n">
-        <v>47</v>
-      </c>
-      <c r="O9" t="n">
-        <v>101.1</v>
-      </c>
-      <c r="P9" t="n">
-        <v>1.1</v>
-      </c>
       <c r="Q9" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>828955</v>
+        <v>953327</v>
       </c>
       <c r="S9" t="n">
-        <v>5250200</v>
+        <v>3039834</v>
       </c>
       <c r="T9" t="n">
         <v>2</v>
@@ -5328,40 +5426,40 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="D10" t="n">
-        <v>74.8</v>
+        <v>69</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="G10" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H10" t="n">
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="J10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -5370,69 +5468,69 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="O10" t="n">
-        <v>101.3</v>
+        <v>100.5</v>
       </c>
       <c r="P10" t="n">
-        <v>1.3</v>
+        <v>0.5</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.2</v>
+        <v>2.5</v>
       </c>
       <c r="R10" t="n">
-        <v>923810</v>
+        <v>976059</v>
       </c>
       <c r="S10" t="n">
-        <v>1034411</v>
+        <v>166751</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="D11" t="n">
-        <v>78.5</v>
+        <v>68.8</v>
       </c>
       <c r="E11" t="n">
         <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>78</v>
+        <v>107</v>
       </c>
       <c r="G11" t="n">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="H11" t="n">
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="J11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -5441,137 +5539,137 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>92</v>
+        <v>65</v>
       </c>
       <c r="O11" t="n">
-        <v>101.6</v>
+        <v>100.9</v>
       </c>
       <c r="P11" t="n">
-        <v>1.6</v>
+        <v>0.9</v>
       </c>
       <c r="Q11" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="R11" t="n">
-        <v>1019924</v>
+        <v>996186</v>
       </c>
       <c r="S11" t="n">
-        <v>266328</v>
+        <v>5881370</v>
       </c>
       <c r="T11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="D12" t="n">
-        <v>72.2</v>
+        <v>68.8</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12" t="n">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="G12" t="n">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="H12" t="n">
         <v>2</v>
       </c>
       <c r="I12" t="n">
+        <v>42</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
+        <v>2</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
         <v>47</v>
       </c>
-      <c r="J12" t="n">
-        <v>3</v>
-      </c>
-      <c r="K12" t="n">
-        <v>2</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" t="n">
-        <v>80</v>
-      </c>
       <c r="O12" t="n">
-        <v>101.4</v>
+        <v>101.1</v>
       </c>
       <c r="P12" t="n">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="R12" t="n">
-        <v>1129549</v>
+        <v>1003072</v>
       </c>
       <c r="S12" t="n">
-        <v>878473</v>
+        <v>5250200</v>
       </c>
       <c r="T12" t="n">
         <v>2</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="D13" t="n">
-        <v>71.5</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="G13" t="n">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H13" t="n">
         <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K13" t="n">
         <v>2</v>
@@ -5583,69 +5681,69 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="O13" t="n">
-        <v>100.4</v>
+        <v>101.3</v>
       </c>
       <c r="P13" t="n">
-        <v>0.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q13" t="n">
-        <v>1.3</v>
+        <v>0.2</v>
       </c>
       <c r="R13" t="n">
-        <v>1185799</v>
+        <v>1054718</v>
       </c>
       <c r="S13" t="n">
-        <v>3009015</v>
+        <v>1034411</v>
       </c>
       <c r="T13" t="n">
         <v>2</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="D14" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="G14" t="n">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="H14" t="n">
         <v>2</v>
       </c>
       <c r="I14" t="n">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -5654,29 +5752,29 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="O14" t="n">
-        <v>100.9</v>
+        <v>101.4</v>
       </c>
       <c r="P14" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="R14" t="n">
-        <v>1236521</v>
+        <v>1218344</v>
       </c>
       <c r="S14" t="n">
-        <v>5881370</v>
+        <v>878473</v>
       </c>
       <c r="T14" t="n">
         <v>2</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
@@ -5692,16 +5790,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="D15" t="n">
-        <v>71.8</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
         <v>90</v>
@@ -5710,10 +5808,10 @@
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5725,7 +5823,7 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
         <v>101.2</v>
@@ -5737,7 +5835,7 @@
         <v>1.1</v>
       </c>
       <c r="R15" t="n">
-        <v>1302824</v>
+        <v>1396886</v>
       </c>
       <c r="S15" t="n">
         <v>101935</v>
@@ -5754,37 +5852,37 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="D16" t="n">
-        <v>76.2</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="E16" t="n">
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5799,63 +5897,63 @@
         <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.8</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.8</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.2</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
-        <v>1363053</v>
+        <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>466127</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="D17" t="n">
-        <v>70</v>
+        <v>66.8</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F17" t="n">
-        <v>81</v>
+        <v>117</v>
       </c>
       <c r="G17" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="H17" t="n">
         <v>2</v>
       </c>
       <c r="I17" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="J17" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K17" t="n">
         <v>2</v>
@@ -5867,66 +5965,66 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="O17" t="n">
-        <v>100.6</v>
+        <v>100.9</v>
       </c>
       <c r="P17" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>1488285</v>
+        <v>1589056</v>
       </c>
       <c r="S17" t="n">
-        <v>4185865</v>
+        <v>1066412</v>
       </c>
       <c r="T17" t="n">
         <v>2</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D18" t="n">
-        <v>71.2</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="E18" t="n">
         <v>3</v>
       </c>
       <c r="F18" t="n">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="G18" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="H18" t="n">
         <v>2</v>
       </c>
       <c r="I18" t="n">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="J18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K18" t="n">
         <v>2</v>
@@ -5938,29 +6036,29 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="O18" t="n">
-        <v>100.9</v>
+        <v>100.6</v>
       </c>
       <c r="P18" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="Q18" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="R18" t="n">
-        <v>1553590</v>
+        <v>1724545</v>
       </c>
       <c r="S18" t="n">
-        <v>1066412</v>
+        <v>4185865</v>
       </c>
       <c r="T18" t="n">
         <v>2</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
@@ -5979,13 +6077,13 @@
         <v>327</v>
       </c>
       <c r="D19" t="n">
-        <v>75</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="E19" t="n">
         <v>3</v>
       </c>
       <c r="F19" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G19" t="n">
         <v>111</v>
@@ -5994,10 +6092,10 @@
         <v>2</v>
       </c>
       <c r="I19" t="n">
-        <v>61</v>
+        <v>27</v>
       </c>
       <c r="J19" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K19" t="n">
         <v>3</v>
@@ -6021,7 +6119,7 @@
         <v>0.6</v>
       </c>
       <c r="R19" t="n">
-        <v>1838986</v>
+        <v>2099042</v>
       </c>
       <c r="S19" t="n">
         <v>637992</v>
@@ -6050,13 +6148,13 @@
         <v>325</v>
       </c>
       <c r="D20" t="n">
-        <v>71.8</v>
+        <v>65</v>
       </c>
       <c r="E20" t="n">
         <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="G20" t="n">
         <v>97</v>
@@ -6065,10 +6163,10 @@
         <v>2</v>
       </c>
       <c r="I20" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K20" t="n">
         <v>5</v>
@@ -6092,7 +6190,7 @@
         <v>0.7</v>
       </c>
       <c r="R20" t="n">
-        <v>2026614</v>
+        <v>2297297</v>
       </c>
       <c r="S20" t="n">
         <v>3048395</v>
@@ -6121,13 +6219,13 @@
         <v>322</v>
       </c>
       <c r="D21" t="n">
-        <v>73.2</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="E21" t="n">
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="G21" t="n">
         <v>120</v>
@@ -6136,10 +6234,10 @@
         <v>2</v>
       </c>
       <c r="I21" t="n">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K21" t="n">
         <v>4</v>
@@ -6163,7 +6261,7 @@
         <v>2.7</v>
       </c>
       <c r="R21" t="n">
-        <v>2234745</v>
+        <v>2516305</v>
       </c>
       <c r="S21" t="n">
         <v>4399137</v>
@@ -6188,13 +6286,13 @@
         <v>321</v>
       </c>
       <c r="D22" t="n">
-        <v>66.5</v>
+        <v>64.2</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="G22" t="n">
         <v>78</v>
@@ -6230,7 +6328,7 @@
         <v>0</v>
       </c>
       <c r="R22" t="n">
-        <v>2313816</v>
+        <v>2598730</v>
       </c>
       <c r="S22" t="n">
         <v>3395267</v>
@@ -6256,16 +6354,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D23" t="n">
-        <v>68.8</v>
+        <v>64</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="G23" t="n">
         <v>93</v>
@@ -6289,7 +6387,7 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="O23" t="n">
         <v>101.7</v>
@@ -6301,7 +6399,7 @@
         <v>0.4</v>
       </c>
       <c r="R23" t="n">
-        <v>2441235</v>
+        <v>2648287</v>
       </c>
       <c r="S23" t="n">
         <v>2735246</v>
@@ -6330,13 +6428,13 @@
         <v>319</v>
       </c>
       <c r="D24" t="n">
-        <v>67.5</v>
+        <v>63.8</v>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="G24" t="n">
         <v>93</v>
@@ -6372,7 +6470,7 @@
         <v>0.6</v>
       </c>
       <c r="R24" t="n">
-        <v>2453794</v>
+        <v>2745198</v>
       </c>
       <c r="S24" t="n">
         <v>2489160</v>
@@ -6389,49 +6487,49 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D25" t="n">
-        <v>66.8</v>
+        <v>63.6</v>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" t="n">
-        <v>58</v>
+        <v>84</v>
       </c>
       <c r="G25" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="H25" t="n">
         <v>2</v>
       </c>
       <c r="I25" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="J25" t="n">
         <v>3</v>
       </c>
       <c r="K25" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="O25" t="n">
         <v>101.1</v>
@@ -6440,48 +6538,44 @@
         <v>1.1</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.1</v>
+        <v>1.1</v>
       </c>
       <c r="R25" t="n">
-        <v>2664369</v>
+        <v>2831164</v>
       </c>
       <c r="S25" t="n">
-        <v>1948104</v>
+        <v>453361</v>
       </c>
       <c r="T25" t="n">
         <v>2</v>
       </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>wildcard</t>
-        </is>
-      </c>
+      <c r="U25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="D26" t="n">
-        <v>67.2</v>
+        <v>63.4</v>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F26" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G26" t="n">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="H26" t="n">
         <v>2</v>
@@ -6490,78 +6584,78 @@
         <v>46</v>
       </c>
       <c r="J26" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K26" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M26" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="N26" t="n">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="O26" t="n">
-        <v>100.2</v>
+        <v>101.1</v>
       </c>
       <c r="P26" t="n">
-        <v>0.2</v>
+        <v>1.1</v>
       </c>
       <c r="Q26" t="n">
-        <v>1.8</v>
+        <v>0.1</v>
       </c>
       <c r="R26" t="n">
-        <v>2874375</v>
+        <v>2963253</v>
       </c>
       <c r="S26" t="n">
-        <v>1595922</v>
+        <v>1948104</v>
       </c>
       <c r="T26" t="n">
         <v>2</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>bboost, 3xc, wildcard</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="D27" t="n">
-        <v>67.5</v>
+        <v>62.8</v>
       </c>
       <c r="E27" t="n">
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="G27" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="H27" t="n">
         <v>2</v>
       </c>
       <c r="I27" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J27" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K27" t="n">
         <v>3</v>
@@ -6573,27 +6667,31 @@
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="O27" t="n">
-        <v>101.1</v>
+        <v>100.2</v>
       </c>
       <c r="P27" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
       <c r="Q27" t="n">
-        <v>1.1</v>
+        <v>1.8</v>
       </c>
       <c r="R27" t="n">
-        <v>3227559</v>
+        <v>3181539</v>
       </c>
       <c r="S27" t="n">
-        <v>453361</v>
+        <v>1595922</v>
       </c>
       <c r="T27" t="n">
         <v>2</v>
       </c>
-      <c r="U27" t="inlineStr"/>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>bboost, 3xc, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6607,16 +6705,16 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="D28" t="n">
-        <v>65.8</v>
+        <v>62.2</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F28" t="n">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="G28" t="n">
         <v>80</v>
@@ -6640,7 +6738,7 @@
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="O28" t="n">
         <v>101.7</v>
@@ -6652,7 +6750,7 @@
         <v>0.7</v>
       </c>
       <c r="R28" t="n">
-        <v>3304136</v>
+        <v>3440315</v>
       </c>
       <c r="S28" t="n">
         <v>614528</v>
@@ -6681,13 +6779,13 @@
         <v>293</v>
       </c>
       <c r="D29" t="n">
-        <v>61.8</v>
+        <v>58.6</v>
       </c>
       <c r="E29" t="n">
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="G29" t="n">
         <v>101</v>
@@ -6723,7 +6821,7 @@
         <v>0</v>
       </c>
       <c r="R29" t="n">
-        <v>4785874</v>
+        <v>5109269</v>
       </c>
       <c r="S29" t="n">
         <v>3963132</v>
@@ -6749,16 +6847,16 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="D30" t="n">
-        <v>58</v>
+        <v>56.8</v>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="G30" t="n">
         <v>89</v>
@@ -6782,7 +6880,7 @@
         <v>-8</v>
       </c>
       <c r="N30" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="O30" t="n">
         <v>101.4</v>
@@ -6794,7 +6892,7 @@
         <v>1</v>
       </c>
       <c r="R30" t="n">
-        <v>6152689</v>
+        <v>5949920</v>
       </c>
       <c r="S30" t="n">
         <v>1952243</v>
@@ -6820,16 +6918,16 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D31" t="n">
-        <v>56.8</v>
+        <v>54.6</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="G31" t="n">
         <v>73</v>
@@ -6853,7 +6951,7 @@
         <v>-4</v>
       </c>
       <c r="N31" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="O31" t="n">
         <v>100.7</v>
@@ -6865,7 +6963,7 @@
         <v>1.2</v>
       </c>
       <c r="R31" t="n">
-        <v>6685768</v>
+        <v>6804394</v>
       </c>
       <c r="S31" t="n">
         <v>553038</v>
@@ -6891,16 +6989,16 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="D32" t="n">
-        <v>46.8</v>
+        <v>46.6</v>
       </c>
       <c r="E32" t="n">
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="G32" t="n">
         <v>55</v>
@@ -6924,7 +7022,7 @@
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="O32" t="n">
         <v>99.2</v>
@@ -6936,7 +7034,7 @@
         <v>2.2</v>
       </c>
       <c r="R32" t="n">
-        <v>8999562</v>
+        <v>8883555</v>
       </c>
       <c r="S32" t="n">
         <v>216389</v>

</xml_diff>

<commit_message>
Update standings 2026-09-21 16:14 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-21 16:50 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-21 21:45 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-22 00:37 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-22 13:08 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-22 21:09 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-23 00:02 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-23 07:25 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-23 13:23 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-23 22:43 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-24 03:27 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-24 09:02 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-24 23:02 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-25 15:01 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-25 19:51 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-26 14:10 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-26 19:03 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-26 22:24 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-27 09:57 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-28 04:00 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-28 13:04 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-29 14:43 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-30 01:07 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-09-30 08:05 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-01 01:06 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-01 08:23 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-02 11:58 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-02 21:52 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-03 13:05 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-03 17:48 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-03 20:39 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-05 00:28 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-05 08:27 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-05 19:09 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-06 01:08 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-06 22:24 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-08 08:29 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-08 17:13 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-09 19:17 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-09 23:49 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-10 04:37 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -787,16 +787,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -811,16 +811,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>453230</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>5483351</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>8188106</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>453230</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>5483351</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>8188106</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -5781,12 +5781,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5799,19 +5799,19 @@
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,41 +5823,41 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>101.2</v>
+        <v>100.4</v>
       </c>
       <c r="P15" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="R15" t="n">
         <v>1396886</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>3009015</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5870,19 +5870,19 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>2</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O16" t="n">
-        <v>100.4</v>
+        <v>101.2</v>
       </c>
       <c r="P16" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="R16" t="n">
         <v>1396886</v>
       </c>
       <c r="S16" t="n">
-        <v>3009015</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-10 12:00 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -484,13 +484,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>51</v>
+        <v>2</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="3">
@@ -508,13 +508,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>58</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="4">
@@ -532,13 +532,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>47</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
         <v>-4</v>
       </c>
       <c r="F4" t="n">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
     <row r="5">
@@ -556,13 +556,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>354</v>
+        <v>360</v>
       </c>
     </row>
     <row r="6">
@@ -580,13 +580,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>64</v>
+        <v>3</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="7">
@@ -604,13 +604,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>46</v>
+        <v>2</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="8">
@@ -619,22 +619,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="9">
@@ -643,22 +643,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>345</v>
+        <v>350</v>
       </c>
     </row>
     <row r="10">
@@ -676,13 +676,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>345</v>
+        <v>349</v>
       </c>
     </row>
     <row r="11">
@@ -691,22 +691,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>60</v>
+        <v>4</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="12">
@@ -715,22 +715,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>61</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="13">
@@ -739,22 +739,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>343</v>
+        <v>346</v>
       </c>
     </row>
     <row r="14">
@@ -772,13 +772,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>340</v>
+        <v>343</v>
       </c>
     </row>
     <row r="15">
@@ -796,61 +796,61 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>337</v>
+        <v>340</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>337</v>
+        <v>340</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>49</v>
+        <v>3</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>334</v>
+        <v>340</v>
       </c>
     </row>
     <row r="18">
@@ -868,13 +868,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>52</v>
+        <v>6</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>332</v>
+        <v>338</v>
       </c>
     </row>
     <row r="19">
@@ -883,22 +883,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="F19" t="n">
-        <v>327</v>
+        <v>330</v>
       </c>
     </row>
     <row r="20">
@@ -907,22 +907,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>42</v>
+        <v>2</v>
       </c>
       <c r="E20" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="21">
@@ -931,22 +931,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>322</v>
+        <v>327</v>
       </c>
     </row>
     <row r="22">
@@ -955,22 +955,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>55</v>
+        <v>6</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>321</v>
+        <v>326</v>
       </c>
     </row>
     <row r="23">
@@ -979,22 +979,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>45</v>
+        <v>3</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
     <row r="24">
@@ -1003,46 +1003,46 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>49</v>
+        <v>3</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>318</v>
+        <v>321</v>
       </c>
     </row>
     <row r="26">
@@ -1051,22 +1051,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="E26" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="27">
@@ -1075,22 +1075,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="F27" t="n">
-        <v>314</v>
+        <v>319</v>
       </c>
     </row>
     <row r="28">
@@ -1108,13 +1108,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="29">
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>46</v>
+        <v>3</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>293</v>
+        <v>296</v>
       </c>
     </row>
     <row r="30">
@@ -1156,13 +1156,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="E30" t="n">
         <v>-8</v>
       </c>
       <c r="F30" t="n">
-        <v>284</v>
+        <v>287</v>
       </c>
     </row>
     <row r="31">
@@ -1180,13 +1180,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>46</v>
+        <v>9</v>
       </c>
       <c r="E31" t="n">
         <v>-4</v>
       </c>
       <c r="F31" t="n">
-        <v>273</v>
+        <v>282</v>
       </c>
     </row>
     <row r="32">
@@ -1204,13 +1204,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>46</v>
+        <v>2</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -1728,45 +1728,45 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>73</v>
+        <v>53</v>
       </c>
       <c r="C8" t="n">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="D8" t="n">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="E8" t="n">
-        <v>91</v>
+        <v>71</v>
       </c>
       <c r="F8" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="C9" t="n">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="D9" t="n">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="E9" t="n">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="F9" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10">
@@ -1794,67 +1794,67 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="n">
+        <v>61</v>
+      </c>
+      <c r="C11" t="n">
+        <v>107</v>
+      </c>
+      <c r="D11" t="n">
         <v>40</v>
       </c>
-      <c r="C11" t="n">
-        <v>118</v>
-      </c>
-      <c r="D11" t="n">
-        <v>55</v>
-      </c>
       <c r="E11" t="n">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="F11" t="n">
-        <v>60</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C12" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D12" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E12" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F12" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B13" t="n">
+        <v>42</v>
+      </c>
+      <c r="C13" t="n">
+        <v>114</v>
+      </c>
+      <c r="D13" t="n">
+        <v>52</v>
+      </c>
+      <c r="E13" t="n">
+        <v>75</v>
+      </c>
+      <c r="F13" t="n">
         <v>61</v>
-      </c>
-      <c r="C13" t="n">
-        <v>107</v>
-      </c>
-      <c r="D13" t="n">
-        <v>40</v>
-      </c>
-      <c r="E13" t="n">
-        <v>91</v>
-      </c>
-      <c r="F13" t="n">
-        <v>44</v>
       </c>
     </row>
     <row r="14">
@@ -1904,45 +1904,45 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="C17" t="n">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="D17" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E17" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="F17" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18">
@@ -1970,199 +1970,199 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="C19" t="n">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="D19" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E19" t="n">
-        <v>62</v>
+        <v>87</v>
       </c>
       <c r="F19" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="C20" t="n">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="D20" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E20" t="n">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="F20" t="n">
-        <v>38</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C21" t="n">
-        <v>120</v>
+        <v>78</v>
       </c>
       <c r="D21" t="n">
-        <v>49</v>
+        <v>78</v>
       </c>
       <c r="E21" t="n">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="F21" t="n">
-        <v>29</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C22" t="n">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="D22" t="n">
-        <v>78</v>
+        <v>50</v>
       </c>
       <c r="E22" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="F22" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C23" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="D23" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E23" t="n">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="F23" t="n">
-        <v>45</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E24" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="F24" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="C25" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D25" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E25" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="F25" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C26" t="n">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="D26" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E26" t="n">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="F26" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B27" t="n">
+        <v>53</v>
+      </c>
+      <c r="C27" t="n">
+        <v>102</v>
+      </c>
+      <c r="D27" t="n">
         <v>46</v>
       </c>
-      <c r="C27" t="n">
-        <v>89</v>
-      </c>
-      <c r="D27" t="n">
+      <c r="E27" t="n">
+        <v>66</v>
+      </c>
+      <c r="F27" t="n">
         <v>50</v>
-      </c>
-      <c r="E27" t="n">
-        <v>84</v>
-      </c>
-      <c r="F27" t="n">
-        <v>45</v>
       </c>
     </row>
     <row r="28">
@@ -2972,7 +2972,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2983,7 +2983,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -3005,7 +3005,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -3016,7 +3016,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -3082,7 +3082,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -3093,7 +3093,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -3838,30 +3838,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E8" t="n">
-        <v>28582</v>
+        <v>182900</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>881388</v>
+        <v>2098988</v>
       </c>
       <c r="H8" t="n">
-        <v>239490</v>
+        <v>182900</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -3875,30 +3875,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E9" t="n">
-        <v>182900</v>
+        <v>28582</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>2098988</v>
+        <v>881388</v>
       </c>
       <c r="H9" t="n">
-        <v>182900</v>
+        <v>239490</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -3949,30 +3949,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E11" t="n">
-        <v>273503</v>
+        <v>30971</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>1994005</v>
+        <v>820221</v>
       </c>
       <c r="H11" t="n">
-        <v>1917309</v>
+        <v>58227</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -3986,19 +3986,19 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E12" t="n">
-        <v>486041</v>
+        <v>273503</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -4006,10 +4006,10 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>2415786</v>
+        <v>1994005</v>
       </c>
       <c r="H12" t="n">
-        <v>1206623</v>
+        <v>1917309</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -4023,30 +4023,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D13" t="n">
         <v>10</v>
       </c>
       <c r="E13" t="n">
-        <v>30971</v>
+        <v>486041</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>820221</v>
+        <v>2415786</v>
       </c>
       <c r="H13" t="n">
-        <v>58227</v>
+        <v>1206623</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -4130,34 +4130,34 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E16" t="n">
-        <v>37120</v>
+        <v>31543</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1571193</v>
+        <v>820692</v>
       </c>
       <c r="H16" t="n">
-        <v>3349378</v>
+        <v>1637750</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -4167,34 +4167,34 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Abhishek Gupte</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Enzotic</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Shivanshu Madan</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Cold Palmer</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>7</v>
-      </c>
       <c r="E17" t="n">
-        <v>31543</v>
+        <v>37120</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>820692</v>
+        <v>1571193</v>
       </c>
       <c r="H17" t="n">
-        <v>1637750</v>
+        <v>3349378</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4245,30 +4245,30 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="E19" t="n">
-        <v>15136</v>
+        <v>1128645</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>983840</v>
+        <v>3434302</v>
       </c>
       <c r="H19" t="n">
-        <v>45077</v>
+        <v>1128645</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -4282,30 +4282,30 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E20" t="n">
-        <v>1128645</v>
+        <v>15136</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>3434302</v>
+        <v>983840</v>
       </c>
       <c r="H20" t="n">
-        <v>1128645</v>
+        <v>45077</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -4319,30 +4319,30 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E21" t="n">
-        <v>60517</v>
+        <v>15288</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2015/16</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>1414622</v>
+        <v>329510</v>
       </c>
       <c r="H21" t="n">
-        <v>339763</v>
+        <v>538046</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -4356,30 +4356,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E22" t="n">
-        <v>15288</v>
+        <v>14603</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2016/17</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>329510</v>
+        <v>949628</v>
       </c>
       <c r="H22" t="n">
-        <v>538046</v>
+        <v>515830</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -4393,30 +4393,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E23" t="n">
-        <v>14603</v>
+        <v>60517</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2016/17</t>
+          <t>2015/16</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>949628</v>
+        <v>1414622</v>
       </c>
       <c r="H23" t="n">
-        <v>515830</v>
+        <v>339763</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4430,30 +4430,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>95791</v>
+        <v>334016</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2404119</v>
+        <v>2156629</v>
       </c>
       <c r="H24" t="n">
-        <v>5124417</v>
+        <v>2691725</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -4463,34 +4463,34 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E25" t="n">
-        <v>334016</v>
+        <v>95791</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>2156629</v>
+        <v>2404119</v>
       </c>
       <c r="H25" t="n">
-        <v>2691725</v>
+        <v>5124417</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -4504,34 +4504,34 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E26" t="n">
-        <v>1320699</v>
+        <v>1615102</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>2490743</v>
+        <v>4234674</v>
       </c>
       <c r="H26" t="n">
-        <v>1861933</v>
+        <v>6092784</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
     </row>
@@ -4541,34 +4541,34 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E27" t="n">
-        <v>1615102</v>
+        <v>1320699</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
+          <t>2020/21</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>2490743</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1861933</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
           <t>2024/25</t>
-        </is>
-      </c>
-      <c r="G27" t="n">
-        <v>4234674</v>
-      </c>
-      <c r="H27" t="n">
-        <v>6092784</v>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>2025/26</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="D2" t="n">
         <v>79</v>
@@ -4907,10 +4907,10 @@
         <v>71</v>
       </c>
       <c r="O2" t="n">
-        <v>101.5</v>
+        <v>102.3</v>
       </c>
       <c r="P2" t="n">
-        <v>1.5</v>
+        <v>2.3</v>
       </c>
       <c r="Q2" t="n">
         <v>2.4</v>
@@ -4942,7 +4942,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="D3" t="n">
         <v>76.59999999999999</v>
@@ -4966,7 +4966,7 @@
         <v>3</v>
       </c>
       <c r="K3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -4978,13 +4978,13 @@
         <v>42</v>
       </c>
       <c r="O3" t="n">
-        <v>100.8</v>
+        <v>101.1</v>
       </c>
       <c r="P3" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="R3" t="n">
         <v>56391</v>
@@ -5009,7 +5009,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="D4" t="n">
         <v>72.40000000000001</v>
@@ -5033,7 +5033,7 @@
         <v>3</v>
       </c>
       <c r="K4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L4" t="n">
         <v>1</v>
@@ -5045,10 +5045,10 @@
         <v>73</v>
       </c>
       <c r="O4" t="n">
-        <v>101.6</v>
+        <v>102.2</v>
       </c>
       <c r="P4" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="Q4" t="n">
         <v>0.7</v>
@@ -5080,7 +5080,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="D5" t="n">
         <v>70.8</v>
@@ -5104,7 +5104,7 @@
         <v>5</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -5116,13 +5116,13 @@
         <v>78</v>
       </c>
       <c r="O5" t="n">
-        <v>101.6</v>
+        <v>101.9</v>
       </c>
       <c r="P5" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="R5" t="n">
         <v>572645</v>
@@ -5151,7 +5151,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="D6" t="n">
         <v>70.2</v>
@@ -5175,7 +5175,7 @@
         <v>3</v>
       </c>
       <c r="K6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
@@ -5187,13 +5187,13 @@
         <v>47</v>
       </c>
       <c r="O6" t="n">
-        <v>100.8</v>
+        <v>101.5</v>
       </c>
       <c r="P6" t="n">
-        <v>0.8</v>
+        <v>1.5</v>
       </c>
       <c r="Q6" t="n">
-        <v>1</v>
+        <v>1.9</v>
       </c>
       <c r="R6" t="n">
         <v>686560</v>
@@ -5222,7 +5222,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D7" t="n">
         <v>70.2</v>
@@ -5258,13 +5258,13 @@
         <v>77</v>
       </c>
       <c r="O7" t="n">
-        <v>101</v>
+        <v>100.9</v>
       </c>
       <c r="P7" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q7" t="n">
         <v>1</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0.5</v>
       </c>
       <c r="R7" t="n">
         <v>706165</v>
@@ -5277,44 +5277,44 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>bboost, 3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="D8" t="n">
-        <v>69.59999999999999</v>
+        <v>69</v>
       </c>
       <c r="E8" t="n">
         <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="G8" t="n">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="H8" t="n">
         <v>2</v>
       </c>
       <c r="I8" t="n">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="J8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K8" t="n">
         <v>2</v>
@@ -5326,69 +5326,69 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>27</v>
+        <v>61</v>
       </c>
       <c r="O8" t="n">
-        <v>101.8</v>
+        <v>101.6</v>
       </c>
       <c r="P8" t="n">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>812352</v>
+        <v>953327</v>
       </c>
       <c r="S8" t="n">
-        <v>466127</v>
+        <v>3039834</v>
       </c>
       <c r="T8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="D9" t="n">
-        <v>69</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="G9" t="n">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="H9" t="n">
         <v>2</v>
       </c>
       <c r="I9" t="n">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="J9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
@@ -5397,29 +5397,29 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>61</v>
+        <v>27</v>
       </c>
       <c r="O9" t="n">
-        <v>101</v>
+        <v>102.2</v>
       </c>
       <c r="P9" t="n">
-        <v>1</v>
+        <v>2.2</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="R9" t="n">
-        <v>953327</v>
+        <v>812352</v>
       </c>
       <c r="S9" t="n">
-        <v>3039834</v>
+        <v>466127</v>
       </c>
       <c r="T9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
@@ -5435,7 +5435,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="D10" t="n">
         <v>69</v>
@@ -5471,13 +5471,13 @@
         <v>54</v>
       </c>
       <c r="O10" t="n">
-        <v>100.5</v>
+        <v>101.3</v>
       </c>
       <c r="P10" t="n">
-        <v>0.5</v>
+        <v>1.3</v>
       </c>
       <c r="Q10" t="n">
-        <v>2.5</v>
+        <v>4.6</v>
       </c>
       <c r="R10" t="n">
         <v>976059</v>
@@ -5490,35 +5490,35 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>bboost, 3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="D11" t="n">
-        <v>68.8</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="E11" t="n">
         <v>3</v>
       </c>
       <c r="F11" t="n">
+        <v>90</v>
+      </c>
+      <c r="G11" t="n">
         <v>107</v>
-      </c>
-      <c r="G11" t="n">
-        <v>118</v>
       </c>
       <c r="H11" t="n">
         <v>2</v>
@@ -5527,10 +5527,10 @@
         <v>40</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -5539,45 +5539,45 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="O11" t="n">
-        <v>100.9</v>
+        <v>101.4</v>
       </c>
       <c r="P11" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="R11" t="n">
-        <v>996186</v>
+        <v>1054718</v>
       </c>
       <c r="S11" t="n">
-        <v>5881370</v>
+        <v>1034411</v>
       </c>
       <c r="T11" t="n">
         <v>2</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D12" t="n">
         <v>68.8</v>
@@ -5586,22 +5586,22 @@
         <v>3</v>
       </c>
       <c r="F12" t="n">
-        <v>69</v>
+        <v>107</v>
       </c>
       <c r="G12" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="H12" t="n">
         <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J12" t="n">
         <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -5610,22 +5610,22 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="O12" t="n">
-        <v>101.1</v>
+        <v>101.2</v>
       </c>
       <c r="P12" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="R12" t="n">
-        <v>1003072</v>
+        <v>996186</v>
       </c>
       <c r="S12" t="n">
-        <v>5250200</v>
+        <v>5881370</v>
       </c>
       <c r="T12" t="n">
         <v>2</v>
@@ -5639,40 +5639,40 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="D13" t="n">
-        <v>68.59999999999999</v>
+        <v>68.8</v>
       </c>
       <c r="E13" t="n">
         <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="G13" t="n">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="H13" t="n">
         <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -5681,7 +5681,7 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="O13" t="n">
         <v>101.3</v>
@@ -5690,20 +5690,20 @@
         <v>1.3</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.2</v>
+        <v>3.5</v>
       </c>
       <c r="R13" t="n">
-        <v>1054718</v>
+        <v>1003072</v>
       </c>
       <c r="S13" t="n">
-        <v>1034411</v>
+        <v>5250200</v>
       </c>
       <c r="T13" t="n">
         <v>2</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, wildcard, bboost</t>
         </is>
       </c>
     </row>
@@ -5719,7 +5719,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="D14" t="n">
         <v>68</v>
@@ -5743,7 +5743,7 @@
         <v>3</v>
       </c>
       <c r="K14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -5755,13 +5755,13 @@
         <v>78</v>
       </c>
       <c r="O14" t="n">
-        <v>101.4</v>
+        <v>101.9</v>
       </c>
       <c r="P14" t="n">
-        <v>1.4</v>
+        <v>1.9</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.2</v>
+        <v>3.1</v>
       </c>
       <c r="R14" t="n">
         <v>1218344</v>
@@ -5790,7 +5790,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="D15" t="n">
         <v>67.40000000000001</v>
@@ -5826,10 +5826,10 @@
         <v>41</v>
       </c>
       <c r="O15" t="n">
-        <v>100.4</v>
+        <v>100.9</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
       <c r="Q15" t="n">
         <v>1.3</v>
@@ -5852,40 +5852,40 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="D16" t="n">
-        <v>67.40000000000001</v>
+        <v>66.8</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>117</v>
       </c>
       <c r="G16" t="n">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J16" t="n">
         <v>5</v>
       </c>
       <c r="K16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
@@ -5894,69 +5894,69 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>43</v>
+        <v>72</v>
       </c>
       <c r="O16" t="n">
-        <v>101.2</v>
+        <v>101.3</v>
       </c>
       <c r="P16" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.1</v>
+        <v>0.1</v>
       </c>
       <c r="R16" t="n">
-        <v>1396886</v>
+        <v>1589056</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>1066412</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="D17" t="n">
-        <v>66.8</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="E17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>117</v>
+        <v>66</v>
       </c>
       <c r="G17" t="n">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="H17" t="n">
         <v>2</v>
       </c>
       <c r="I17" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J17" t="n">
         <v>5</v>
       </c>
       <c r="K17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
@@ -5965,29 +5965,29 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>72</v>
+        <v>43</v>
       </c>
       <c r="O17" t="n">
-        <v>100.9</v>
+        <v>101.4</v>
       </c>
       <c r="P17" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="Q17" t="n">
-        <v>0</v>
+        <v>2.3</v>
       </c>
       <c r="R17" t="n">
-        <v>1589056</v>
+        <v>1396886</v>
       </c>
       <c r="S17" t="n">
-        <v>1066412</v>
+        <v>101935</v>
       </c>
       <c r="T17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
@@ -6003,7 +6003,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="D18" t="n">
         <v>66.40000000000001</v>
@@ -6039,10 +6039,10 @@
         <v>59</v>
       </c>
       <c r="O18" t="n">
-        <v>100.6</v>
+        <v>101.3</v>
       </c>
       <c r="P18" t="n">
-        <v>0.6</v>
+        <v>1.3</v>
       </c>
       <c r="Q18" t="n">
         <v>0.4</v>
@@ -6058,112 +6058,112 @@
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>3xc, freehit, wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="D19" t="n">
-        <v>65.40000000000001</v>
+        <v>65</v>
       </c>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="G19" t="n">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="H19" t="n">
         <v>2</v>
       </c>
       <c r="I19" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="J19" t="n">
         <v>5</v>
       </c>
       <c r="K19" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="N19" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="O19" t="n">
-        <v>100.4</v>
+        <v>100.9</v>
       </c>
       <c r="P19" t="n">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.6</v>
+        <v>3.5</v>
       </c>
       <c r="R19" t="n">
-        <v>2099042</v>
+        <v>2297297</v>
       </c>
       <c r="S19" t="n">
-        <v>637992</v>
+        <v>3048395</v>
       </c>
       <c r="T19" t="n">
         <v>2</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="D20" t="n">
-        <v>65</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="G20" t="n">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="H20" t="n">
         <v>2</v>
       </c>
       <c r="I20" t="n">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="J20" t="n">
         <v>5</v>
@@ -6172,72 +6172,72 @@
         <v>5</v>
       </c>
       <c r="L20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="O20" t="n">
-        <v>100.6</v>
+        <v>100.1</v>
       </c>
       <c r="P20" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="R20" t="n">
-        <v>2297297</v>
+        <v>2099042</v>
       </c>
       <c r="S20" t="n">
-        <v>3048395</v>
+        <v>637992</v>
       </c>
       <c r="T20" t="n">
         <v>2</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="D21" t="n">
-        <v>64.40000000000001</v>
+        <v>64.2</v>
       </c>
       <c r="E21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" t="n">
+        <v>93</v>
+      </c>
+      <c r="G21" t="n">
+        <v>78</v>
+      </c>
+      <c r="H21" t="n">
+        <v>3</v>
+      </c>
+      <c r="I21" t="n">
+        <v>41</v>
+      </c>
+      <c r="J21" t="n">
         <v>1</v>
-      </c>
-      <c r="F21" t="n">
-        <v>90</v>
-      </c>
-      <c r="G21" t="n">
-        <v>120</v>
-      </c>
-      <c r="H21" t="n">
-        <v>2</v>
-      </c>
-      <c r="I21" t="n">
-        <v>29</v>
-      </c>
-      <c r="J21" t="n">
-        <v>5</v>
       </c>
       <c r="K21" t="n">
         <v>4</v>
@@ -6249,65 +6249,69 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>74</v>
+        <v>38</v>
       </c>
       <c r="O21" t="n">
-        <v>100.3</v>
+        <v>101.4</v>
       </c>
       <c r="P21" t="n">
-        <v>0.3</v>
+        <v>1.4</v>
       </c>
       <c r="Q21" t="n">
-        <v>2.7</v>
+        <v>0.5</v>
       </c>
       <c r="R21" t="n">
-        <v>2516305</v>
+        <v>2598730</v>
       </c>
       <c r="S21" t="n">
-        <v>4399137</v>
+        <v>3395267</v>
       </c>
       <c r="T21" t="n">
-        <v>2</v>
-      </c>
-      <c r="U21" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>3xc, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="D22" t="n">
-        <v>64.2</v>
+        <v>64</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
+        <v>70</v>
+      </c>
+      <c r="G22" t="n">
         <v>93</v>
       </c>
-      <c r="G22" t="n">
-        <v>78</v>
-      </c>
       <c r="H22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I22" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J22" t="n">
         <v>1</v>
       </c>
       <c r="K22" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
@@ -6316,69 +6320,69 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="O22" t="n">
-        <v>100.8</v>
+        <v>102.4</v>
       </c>
       <c r="P22" t="n">
-        <v>0.8</v>
+        <v>2.4</v>
       </c>
       <c r="Q22" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="R22" t="n">
-        <v>2598730</v>
+        <v>2648287</v>
       </c>
       <c r="S22" t="n">
-        <v>3395267</v>
+        <v>2735246</v>
       </c>
       <c r="T22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>3xc</t>
+          <t>wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="D23" t="n">
-        <v>64</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="G23" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="H23" t="n">
         <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="J23" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L23" t="n">
         <v>0</v>
@@ -6387,22 +6391,22 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="O23" t="n">
-        <v>101.7</v>
+        <v>100.3</v>
       </c>
       <c r="P23" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Q23" t="n">
         <v>1.7</v>
       </c>
-      <c r="Q23" t="n">
-        <v>0.4</v>
-      </c>
       <c r="R23" t="n">
-        <v>2648287</v>
+        <v>2516305</v>
       </c>
       <c r="S23" t="n">
-        <v>2735246</v>
+        <v>4399137</v>
       </c>
       <c r="T23" t="n">
         <v>2</v>
@@ -6416,37 +6420,37 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="D24" t="n">
-        <v>63.8</v>
+        <v>63.6</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="G24" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K24" t="n">
         <v>3</v>
@@ -6458,25 +6462,25 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="O24" t="n">
-        <v>101.9</v>
+        <v>101.7</v>
       </c>
       <c r="P24" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="R24" t="n">
-        <v>2745198</v>
+        <v>2831164</v>
       </c>
       <c r="S24" t="n">
-        <v>2489160</v>
+        <v>453361</v>
       </c>
       <c r="T24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U24" t="inlineStr">
         <is>
@@ -6487,37 +6491,37 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="D25" t="n">
-        <v>63.6</v>
+        <v>63.8</v>
       </c>
       <c r="E25" t="n">
         <v>2</v>
       </c>
       <c r="F25" t="n">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="G25" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I25" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="J25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K25" t="n">
         <v>3</v>
@@ -6529,167 +6533,171 @@
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="O25" t="n">
-        <v>101.1</v>
+        <v>102.6</v>
       </c>
       <c r="P25" t="n">
-        <v>1.1</v>
+        <v>2.6</v>
       </c>
       <c r="Q25" t="n">
-        <v>1.1</v>
+        <v>0.6</v>
       </c>
       <c r="R25" t="n">
-        <v>2831164</v>
+        <v>2745198</v>
       </c>
       <c r="S25" t="n">
-        <v>453361</v>
+        <v>2489160</v>
       </c>
       <c r="T25" t="n">
-        <v>2</v>
-      </c>
-      <c r="U25" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D26" t="n">
-        <v>63.4</v>
+        <v>62.8</v>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="G26" t="n">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="H26" t="n">
         <v>2</v>
       </c>
       <c r="I26" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J26" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="O26" t="n">
-        <v>101.1</v>
+        <v>100.6</v>
       </c>
       <c r="P26" t="n">
-        <v>1.1</v>
+        <v>0.6</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.1</v>
+        <v>2.5</v>
       </c>
       <c r="R26" t="n">
-        <v>2963253</v>
+        <v>3181539</v>
       </c>
       <c r="S26" t="n">
-        <v>1948104</v>
+        <v>1595922</v>
       </c>
       <c r="T26" t="n">
         <v>2</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>bboost, 3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="D27" t="n">
-        <v>62.8</v>
+        <v>63.4</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="G27" t="n">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="H27" t="n">
         <v>2</v>
       </c>
       <c r="I27" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J27" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K27" t="n">
+        <v>7</v>
+      </c>
+      <c r="L27" t="n">
         <v>3</v>
       </c>
-      <c r="L27" t="n">
-        <v>0</v>
-      </c>
       <c r="M27" t="n">
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="N27" t="n">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="O27" t="n">
-        <v>100.2</v>
+        <v>101.3</v>
       </c>
       <c r="P27" t="n">
-        <v>0.2</v>
+        <v>1.3</v>
       </c>
       <c r="Q27" t="n">
-        <v>1.8</v>
+        <v>0.6</v>
       </c>
       <c r="R27" t="n">
-        <v>3181539</v>
+        <v>2963253</v>
       </c>
       <c r="S27" t="n">
-        <v>1595922</v>
+        <v>1948104</v>
       </c>
       <c r="T27" t="n">
         <v>2</v>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>bboost, 3xc, wildcard</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
@@ -6705,7 +6713,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D28" t="n">
         <v>62.2</v>
@@ -6741,10 +6749,10 @@
         <v>68</v>
       </c>
       <c r="O28" t="n">
-        <v>101.7</v>
+        <v>101.9</v>
       </c>
       <c r="P28" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="Q28" t="n">
         <v>0.7</v>
@@ -6776,7 +6784,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="D29" t="n">
         <v>58.6</v>
@@ -6800,7 +6808,7 @@
         <v>1</v>
       </c>
       <c r="K29" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L29" t="n">
         <v>0</v>
@@ -6812,13 +6820,13 @@
         <v>74</v>
       </c>
       <c r="O29" t="n">
-        <v>100.7</v>
+        <v>101.1</v>
       </c>
       <c r="P29" t="n">
-        <v>0.7</v>
+        <v>1.1</v>
       </c>
       <c r="Q29" t="n">
-        <v>0</v>
+        <v>2.3</v>
       </c>
       <c r="R29" t="n">
         <v>5109269</v>
@@ -6847,7 +6855,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="D30" t="n">
         <v>56.8</v>
@@ -6883,10 +6891,10 @@
         <v>36</v>
       </c>
       <c r="O30" t="n">
-        <v>101.4</v>
+        <v>101.6</v>
       </c>
       <c r="P30" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="Q30" t="n">
         <v>1</v>
@@ -6918,7 +6926,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>273</v>
+        <v>282</v>
       </c>
       <c r="D31" t="n">
         <v>54.6</v>
@@ -6954,10 +6962,10 @@
         <v>85</v>
       </c>
       <c r="O31" t="n">
-        <v>100.7</v>
+        <v>101.2</v>
       </c>
       <c r="P31" t="n">
-        <v>0.7</v>
+        <v>1.2</v>
       </c>
       <c r="Q31" t="n">
         <v>1.2</v>
@@ -6989,7 +6997,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D32" t="n">
         <v>46.6</v>
@@ -7025,10 +7033,10 @@
         <v>9</v>
       </c>
       <c r="O32" t="n">
-        <v>99.2</v>
+        <v>98.7</v>
       </c>
       <c r="P32" t="n">
-        <v>-0.8</v>
+        <v>-1.3</v>
       </c>
       <c r="Q32" t="n">
         <v>2.2</v>

</xml_diff>

<commit_message>
Update standings 2026-10-10 17:17 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -484,13 +484,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>60</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>397</v>
+        <v>455</v>
       </c>
     </row>
     <row r="3">
@@ -499,22 +499,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>66</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F3" t="n">
-        <v>385</v>
+        <v>428</v>
       </c>
     </row>
     <row r="4">
@@ -523,22 +523,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>41</v>
       </c>
       <c r="E4" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>365</v>
+        <v>424</v>
       </c>
     </row>
     <row r="5">
@@ -556,13 +556,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>6</v>
+        <v>69</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>360</v>
+        <v>423</v>
       </c>
     </row>
     <row r="6">
@@ -571,22 +571,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>69</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>354</v>
+        <v>413</v>
       </c>
     </row>
     <row r="7">
@@ -595,22 +595,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>60</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>353</v>
+        <v>411</v>
       </c>
     </row>
     <row r="8">
@@ -619,22 +619,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>66</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>350</v>
+        <v>410</v>
       </c>
     </row>
     <row r="9">
@@ -643,22 +643,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>350</v>
+        <v>405</v>
       </c>
     </row>
     <row r="10">
@@ -667,22 +667,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>349</v>
+        <v>401</v>
       </c>
     </row>
     <row r="11">
@@ -691,22 +691,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>4</v>
+        <v>56</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>347</v>
+        <v>396</v>
       </c>
     </row>
     <row r="12">
@@ -715,22 +715,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>346</v>
+        <v>396</v>
       </c>
     </row>
     <row r="13">
@@ -739,22 +739,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>71</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>346</v>
+        <v>391</v>
       </c>
     </row>
     <row r="14">
@@ -763,22 +763,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>45</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>343</v>
+        <v>390</v>
       </c>
     </row>
     <row r="15">
@@ -787,22 +787,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3</v>
+        <v>45</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>340</v>
+        <v>388</v>
       </c>
     </row>
     <row r="16">
@@ -811,46 +811,46 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>6</v>
+        <v>41</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>340</v>
+        <v>386</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3</v>
+        <v>64</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>340</v>
+        <v>385</v>
       </c>
     </row>
     <row r="18">
@@ -859,22 +859,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>6</v>
+        <v>65</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>338</v>
+        <v>384</v>
       </c>
     </row>
     <row r="19">
@@ -883,22 +883,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="E19" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>330</v>
+        <v>384</v>
       </c>
     </row>
     <row r="20">
@@ -907,22 +907,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>329</v>
+        <v>382</v>
       </c>
     </row>
     <row r="21">
@@ -931,22 +931,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>327</v>
+        <v>381</v>
       </c>
     </row>
     <row r="22">
@@ -955,22 +955,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>6</v>
+        <v>54</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>326</v>
+        <v>381</v>
       </c>
     </row>
     <row r="23">
@@ -979,22 +979,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>3</v>
+        <v>58</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>325</v>
+        <v>376</v>
       </c>
     </row>
     <row r="24">
@@ -1003,46 +1003,46 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3</v>
+        <v>60</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="F24" t="n">
-        <v>321</v>
+        <v>373</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>2</v>
+        <v>49</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>321</v>
+        <v>371</v>
       </c>
     </row>
     <row r="26">
@@ -1060,13 +1060,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>319</v>
+        <v>370</v>
       </c>
     </row>
     <row r="27">
@@ -1075,22 +1075,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="E27" t="n">
-        <v>-12</v>
+        <v>-8</v>
       </c>
       <c r="F27" t="n">
-        <v>319</v>
+        <v>364</v>
       </c>
     </row>
     <row r="28">
@@ -1108,13 +1108,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>313</v>
+        <v>357</v>
       </c>
     </row>
     <row r="29">
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>3</v>
+        <v>63</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>296</v>
+        <v>356</v>
       </c>
     </row>
     <row r="30">
@@ -1147,22 +1147,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Redsbay</t>
+          <t>Slumber FC</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>3</v>
+        <v>60</v>
       </c>
       <c r="E30" t="n">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="F30" t="n">
-        <v>287</v>
+        <v>333</v>
       </c>
     </row>
     <row r="31">
@@ -1171,22 +1171,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Slumber FC</t>
+          <t>Redsbay</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>9</v>
+        <v>47</v>
       </c>
       <c r="E31" t="n">
-        <v>-4</v>
+        <v>-8</v>
       </c>
       <c r="F31" t="n">
-        <v>282</v>
+        <v>331</v>
       </c>
     </row>
     <row r="32">
@@ -1204,13 +1204,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>235</v>
+        <v>270</v>
       </c>
     </row>
   </sheetData>
@@ -1478,17 +1478,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C11" t="n">
         <v>38</v>
       </c>
       <c r="D11" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -1502,17 +1502,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C12" t="n">
         <v>38</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
@@ -1618,45 +1618,45 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C3" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D3" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="E3" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="F3" t="n">
-        <v>58</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C4" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="E4" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="F4" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5">
@@ -1684,55 +1684,55 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B6" t="n">
+        <v>42</v>
+      </c>
+      <c r="C6" t="n">
+        <v>114</v>
+      </c>
+      <c r="D6" t="n">
         <v>52</v>
       </c>
-      <c r="C6" t="n">
-        <v>113</v>
-      </c>
-      <c r="D6" t="n">
-        <v>45</v>
-      </c>
       <c r="E6" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F6" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B7" t="n">
+        <v>52</v>
+      </c>
+      <c r="C7" t="n">
+        <v>113</v>
+      </c>
+      <c r="D7" t="n">
+        <v>45</v>
+      </c>
+      <c r="E7" t="n">
+        <v>77</v>
+      </c>
+      <c r="F7" t="n">
         <v>64</v>
-      </c>
-      <c r="C7" t="n">
-        <v>105</v>
-      </c>
-      <c r="D7" t="n">
-        <v>60</v>
-      </c>
-      <c r="E7" t="n">
-        <v>76</v>
-      </c>
-      <c r="F7" t="n">
-        <v>46</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="C8" t="n">
         <v>118</v>
@@ -1744,381 +1744,381 @@
         <v>71</v>
       </c>
       <c r="F8" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>73</v>
       </c>
       <c r="C9" t="n">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="D9" t="n">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="E9" t="n">
-        <v>91</v>
+        <v>69</v>
       </c>
       <c r="F9" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="C10" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D10" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="E10" t="n">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="F10" t="n">
-        <v>32</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C11" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D11" t="n">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="E11" t="n">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="F11" t="n">
-        <v>44</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="C12" t="n">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="D12" t="n">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="E12" t="n">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="F12" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>42</v>
       </c>
       <c r="C13" t="n">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="D13" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E13" t="n">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="F13" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="C14" t="n">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="D14" t="n">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="E14" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F14" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="C15" t="n">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>40</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="F15" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="C16" t="n">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="D16" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E16" t="n">
-        <v>58</v>
+        <v>84</v>
       </c>
       <c r="F16" t="n">
-        <v>49</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>73</v>
+        <v>41</v>
       </c>
       <c r="C17" t="n">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="D17" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="E17" t="n">
         <v>69</v>
       </c>
       <c r="F17" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C18" t="n">
-        <v>107</v>
+        <v>86</v>
       </c>
       <c r="D18" t="n">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="E18" t="n">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="F18" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="C19" t="n">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="D19" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="E19" t="n">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="F19" t="n">
-        <v>38</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="C20" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D20" t="n">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E20" t="n">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="F20" t="n">
-        <v>27</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C21" t="n">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="D21" t="n">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="E21" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F21" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="C22" t="n">
-        <v>93</v>
+        <v>111</v>
       </c>
       <c r="D22" t="n">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="E22" t="n">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="F22" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="n">
+        <v>59</v>
+      </c>
+      <c r="C23" t="n">
+        <v>96</v>
+      </c>
+      <c r="D23" t="n">
+        <v>38</v>
+      </c>
+      <c r="E23" t="n">
+        <v>77</v>
+      </c>
+      <c r="F23" t="n">
         <v>48</v>
-      </c>
-      <c r="C23" t="n">
-        <v>120</v>
-      </c>
-      <c r="D23" t="n">
-        <v>49</v>
-      </c>
-      <c r="E23" t="n">
-        <v>76</v>
-      </c>
-      <c r="F23" t="n">
-        <v>29</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E24" t="n">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="F24" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C25" t="n">
-        <v>86</v>
+        <v>120</v>
       </c>
       <c r="D25" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E25" t="n">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="F25" t="n">
-        <v>49</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26">
@@ -2146,23 +2146,23 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="C27" t="n">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="D27" t="n">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="E27" t="n">
-        <v>66</v>
+        <v>87</v>
       </c>
       <c r="F27" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
     </row>
     <row r="28">
@@ -2212,45 +2212,45 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="C30" t="n">
+        <v>73</v>
+      </c>
+      <c r="D30" t="n">
+        <v>32</v>
+      </c>
+      <c r="E30" t="n">
         <v>69</v>
       </c>
-      <c r="D30" t="n">
-        <v>37</v>
-      </c>
-      <c r="E30" t="n">
-        <v>89</v>
-      </c>
       <c r="F30" t="n">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="C31" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D31" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="E31" t="n">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="F31" t="n">
-        <v>46</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -2472,7 +2472,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -2483,7 +2483,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -2530,16 +2530,12 @@
       <c r="B11" t="n">
         <v>90</v>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2550,7 +2546,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2561,7 +2557,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2594,7 +2590,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2609,7 +2605,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -2657,7 +2653,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -2668,7 +2664,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2740,7 +2736,11 @@
       <c r="B29" t="n">
         <v>69</v>
       </c>
-      <c r="C29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2835,7 +2835,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -2846,7 +2846,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -2857,7 +2857,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -2868,7 +2868,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -2879,7 +2879,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -2946,7 +2946,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2961,7 +2961,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2972,7 +2972,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2983,7 +2983,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2994,7 +2994,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -3005,7 +3005,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -3016,7 +3016,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -3027,7 +3027,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -3038,7 +3038,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -3049,7 +3049,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -3060,7 +3060,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -3082,7 +3082,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -3093,7 +3093,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -3258,7 +3258,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3279,7 +3279,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3653,30 +3653,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>545267</v>
+        <v>281617</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>604934</v>
+        <v>1051323</v>
       </c>
       <c r="H3" t="n">
-        <v>545267</v>
+        <v>1076546</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -3690,30 +3690,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>281617</v>
+        <v>545267</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1051323</v>
+        <v>604934</v>
       </c>
       <c r="H4" t="n">
-        <v>1076546</v>
+        <v>545267</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -3764,19 +3764,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E6" t="n">
-        <v>189374</v>
+        <v>486041</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -3784,10 +3784,10 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1757289</v>
+        <v>2415786</v>
       </c>
       <c r="H6" t="n">
-        <v>250879</v>
+        <v>1206623</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -3801,30 +3801,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E7" t="n">
-        <v>6474</v>
+        <v>189374</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1177681</v>
+        <v>1757289</v>
       </c>
       <c r="H7" t="n">
-        <v>6474</v>
+        <v>250879</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -3838,30 +3838,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E8" t="n">
-        <v>182900</v>
+        <v>273503</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>2098988</v>
+        <v>1994005</v>
       </c>
       <c r="H8" t="n">
-        <v>182900</v>
+        <v>1917309</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -3875,30 +3875,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E9" t="n">
-        <v>28582</v>
+        <v>37120</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>881388</v>
+        <v>1571193</v>
       </c>
       <c r="H9" t="n">
-        <v>239490</v>
+        <v>3349378</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -3912,30 +3912,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E10" t="n">
-        <v>27153</v>
+        <v>6474</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>606381</v>
+        <v>1177681</v>
       </c>
       <c r="H10" t="n">
-        <v>240451</v>
+        <v>6474</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -3949,30 +3949,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E11" t="n">
-        <v>30971</v>
+        <v>8917</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>820221</v>
+        <v>2118382</v>
       </c>
       <c r="H11" t="n">
-        <v>58227</v>
+        <v>9146930</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -3986,30 +3986,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E12" t="n">
-        <v>273503</v>
+        <v>28582</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1994005</v>
+        <v>881388</v>
       </c>
       <c r="H12" t="n">
-        <v>1917309</v>
+        <v>239490</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -4023,30 +4023,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>486041</v>
+        <v>14603</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2016/17</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>2415786</v>
+        <v>949628</v>
       </c>
       <c r="H13" t="n">
-        <v>1206623</v>
+        <v>515830</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -4060,30 +4060,30 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E14" t="n">
-        <v>8917</v>
+        <v>182900</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>2118382</v>
+        <v>2098988</v>
       </c>
       <c r="H14" t="n">
-        <v>9146930</v>
+        <v>182900</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E15" t="n">
-        <v>453230</v>
+        <v>30971</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5483351</v>
+        <v>820221</v>
       </c>
       <c r="H15" t="n">
-        <v>8188106</v>
+        <v>58227</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,19 +4134,19 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E16" t="n">
-        <v>31543</v>
+        <v>27153</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -4154,10 +4154,10 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>820692</v>
+        <v>606381</v>
       </c>
       <c r="H16" t="n">
-        <v>1637750</v>
+        <v>240451</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -4167,34 +4167,34 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E17" t="n">
-        <v>37120</v>
+        <v>15288</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>1571193</v>
+        <v>329510</v>
       </c>
       <c r="H17" t="n">
-        <v>3349378</v>
+        <v>538046</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4208,30 +4208,30 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E18" t="n">
-        <v>410102</v>
+        <v>95791</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>2088802</v>
+        <v>2404119</v>
       </c>
       <c r="H18" t="n">
-        <v>5360778</v>
+        <v>5124417</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -4245,30 +4245,30 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E19" t="n">
-        <v>1128645</v>
+        <v>31543</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>3434302</v>
+        <v>820692</v>
       </c>
       <c r="H19" t="n">
-        <v>1128645</v>
+        <v>1637750</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -4282,30 +4282,30 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E20" t="n">
-        <v>15136</v>
+        <v>410102</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>983840</v>
+        <v>2088802</v>
       </c>
       <c r="H20" t="n">
-        <v>45077</v>
+        <v>5360778</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -4319,30 +4319,30 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E21" t="n">
-        <v>15288</v>
+        <v>453230</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>329510</v>
+        <v>5483351</v>
       </c>
       <c r="H21" t="n">
-        <v>538046</v>
+        <v>8188106</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -4356,30 +4356,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E22" t="n">
-        <v>14603</v>
+        <v>15136</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2016/17</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>949628</v>
+        <v>983840</v>
       </c>
       <c r="H22" t="n">
-        <v>515830</v>
+        <v>45077</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -4393,30 +4393,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
-        <v>60517</v>
+        <v>334016</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2015/16</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>1414622</v>
+        <v>2156629</v>
       </c>
       <c r="H23" t="n">
-        <v>339763</v>
+        <v>2691725</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4430,19 +4430,19 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E24" t="n">
-        <v>334016</v>
+        <v>1320699</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -4450,47 +4450,47 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2156629</v>
+        <v>2490743</v>
       </c>
       <c r="H24" t="n">
-        <v>2691725</v>
+        <v>1861933</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2024/25</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E25" t="n">
-        <v>95791</v>
+        <v>60517</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2015/16</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>2404119</v>
+        <v>1414622</v>
       </c>
       <c r="H25" t="n">
-        <v>5124417</v>
+        <v>339763</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -4541,34 +4541,34 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E27" t="n">
-        <v>1320699</v>
+        <v>1128645</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>2490743</v>
+        <v>3434302</v>
       </c>
       <c r="H27" t="n">
-        <v>1861933</v>
+        <v>1128645</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
     </row>
@@ -4652,19 +4652,19 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Redsbay</t>
+          <t>Slumber FC</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E30" t="n">
-        <v>4884220</v>
+        <v>676529</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -4672,10 +4672,10 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>4884220</v>
+        <v>998938</v>
       </c>
       <c r="H30" t="n">
-        <v>4884220</v>
+        <v>676529</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -4689,19 +4689,19 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Slumber FC</t>
+          <t>Redsbay</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E31" t="n">
-        <v>676529</v>
+        <v>4884220</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -4709,10 +4709,10 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>998938</v>
+        <v>4884220</v>
       </c>
       <c r="H31" t="n">
-        <v>676529</v>
+        <v>4884220</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -4871,7 +4871,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>397</v>
+        <v>455</v>
       </c>
       <c r="D2" t="n">
         <v>79</v>
@@ -4933,34 +4933,34 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>385</v>
+        <v>428</v>
       </c>
       <c r="D3" t="n">
-        <v>76.59999999999999</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
         <v>84</v>
       </c>
       <c r="G3" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="H3" t="n">
         <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="J3" t="n">
         <v>3</v>
@@ -4969,65 +4969,69 @@
         <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N3" t="n">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="O3" t="n">
-        <v>101.1</v>
+        <v>102.2</v>
       </c>
       <c r="P3" t="n">
-        <v>1.1</v>
+        <v>2.2</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="R3" t="n">
-        <v>56391</v>
+        <v>352905</v>
       </c>
       <c r="S3" t="n">
-        <v>1461471</v>
+        <v>1229264</v>
       </c>
       <c r="T3" t="n">
-        <v>2</v>
-      </c>
-      <c r="U3" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>bboost, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>365</v>
+        <v>424</v>
       </c>
       <c r="D4" t="n">
-        <v>72.40000000000001</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
         <v>84</v>
       </c>
       <c r="G4" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="H4" t="n">
         <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="J4" t="n">
         <v>3</v>
@@ -5036,37 +5040,33 @@
         <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>73</v>
+        <v>42</v>
       </c>
       <c r="O4" t="n">
-        <v>102.2</v>
+        <v>101.1</v>
       </c>
       <c r="P4" t="n">
-        <v>2.2</v>
+        <v>1.1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="R4" t="n">
-        <v>352905</v>
+        <v>56391</v>
       </c>
       <c r="S4" t="n">
-        <v>1229264</v>
+        <v>1461471</v>
       </c>
       <c r="T4" t="n">
-        <v>4</v>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>bboost, wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5080,7 +5080,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>360</v>
+        <v>423</v>
       </c>
       <c r="D5" t="n">
         <v>70.8</v>
@@ -5142,40 +5142,40 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>354</v>
+        <v>413</v>
       </c>
       <c r="D6" t="n">
-        <v>70.2</v>
+        <v>68.8</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="G6" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H6" t="n">
         <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="J6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
@@ -5187,66 +5187,66 @@
         <v>47</v>
       </c>
       <c r="O6" t="n">
-        <v>101.5</v>
+        <v>101.3</v>
       </c>
       <c r="P6" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="Q6" t="n">
-        <v>1.9</v>
+        <v>3.5</v>
       </c>
       <c r="R6" t="n">
-        <v>686560</v>
+        <v>1003072</v>
       </c>
       <c r="S6" t="n">
-        <v>3046343</v>
+        <v>5250200</v>
       </c>
       <c r="T6" t="n">
         <v>2</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>3xc, wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>353</v>
+        <v>411</v>
       </c>
       <c r="D7" t="n">
         <v>70.2</v>
       </c>
       <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>90</v>
+      </c>
+      <c r="G7" t="n">
+        <v>113</v>
+      </c>
+      <c r="H7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" t="n">
+        <v>45</v>
+      </c>
+      <c r="J7" t="n">
         <v>3</v>
       </c>
-      <c r="F7" t="n">
-        <v>79</v>
-      </c>
-      <c r="G7" t="n">
-        <v>105</v>
-      </c>
-      <c r="H7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I7" t="n">
-        <v>46</v>
-      </c>
-      <c r="J7" t="n">
-        <v>5</v>
-      </c>
       <c r="K7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -5255,54 +5255,54 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>77</v>
+        <v>47</v>
       </c>
       <c r="O7" t="n">
-        <v>100.9</v>
+        <v>101.5</v>
       </c>
       <c r="P7" t="n">
-        <v>0.9</v>
+        <v>1.5</v>
       </c>
       <c r="Q7" t="n">
-        <v>1</v>
+        <v>1.9</v>
       </c>
       <c r="R7" t="n">
-        <v>706165</v>
+        <v>686560</v>
       </c>
       <c r="S7" t="n">
-        <v>617418</v>
+        <v>3046343</v>
       </c>
       <c r="T7" t="n">
         <v>2</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>bboost, 3xc, wildcard</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>350</v>
+        <v>410</v>
       </c>
       <c r="D8" t="n">
-        <v>69</v>
+        <v>68.8</v>
       </c>
       <c r="E8" t="n">
         <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="G8" t="n">
         <v>118</v>
@@ -5311,13 +5311,13 @@
         <v>2</v>
       </c>
       <c r="I8" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="J8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -5326,22 +5326,22 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="O8" t="n">
-        <v>101.6</v>
+        <v>101.2</v>
       </c>
       <c r="P8" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="R8" t="n">
-        <v>953327</v>
+        <v>996186</v>
       </c>
       <c r="S8" t="n">
-        <v>3039834</v>
+        <v>5881370</v>
       </c>
       <c r="T8" t="n">
         <v>2</v>
@@ -5355,37 +5355,37 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>350</v>
+        <v>405</v>
       </c>
       <c r="D9" t="n">
-        <v>69.59999999999999</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
       </c>
       <c r="F9" t="n">
+        <v>66</v>
+      </c>
+      <c r="G9" t="n">
         <v>90</v>
       </c>
-      <c r="G9" t="n">
-        <v>104</v>
-      </c>
       <c r="H9" t="n">
         <v>2</v>
       </c>
       <c r="I9" t="n">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="J9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K9" t="n">
         <v>4</v>
@@ -5397,63 +5397,63 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="O9" t="n">
-        <v>102.2</v>
+        <v>101.4</v>
       </c>
       <c r="P9" t="n">
-        <v>2.2</v>
+        <v>1.4</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.1</v>
+        <v>2.3</v>
       </c>
       <c r="R9" t="n">
-        <v>812352</v>
+        <v>1396886</v>
       </c>
       <c r="S9" t="n">
-        <v>466127</v>
+        <v>101935</v>
       </c>
       <c r="T9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>349</v>
+        <v>401</v>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>70.2</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G10" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H10" t="n">
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="J10" t="n">
         <v>5</v>
@@ -5468,22 +5468,22 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="O10" t="n">
-        <v>101.3</v>
+        <v>100.9</v>
       </c>
       <c r="P10" t="n">
-        <v>1.3</v>
+        <v>0.9</v>
       </c>
       <c r="Q10" t="n">
-        <v>4.6</v>
+        <v>1</v>
       </c>
       <c r="R10" t="n">
-        <v>976059</v>
+        <v>706165</v>
       </c>
       <c r="S10" t="n">
-        <v>166751</v>
+        <v>617418</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
@@ -5497,19 +5497,19 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>347</v>
+        <v>396</v>
       </c>
       <c r="D11" t="n">
-        <v>68.59999999999999</v>
+        <v>68</v>
       </c>
       <c r="E11" t="n">
         <v>3</v>
@@ -5518,19 +5518,19 @@
         <v>90</v>
       </c>
       <c r="G11" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H11" t="n">
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="J11" t="n">
         <v>3</v>
       </c>
       <c r="K11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -5539,22 +5539,22 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>25</v>
+        <v>78</v>
       </c>
       <c r="O11" t="n">
-        <v>101.4</v>
+        <v>101.9</v>
       </c>
       <c r="P11" t="n">
-        <v>1.4</v>
+        <v>1.9</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.2</v>
+        <v>3.1</v>
       </c>
       <c r="R11" t="n">
-        <v>1054718</v>
+        <v>1218344</v>
       </c>
       <c r="S11" t="n">
-        <v>1034411</v>
+        <v>878473</v>
       </c>
       <c r="T11" t="n">
         <v>2</v>
@@ -5568,40 +5568,40 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>346</v>
+        <v>396</v>
       </c>
       <c r="D12" t="n">
-        <v>68.8</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="E12" t="n">
         <v>3</v>
       </c>
       <c r="F12" t="n">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="G12" t="n">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="H12" t="n">
         <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="J12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -5610,57 +5610,57 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>65</v>
+        <v>27</v>
       </c>
       <c r="O12" t="n">
-        <v>101.2</v>
+        <v>102.2</v>
       </c>
       <c r="P12" t="n">
-        <v>1.2</v>
+        <v>2.2</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="R12" t="n">
-        <v>996186</v>
+        <v>812352</v>
       </c>
       <c r="S12" t="n">
-        <v>5881370</v>
+        <v>466127</v>
       </c>
       <c r="T12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>346</v>
+        <v>391</v>
       </c>
       <c r="D13" t="n">
-        <v>68.8</v>
+        <v>64</v>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G13" t="n">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="H13" t="n">
         <v>2</v>
@@ -5672,7 +5672,7 @@
         <v>1</v>
       </c>
       <c r="K13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -5681,69 +5681,69 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="O13" t="n">
-        <v>101.3</v>
+        <v>102.4</v>
       </c>
       <c r="P13" t="n">
-        <v>1.3</v>
+        <v>2.4</v>
       </c>
       <c r="Q13" t="n">
-        <v>3.5</v>
+        <v>0.4</v>
       </c>
       <c r="R13" t="n">
-        <v>1003072</v>
+        <v>2648287</v>
       </c>
       <c r="S13" t="n">
-        <v>5250200</v>
+        <v>2735246</v>
       </c>
       <c r="T13" t="n">
         <v>2</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>3xc, wildcard, bboost</t>
+          <t>wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>343</v>
+        <v>390</v>
       </c>
       <c r="D14" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E14" t="n">
         <v>3</v>
       </c>
       <c r="F14" t="n">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="G14" t="n">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="H14" t="n">
         <v>2</v>
       </c>
       <c r="I14" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J14" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -5752,66 +5752,66 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="O14" t="n">
-        <v>101.9</v>
+        <v>101.6</v>
       </c>
       <c r="P14" t="n">
-        <v>1.9</v>
+        <v>1.6</v>
       </c>
       <c r="Q14" t="n">
-        <v>3.1</v>
+        <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>1218344</v>
+        <v>953327</v>
       </c>
       <c r="S14" t="n">
-        <v>878473</v>
+        <v>3039834</v>
       </c>
       <c r="T14" t="n">
         <v>2</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>340</v>
+        <v>388</v>
       </c>
       <c r="D15" t="n">
-        <v>67.40000000000001</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="E15" t="n">
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="G15" t="n">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,63 +5823,63 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="O15" t="n">
-        <v>100.9</v>
+        <v>101.4</v>
       </c>
       <c r="P15" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.3</v>
+        <v>0.2</v>
       </c>
       <c r="R15" t="n">
-        <v>1396886</v>
+        <v>1054718</v>
       </c>
       <c r="S15" t="n">
-        <v>3009015</v>
+        <v>1034411</v>
       </c>
       <c r="T15" t="n">
         <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>340</v>
+        <v>386</v>
       </c>
       <c r="D16" t="n">
-        <v>66.8</v>
+        <v>69</v>
       </c>
       <c r="E16" t="n">
         <v>4</v>
       </c>
       <c r="F16" t="n">
-        <v>117</v>
+        <v>81</v>
       </c>
       <c r="G16" t="n">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="J16" t="n">
         <v>5</v>
@@ -5894,7 +5894,7 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="O16" t="n">
         <v>101.3</v>
@@ -5903,57 +5903,57 @@
         <v>1.3</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.1</v>
+        <v>4.6</v>
       </c>
       <c r="R16" t="n">
-        <v>1589056</v>
+        <v>976059</v>
       </c>
       <c r="S16" t="n">
-        <v>1066412</v>
+        <v>166751</v>
       </c>
       <c r="T16" t="n">
         <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, 3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>340</v>
+        <v>385</v>
       </c>
       <c r="D17" t="n">
-        <v>67.40000000000001</v>
+        <v>64.2</v>
       </c>
       <c r="E17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" t="n">
+        <v>93</v>
+      </c>
+      <c r="G17" t="n">
+        <v>78</v>
+      </c>
+      <c r="H17" t="n">
         <v>3</v>
       </c>
-      <c r="F17" t="n">
-        <v>66</v>
-      </c>
-      <c r="G17" t="n">
-        <v>90</v>
-      </c>
-      <c r="H17" t="n">
-        <v>2</v>
-      </c>
       <c r="I17" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="J17" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K17" t="n">
         <v>4</v>
@@ -5965,7 +5965,7 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="O17" t="n">
         <v>101.4</v>
@@ -5974,60 +5974,60 @@
         <v>1.4</v>
       </c>
       <c r="Q17" t="n">
-        <v>2.3</v>
+        <v>0.5</v>
       </c>
       <c r="R17" t="n">
-        <v>1396886</v>
+        <v>2598730</v>
       </c>
       <c r="S17" t="n">
-        <v>101935</v>
+        <v>3395267</v>
       </c>
       <c r="T17" t="n">
         <v>3</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>338</v>
+        <v>384</v>
       </c>
       <c r="D18" t="n">
-        <v>66.40000000000001</v>
+        <v>63.8</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
+        <v>70</v>
+      </c>
+      <c r="G18" t="n">
         <v>93</v>
       </c>
-      <c r="G18" t="n">
-        <v>107</v>
-      </c>
       <c r="H18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I18" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J18" t="n">
         <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L18" t="n">
         <v>0</v>
@@ -6036,93 +6036,93 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>59</v>
+        <v>87</v>
       </c>
       <c r="O18" t="n">
-        <v>101.3</v>
+        <v>102.6</v>
       </c>
       <c r="P18" t="n">
-        <v>1.3</v>
+        <v>2.6</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="R18" t="n">
-        <v>1724545</v>
+        <v>2745198</v>
       </c>
       <c r="S18" t="n">
-        <v>4185865</v>
+        <v>2489160</v>
       </c>
       <c r="T18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard, bboost</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>330</v>
+        <v>384</v>
       </c>
       <c r="D19" t="n">
-        <v>65</v>
+        <v>66.8</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F19" t="n">
-        <v>79</v>
+        <v>117</v>
       </c>
       <c r="G19" t="n">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="H19" t="n">
         <v>2</v>
       </c>
       <c r="I19" t="n">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="J19" t="n">
         <v>5</v>
       </c>
       <c r="K19" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="O19" t="n">
-        <v>100.9</v>
+        <v>101.3</v>
       </c>
       <c r="P19" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="Q19" t="n">
-        <v>3.5</v>
+        <v>0.1</v>
       </c>
       <c r="R19" t="n">
-        <v>2297297</v>
+        <v>1589056</v>
       </c>
       <c r="S19" t="n">
-        <v>3048395</v>
+        <v>1066412</v>
       </c>
       <c r="T19" t="n">
         <v>2</v>
@@ -6136,40 +6136,40 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>329</v>
+        <v>382</v>
       </c>
       <c r="D20" t="n">
-        <v>65.40000000000001</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="E20" t="n">
         <v>3</v>
       </c>
       <c r="F20" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="G20" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="H20" t="n">
         <v>2</v>
       </c>
       <c r="I20" t="n">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="J20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L20" t="n">
         <v>0</v>
@@ -6178,69 +6178,69 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="O20" t="n">
-        <v>100.1</v>
+        <v>101.3</v>
       </c>
       <c r="P20" t="n">
-        <v>0.1</v>
+        <v>1.3</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="R20" t="n">
-        <v>2099042</v>
+        <v>1724545</v>
       </c>
       <c r="S20" t="n">
-        <v>637992</v>
+        <v>4185865</v>
       </c>
       <c r="T20" t="n">
         <v>2</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>3xc, freehit, wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>327</v>
+        <v>381</v>
       </c>
       <c r="D21" t="n">
-        <v>64.2</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="G21" t="n">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="H21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I21" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="J21" t="n">
         <v>1</v>
       </c>
       <c r="K21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L21" t="n">
         <v>0</v>
@@ -6249,69 +6249,69 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="O21" t="n">
-        <v>101.4</v>
+        <v>100.9</v>
       </c>
       <c r="P21" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.5</v>
+        <v>1.3</v>
       </c>
       <c r="R21" t="n">
-        <v>2598730</v>
+        <v>1396886</v>
       </c>
       <c r="S21" t="n">
-        <v>3395267</v>
+        <v>3009015</v>
       </c>
       <c r="T21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>326</v>
+        <v>381</v>
       </c>
       <c r="D22" t="n">
-        <v>64</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F22" t="n">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="G22" t="n">
-        <v>93</v>
+        <v>111</v>
       </c>
       <c r="H22" t="n">
         <v>2</v>
       </c>
       <c r="I22" t="n">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K22" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
@@ -6320,69 +6320,69 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="O22" t="n">
-        <v>102.4</v>
+        <v>100.1</v>
       </c>
       <c r="P22" t="n">
-        <v>2.4</v>
+        <v>0.1</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="R22" t="n">
-        <v>2648287</v>
+        <v>2099042</v>
       </c>
       <c r="S22" t="n">
-        <v>2735246</v>
+        <v>637992</v>
       </c>
       <c r="T22" t="n">
         <v>2</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>wildcard, bboost</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>325</v>
+        <v>376</v>
       </c>
       <c r="D23" t="n">
-        <v>64.40000000000001</v>
+        <v>63.6</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="G23" t="n">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="H23" t="n">
         <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="J23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L23" t="n">
         <v>0</v>
@@ -6391,22 +6391,22 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="O23" t="n">
-        <v>100.3</v>
+        <v>101.7</v>
       </c>
       <c r="P23" t="n">
-        <v>0.3</v>
+        <v>1.7</v>
       </c>
       <c r="Q23" t="n">
-        <v>1.7</v>
+        <v>1.2</v>
       </c>
       <c r="R23" t="n">
-        <v>2516305</v>
+        <v>2831164</v>
       </c>
       <c r="S23" t="n">
-        <v>4399137</v>
+        <v>453361</v>
       </c>
       <c r="T23" t="n">
         <v>2</v>
@@ -6420,64 +6420,64 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>321</v>
+        <v>373</v>
       </c>
       <c r="D24" t="n">
-        <v>63.6</v>
+        <v>63.4</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="G24" t="n">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="H24" t="n">
         <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="J24" t="n">
         <v>3</v>
       </c>
       <c r="K24" t="n">
+        <v>7</v>
+      </c>
+      <c r="L24" t="n">
         <v>3</v>
       </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
       <c r="M24" t="n">
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="N24" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="O24" t="n">
-        <v>101.7</v>
+        <v>101.3</v>
       </c>
       <c r="P24" t="n">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
       <c r="Q24" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="R24" t="n">
-        <v>2831164</v>
+        <v>2963253</v>
       </c>
       <c r="S24" t="n">
-        <v>453361</v>
+        <v>1948104</v>
       </c>
       <c r="T24" t="n">
         <v>2</v>
@@ -6491,41 +6491,41 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>321</v>
+        <v>371</v>
       </c>
       <c r="D25" t="n">
-        <v>63.8</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="G25" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="H25" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" t="n">
+        <v>29</v>
+      </c>
+      <c r="J25" t="n">
+        <v>5</v>
+      </c>
+      <c r="K25" t="n">
         <v>4</v>
       </c>
-      <c r="I25" t="n">
-        <v>45</v>
-      </c>
-      <c r="J25" t="n">
-        <v>1</v>
-      </c>
-      <c r="K25" t="n">
-        <v>3</v>
-      </c>
       <c r="L25" t="n">
         <v>0</v>
       </c>
@@ -6533,25 +6533,25 @@
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="O25" t="n">
-        <v>102.6</v>
+        <v>100.3</v>
       </c>
       <c r="P25" t="n">
-        <v>2.6</v>
+        <v>0.3</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.6</v>
+        <v>1.7</v>
       </c>
       <c r="R25" t="n">
-        <v>2745198</v>
+        <v>2516305</v>
       </c>
       <c r="S25" t="n">
-        <v>2489160</v>
+        <v>4399137</v>
       </c>
       <c r="T25" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U25" t="inlineStr">
         <is>
@@ -6571,7 +6571,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>319</v>
+        <v>370</v>
       </c>
       <c r="D26" t="n">
         <v>62.8</v>
@@ -6633,71 +6633,71 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>319</v>
+        <v>364</v>
       </c>
       <c r="D27" t="n">
-        <v>63.4</v>
+        <v>65</v>
       </c>
       <c r="E27" t="n">
         <v>2</v>
       </c>
       <c r="F27" t="n">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="G27" t="n">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="H27" t="n">
         <v>2</v>
       </c>
       <c r="I27" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="J27" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M27" t="n">
-        <v>-12</v>
+        <v>-8</v>
       </c>
       <c r="N27" t="n">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="O27" t="n">
-        <v>101.3</v>
+        <v>100.9</v>
       </c>
       <c r="P27" t="n">
-        <v>1.3</v>
+        <v>0.9</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.6</v>
+        <v>3.5</v>
       </c>
       <c r="R27" t="n">
-        <v>2963253</v>
+        <v>2297297</v>
       </c>
       <c r="S27" t="n">
-        <v>1948104</v>
+        <v>3048395</v>
       </c>
       <c r="T27" t="n">
         <v>2</v>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
@@ -6713,7 +6713,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>313</v>
+        <v>357</v>
       </c>
       <c r="D28" t="n">
         <v>62.2</v>
@@ -6784,7 +6784,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>296</v>
+        <v>356</v>
       </c>
       <c r="D29" t="n">
         <v>58.6</v>
@@ -6846,64 +6846,64 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Redsbay</t>
+          <t>Slumber FC</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>287</v>
+        <v>333</v>
       </c>
       <c r="D30" t="n">
-        <v>56.8</v>
+        <v>54.6</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="G30" t="n">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="H30" t="n">
+        <v>2</v>
+      </c>
+      <c r="I30" t="n">
+        <v>32</v>
+      </c>
+      <c r="J30" t="n">
+        <v>3</v>
+      </c>
+      <c r="K30" t="n">
         <v>4</v>
       </c>
-      <c r="I30" t="n">
-        <v>37</v>
-      </c>
-      <c r="J30" t="n">
+      <c r="L30" t="n">
         <v>1</v>
       </c>
-      <c r="K30" t="n">
-        <v>5</v>
-      </c>
-      <c r="L30" t="n">
-        <v>2</v>
-      </c>
       <c r="M30" t="n">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="N30" t="n">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="O30" t="n">
-        <v>101.6</v>
+        <v>101.2</v>
       </c>
       <c r="P30" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="Q30" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="R30" t="n">
-        <v>5949920</v>
+        <v>6804394</v>
       </c>
       <c r="S30" t="n">
-        <v>1952243</v>
+        <v>553038</v>
       </c>
       <c r="T30" t="n">
         <v>4</v>
@@ -6917,64 +6917,64 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Slumber FC</t>
+          <t>Redsbay</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>282</v>
+        <v>331</v>
       </c>
       <c r="D31" t="n">
-        <v>54.6</v>
+        <v>56.8</v>
       </c>
       <c r="E31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F31" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G31" t="n">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="H31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I31" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="J31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K31" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L31" t="n">
+        <v>2</v>
+      </c>
+      <c r="M31" t="n">
+        <v>-8</v>
+      </c>
+      <c r="N31" t="n">
+        <v>36</v>
+      </c>
+      <c r="O31" t="n">
+        <v>101.6</v>
+      </c>
+      <c r="P31" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="Q31" t="n">
         <v>1</v>
       </c>
-      <c r="M31" t="n">
-        <v>-4</v>
-      </c>
-      <c r="N31" t="n">
-        <v>85</v>
-      </c>
-      <c r="O31" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P31" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>1.2</v>
-      </c>
       <c r="R31" t="n">
-        <v>6804394</v>
+        <v>5949920</v>
       </c>
       <c r="S31" t="n">
-        <v>553038</v>
+        <v>1952243</v>
       </c>
       <c r="T31" t="n">
         <v>4</v>
@@ -6997,7 +6997,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>235</v>
+        <v>270</v>
       </c>
       <c r="D32" t="n">
         <v>46.6</v>

</xml_diff>

<commit_message>
Update standings 2026-10-10 21:14 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -652,13 +652,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="10">
@@ -700,13 +700,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>396</v>
+        <v>400</v>
       </c>
     </row>
     <row r="12">
@@ -931,22 +931,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="22">
@@ -955,16 +955,16 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
@@ -1084,13 +1084,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E27" t="n">
         <v>-8</v>
       </c>
       <c r="F27" t="n">
-        <v>364</v>
+        <v>366</v>
       </c>
     </row>
     <row r="28">
@@ -1099,22 +1099,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>sakalaka</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>357</v>
+        <v>363</v>
       </c>
     </row>
     <row r="29">
@@ -1123,22 +1123,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>sakalaka</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>356</v>
+        <v>359</v>
       </c>
     </row>
     <row r="30">
@@ -1204,13 +1204,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -2014,45 +2014,45 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="C21" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="D21" t="n">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="E21" t="n">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="F21" t="n">
-        <v>51</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="C22" t="n">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="D22" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="E22" t="n">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="F22" t="n">
-        <v>27</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23">
@@ -2168,45 +2168,45 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="C28" t="n">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="D28" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E28" t="n">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="F28" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="C29" t="n">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="D29" t="n">
+        <v>47</v>
+      </c>
+      <c r="E29" t="n">
+        <v>77</v>
+      </c>
+      <c r="F29" t="n">
         <v>48</v>
-      </c>
-      <c r="E29" t="n">
-        <v>69</v>
-      </c>
-      <c r="F29" t="n">
-        <v>46</v>
       </c>
     </row>
     <row r="30">
@@ -4319,30 +4319,30 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E21" t="n">
-        <v>453230</v>
+        <v>15136</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>5483351</v>
+        <v>983840</v>
       </c>
       <c r="H21" t="n">
-        <v>8188106</v>
+        <v>45077</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -4356,30 +4356,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E22" t="n">
-        <v>15136</v>
+        <v>453230</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>983840</v>
+        <v>5483351</v>
       </c>
       <c r="H22" t="n">
-        <v>45077</v>
+        <v>8188106</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -4578,30 +4578,30 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>sakalaka</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E28" t="n">
-        <v>81907</v>
+        <v>117338</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>3252487</v>
+        <v>4684930</v>
       </c>
       <c r="H28" t="n">
-        <v>11118394</v>
+        <v>117338</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -4615,30 +4615,30 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>sakalaka</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E29" t="n">
-        <v>117338</v>
+        <v>81907</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>4684930</v>
+        <v>3252487</v>
       </c>
       <c r="H29" t="n">
-        <v>117338</v>
+        <v>11118394</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -4904,7 +4904,7 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="O2" t="n">
         <v>102.3</v>
@@ -4916,7 +4916,7 @@
         <v>2.4</v>
       </c>
       <c r="R2" t="n">
-        <v>14101</v>
+        <v>14788</v>
       </c>
       <c r="S2" t="n">
         <v>270274</v>
@@ -4975,7 +4975,7 @@
         <v>-4</v>
       </c>
       <c r="N3" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="O3" t="n">
         <v>102.2</v>
@@ -4987,7 +4987,7 @@
         <v>0.7</v>
       </c>
       <c r="R3" t="n">
-        <v>352905</v>
+        <v>167799</v>
       </c>
       <c r="S3" t="n">
         <v>1229264</v>
@@ -5046,7 +5046,7 @@
         <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="O4" t="n">
         <v>101.1</v>
@@ -5058,7 +5058,7 @@
         <v>0.3</v>
       </c>
       <c r="R4" t="n">
-        <v>56391</v>
+        <v>218204</v>
       </c>
       <c r="S4" t="n">
         <v>1461471</v>
@@ -5113,7 +5113,7 @@
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="O5" t="n">
         <v>101.9</v>
@@ -5125,7 +5125,7 @@
         <v>1.3</v>
       </c>
       <c r="R5" t="n">
-        <v>572645</v>
+        <v>222828</v>
       </c>
       <c r="S5" t="n">
         <v>266328</v>
@@ -5196,7 +5196,7 @@
         <v>3.5</v>
       </c>
       <c r="R6" t="n">
-        <v>1003072</v>
+        <v>410385</v>
       </c>
       <c r="S6" t="n">
         <v>5250200</v>
@@ -5255,7 +5255,7 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="O7" t="n">
         <v>101.5</v>
@@ -5267,7 +5267,7 @@
         <v>1.9</v>
       </c>
       <c r="R7" t="n">
-        <v>686560</v>
+        <v>451158</v>
       </c>
       <c r="S7" t="n">
         <v>3046343</v>
@@ -5326,7 +5326,7 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="O8" t="n">
         <v>101.2</v>
@@ -5338,7 +5338,7 @@
         <v>0.3</v>
       </c>
       <c r="R8" t="n">
-        <v>996186</v>
+        <v>475447</v>
       </c>
       <c r="S8" t="n">
         <v>5881370</v>
@@ -5364,7 +5364,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D9" t="n">
         <v>67.40000000000001</v>
@@ -5397,7 +5397,7 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="O9" t="n">
         <v>101.4</v>
@@ -5409,7 +5409,7 @@
         <v>2.3</v>
       </c>
       <c r="R9" t="n">
-        <v>1396886</v>
+        <v>589590</v>
       </c>
       <c r="S9" t="n">
         <v>101935</v>
@@ -5468,7 +5468,7 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="O10" t="n">
         <v>100.9</v>
@@ -5480,7 +5480,7 @@
         <v>1</v>
       </c>
       <c r="R10" t="n">
-        <v>706165</v>
+        <v>744178</v>
       </c>
       <c r="S10" t="n">
         <v>617418</v>
@@ -5506,7 +5506,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D11" t="n">
         <v>68</v>
@@ -5539,7 +5539,7 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="O11" t="n">
         <v>101.9</v>
@@ -5551,7 +5551,7 @@
         <v>3.1</v>
       </c>
       <c r="R11" t="n">
-        <v>1218344</v>
+        <v>770553</v>
       </c>
       <c r="S11" t="n">
         <v>878473</v>
@@ -5610,7 +5610,7 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="O12" t="n">
         <v>102.2</v>
@@ -5622,7 +5622,7 @@
         <v>0.1</v>
       </c>
       <c r="R12" t="n">
-        <v>812352</v>
+        <v>923827</v>
       </c>
       <c r="S12" t="n">
         <v>466127</v>
@@ -5693,7 +5693,7 @@
         <v>0.4</v>
       </c>
       <c r="R13" t="n">
-        <v>2648287</v>
+        <v>1114650</v>
       </c>
       <c r="S13" t="n">
         <v>2735246</v>
@@ -5752,7 +5752,7 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="O14" t="n">
         <v>101.6</v>
@@ -5764,7 +5764,7 @@
         <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>953327</v>
+        <v>1158371</v>
       </c>
       <c r="S14" t="n">
         <v>3039834</v>
@@ -5823,7 +5823,7 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="O15" t="n">
         <v>101.4</v>
@@ -5835,7 +5835,7 @@
         <v>0.2</v>
       </c>
       <c r="R15" t="n">
-        <v>1054718</v>
+        <v>1248989</v>
       </c>
       <c r="S15" t="n">
         <v>1034411</v>
@@ -5894,7 +5894,7 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="O16" t="n">
         <v>101.3</v>
@@ -5906,7 +5906,7 @@
         <v>4.6</v>
       </c>
       <c r="R16" t="n">
-        <v>976059</v>
+        <v>1356607</v>
       </c>
       <c r="S16" t="n">
         <v>166751</v>
@@ -5965,7 +5965,7 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="O17" t="n">
         <v>101.4</v>
@@ -5977,7 +5977,7 @@
         <v>0.5</v>
       </c>
       <c r="R17" t="n">
-        <v>2598730</v>
+        <v>1404615</v>
       </c>
       <c r="S17" t="n">
         <v>3395267</v>
@@ -6036,7 +6036,7 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>87</v>
+        <v>108</v>
       </c>
       <c r="O18" t="n">
         <v>102.6</v>
@@ -6048,7 +6048,7 @@
         <v>0.6</v>
       </c>
       <c r="R18" t="n">
-        <v>2745198</v>
+        <v>1444509</v>
       </c>
       <c r="S18" t="n">
         <v>2489160</v>
@@ -6107,7 +6107,7 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="O19" t="n">
         <v>101.3</v>
@@ -6119,7 +6119,7 @@
         <v>0.1</v>
       </c>
       <c r="R19" t="n">
-        <v>1589056</v>
+        <v>1454273</v>
       </c>
       <c r="S19" t="n">
         <v>1066412</v>
@@ -6190,7 +6190,7 @@
         <v>0.4</v>
       </c>
       <c r="R20" t="n">
-        <v>1724545</v>
+        <v>1541290</v>
       </c>
       <c r="S20" t="n">
         <v>4185865</v>
@@ -6207,40 +6207,40 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D21" t="n">
-        <v>67.40000000000001</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="E21" t="n">
         <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="G21" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="H21" t="n">
         <v>2</v>
       </c>
       <c r="I21" t="n">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K21" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L21" t="n">
         <v>0</v>
@@ -6249,69 +6249,69 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="O21" t="n">
-        <v>100.9</v>
+        <v>100.1</v>
       </c>
       <c r="P21" t="n">
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
       <c r="Q21" t="n">
-        <v>1.3</v>
+        <v>0.3</v>
       </c>
       <c r="R21" t="n">
-        <v>1396886</v>
+        <v>1570675</v>
       </c>
       <c r="S21" t="n">
-        <v>3009015</v>
+        <v>637992</v>
       </c>
       <c r="T21" t="n">
         <v>2</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C22" t="n">
         <v>381</v>
       </c>
       <c r="D22" t="n">
-        <v>65.40000000000001</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="E22" t="n">
         <v>3</v>
       </c>
       <c r="F22" t="n">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="G22" t="n">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="H22" t="n">
         <v>2</v>
       </c>
       <c r="I22" t="n">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="J22" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K22" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
@@ -6320,29 +6320,29 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="O22" t="n">
-        <v>100.1</v>
+        <v>100.9</v>
       </c>
       <c r="P22" t="n">
-        <v>0.1</v>
+        <v>0.9</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.3</v>
+        <v>1.3</v>
       </c>
       <c r="R22" t="n">
-        <v>2099042</v>
+        <v>1593374</v>
       </c>
       <c r="S22" t="n">
-        <v>637992</v>
+        <v>3009015</v>
       </c>
       <c r="T22" t="n">
         <v>2</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
@@ -6391,7 +6391,7 @@
         <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="O23" t="n">
         <v>101.7</v>
@@ -6403,7 +6403,7 @@
         <v>1.2</v>
       </c>
       <c r="R23" t="n">
-        <v>2831164</v>
+        <v>1870917</v>
       </c>
       <c r="S23" t="n">
         <v>453361</v>
@@ -6462,7 +6462,7 @@
         <v>-12</v>
       </c>
       <c r="N24" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="O24" t="n">
         <v>101.3</v>
@@ -6474,7 +6474,7 @@
         <v>0.6</v>
       </c>
       <c r="R24" t="n">
-        <v>2963253</v>
+        <v>2090174</v>
       </c>
       <c r="S24" t="n">
         <v>1948104</v>
@@ -6533,7 +6533,7 @@
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>74</v>
+        <v>90</v>
       </c>
       <c r="O25" t="n">
         <v>100.3</v>
@@ -6545,7 +6545,7 @@
         <v>1.7</v>
       </c>
       <c r="R25" t="n">
-        <v>2516305</v>
+        <v>2176286</v>
       </c>
       <c r="S25" t="n">
         <v>4399137</v>
@@ -6604,7 +6604,7 @@
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="O26" t="n">
         <v>100.6</v>
@@ -6616,7 +6616,7 @@
         <v>2.5</v>
       </c>
       <c r="R26" t="n">
-        <v>3181539</v>
+        <v>2237832</v>
       </c>
       <c r="S26" t="n">
         <v>1595922</v>
@@ -6642,7 +6642,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="D27" t="n">
         <v>65</v>
@@ -6675,7 +6675,7 @@
         <v>-8</v>
       </c>
       <c r="N27" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="O27" t="n">
         <v>100.9</v>
@@ -6687,7 +6687,7 @@
         <v>3.5</v>
       </c>
       <c r="R27" t="n">
-        <v>2297297</v>
+        <v>2521847</v>
       </c>
       <c r="S27" t="n">
         <v>3048395</v>
@@ -6704,40 +6704,40 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>sakalaka</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="D28" t="n">
-        <v>62.2</v>
+        <v>58.6</v>
       </c>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="G28" t="n">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="H28" t="n">
         <v>2</v>
       </c>
       <c r="I28" t="n">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="J28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
@@ -6746,25 +6746,25 @@
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="O28" t="n">
-        <v>101.9</v>
+        <v>101.1</v>
       </c>
       <c r="P28" t="n">
-        <v>1.9</v>
+        <v>1.1</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.7</v>
+        <v>2.3</v>
       </c>
       <c r="R28" t="n">
-        <v>3440315</v>
+        <v>2687602</v>
       </c>
       <c r="S28" t="n">
-        <v>614528</v>
+        <v>3963132</v>
       </c>
       <c r="T28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U28" t="inlineStr">
         <is>
@@ -6775,67 +6775,67 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>sakalaka</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D29" t="n">
-        <v>58.6</v>
+        <v>62.2</v>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F29" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="G29" t="n">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="H29" t="n">
         <v>2</v>
       </c>
       <c r="I29" t="n">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="J29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K29" t="n">
+        <v>2</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" t="n">
+        <v>81</v>
+      </c>
+      <c r="O29" t="n">
+        <v>101.9</v>
+      </c>
+      <c r="P29" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="R29" t="n">
+        <v>2941655</v>
+      </c>
+      <c r="S29" t="n">
+        <v>614528</v>
+      </c>
+      <c r="T29" t="n">
         <v>4</v>
-      </c>
-      <c r="L29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N29" t="n">
-        <v>74</v>
-      </c>
-      <c r="O29" t="n">
-        <v>101.1</v>
-      </c>
-      <c r="P29" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="R29" t="n">
-        <v>5109269</v>
-      </c>
-      <c r="S29" t="n">
-        <v>3963132</v>
-      </c>
-      <c r="T29" t="n">
-        <v>2</v>
       </c>
       <c r="U29" t="inlineStr">
         <is>
@@ -6888,7 +6888,7 @@
         <v>-4</v>
       </c>
       <c r="N30" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O30" t="n">
         <v>101.2</v>
@@ -6900,7 +6900,7 @@
         <v>1.2</v>
       </c>
       <c r="R30" t="n">
-        <v>6804394</v>
+        <v>4842912</v>
       </c>
       <c r="S30" t="n">
         <v>553038</v>
@@ -6959,7 +6959,7 @@
         <v>-8</v>
       </c>
       <c r="N31" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="O31" t="n">
         <v>101.6</v>
@@ -6971,7 +6971,7 @@
         <v>1</v>
       </c>
       <c r="R31" t="n">
-        <v>5949920</v>
+        <v>5004268</v>
       </c>
       <c r="S31" t="n">
         <v>1952243</v>
@@ -6997,7 +6997,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D32" t="n">
         <v>46.6</v>
@@ -7030,7 +7030,7 @@
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O32" t="n">
         <v>98.7</v>
@@ -7042,7 +7042,7 @@
         <v>2.2</v>
       </c>
       <c r="R32" t="n">
-        <v>8883555</v>
+        <v>8607260</v>
       </c>
       <c r="S32" t="n">
         <v>216389</v>

</xml_diff>

<commit_message>
Update standings 2026-10-11 16:10 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -484,13 +484,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>455</v>
+        <v>465</v>
       </c>
     </row>
     <row r="3">
@@ -508,13 +508,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E3" t="n">
         <v>-4</v>
       </c>
       <c r="F3" t="n">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="4">
@@ -532,13 +532,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>424</v>
+        <v>428</v>
       </c>
     </row>
     <row r="5">
@@ -556,13 +556,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="6">
@@ -580,13 +580,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>413</v>
+        <v>420</v>
       </c>
     </row>
     <row r="7">
@@ -595,46 +595,46 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="9">
@@ -676,13 +676,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="11">
@@ -700,13 +700,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="12">
@@ -724,13 +724,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>396</v>
+        <v>400</v>
       </c>
     </row>
     <row r="13">
@@ -739,22 +739,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>391</v>
+        <v>396</v>
       </c>
     </row>
     <row r="14">
@@ -763,46 +763,46 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>45</v>
+        <v>74</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>390</v>
+        <v>394</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>388</v>
+        <v>394</v>
       </c>
     </row>
     <row r="16">
@@ -811,22 +811,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>41</v>
+        <v>74</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>386</v>
+        <v>393</v>
       </c>
     </row>
     <row r="17">
@@ -835,22 +835,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>385</v>
+        <v>391</v>
       </c>
     </row>
     <row r="18">
@@ -859,22 +859,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>384</v>
+        <v>390</v>
       </c>
     </row>
     <row r="19">
@@ -883,22 +883,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>384</v>
+        <v>387</v>
       </c>
     </row>
     <row r="20">
@@ -907,22 +907,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>382</v>
+        <v>386</v>
       </c>
     </row>
     <row r="21">
@@ -931,22 +931,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>382</v>
+        <v>385</v>
       </c>
     </row>
     <row r="22">
@@ -955,22 +955,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="23">
@@ -979,22 +979,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="F23" t="n">
-        <v>376</v>
+        <v>382</v>
       </c>
     </row>
     <row r="24">
@@ -1003,22 +1003,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E24" t="n">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>373</v>
+        <v>377</v>
       </c>
     </row>
     <row r="25">
@@ -1027,22 +1027,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>371</v>
+        <v>377</v>
       </c>
     </row>
     <row r="26">
@@ -1051,22 +1051,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="F26" t="n">
-        <v>370</v>
+        <v>375</v>
       </c>
     </row>
     <row r="27">
@@ -1075,22 +1075,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="E27" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>366</v>
+        <v>372</v>
       </c>
     </row>
     <row r="28">
@@ -1108,13 +1108,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="29">
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>359</v>
+        <v>362</v>
       </c>
     </row>
     <row r="30">
@@ -1156,13 +1156,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E30" t="n">
         <v>-4</v>
       </c>
       <c r="F30" t="n">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="31">
@@ -1180,13 +1180,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E31" t="n">
         <v>-8</v>
       </c>
       <c r="F31" t="n">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="32">
@@ -1204,13 +1204,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -1706,45 +1706,45 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="C7" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D7" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="E7" t="n">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F7" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="C8" t="n">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D8" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="E8" t="n">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F8" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9">
@@ -1838,331 +1838,331 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C13" t="n">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="D13" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="E13" t="n">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="F13" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="C14" t="n">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="D14" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E14" t="n">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="F14" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="C15" t="n">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="D15" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>91</v>
+        <v>71</v>
       </c>
       <c r="F15" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>72</v>
+        <v>45</v>
       </c>
       <c r="C16" t="n">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="D16" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="E16" t="n">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="F16" t="n">
-        <v>32</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="C17" t="n">
-        <v>78</v>
+        <v>107</v>
       </c>
       <c r="D17" t="n">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="E17" t="n">
-        <v>69</v>
+        <v>91</v>
       </c>
       <c r="F17" t="n">
-        <v>55</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C18" t="n">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="D18" t="n">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="E18" t="n">
-        <v>93</v>
+        <v>71</v>
       </c>
       <c r="F18" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="C19" t="n">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="D19" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E19" t="n">
-        <v>58</v>
+        <v>84</v>
       </c>
       <c r="F19" t="n">
-        <v>49</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C20" t="n">
-        <v>107</v>
+        <v>78</v>
       </c>
       <c r="D20" t="n">
-        <v>56</v>
+        <v>78</v>
       </c>
       <c r="E20" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F20" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C21" t="n">
         <v>111</v>
       </c>
       <c r="D21" t="n">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E21" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F21" t="n">
-        <v>27</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="C22" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="D22" t="n">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="E22" t="n">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="F22" t="n">
-        <v>51</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C23" t="n">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E23" t="n">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="F23" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E24" t="n">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="F24" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C25" t="n">
-        <v>120</v>
+        <v>89</v>
       </c>
       <c r="D25" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E25" t="n">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F25" t="n">
-        <v>29</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C26" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="D26" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="E26" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F26" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C27" t="n">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="D27" t="n">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="E27" t="n">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="F27" t="n">
-        <v>38</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28">
@@ -2472,7 +2472,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -2483,7 +2483,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -2835,7 +2835,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -2857,7 +2857,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -2868,7 +2868,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -3071,7 +3071,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -3082,7 +3082,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -3531,7 +3531,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3801,19 +3801,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E7" t="n">
-        <v>189374</v>
+        <v>273503</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -3821,10 +3821,10 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1757289</v>
+        <v>1994005</v>
       </c>
       <c r="H7" t="n">
-        <v>250879</v>
+        <v>1917309</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -3834,23 +3834,23 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E8" t="n">
-        <v>273503</v>
+        <v>189374</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -3858,10 +3858,10 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>1994005</v>
+        <v>1757289</v>
       </c>
       <c r="H8" t="n">
-        <v>1917309</v>
+        <v>250879</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -4023,30 +4023,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E13" t="n">
-        <v>14603</v>
+        <v>410102</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2016/17</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>949628</v>
+        <v>2088802</v>
       </c>
       <c r="H13" t="n">
-        <v>515830</v>
+        <v>5360778</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -4060,30 +4060,30 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>182900</v>
+        <v>14603</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2016/17</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>2098988</v>
+        <v>949628</v>
       </c>
       <c r="H14" t="n">
-        <v>182900</v>
+        <v>515830</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -4093,34 +4093,34 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E15" t="n">
-        <v>30971</v>
+        <v>182900</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>820221</v>
+        <v>2098988</v>
       </c>
       <c r="H15" t="n">
-        <v>58227</v>
+        <v>182900</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E16" t="n">
-        <v>27153</v>
+        <v>95791</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>606381</v>
+        <v>2404119</v>
       </c>
       <c r="H16" t="n">
-        <v>240451</v>
+        <v>5124417</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -4171,30 +4171,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>15288</v>
+        <v>30971</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>329510</v>
+        <v>820221</v>
       </c>
       <c r="H17" t="n">
-        <v>538046</v>
+        <v>58227</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4208,30 +4208,30 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E18" t="n">
-        <v>95791</v>
+        <v>453230</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>2404119</v>
+        <v>5483351</v>
       </c>
       <c r="H18" t="n">
-        <v>5124417</v>
+        <v>8188106</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -4245,19 +4245,19 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E19" t="n">
-        <v>31543</v>
+        <v>27153</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4265,10 +4265,10 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>820692</v>
+        <v>606381</v>
       </c>
       <c r="H19" t="n">
-        <v>1637750</v>
+        <v>240451</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -4282,30 +4282,30 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E20" t="n">
-        <v>410102</v>
+        <v>15288</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>2088802</v>
+        <v>329510</v>
       </c>
       <c r="H20" t="n">
-        <v>5360778</v>
+        <v>538046</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -4319,30 +4319,30 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E21" t="n">
-        <v>15136</v>
+        <v>31543</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>983840</v>
+        <v>820692</v>
       </c>
       <c r="H21" t="n">
-        <v>45077</v>
+        <v>1637750</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -4356,30 +4356,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E22" t="n">
-        <v>453230</v>
+        <v>15136</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>5483351</v>
+        <v>983840</v>
       </c>
       <c r="H22" t="n">
-        <v>8188106</v>
+        <v>45077</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -4393,19 +4393,19 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E23" t="n">
-        <v>334016</v>
+        <v>1320699</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -4413,14 +4413,14 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2156629</v>
+        <v>2490743</v>
       </c>
       <c r="H23" t="n">
-        <v>2691725</v>
+        <v>1861933</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2024/25</t>
         </is>
       </c>
     </row>
@@ -4430,19 +4430,19 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>1320699</v>
+        <v>334016</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -4450,14 +4450,14 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2490743</v>
+        <v>2156629</v>
       </c>
       <c r="H24" t="n">
-        <v>1861933</v>
+        <v>2691725</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
     </row>
@@ -4467,30 +4467,30 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E25" t="n">
-        <v>60517</v>
+        <v>1615102</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2015/16</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>1414622</v>
+        <v>4234674</v>
       </c>
       <c r="H25" t="n">
-        <v>339763</v>
+        <v>6092784</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -4504,30 +4504,30 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E26" t="n">
-        <v>1615102</v>
+        <v>1128645</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>4234674</v>
+        <v>3434302</v>
       </c>
       <c r="H26" t="n">
-        <v>6092784</v>
+        <v>1128645</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -4541,30 +4541,30 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="E27" t="n">
-        <v>1128645</v>
+        <v>60517</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2015/16</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>3434302</v>
+        <v>1414622</v>
       </c>
       <c r="H27" t="n">
-        <v>1128645</v>
+        <v>339763</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -4871,7 +4871,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>455</v>
+        <v>465</v>
       </c>
       <c r="D2" t="n">
         <v>79</v>
@@ -4942,7 +4942,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="D3" t="n">
         <v>72.40000000000001</v>
@@ -5013,7 +5013,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="D4" t="n">
         <v>76.59999999999999</v>
@@ -5080,7 +5080,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D5" t="n">
         <v>70.8</v>
@@ -5151,7 +5151,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="D6" t="n">
         <v>68.8</v>
@@ -5213,37 +5213,37 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Danish Javed</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Old Reijnders Nagar</t>
+          <t>ItDzntMata</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D7" t="n">
-        <v>70.2</v>
+        <v>68.8</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="G7" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="H7" t="n">
         <v>2</v>
       </c>
       <c r="I7" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="J7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K7" t="n">
         <v>3</v>
@@ -5255,66 +5255,66 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="O7" t="n">
-        <v>101.5</v>
+        <v>101.2</v>
       </c>
       <c r="P7" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="Q7" t="n">
-        <v>1.9</v>
+        <v>0.3</v>
       </c>
       <c r="R7" t="n">
-        <v>451158</v>
+        <v>475447</v>
       </c>
       <c r="S7" t="n">
-        <v>3046343</v>
+        <v>5881370</v>
       </c>
       <c r="T7" t="n">
         <v>2</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Danish Javed</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ItDzntMata</t>
+          <t>Old Reijnders Nagar</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="D8" t="n">
-        <v>68.8</v>
+        <v>70.2</v>
       </c>
       <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>90</v>
+      </c>
+      <c r="G8" t="n">
+        <v>113</v>
+      </c>
+      <c r="H8" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" t="n">
+        <v>45</v>
+      </c>
+      <c r="J8" t="n">
         <v>3</v>
-      </c>
-      <c r="F8" t="n">
-        <v>107</v>
-      </c>
-      <c r="G8" t="n">
-        <v>118</v>
-      </c>
-      <c r="H8" t="n">
-        <v>2</v>
-      </c>
-      <c r="I8" t="n">
-        <v>40</v>
-      </c>
-      <c r="J8" t="n">
-        <v>1</v>
       </c>
       <c r="K8" t="n">
         <v>3</v>
@@ -5326,29 +5326,29 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>73</v>
+        <v>51</v>
       </c>
       <c r="O8" t="n">
-        <v>101.2</v>
+        <v>101.5</v>
       </c>
       <c r="P8" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.3</v>
+        <v>1.9</v>
       </c>
       <c r="R8" t="n">
-        <v>475447</v>
+        <v>451158</v>
       </c>
       <c r="S8" t="n">
-        <v>5881370</v>
+        <v>3046343</v>
       </c>
       <c r="T8" t="n">
         <v>2</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
@@ -5435,7 +5435,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D10" t="n">
         <v>70.2</v>
@@ -5506,7 +5506,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D11" t="n">
         <v>68</v>
@@ -5577,7 +5577,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D12" t="n">
         <v>69.59999999999999</v>
@@ -5639,34 +5639,34 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="D13" t="n">
-        <v>64</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="G13" t="n">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="H13" t="n">
         <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="J13" t="n">
         <v>1</v>
@@ -5684,63 +5684,63 @@
         <v>59</v>
       </c>
       <c r="O13" t="n">
-        <v>102.4</v>
+        <v>101.3</v>
       </c>
       <c r="P13" t="n">
-        <v>2.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q13" t="n">
         <v>0.4</v>
       </c>
       <c r="R13" t="n">
-        <v>1114650</v>
+        <v>1541290</v>
       </c>
       <c r="S13" t="n">
-        <v>2735246</v>
+        <v>4185865</v>
       </c>
       <c r="T13" t="n">
         <v>2</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>wildcard, bboost</t>
+          <t>3xc, freehit, wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="D14" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>99</v>
+        <v>70</v>
       </c>
       <c r="G14" t="n">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="H14" t="n">
         <v>2</v>
       </c>
       <c r="I14" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="J14" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
         <v>2</v>
@@ -5752,66 +5752,66 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="O14" t="n">
-        <v>101.6</v>
+        <v>102.4</v>
       </c>
       <c r="P14" t="n">
-        <v>1.6</v>
+        <v>2.4</v>
       </c>
       <c r="Q14" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="R14" t="n">
-        <v>1158371</v>
+        <v>1114650</v>
       </c>
       <c r="S14" t="n">
-        <v>3039834</v>
+        <v>2735246</v>
       </c>
       <c r="T14" t="n">
         <v>2</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="D15" t="n">
-        <v>68.59999999999999</v>
+        <v>69</v>
       </c>
       <c r="E15" t="n">
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="G15" t="n">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="J15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>2</v>
@@ -5823,140 +5823,140 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>26</v>
+        <v>70</v>
       </c>
       <c r="O15" t="n">
-        <v>101.4</v>
+        <v>101.6</v>
       </c>
       <c r="P15" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="R15" t="n">
-        <v>1248989</v>
+        <v>1158371</v>
       </c>
       <c r="S15" t="n">
-        <v>1034411</v>
+        <v>3039834</v>
       </c>
       <c r="T15" t="n">
         <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="D16" t="n">
-        <v>69</v>
+        <v>63.8</v>
       </c>
       <c r="E16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" t="n">
+        <v>70</v>
+      </c>
+      <c r="G16" t="n">
+        <v>93</v>
+      </c>
+      <c r="H16" t="n">
         <v>4</v>
       </c>
-      <c r="F16" t="n">
-        <v>81</v>
-      </c>
-      <c r="G16" t="n">
-        <v>106</v>
-      </c>
-      <c r="H16" t="n">
-        <v>2</v>
-      </c>
       <c r="I16" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
+        <v>3</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>108</v>
+      </c>
+      <c r="O16" t="n">
+        <v>102.6</v>
+      </c>
+      <c r="P16" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="R16" t="n">
+        <v>1444509</v>
+      </c>
+      <c r="S16" t="n">
+        <v>2489160</v>
+      </c>
+      <c r="T16" t="n">
         <v>4</v>
       </c>
-      <c r="L16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" t="n">
-        <v>57</v>
-      </c>
-      <c r="O16" t="n">
-        <v>101.3</v>
-      </c>
-      <c r="P16" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="R16" t="n">
-        <v>1356607</v>
-      </c>
-      <c r="S16" t="n">
-        <v>166751</v>
-      </c>
-      <c r="T16" t="n">
-        <v>2</v>
-      </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost, 3xc, wildcard</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="D17" t="n">
-        <v>64.2</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G17" t="n">
-        <v>78</v>
+        <v>107</v>
       </c>
       <c r="H17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I17" t="n">
+        <v>40</v>
+      </c>
+      <c r="J17" t="n">
         <v>3</v>
       </c>
-      <c r="I17" t="n">
-        <v>41</v>
-      </c>
-      <c r="J17" t="n">
-        <v>1</v>
-      </c>
       <c r="K17" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
@@ -5965,7 +5965,7 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="O17" t="n">
         <v>101.4</v>
@@ -5974,60 +5974,60 @@
         <v>1.4</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="R17" t="n">
-        <v>1404615</v>
+        <v>1248989</v>
       </c>
       <c r="S17" t="n">
-        <v>3395267</v>
+        <v>1034411</v>
       </c>
       <c r="T17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Amad Aura</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="D18" t="n">
-        <v>63.8</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
-        <v>70</v>
+        <v>103</v>
       </c>
       <c r="G18" t="n">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="H18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I18" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J18" t="n">
         <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L18" t="n">
         <v>0</v>
@@ -6036,63 +6036,63 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>108</v>
+        <v>44</v>
       </c>
       <c r="O18" t="n">
-        <v>102.6</v>
+        <v>100.9</v>
       </c>
       <c r="P18" t="n">
-        <v>2.6</v>
+        <v>0.9</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.6</v>
+        <v>1.3</v>
       </c>
       <c r="R18" t="n">
-        <v>1444509</v>
+        <v>1593374</v>
       </c>
       <c r="S18" t="n">
-        <v>2489160</v>
+        <v>3009015</v>
       </c>
       <c r="T18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>3xc, freehit, wildcard</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="D19" t="n">
-        <v>66.8</v>
+        <v>69</v>
       </c>
       <c r="E19" t="n">
         <v>4</v>
       </c>
       <c r="F19" t="n">
-        <v>117</v>
+        <v>81</v>
       </c>
       <c r="G19" t="n">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="H19" t="n">
         <v>2</v>
       </c>
       <c r="I19" t="n">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="J19" t="n">
         <v>5</v>
@@ -6107,7 +6107,7 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="O19" t="n">
         <v>101.3</v>
@@ -6116,60 +6116,60 @@
         <v>1.3</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.1</v>
+        <v>4.6</v>
       </c>
       <c r="R19" t="n">
-        <v>1454273</v>
+        <v>1356607</v>
       </c>
       <c r="S19" t="n">
-        <v>1066412</v>
+        <v>166751</v>
       </c>
       <c r="T19" t="n">
         <v>2</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, 3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="D20" t="n">
-        <v>66.40000000000001</v>
+        <v>64.2</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
         <v>93</v>
       </c>
       <c r="G20" t="n">
-        <v>107</v>
+        <v>78</v>
       </c>
       <c r="H20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I20" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="J20" t="n">
         <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L20" t="n">
         <v>0</v>
@@ -6178,54 +6178,54 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="O20" t="n">
-        <v>101.3</v>
+        <v>101.4</v>
       </c>
       <c r="P20" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="R20" t="n">
-        <v>1541290</v>
+        <v>1404615</v>
       </c>
       <c r="S20" t="n">
-        <v>4185865</v>
+        <v>3395267</v>
       </c>
       <c r="T20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard, bboost</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="D21" t="n">
-        <v>65.40000000000001</v>
+        <v>66.8</v>
       </c>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
-        <v>95</v>
+        <v>117</v>
       </c>
       <c r="G21" t="n">
         <v>111</v>
@@ -6234,13 +6234,13 @@
         <v>2</v>
       </c>
       <c r="I21" t="n">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="J21" t="n">
         <v>5</v>
       </c>
       <c r="K21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L21" t="n">
         <v>0</v>
@@ -6249,69 +6249,69 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="O21" t="n">
-        <v>100.1</v>
+        <v>101.3</v>
       </c>
       <c r="P21" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="Q21" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q21" t="n">
-        <v>0.3</v>
-      </c>
       <c r="R21" t="n">
-        <v>1570675</v>
+        <v>1454273</v>
       </c>
       <c r="S21" t="n">
-        <v>637992</v>
+        <v>1066412</v>
       </c>
       <c r="T21" t="n">
         <v>2</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Amad Aura</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="D22" t="n">
-        <v>67.40000000000001</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="E22" t="n">
         <v>3</v>
       </c>
       <c r="F22" t="n">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="G22" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="H22" t="n">
         <v>2</v>
       </c>
       <c r="I22" t="n">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K22" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
@@ -6320,93 +6320,93 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="O22" t="n">
-        <v>100.9</v>
+        <v>100.1</v>
       </c>
       <c r="P22" t="n">
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
       <c r="Q22" t="n">
-        <v>1.3</v>
+        <v>0.3</v>
       </c>
       <c r="R22" t="n">
-        <v>1593374</v>
+        <v>1570675</v>
       </c>
       <c r="S22" t="n">
-        <v>3009015</v>
+        <v>637992</v>
       </c>
       <c r="T22" t="n">
         <v>2</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="D23" t="n">
-        <v>63.6</v>
+        <v>63.4</v>
       </c>
       <c r="E23" t="n">
         <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="G23" t="n">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="H23" t="n">
         <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="J23" t="n">
         <v>3</v>
       </c>
       <c r="K23" t="n">
+        <v>7</v>
+      </c>
+      <c r="L23" t="n">
         <v>3</v>
       </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
       <c r="M23" t="n">
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="N23" t="n">
         <v>72</v>
       </c>
       <c r="O23" t="n">
-        <v>101.7</v>
+        <v>101.3</v>
       </c>
       <c r="P23" t="n">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
       <c r="Q23" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="R23" t="n">
-        <v>1870917</v>
+        <v>2090174</v>
       </c>
       <c r="S23" t="n">
-        <v>453361</v>
+        <v>1948104</v>
       </c>
       <c r="T23" t="n">
         <v>2</v>
@@ -6420,64 +6420,64 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="D24" t="n">
-        <v>63.4</v>
+        <v>63.6</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="G24" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="H24" t="n">
         <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="J24" t="n">
         <v>3</v>
       </c>
       <c r="K24" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M24" t="n">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="N24" t="n">
         <v>72</v>
       </c>
       <c r="O24" t="n">
-        <v>101.3</v>
+        <v>101.7</v>
       </c>
       <c r="P24" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="R24" t="n">
-        <v>2090174</v>
+        <v>1870917</v>
       </c>
       <c r="S24" t="n">
-        <v>1948104</v>
+        <v>453361</v>
       </c>
       <c r="T24" t="n">
         <v>2</v>
@@ -6491,34 +6491,34 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="D25" t="n">
-        <v>64.40000000000001</v>
+        <v>62.8</v>
       </c>
       <c r="E25" t="n">
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="G25" t="n">
-        <v>120</v>
+        <v>89</v>
       </c>
       <c r="H25" t="n">
         <v>2</v>
       </c>
       <c r="I25" t="n">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="J25" t="n">
         <v>5</v>
@@ -6533,171 +6533,171 @@
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="O25" t="n">
-        <v>100.3</v>
+        <v>100.6</v>
       </c>
       <c r="P25" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="Q25" t="n">
-        <v>1.7</v>
+        <v>2.5</v>
       </c>
       <c r="R25" t="n">
-        <v>2176286</v>
+        <v>2237832</v>
       </c>
       <c r="S25" t="n">
-        <v>4399137</v>
+        <v>1595922</v>
       </c>
       <c r="T25" t="n">
         <v>2</v>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>bboost, 3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="D26" t="n">
-        <v>62.8</v>
+        <v>65</v>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F26" t="n">
         <v>79</v>
       </c>
       <c r="G26" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="H26" t="n">
         <v>2</v>
       </c>
       <c r="I26" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="J26" t="n">
         <v>5</v>
       </c>
       <c r="K26" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M26" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="N26" t="n">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="O26" t="n">
-        <v>100.6</v>
+        <v>100.9</v>
       </c>
       <c r="P26" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="Q26" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="R26" t="n">
-        <v>2237832</v>
+        <v>2521847</v>
       </c>
       <c r="S26" t="n">
-        <v>1595922</v>
+        <v>3048395</v>
       </c>
       <c r="T26" t="n">
         <v>2</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>bboost, 3xc, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="D27" t="n">
-        <v>65</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="G27" t="n">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="H27" t="n">
         <v>2</v>
       </c>
       <c r="I27" t="n">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="J27" t="n">
         <v>5</v>
       </c>
       <c r="K27" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L27" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M27" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>58</v>
+        <v>90</v>
       </c>
       <c r="O27" t="n">
-        <v>100.9</v>
+        <v>100.3</v>
       </c>
       <c r="P27" t="n">
-        <v>0.9</v>
+        <v>0.3</v>
       </c>
       <c r="Q27" t="n">
-        <v>3.5</v>
+        <v>1.7</v>
       </c>
       <c r="R27" t="n">
-        <v>2521847</v>
+        <v>2176286</v>
       </c>
       <c r="S27" t="n">
-        <v>3048395</v>
+        <v>4399137</v>
       </c>
       <c r="T27" t="n">
         <v>2</v>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
@@ -6713,7 +6713,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="D28" t="n">
         <v>58.6</v>
@@ -6784,7 +6784,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="D29" t="n">
         <v>62.2</v>
@@ -6855,7 +6855,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D30" t="n">
         <v>54.6</v>
@@ -6926,7 +6926,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="D31" t="n">
         <v>56.8</v>
@@ -6997,7 +6997,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D32" t="n">
         <v>46.6</v>

</xml_diff>

<commit_message>
Update standings 2026-10-11 21:34 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -484,13 +484,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>465</v>
+        <v>470</v>
       </c>
     </row>
     <row r="3">
@@ -508,13 +508,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="E3" t="n">
         <v>-4</v>
       </c>
       <c r="F3" t="n">
-        <v>430</v>
+        <v>444</v>
       </c>
     </row>
     <row r="4">
@@ -532,13 +532,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>428</v>
+        <v>442</v>
       </c>
     </row>
     <row r="5">
@@ -547,22 +547,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>424</v>
+        <v>430</v>
       </c>
     </row>
     <row r="6">
@@ -571,22 +571,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>420</v>
+        <v>429</v>
       </c>
     </row>
     <row r="7">
@@ -604,18 +604,18 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>412</v>
+        <v>422</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -628,13 +628,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>412</v>
+        <v>417</v>
       </c>
     </row>
     <row r="9">
@@ -643,46 +643,46 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>406</v>
+        <v>410</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>402</v>
+        <v>410</v>
       </c>
     </row>
     <row r="11">
@@ -691,22 +691,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>61</v>
+        <v>88</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>401</v>
+        <v>408</v>
       </c>
     </row>
     <row r="12">
@@ -715,22 +715,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>400</v>
+        <v>407</v>
       </c>
     </row>
     <row r="13">
@@ -739,22 +739,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>396</v>
+        <v>406</v>
       </c>
     </row>
     <row r="14">
@@ -763,46 +763,46 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>394</v>
+        <v>406</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>394</v>
+        <v>405</v>
       </c>
     </row>
     <row r="16">
@@ -811,22 +811,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>393</v>
+        <v>404</v>
       </c>
     </row>
     <row r="17">
@@ -835,22 +835,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>48</v>
+        <v>79</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>391</v>
+        <v>398</v>
       </c>
     </row>
     <row r="18">
@@ -868,13 +868,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>390</v>
+        <v>395</v>
       </c>
     </row>
     <row r="19">
@@ -883,22 +883,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>42</v>
+        <v>69</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="F19" t="n">
-        <v>387</v>
+        <v>394</v>
       </c>
     </row>
     <row r="20">
@@ -907,22 +907,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>386</v>
+        <v>392</v>
       </c>
     </row>
     <row r="21">
@@ -931,22 +931,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>385</v>
+        <v>391</v>
       </c>
     </row>
     <row r="22">
@@ -955,12 +955,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -970,7 +970,7 @@
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>383</v>
+        <v>390</v>
       </c>
     </row>
     <row r="23">
@@ -988,13 +988,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E23" t="n">
         <v>-12</v>
       </c>
       <c r="F23" t="n">
-        <v>382</v>
+        <v>387</v>
       </c>
     </row>
     <row r="24">
@@ -1003,22 +1003,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>377</v>
+        <v>385</v>
       </c>
     </row>
     <row r="25">
@@ -1027,22 +1027,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>377</v>
+        <v>383</v>
       </c>
     </row>
     <row r="26">
@@ -1051,22 +1051,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="E26" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>375</v>
+        <v>382</v>
       </c>
     </row>
     <row r="27">
@@ -1075,22 +1075,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>372</v>
+        <v>382</v>
       </c>
     </row>
     <row r="28">
@@ -1099,22 +1099,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>sakalaka</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>365</v>
+        <v>377</v>
       </c>
     </row>
     <row r="29">
@@ -1123,22 +1123,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>sakalaka</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>51</v>
+        <v>82</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>362</v>
+        <v>375</v>
       </c>
     </row>
     <row r="30">
@@ -1147,22 +1147,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Slumber FC</t>
+          <t>Redsbay</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E30" t="n">
-        <v>-4</v>
+        <v>-8</v>
       </c>
       <c r="F30" t="n">
-        <v>334</v>
+        <v>343</v>
       </c>
     </row>
     <row r="31">
@@ -1171,22 +1171,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Redsbay</t>
+          <t>Slumber FC</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="E31" t="n">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="F31" t="n">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="32">
@@ -1204,13 +1204,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>274</v>
+        <v>282</v>
       </c>
     </row>
   </sheetData>
@@ -1478,17 +1478,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C11" t="n">
         <v>38</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -1502,17 +1502,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C12" t="n">
         <v>38</v>
       </c>
       <c r="D12" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
@@ -1662,45 +1662,45 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="C5" t="n">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="D5" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="E5" t="n">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="F5" t="n">
-        <v>40</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>42</v>
+        <v>74</v>
       </c>
       <c r="C6" t="n">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="D6" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="E6" t="n">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="F6" t="n">
-        <v>61</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7">
@@ -1750,199 +1750,199 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B9" t="n">
+        <v>44</v>
+      </c>
+      <c r="C9" t="n">
+        <v>107</v>
+      </c>
+      <c r="D9" t="n">
+        <v>56</v>
+      </c>
+      <c r="E9" t="n">
         <v>73</v>
       </c>
-      <c r="C9" t="n">
-        <v>90</v>
-      </c>
-      <c r="D9" t="n">
-        <v>55</v>
-      </c>
-      <c r="E9" t="n">
-        <v>69</v>
-      </c>
       <c r="F9" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C10" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D10" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="E10" t="n">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="F10" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="C11" t="n">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="D11" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E11" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="F11" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="C12" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D12" t="n">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="E12" t="n">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="F12" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="C13" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D13" t="n">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="E13" t="n">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="F13" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="C14" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D14" t="n">
+        <v>55</v>
+      </c>
+      <c r="E14" t="n">
+        <v>69</v>
+      </c>
+      <c r="F14" t="n">
         <v>50</v>
-      </c>
-      <c r="E14" t="n">
-        <v>90</v>
-      </c>
-      <c r="F14" t="n">
-        <v>45</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="F15" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="C16" t="n">
-        <v>86</v>
+        <v>118</v>
       </c>
       <c r="D16" t="n">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>93</v>
+        <v>71</v>
       </c>
       <c r="F16" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="C17" t="n">
-        <v>107</v>
+        <v>86</v>
       </c>
       <c r="D17" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="E17" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F17" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18">
@@ -1970,89 +1970,89 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>72</v>
+        <v>43</v>
       </c>
       <c r="C19" t="n">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="D19" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="E19" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F19" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="C20" t="n">
-        <v>78</v>
+        <v>106</v>
       </c>
       <c r="D20" t="n">
-        <v>78</v>
+        <v>51</v>
       </c>
       <c r="E20" t="n">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="F20" t="n">
-        <v>55</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="C21" t="n">
-        <v>111</v>
+        <v>78</v>
       </c>
       <c r="D21" t="n">
-        <v>54</v>
+        <v>78</v>
       </c>
       <c r="E21" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="F21" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C22" t="n">
         <v>111</v>
       </c>
       <c r="D22" t="n">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E22" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F22" t="n">
-        <v>27</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23">
@@ -2080,17 +2080,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="D24" t="n">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="E24" t="n">
         <v>77</v>
@@ -2102,155 +2102,155 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="C25" t="n">
-        <v>89</v>
+        <v>111</v>
       </c>
       <c r="D25" t="n">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="E25" t="n">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="F25" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="C26" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D26" t="n">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="E26" t="n">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F26" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C27" t="n">
-        <v>120</v>
+        <v>89</v>
       </c>
       <c r="D27" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E27" t="n">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F27" t="n">
-        <v>29</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B28" t="n">
+        <v>48</v>
+      </c>
+      <c r="C28" t="n">
+        <v>120</v>
+      </c>
+      <c r="D28" t="n">
+        <v>49</v>
+      </c>
+      <c r="E28" t="n">
+        <v>76</v>
+      </c>
+      <c r="F28" t="n">
         <v>29</v>
-      </c>
-      <c r="C28" t="n">
-        <v>101</v>
-      </c>
-      <c r="D28" t="n">
-        <v>48</v>
-      </c>
-      <c r="E28" t="n">
-        <v>69</v>
-      </c>
-      <c r="F28" t="n">
-        <v>46</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="C29" t="n">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="D29" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E29" t="n">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="F29" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="C30" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D30" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="E30" t="n">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="F30" t="n">
-        <v>46</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="C31" t="n">
+        <v>73</v>
+      </c>
+      <c r="D31" t="n">
+        <v>32</v>
+      </c>
+      <c r="E31" t="n">
         <v>69</v>
       </c>
-      <c r="D31" t="n">
-        <v>37</v>
-      </c>
-      <c r="E31" t="n">
-        <v>89</v>
-      </c>
       <c r="F31" t="n">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="32">
@@ -2535,7 +2535,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2546,7 +2546,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2557,7 +2557,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2653,7 +2653,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -2664,7 +2664,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2868,7 +2868,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -2879,7 +2879,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -2931,7 +2931,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2946,7 +2946,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2972,7 +2972,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2983,7 +2983,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2994,7 +2994,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -3005,7 +3005,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -3016,7 +3016,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -3027,7 +3027,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -3038,7 +3038,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -3060,7 +3060,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -3071,7 +3071,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -3137,7 +3137,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -3148,7 +3148,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -3727,30 +3727,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>71857</v>
+        <v>486041</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>1929309</v>
+        <v>2415786</v>
       </c>
       <c r="H5" t="n">
-        <v>297407</v>
+        <v>1206623</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -3764,30 +3764,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>486041</v>
+        <v>71857</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>2415786</v>
+        <v>1929309</v>
       </c>
       <c r="H6" t="n">
-        <v>1206623</v>
+        <v>297407</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -3834,7 +3834,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -3875,30 +3875,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E9" t="n">
-        <v>37120</v>
+        <v>410102</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>1571193</v>
+        <v>2088802</v>
       </c>
       <c r="H9" t="n">
-        <v>3349378</v>
+        <v>5360778</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -3908,34 +3908,34 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E10" t="n">
-        <v>6474</v>
+        <v>30971</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>1177681</v>
+        <v>820221</v>
       </c>
       <c r="H10" t="n">
-        <v>6474</v>
+        <v>58227</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -3949,30 +3949,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>8917</v>
+        <v>14603</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2016/17</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2118382</v>
+        <v>949628</v>
       </c>
       <c r="H11" t="n">
-        <v>9146930</v>
+        <v>515830</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -3986,30 +3986,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E12" t="n">
-        <v>28582</v>
+        <v>6474</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>881388</v>
+        <v>1177681</v>
       </c>
       <c r="H12" t="n">
-        <v>239490</v>
+        <v>6474</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -4023,30 +4023,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="E13" t="n">
-        <v>410102</v>
+        <v>8917</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>2088802</v>
+        <v>2118382</v>
       </c>
       <c r="H13" t="n">
-        <v>5360778</v>
+        <v>9146930</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -4060,30 +4060,30 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E14" t="n">
-        <v>14603</v>
+        <v>37120</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2016/17</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>949628</v>
+        <v>1571193</v>
       </c>
       <c r="H14" t="n">
-        <v>515830</v>
+        <v>3349378</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -4093,34 +4093,34 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E15" t="n">
-        <v>182900</v>
+        <v>28582</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>2098988</v>
+        <v>881388</v>
       </c>
       <c r="H15" t="n">
-        <v>182900</v>
+        <v>239490</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4134,30 +4134,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E16" t="n">
-        <v>95791</v>
+        <v>182900</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>2404119</v>
+        <v>2098988</v>
       </c>
       <c r="H16" t="n">
-        <v>5124417</v>
+        <v>182900</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -4171,19 +4171,19 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E17" t="n">
-        <v>30971</v>
+        <v>95791</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4191,10 +4191,10 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>820221</v>
+        <v>2404119</v>
       </c>
       <c r="H17" t="n">
-        <v>58227</v>
+        <v>5124417</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -4245,30 +4245,30 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E19" t="n">
-        <v>27153</v>
+        <v>1128645</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>606381</v>
+        <v>3434302</v>
       </c>
       <c r="H19" t="n">
-        <v>240451</v>
+        <v>1128645</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -4282,30 +4282,30 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D20" t="n">
         <v>12</v>
       </c>
       <c r="E20" t="n">
-        <v>15288</v>
+        <v>27153</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>329510</v>
+        <v>606381</v>
       </c>
       <c r="H20" t="n">
-        <v>538046</v>
+        <v>240451</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -4319,30 +4319,30 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E21" t="n">
-        <v>31543</v>
+        <v>15288</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>820692</v>
+        <v>329510</v>
       </c>
       <c r="H21" t="n">
-        <v>1637750</v>
+        <v>538046</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -4356,30 +4356,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E22" t="n">
-        <v>15136</v>
+        <v>31543</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>983840</v>
+        <v>820692</v>
       </c>
       <c r="H22" t="n">
-        <v>45077</v>
+        <v>1637750</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -4430,19 +4430,19 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E24" t="n">
-        <v>334016</v>
+        <v>81907</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -4450,10 +4450,10 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2156629</v>
+        <v>3252487</v>
       </c>
       <c r="H24" t="n">
-        <v>2691725</v>
+        <v>11118394</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -4467,30 +4467,30 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E25" t="n">
-        <v>1615102</v>
+        <v>15136</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>4234674</v>
+        <v>983840</v>
       </c>
       <c r="H25" t="n">
-        <v>6092784</v>
+        <v>45077</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -4504,30 +4504,30 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E26" t="n">
-        <v>1128645</v>
+        <v>334016</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>3434302</v>
+        <v>2156629</v>
       </c>
       <c r="H26" t="n">
-        <v>1128645</v>
+        <v>2691725</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -4541,30 +4541,30 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>60517</v>
+        <v>1615102</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2015/16</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>1414622</v>
+        <v>4234674</v>
       </c>
       <c r="H27" t="n">
-        <v>339763</v>
+        <v>6092784</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -4578,30 +4578,30 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>sakalaka</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E28" t="n">
-        <v>117338</v>
+        <v>60517</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2015/16</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>4684930</v>
+        <v>1414622</v>
       </c>
       <c r="H28" t="n">
-        <v>117338</v>
+        <v>339763</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -4615,30 +4615,30 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>sakalaka</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E29" t="n">
-        <v>81907</v>
+        <v>117338</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>3252487</v>
+        <v>4684930</v>
       </c>
       <c r="H29" t="n">
-        <v>11118394</v>
+        <v>117338</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -4652,19 +4652,19 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Slumber FC</t>
+          <t>Redsbay</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E30" t="n">
-        <v>676529</v>
+        <v>4884220</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -4672,10 +4672,10 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>998938</v>
+        <v>4884220</v>
       </c>
       <c r="H30" t="n">
-        <v>676529</v>
+        <v>4884220</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -4689,19 +4689,19 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Redsbay</t>
+          <t>Slumber FC</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E31" t="n">
-        <v>4884220</v>
+        <v>676529</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -4709,10 +4709,10 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>4884220</v>
+        <v>998938</v>
       </c>
       <c r="H31" t="n">
-        <v>4884220</v>
+        <v>676529</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -4871,7 +4871,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>465</v>
+        <v>470</v>
       </c>
       <c r="D2" t="n">
         <v>79</v>
@@ -4904,7 +4904,7 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="O2" t="n">
         <v>102.3</v>
@@ -4916,7 +4916,7 @@
         <v>2.4</v>
       </c>
       <c r="R2" t="n">
-        <v>14788</v>
+        <v>11041</v>
       </c>
       <c r="S2" t="n">
         <v>270274</v>
@@ -4942,7 +4942,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>430</v>
+        <v>444</v>
       </c>
       <c r="D3" t="n">
         <v>72.40000000000001</v>
@@ -4975,7 +4975,7 @@
         <v>-4</v>
       </c>
       <c r="N3" t="n">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="O3" t="n">
         <v>102.2</v>
@@ -4987,7 +4987,7 @@
         <v>0.7</v>
       </c>
       <c r="R3" t="n">
-        <v>167799</v>
+        <v>138579</v>
       </c>
       <c r="S3" t="n">
         <v>1229264</v>
@@ -5013,7 +5013,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>428</v>
+        <v>442</v>
       </c>
       <c r="D4" t="n">
         <v>76.59999999999999</v>
@@ -5046,7 +5046,7 @@
         <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="O4" t="n">
         <v>101.1</v>
@@ -5058,7 +5058,7 @@
         <v>0.3</v>
       </c>
       <c r="R4" t="n">
-        <v>218204</v>
+        <v>160619</v>
       </c>
       <c r="S4" t="n">
         <v>1461471</v>
@@ -5071,40 +5071,40 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BattleBorn</t>
+          <t>Loading...</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>424</v>
+        <v>430</v>
       </c>
       <c r="D5" t="n">
-        <v>70.8</v>
+        <v>68.8</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="G5" t="n">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="H5" t="n">
         <v>2</v>
       </c>
       <c r="I5" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -5113,100 +5113,100 @@
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>88</v>
+        <v>47</v>
       </c>
       <c r="O5" t="n">
-        <v>101.9</v>
+        <v>101.3</v>
       </c>
       <c r="P5" t="n">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
       <c r="Q5" t="n">
-        <v>1.3</v>
+        <v>3.5</v>
       </c>
       <c r="R5" t="n">
-        <v>222828</v>
+        <v>346688</v>
       </c>
       <c r="S5" t="n">
-        <v>266328</v>
+        <v>5250200</v>
       </c>
       <c r="T5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Loading...</t>
+          <t>BattleBorn</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>420</v>
+        <v>429</v>
       </c>
       <c r="D6" t="n">
-        <v>68.8</v>
+        <v>70.8</v>
       </c>
       <c r="E6" t="n">
         <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="G6" t="n">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="H6" t="n">
         <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K6" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>92</v>
+      </c>
+      <c r="O6" t="n">
+        <v>101.9</v>
+      </c>
+      <c r="P6" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="R6" t="n">
+        <v>360389</v>
+      </c>
+      <c r="S6" t="n">
+        <v>266328</v>
+      </c>
+      <c r="T6" t="n">
         <v>4</v>
       </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="n">
-        <v>47</v>
-      </c>
-      <c r="O6" t="n">
-        <v>101.3</v>
-      </c>
-      <c r="P6" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="R6" t="n">
-        <v>410385</v>
-      </c>
-      <c r="S6" t="n">
-        <v>5250200</v>
-      </c>
-      <c r="T6" t="n">
-        <v>2</v>
-      </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>3xc, wildcard, bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
@@ -5222,7 +5222,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>412</v>
+        <v>422</v>
       </c>
       <c r="D7" t="n">
         <v>68.8</v>
@@ -5255,7 +5255,7 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O7" t="n">
         <v>101.2</v>
@@ -5267,7 +5267,7 @@
         <v>0.3</v>
       </c>
       <c r="R7" t="n">
-        <v>475447</v>
+        <v>537268</v>
       </c>
       <c r="S7" t="n">
         <v>5881370</v>
@@ -5293,7 +5293,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="D8" t="n">
         <v>70.2</v>
@@ -5326,7 +5326,7 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="O8" t="n">
         <v>101.5</v>
@@ -5338,7 +5338,7 @@
         <v>1.9</v>
       </c>
       <c r="R8" t="n">
-        <v>451158</v>
+        <v>693079</v>
       </c>
       <c r="S8" t="n">
         <v>3046343</v>
@@ -5355,40 +5355,40 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="D9" t="n">
-        <v>67.40000000000001</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>66</v>
+        <v>93</v>
       </c>
       <c r="G9" t="n">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="H9" t="n">
         <v>2</v>
       </c>
       <c r="I9" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="J9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
@@ -5397,69 +5397,69 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="O9" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="P9" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q9" t="n">
-        <v>2.3</v>
+        <v>0.4</v>
       </c>
       <c r="R9" t="n">
-        <v>589590</v>
+        <v>952624</v>
       </c>
       <c r="S9" t="n">
-        <v>101935</v>
+        <v>4185865</v>
       </c>
       <c r="T9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>3xc, freehit, wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>402</v>
+        <v>410</v>
       </c>
       <c r="D10" t="n">
-        <v>70.2</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="E10" t="n">
         <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="G10" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H10" t="n">
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="J10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -5468,69 +5468,69 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>80</v>
+        <v>27</v>
       </c>
       <c r="O10" t="n">
-        <v>100.9</v>
+        <v>101.4</v>
       </c>
       <c r="P10" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="Q10" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="R10" t="n">
-        <v>744178</v>
+        <v>952624</v>
       </c>
       <c r="S10" t="n">
-        <v>617418</v>
+        <v>1034411</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>bboost, 3xc, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="D11" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="G11" t="n">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="H11" t="n">
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="J11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -5539,66 +5539,66 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="O11" t="n">
-        <v>101.9</v>
+        <v>102.4</v>
       </c>
       <c r="P11" t="n">
-        <v>1.9</v>
+        <v>2.4</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.1</v>
+        <v>0.4</v>
       </c>
       <c r="R11" t="n">
-        <v>770553</v>
+        <v>1037797</v>
       </c>
       <c r="S11" t="n">
-        <v>878473</v>
+        <v>2735246</v>
       </c>
       <c r="T11" t="n">
         <v>2</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="D12" t="n">
-        <v>69.59999999999999</v>
+        <v>70.2</v>
       </c>
       <c r="E12" t="n">
         <v>3</v>
       </c>
       <c r="F12" t="n">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="G12" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H12" t="n">
         <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="J12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K12" t="n">
         <v>4</v>
@@ -5610,69 +5610,69 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>46</v>
+        <v>80</v>
       </c>
       <c r="O12" t="n">
-        <v>102.2</v>
+        <v>100.9</v>
       </c>
       <c r="P12" t="n">
-        <v>2.2</v>
+        <v>0.9</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="R12" t="n">
-        <v>923827</v>
+        <v>1095162</v>
       </c>
       <c r="S12" t="n">
-        <v>466127</v>
+        <v>617418</v>
       </c>
       <c r="T12" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>bboost, 3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>396</v>
+        <v>406</v>
       </c>
       <c r="D13" t="n">
-        <v>66.40000000000001</v>
+        <v>68</v>
       </c>
       <c r="E13" t="n">
         <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G13" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H13" t="n">
         <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -5681,69 +5681,69 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="O13" t="n">
-        <v>101.3</v>
+        <v>101.9</v>
       </c>
       <c r="P13" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.4</v>
+        <v>3.1</v>
       </c>
       <c r="R13" t="n">
-        <v>1541290</v>
+        <v>1131411</v>
       </c>
       <c r="S13" t="n">
-        <v>4185865</v>
+        <v>878473</v>
       </c>
       <c r="T13" t="n">
         <v>2</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard, bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>394</v>
+        <v>406</v>
       </c>
       <c r="D14" t="n">
-        <v>64</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="G14" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="H14" t="n">
         <v>2</v>
       </c>
       <c r="I14" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -5752,69 +5752,69 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="O14" t="n">
-        <v>102.4</v>
+        <v>101.4</v>
       </c>
       <c r="P14" t="n">
-        <v>2.4</v>
+        <v>1.4</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.4</v>
+        <v>2.3</v>
       </c>
       <c r="R14" t="n">
-        <v>1114650</v>
+        <v>1140818</v>
       </c>
       <c r="S14" t="n">
-        <v>2735246</v>
+        <v>101935</v>
       </c>
       <c r="T14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>wildcard, bboost</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>394</v>
+        <v>405</v>
       </c>
       <c r="D15" t="n">
-        <v>69</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="E15" t="n">
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="G15" t="n">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
@@ -5823,69 +5823,69 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="O15" t="n">
-        <v>101.6</v>
+        <v>102.2</v>
       </c>
       <c r="P15" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="R15" t="n">
-        <v>1158371</v>
+        <v>1187333</v>
       </c>
       <c r="S15" t="n">
-        <v>3039834</v>
+        <v>466127</v>
       </c>
       <c r="T15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Pole Calmer �</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>393</v>
+        <v>404</v>
       </c>
       <c r="D16" t="n">
-        <v>63.8</v>
+        <v>69</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="G16" t="n">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="H16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
@@ -5894,70 +5894,70 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>108</v>
+        <v>71</v>
       </c>
       <c r="O16" t="n">
-        <v>102.6</v>
+        <v>101.6</v>
       </c>
       <c r="P16" t="n">
-        <v>2.6</v>
+        <v>1.6</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="R16" t="n">
-        <v>1444509</v>
+        <v>1220869</v>
       </c>
       <c r="S16" t="n">
-        <v>2489160</v>
+        <v>3039834</v>
       </c>
       <c r="T16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Pole Calmer �</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="D17" t="n">
-        <v>68.59999999999999</v>
+        <v>63.8</v>
       </c>
       <c r="E17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" t="n">
+        <v>70</v>
+      </c>
+      <c r="G17" t="n">
+        <v>93</v>
+      </c>
+      <c r="H17" t="n">
+        <v>4</v>
+      </c>
+      <c r="I17" t="n">
+        <v>45</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" t="n">
         <v>3</v>
       </c>
-      <c r="F17" t="n">
-        <v>90</v>
-      </c>
-      <c r="G17" t="n">
-        <v>107</v>
-      </c>
-      <c r="H17" t="n">
-        <v>2</v>
-      </c>
-      <c r="I17" t="n">
-        <v>40</v>
-      </c>
-      <c r="J17" t="n">
-        <v>3</v>
-      </c>
-      <c r="K17" t="n">
-        <v>2</v>
-      </c>
       <c r="L17" t="n">
         <v>0</v>
       </c>
@@ -5965,29 +5965,29 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>26</v>
+        <v>108</v>
       </c>
       <c r="O17" t="n">
-        <v>101.4</v>
+        <v>102.6</v>
       </c>
       <c r="P17" t="n">
-        <v>1.4</v>
+        <v>2.6</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="R17" t="n">
-        <v>1248989</v>
+        <v>1533467</v>
       </c>
       <c r="S17" t="n">
-        <v>1034411</v>
+        <v>2489160</v>
       </c>
       <c r="T17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
@@ -6003,7 +6003,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="D18" t="n">
         <v>67.40000000000001</v>
@@ -6036,7 +6036,7 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O18" t="n">
         <v>100.9</v>
@@ -6048,7 +6048,7 @@
         <v>1.3</v>
       </c>
       <c r="R18" t="n">
-        <v>1593374</v>
+        <v>1694595</v>
       </c>
       <c r="S18" t="n">
         <v>3009015</v>
@@ -6065,108 +6065,108 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="D19" t="n">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G19" t="n">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="H19" t="n">
         <v>2</v>
       </c>
       <c r="I19" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="J19" t="n">
         <v>5</v>
       </c>
       <c r="K19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="N19" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="O19" t="n">
-        <v>101.3</v>
+        <v>100.9</v>
       </c>
       <c r="P19" t="n">
-        <v>1.3</v>
+        <v>0.9</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.6</v>
+        <v>3.5</v>
       </c>
       <c r="R19" t="n">
-        <v>1356607</v>
+        <v>1797324</v>
       </c>
       <c r="S19" t="n">
-        <v>166751</v>
+        <v>3048395</v>
       </c>
       <c r="T19" t="n">
         <v>2</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>bboost, 3xc, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>386</v>
+        <v>392</v>
       </c>
       <c r="D20" t="n">
-        <v>64.2</v>
+        <v>69</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F20" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="G20" t="n">
-        <v>78</v>
+        <v>106</v>
       </c>
       <c r="H20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I20" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K20" t="n">
         <v>4</v>
@@ -6178,66 +6178,66 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="O20" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="P20" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.5</v>
+        <v>4.6</v>
       </c>
       <c r="R20" t="n">
-        <v>1404615</v>
+        <v>1885922</v>
       </c>
       <c r="S20" t="n">
-        <v>3395267</v>
+        <v>166751</v>
       </c>
       <c r="T20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, 3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="D21" t="n">
-        <v>66.8</v>
+        <v>64.2</v>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>117</v>
+        <v>93</v>
       </c>
       <c r="G21" t="n">
-        <v>111</v>
+        <v>78</v>
       </c>
       <c r="H21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I21" t="n">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="J21" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K21" t="n">
         <v>4</v>
@@ -6249,25 +6249,25 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="O21" t="n">
-        <v>101.3</v>
+        <v>101.4</v>
       </c>
       <c r="P21" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="R21" t="n">
-        <v>1454273</v>
+        <v>1946361</v>
       </c>
       <c r="S21" t="n">
-        <v>1066412</v>
+        <v>3395267</v>
       </c>
       <c r="T21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
@@ -6278,25 +6278,25 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="D22" t="n">
-        <v>65.40000000000001</v>
+        <v>66.8</v>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
-        <v>95</v>
+        <v>117</v>
       </c>
       <c r="G22" t="n">
         <v>111</v>
@@ -6305,13 +6305,13 @@
         <v>2</v>
       </c>
       <c r="I22" t="n">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="J22" t="n">
         <v>5</v>
       </c>
       <c r="K22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
@@ -6320,29 +6320,29 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="O22" t="n">
-        <v>100.1</v>
+        <v>101.3</v>
       </c>
       <c r="P22" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="Q22" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q22" t="n">
-        <v>0.3</v>
-      </c>
       <c r="R22" t="n">
-        <v>1570675</v>
+        <v>2007432</v>
       </c>
       <c r="S22" t="n">
-        <v>637992</v>
+        <v>1066412</v>
       </c>
       <c r="T22" t="n">
         <v>2</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
@@ -6358,7 +6358,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="D23" t="n">
         <v>63.4</v>
@@ -6403,7 +6403,7 @@
         <v>0.6</v>
       </c>
       <c r="R23" t="n">
-        <v>2090174</v>
+        <v>2231895</v>
       </c>
       <c r="S23" t="n">
         <v>1948104</v>
@@ -6420,40 +6420,40 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="D24" t="n">
-        <v>63.6</v>
+        <v>62.2</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="G24" t="n">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="H24" t="n">
         <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="J24" t="n">
         <v>3</v>
       </c>
       <c r="K24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
@@ -6462,25 +6462,25 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="O24" t="n">
-        <v>101.7</v>
+        <v>101.9</v>
       </c>
       <c r="P24" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="Q24" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="R24" t="n">
-        <v>1870917</v>
+        <v>2308052</v>
       </c>
       <c r="S24" t="n">
-        <v>453361</v>
+        <v>614528</v>
       </c>
       <c r="T24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U24" t="inlineStr">
         <is>
@@ -6491,40 +6491,40 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="D25" t="n">
-        <v>62.8</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F25" t="n">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="G25" t="n">
-        <v>89</v>
+        <v>111</v>
       </c>
       <c r="H25" t="n">
         <v>2</v>
       </c>
       <c r="I25" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="J25" t="n">
         <v>5</v>
       </c>
       <c r="K25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
@@ -6533,57 +6533,57 @@
         <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="O25" t="n">
-        <v>100.6</v>
+        <v>100.1</v>
       </c>
       <c r="P25" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="Q25" t="n">
-        <v>2.5</v>
+        <v>0.3</v>
       </c>
       <c r="R25" t="n">
-        <v>2237832</v>
+        <v>2475208</v>
       </c>
       <c r="S25" t="n">
-        <v>1595922</v>
+        <v>637992</v>
       </c>
       <c r="T25" t="n">
         <v>2</v>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>bboost, 3xc, wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>375</v>
+        <v>382</v>
       </c>
       <c r="D26" t="n">
-        <v>65</v>
+        <v>63.6</v>
       </c>
       <c r="E26" t="n">
         <v>2</v>
       </c>
       <c r="F26" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="G26" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H26" t="n">
         <v>2</v>
@@ -6592,75 +6592,75 @@
         <v>38</v>
       </c>
       <c r="J26" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K26" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="O26" t="n">
-        <v>100.9</v>
+        <v>101.7</v>
       </c>
       <c r="P26" t="n">
-        <v>0.9</v>
+        <v>1.7</v>
       </c>
       <c r="Q26" t="n">
-        <v>3.5</v>
+        <v>1.2</v>
       </c>
       <c r="R26" t="n">
-        <v>2521847</v>
+        <v>2513181</v>
       </c>
       <c r="S26" t="n">
-        <v>3048395</v>
+        <v>453361</v>
       </c>
       <c r="T26" t="n">
         <v>2</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Malisahi Randuas</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>372</v>
+        <v>382</v>
       </c>
       <c r="D27" t="n">
-        <v>64.40000000000001</v>
+        <v>62.8</v>
       </c>
       <c r="E27" t="n">
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="G27" t="n">
-        <v>120</v>
+        <v>89</v>
       </c>
       <c r="H27" t="n">
         <v>2</v>
       </c>
       <c r="I27" t="n">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="J27" t="n">
         <v>5</v>
@@ -6675,48 +6675,48 @@
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="O27" t="n">
-        <v>100.3</v>
+        <v>100.6</v>
       </c>
       <c r="P27" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="Q27" t="n">
-        <v>1.7</v>
+        <v>2.5</v>
       </c>
       <c r="R27" t="n">
-        <v>2176286</v>
+        <v>2524915</v>
       </c>
       <c r="S27" t="n">
-        <v>4399137</v>
+        <v>1595922</v>
       </c>
       <c r="T27" t="n">
         <v>2</v>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>bboost, 3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>sakalaka</t>
+          <t>Malisahi Randuas</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>365</v>
+        <v>377</v>
       </c>
       <c r="D28" t="n">
-        <v>58.6</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="E28" t="n">
         <v>1</v>
@@ -6725,7 +6725,7 @@
         <v>90</v>
       </c>
       <c r="G28" t="n">
-        <v>101</v>
+        <v>120</v>
       </c>
       <c r="H28" t="n">
         <v>2</v>
@@ -6734,7 +6734,7 @@
         <v>29</v>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K28" t="n">
         <v>4</v>
@@ -6746,22 +6746,22 @@
         <v>0</v>
       </c>
       <c r="N28" t="n">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="O28" t="n">
-        <v>101.1</v>
+        <v>100.3</v>
       </c>
       <c r="P28" t="n">
-        <v>1.1</v>
+        <v>0.3</v>
       </c>
       <c r="Q28" t="n">
-        <v>2.3</v>
+        <v>1.7</v>
       </c>
       <c r="R28" t="n">
-        <v>2687602</v>
+        <v>2871388</v>
       </c>
       <c r="S28" t="n">
-        <v>3963132</v>
+        <v>4399137</v>
       </c>
       <c r="T28" t="n">
         <v>2</v>
@@ -6775,40 +6775,40 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>sakalaka</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>362</v>
+        <v>375</v>
       </c>
       <c r="D29" t="n">
-        <v>62.2</v>
+        <v>58.6</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="G29" t="n">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="H29" t="n">
         <v>2</v>
       </c>
       <c r="I29" t="n">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="J29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K29" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L29" t="n">
         <v>0</v>
@@ -6817,25 +6817,25 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="O29" t="n">
-        <v>101.9</v>
+        <v>101.1</v>
       </c>
       <c r="P29" t="n">
-        <v>1.9</v>
+        <v>1.1</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.7</v>
+        <v>2.3</v>
       </c>
       <c r="R29" t="n">
-        <v>2941655</v>
+        <v>3013315</v>
       </c>
       <c r="S29" t="n">
-        <v>614528</v>
+        <v>3963132</v>
       </c>
       <c r="T29" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U29" t="inlineStr">
         <is>
@@ -6846,64 +6846,64 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Slumber FC</t>
+          <t>Redsbay</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>334</v>
+        <v>343</v>
       </c>
       <c r="D30" t="n">
-        <v>54.6</v>
+        <v>56.8</v>
       </c>
       <c r="E30" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F30" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="G30" t="n">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="H30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I30" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="J30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K30" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L30" t="n">
+        <v>2</v>
+      </c>
+      <c r="M30" t="n">
+        <v>-8</v>
+      </c>
+      <c r="N30" t="n">
+        <v>39</v>
+      </c>
+      <c r="O30" t="n">
+        <v>101.6</v>
+      </c>
+      <c r="P30" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="Q30" t="n">
         <v>1</v>
       </c>
-      <c r="M30" t="n">
-        <v>-4</v>
-      </c>
-      <c r="N30" t="n">
-        <v>87</v>
-      </c>
-      <c r="O30" t="n">
-        <v>101.2</v>
-      </c>
-      <c r="P30" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>1.2</v>
-      </c>
       <c r="R30" t="n">
-        <v>4842912</v>
+        <v>5407173</v>
       </c>
       <c r="S30" t="n">
-        <v>553038</v>
+        <v>1952243</v>
       </c>
       <c r="T30" t="n">
         <v>4</v>
@@ -6917,64 +6917,64 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Redsbay</t>
+          <t>Slumber FC</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="D31" t="n">
-        <v>56.8</v>
+        <v>54.6</v>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="G31" t="n">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="H31" t="n">
+        <v>2</v>
+      </c>
+      <c r="I31" t="n">
+        <v>32</v>
+      </c>
+      <c r="J31" t="n">
+        <v>3</v>
+      </c>
+      <c r="K31" t="n">
         <v>4</v>
       </c>
-      <c r="I31" t="n">
-        <v>37</v>
-      </c>
-      <c r="J31" t="n">
+      <c r="L31" t="n">
         <v>1</v>
       </c>
-      <c r="K31" t="n">
-        <v>5</v>
-      </c>
-      <c r="L31" t="n">
-        <v>2</v>
-      </c>
       <c r="M31" t="n">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="N31" t="n">
-        <v>37</v>
+        <v>103</v>
       </c>
       <c r="O31" t="n">
-        <v>101.6</v>
+        <v>101.2</v>
       </c>
       <c r="P31" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="Q31" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="R31" t="n">
-        <v>5004268</v>
+        <v>5751989</v>
       </c>
       <c r="S31" t="n">
-        <v>1952243</v>
+        <v>553038</v>
       </c>
       <c r="T31" t="n">
         <v>4</v>
@@ -6997,7 +6997,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="D32" t="n">
         <v>46.6</v>
@@ -7042,7 +7042,7 @@
         <v>2.2</v>
       </c>
       <c r="R32" t="n">
-        <v>8607260</v>
+        <v>8713733</v>
       </c>
       <c r="S32" t="n">
         <v>216389</v>

</xml_diff>

<commit_message>
Update standings 2026-10-12 01:02 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -643,16 +643,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -667,16 +667,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -1750,45 +1750,45 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="C9" t="n">
         <v>107</v>
       </c>
       <c r="D9" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="E9" t="n">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="F9" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="C10" t="n">
         <v>107</v>
       </c>
       <c r="D10" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E10" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="F10" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11">
@@ -3875,30 +3875,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>410102</v>
+        <v>30971</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>2088802</v>
+        <v>820221</v>
       </c>
       <c r="H9" t="n">
-        <v>5360778</v>
+        <v>58227</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -3912,30 +3912,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E10" t="n">
-        <v>30971</v>
+        <v>410102</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>820221</v>
+        <v>2088802</v>
       </c>
       <c r="H10" t="n">
-        <v>58227</v>
+        <v>5360778</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -5355,25 +5355,25 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>410</v>
       </c>
       <c r="D9" t="n">
-        <v>66.40000000000001</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G9" t="n">
         <v>107</v>
@@ -5382,10 +5382,10 @@
         <v>2</v>
       </c>
       <c r="I9" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K9" t="n">
         <v>2</v>
@@ -5397,54 +5397,54 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="O9" t="n">
-        <v>101.3</v>
+        <v>101.4</v>
       </c>
       <c r="P9" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="R9" t="n">
         <v>952624</v>
       </c>
       <c r="S9" t="n">
-        <v>4185865</v>
+        <v>1034411</v>
       </c>
       <c r="T9" t="n">
         <v>2</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard, bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>410</v>
       </c>
       <c r="D10" t="n">
-        <v>68.59999999999999</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="E10" t="n">
         <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G10" t="n">
         <v>107</v>
@@ -5453,10 +5453,10 @@
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
@@ -5468,29 +5468,29 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="O10" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="P10" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="R10" t="n">
         <v>952624</v>
       </c>
       <c r="S10" t="n">
-        <v>1034411</v>
+        <v>4185865</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard, bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-12 08:42 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -643,16 +643,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -667,16 +667,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -1750,45 +1750,45 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="C9" t="n">
         <v>107</v>
       </c>
       <c r="D9" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E9" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="F9" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="C10" t="n">
         <v>107</v>
       </c>
       <c r="D10" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="E10" t="n">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="F10" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11">
@@ -3875,30 +3875,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E9" t="n">
-        <v>30971</v>
+        <v>410102</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>820221</v>
+        <v>2088802</v>
       </c>
       <c r="H9" t="n">
-        <v>58227</v>
+        <v>5360778</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -3912,30 +3912,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E10" t="n">
-        <v>410102</v>
+        <v>30971</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2088802</v>
+        <v>820221</v>
       </c>
       <c r="H10" t="n">
-        <v>5360778</v>
+        <v>58227</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -5355,25 +5355,25 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>410</v>
       </c>
       <c r="D9" t="n">
-        <v>68.59999999999999</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G9" t="n">
         <v>107</v>
@@ -5382,10 +5382,10 @@
         <v>2</v>
       </c>
       <c r="I9" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
         <v>2</v>
@@ -5397,54 +5397,54 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="O9" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="P9" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="R9" t="n">
         <v>952624</v>
       </c>
       <c r="S9" t="n">
-        <v>1034411</v>
+        <v>4185865</v>
       </c>
       <c r="T9" t="n">
         <v>2</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>410</v>
       </c>
       <c r="D10" t="n">
-        <v>66.40000000000001</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="E10" t="n">
         <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G10" t="n">
         <v>107</v>
@@ -5453,10 +5453,10 @@
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
@@ -5468,29 +5468,29 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="O10" t="n">
-        <v>101.3</v>
+        <v>101.4</v>
       </c>
       <c r="P10" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="R10" t="n">
         <v>952624</v>
       </c>
       <c r="S10" t="n">
-        <v>4185865</v>
+        <v>1034411</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard, bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-12 19:38 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -484,13 +484,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>470</v>
+        <v>473</v>
       </c>
     </row>
     <row r="3">
@@ -508,13 +508,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E3" t="n">
         <v>-4</v>
       </c>
       <c r="F3" t="n">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="4">
@@ -532,13 +532,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="5">
@@ -556,13 +556,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>430</v>
+        <v>433</v>
       </c>
     </row>
     <row r="6">
@@ -580,13 +580,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="7">
@@ -604,13 +604,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>422</v>
+        <v>425</v>
       </c>
     </row>
     <row r="8">
@@ -628,13 +628,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>417</v>
+        <v>420</v>
       </c>
     </row>
     <row r="9">
@@ -643,70 +643,70 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>408</v>
+        <v>411</v>
       </c>
     </row>
     <row r="12">
@@ -715,22 +715,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>56</v>
+        <v>90</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>407</v>
+        <v>410</v>
       </c>
     </row>
     <row r="13">
@@ -739,22 +739,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>406</v>
+        <v>408</v>
       </c>
     </row>
     <row r="14">
@@ -763,22 +763,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>406</v>
+        <v>408</v>
       </c>
     </row>
     <row r="15">
@@ -787,46 +787,46 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="17">
@@ -844,13 +844,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="18">
@@ -868,13 +868,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="19">
@@ -883,22 +883,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="E19" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="20">
@@ -907,22 +907,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>47</v>
+        <v>69</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="F20" t="n">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="21">
@@ -931,22 +931,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="22">
@@ -955,22 +955,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="23">
@@ -979,22 +979,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="E23" t="n">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="24">
@@ -1003,22 +1003,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="25">
@@ -1027,22 +1027,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="F25" t="n">
-        <v>383</v>
+        <v>387</v>
       </c>
     </row>
     <row r="26">
@@ -1051,22 +1051,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="27">
@@ -1108,13 +1108,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>377</v>
+        <v>380</v>
       </c>
     </row>
     <row r="29">
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="30">
@@ -1156,13 +1156,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E30" t="n">
         <v>-8</v>
       </c>
       <c r="F30" t="n">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="31">
@@ -1750,177 +1750,177 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="C9" t="n">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D9" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E9" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F9" t="n">
-        <v>52</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="C10" t="n">
         <v>107</v>
       </c>
       <c r="D10" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E10" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="F10" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="C11" t="n">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="D11" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="E11" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F11" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="C12" t="n">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="D12" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E12" t="n">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="F12" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="C13" t="n">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="D13" t="n">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="E13" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F13" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="C14" t="n">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="D14" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E14" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F14" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>91</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="E16" t="n">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="F16" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17">
@@ -1970,127 +1970,127 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>43</v>
+        <v>72</v>
       </c>
       <c r="C19" t="n">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="D19" t="n">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="E19" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F19" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>72</v>
+        <v>43</v>
       </c>
       <c r="C20" t="n">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="D20" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="E20" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F20" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>41</v>
+        <v>62</v>
       </c>
       <c r="C21" t="n">
-        <v>78</v>
+        <v>111</v>
       </c>
       <c r="D21" t="n">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="E21" t="n">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="F21" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="C22" t="n">
-        <v>111</v>
+        <v>78</v>
       </c>
       <c r="D22" t="n">
-        <v>54</v>
+        <v>78</v>
       </c>
       <c r="E22" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="F22" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C23" t="n">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="D23" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E23" t="n">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="F23" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D24" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="E24" t="n">
         <v>77</v>
@@ -2102,45 +2102,45 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B25" t="n">
+        <v>53</v>
+      </c>
+      <c r="C25" t="n">
+        <v>102</v>
+      </c>
+      <c r="D25" t="n">
+        <v>46</v>
+      </c>
+      <c r="E25" t="n">
         <v>66</v>
       </c>
-      <c r="C25" t="n">
-        <v>111</v>
-      </c>
-      <c r="D25" t="n">
-        <v>61</v>
-      </c>
-      <c r="E25" t="n">
-        <v>62</v>
-      </c>
       <c r="F25" t="n">
-        <v>27</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="C26" t="n">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="D26" t="n">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="E26" t="n">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="F26" t="n">
-        <v>48</v>
+        <v>27</v>
       </c>
     </row>
     <row r="27">
@@ -2708,7 +2708,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2719,7 +2719,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2972,7 +2972,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2983,7 +2983,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2994,7 +2994,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -3005,7 +3005,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -3016,7 +3016,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -3027,7 +3027,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -3038,7 +3038,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -3060,7 +3060,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -3071,7 +3071,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -3082,7 +3082,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -3875,30 +3875,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E9" t="n">
-        <v>410102</v>
+        <v>6474</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>2088802</v>
+        <v>1177681</v>
       </c>
       <c r="H9" t="n">
-        <v>5360778</v>
+        <v>6474</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -3908,34 +3908,34 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E10" t="n">
-        <v>30971</v>
+        <v>410102</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>820221</v>
+        <v>2088802</v>
       </c>
       <c r="H10" t="n">
-        <v>58227</v>
+        <v>5360778</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -3945,34 +3945,34 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Yash Beohar</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Fluente in Football</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Satweek Nayak</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Xa bing chilling</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>14</v>
-      </c>
       <c r="E11" t="n">
-        <v>14603</v>
+        <v>30971</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2016/17</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>949628</v>
+        <v>820221</v>
       </c>
       <c r="H11" t="n">
-        <v>515830</v>
+        <v>58227</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -3986,30 +3986,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E12" t="n">
-        <v>6474</v>
+        <v>14603</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2016/17</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1177681</v>
+        <v>949628</v>
       </c>
       <c r="H12" t="n">
-        <v>6474</v>
+        <v>515830</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -4023,30 +4023,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E13" t="n">
-        <v>8917</v>
+        <v>182900</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>2118382</v>
+        <v>2098988</v>
       </c>
       <c r="H13" t="n">
-        <v>9146930</v>
+        <v>182900</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -4060,30 +4060,30 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E14" t="n">
-        <v>37120</v>
+        <v>8917</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>1571193</v>
+        <v>2118382</v>
       </c>
       <c r="H14" t="n">
-        <v>3349378</v>
+        <v>9146930</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>28582</v>
+        <v>37120</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>881388</v>
+        <v>1571193</v>
       </c>
       <c r="H15" t="n">
-        <v>239490</v>
+        <v>3349378</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4130,34 +4130,34 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E16" t="n">
-        <v>182900</v>
+        <v>28582</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>2098988</v>
+        <v>881388</v>
       </c>
       <c r="H16" t="n">
-        <v>182900</v>
+        <v>239490</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -4245,30 +4245,30 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E19" t="n">
-        <v>1128645</v>
+        <v>27153</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>3434302</v>
+        <v>606381</v>
       </c>
       <c r="H19" t="n">
-        <v>1128645</v>
+        <v>240451</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -4282,30 +4282,30 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E20" t="n">
-        <v>27153</v>
+        <v>1128645</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>606381</v>
+        <v>3434302</v>
       </c>
       <c r="H20" t="n">
-        <v>240451</v>
+        <v>1128645</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -4319,30 +4319,30 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E21" t="n">
-        <v>15288</v>
+        <v>31543</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>329510</v>
+        <v>820692</v>
       </c>
       <c r="H21" t="n">
-        <v>538046</v>
+        <v>1637750</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -4356,30 +4356,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E22" t="n">
-        <v>31543</v>
+        <v>15288</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>820692</v>
+        <v>329510</v>
       </c>
       <c r="H22" t="n">
-        <v>1637750</v>
+        <v>538046</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -4393,19 +4393,19 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E23" t="n">
-        <v>1320699</v>
+        <v>81907</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -4413,14 +4413,14 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2490743</v>
+        <v>3252487</v>
       </c>
       <c r="H23" t="n">
-        <v>1861933</v>
+        <v>11118394</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
     </row>
@@ -4430,19 +4430,19 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
-        <v>81907</v>
+        <v>334016</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -4450,10 +4450,10 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>3252487</v>
+        <v>2156629</v>
       </c>
       <c r="H24" t="n">
-        <v>11118394</v>
+        <v>2691725</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -4467,34 +4467,34 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E25" t="n">
-        <v>15136</v>
+        <v>1320699</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>983840</v>
+        <v>2490743</v>
       </c>
       <c r="H25" t="n">
-        <v>45077</v>
+        <v>1861933</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2024/25</t>
         </is>
       </c>
     </row>
@@ -4504,30 +4504,30 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E26" t="n">
-        <v>334016</v>
+        <v>15136</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>2156629</v>
+        <v>983840</v>
       </c>
       <c r="H26" t="n">
-        <v>2691725</v>
+        <v>45077</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -4871,7 +4871,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="D2" t="n">
         <v>79</v>
@@ -4942,7 +4942,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D3" t="n">
         <v>72.40000000000001</v>
@@ -5013,7 +5013,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="D4" t="n">
         <v>76.59999999999999</v>
@@ -5080,7 +5080,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="D5" t="n">
         <v>68.8</v>
@@ -5151,7 +5151,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="D6" t="n">
         <v>70.8</v>
@@ -5222,7 +5222,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="D7" t="n">
         <v>68.8</v>
@@ -5293,7 +5293,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="D8" t="n">
         <v>70.2</v>
@@ -5355,96 +5355,96 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="D9" t="n">
-        <v>66.40000000000001</v>
+        <v>70.2</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="G9" t="n">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="H9" t="n">
         <v>2</v>
       </c>
       <c r="I9" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="J9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K9" t="n">
+        <v>4</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>80</v>
+      </c>
+      <c r="O9" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Q9" t="n">
         <v>1</v>
       </c>
-      <c r="K9" t="n">
-        <v>2</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" t="n">
-        <v>59</v>
-      </c>
-      <c r="O9" t="n">
-        <v>101.3</v>
-      </c>
-      <c r="P9" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0.4</v>
-      </c>
       <c r="R9" t="n">
-        <v>952624</v>
+        <v>1095162</v>
       </c>
       <c r="S9" t="n">
-        <v>4185865</v>
+        <v>617418</v>
       </c>
       <c r="T9" t="n">
         <v>2</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard, bboost</t>
+          <t>bboost, 3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D10" t="n">
-        <v>68.59999999999999</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="E10" t="n">
         <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G10" t="n">
         <v>107</v>
@@ -5453,10 +5453,10 @@
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
@@ -5468,66 +5468,66 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="O10" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="P10" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="R10" t="n">
         <v>952624</v>
       </c>
       <c r="S10" t="n">
-        <v>1034411</v>
+        <v>4185865</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Xa bing chilling</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="D11" t="n">
-        <v>64</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="G11" t="n">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="H11" t="n">
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K11" t="n">
         <v>2</v>
@@ -5539,69 +5539,69 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="O11" t="n">
-        <v>102.4</v>
+        <v>101.4</v>
       </c>
       <c r="P11" t="n">
-        <v>2.4</v>
+        <v>1.4</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="R11" t="n">
-        <v>1037797</v>
+        <v>952624</v>
       </c>
       <c r="S11" t="n">
-        <v>2735246</v>
+        <v>1034411</v>
       </c>
       <c r="T11" t="n">
         <v>2</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>wildcard, bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Xa bing chilling</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="D12" t="n">
-        <v>70.2</v>
+        <v>64</v>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="G12" t="n">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="H12" t="n">
         <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="J12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -5610,69 +5610,69 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="O12" t="n">
-        <v>100.9</v>
+        <v>102.4</v>
       </c>
       <c r="P12" t="n">
-        <v>0.9</v>
+        <v>2.4</v>
       </c>
       <c r="Q12" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="R12" t="n">
-        <v>1095162</v>
+        <v>1037797</v>
       </c>
       <c r="S12" t="n">
-        <v>617418</v>
+        <v>2735246</v>
       </c>
       <c r="T12" t="n">
         <v>2</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>bboost, 3xc, wildcard</t>
+          <t>wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MaSalah</t>
+          <t>Carrick Janta Party</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="D13" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E13" t="n">
         <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="G13" t="n">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="H13" t="n">
         <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J13" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -5681,69 +5681,69 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="O13" t="n">
-        <v>101.9</v>
+        <v>101.6</v>
       </c>
       <c r="P13" t="n">
-        <v>1.9</v>
+        <v>1.6</v>
       </c>
       <c r="Q13" t="n">
-        <v>3.1</v>
+        <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>1131411</v>
+        <v>1220869</v>
       </c>
       <c r="S13" t="n">
-        <v>878473</v>
+        <v>3039834</v>
       </c>
       <c r="T13" t="n">
         <v>2</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>MaSalah</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="D14" t="n">
-        <v>67.40000000000001</v>
+        <v>68</v>
       </c>
       <c r="E14" t="n">
         <v>3</v>
       </c>
       <c r="F14" t="n">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="G14" t="n">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="H14" t="n">
         <v>2</v>
       </c>
       <c r="I14" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J14" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -5752,66 +5752,66 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>56</v>
+        <v>83</v>
       </c>
       <c r="O14" t="n">
-        <v>101.4</v>
+        <v>101.9</v>
       </c>
       <c r="P14" t="n">
-        <v>1.4</v>
+        <v>1.9</v>
       </c>
       <c r="Q14" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="R14" t="n">
-        <v>1140818</v>
+        <v>1131411</v>
       </c>
       <c r="S14" t="n">
-        <v>101935</v>
+        <v>878473</v>
       </c>
       <c r="T14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D15" t="n">
-        <v>69.59999999999999</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="E15" t="n">
         <v>3</v>
       </c>
       <c r="F15" t="n">
+        <v>66</v>
+      </c>
+      <c r="G15" t="n">
         <v>90</v>
       </c>
-      <c r="G15" t="n">
-        <v>104</v>
-      </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="J15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
         <v>4</v>
@@ -5826,66 +5826,66 @@
         <v>56</v>
       </c>
       <c r="O15" t="n">
-        <v>102.2</v>
+        <v>101.4</v>
       </c>
       <c r="P15" t="n">
-        <v>2.2</v>
+        <v>1.4</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.1</v>
+        <v>2.3</v>
       </c>
       <c r="R15" t="n">
-        <v>1187333</v>
+        <v>1140818</v>
       </c>
       <c r="S15" t="n">
-        <v>466127</v>
+        <v>101935</v>
       </c>
       <c r="T15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Carrick Janta Party</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="D16" t="n">
-        <v>69</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="E16" t="n">
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="G16" t="n">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="J16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="O16" t="n">
-        <v>101.6</v>
+        <v>102.2</v>
       </c>
       <c r="P16" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="R16" t="n">
-        <v>1220869</v>
+        <v>1187333</v>
       </c>
       <c r="S16" t="n">
-        <v>3039834</v>
+        <v>466127</v>
       </c>
       <c r="T16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
@@ -5932,7 +5932,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D17" t="n">
         <v>63.8</v>
@@ -6003,7 +6003,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="D18" t="n">
         <v>67.40000000000001</v>
@@ -6065,179 +6065,179 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cment_mixers</t>
+          <t>Totally Szobo</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D19" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F19" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G19" t="n">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="H19" t="n">
         <v>2</v>
       </c>
       <c r="I19" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="J19" t="n">
         <v>5</v>
       </c>
       <c r="K19" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="N19" t="n">
         <v>58</v>
       </c>
       <c r="O19" t="n">
-        <v>100.9</v>
+        <v>101.3</v>
       </c>
       <c r="P19" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="Q19" t="n">
-        <v>3.5</v>
+        <v>4.6</v>
       </c>
       <c r="R19" t="n">
-        <v>1797324</v>
+        <v>1885922</v>
       </c>
       <c r="S19" t="n">
-        <v>3048395</v>
+        <v>166751</v>
       </c>
       <c r="T19" t="n">
         <v>2</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>3xc, wildcard</t>
+          <t>bboost, 3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Totally Szobo</t>
+          <t>Cment_mixers</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="D20" t="n">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G20" t="n">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="H20" t="n">
         <v>2</v>
       </c>
       <c r="I20" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="J20" t="n">
         <v>5</v>
       </c>
       <c r="K20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M20" t="n">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="N20" t="n">
         <v>58</v>
       </c>
       <c r="O20" t="n">
-        <v>101.3</v>
+        <v>100.9</v>
       </c>
       <c r="P20" t="n">
-        <v>1.3</v>
+        <v>0.9</v>
       </c>
       <c r="Q20" t="n">
-        <v>4.6</v>
+        <v>3.5</v>
       </c>
       <c r="R20" t="n">
-        <v>1885922</v>
+        <v>1797324</v>
       </c>
       <c r="S20" t="n">
-        <v>166751</v>
+        <v>3048395</v>
       </c>
       <c r="T20" t="n">
         <v>2</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>bboost, 3xc, wildcard</t>
+          <t>3xc, wildcard</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D21" t="n">
-        <v>64.2</v>
+        <v>66.8</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="G21" t="n">
-        <v>78</v>
+        <v>111</v>
       </c>
       <c r="H21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I21" t="n">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K21" t="n">
         <v>4</v>
@@ -6249,25 +6249,25 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>56</v>
+        <v>82</v>
       </c>
       <c r="O21" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="P21" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="R21" t="n">
-        <v>1946361</v>
+        <v>2007432</v>
       </c>
       <c r="S21" t="n">
-        <v>3395267</v>
+        <v>1066412</v>
       </c>
       <c r="T21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
@@ -6278,37 +6278,37 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D22" t="n">
-        <v>66.8</v>
+        <v>64.2</v>
       </c>
       <c r="E22" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>117</v>
+        <v>93</v>
       </c>
       <c r="G22" t="n">
-        <v>111</v>
+        <v>78</v>
       </c>
       <c r="H22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I22" t="n">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="J22" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K22" t="n">
         <v>4</v>
@@ -6320,25 +6320,25 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="O22" t="n">
-        <v>101.3</v>
+        <v>101.4</v>
       </c>
       <c r="P22" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="R22" t="n">
-        <v>2007432</v>
+        <v>1946361</v>
       </c>
       <c r="S22" t="n">
-        <v>1066412</v>
+        <v>3395267</v>
       </c>
       <c r="T22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
@@ -6349,19 +6349,19 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D23" t="n">
-        <v>63.4</v>
+        <v>62.2</v>
       </c>
       <c r="E23" t="n">
         <v>2</v>
@@ -6370,46 +6370,46 @@
         <v>70</v>
       </c>
       <c r="G23" t="n">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="H23" t="n">
         <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J23" t="n">
         <v>3</v>
       </c>
       <c r="K23" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L23" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M23" t="n">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="N23" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="O23" t="n">
-        <v>101.3</v>
+        <v>101.9</v>
       </c>
       <c r="P23" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="R23" t="n">
-        <v>2231895</v>
+        <v>2308052</v>
       </c>
       <c r="S23" t="n">
-        <v>1948104</v>
+        <v>614528</v>
       </c>
       <c r="T23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U23" t="inlineStr">
         <is>
@@ -6420,40 +6420,40 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="D24" t="n">
-        <v>62.2</v>
+        <v>63.6</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="G24" t="n">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="H24" t="n">
         <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="J24" t="n">
         <v>3</v>
       </c>
       <c r="K24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
@@ -6462,25 +6462,25 @@
         <v>0</v>
       </c>
       <c r="N24" t="n">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="O24" t="n">
-        <v>101.9</v>
+        <v>101.7</v>
       </c>
       <c r="P24" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.7</v>
+        <v>1.2</v>
       </c>
       <c r="R24" t="n">
-        <v>2308052</v>
+        <v>2513181</v>
       </c>
       <c r="S24" t="n">
-        <v>614528</v>
+        <v>453361</v>
       </c>
       <c r="T24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U24" t="inlineStr">
         <is>
@@ -6491,111 +6491,111 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="D25" t="n">
-        <v>65.40000000000001</v>
+        <v>63.4</v>
       </c>
       <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="n">
+        <v>70</v>
+      </c>
+      <c r="G25" t="n">
+        <v>102</v>
+      </c>
+      <c r="H25" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" t="n">
+        <v>46</v>
+      </c>
+      <c r="J25" t="n">
         <v>3</v>
       </c>
-      <c r="F25" t="n">
-        <v>95</v>
-      </c>
-      <c r="G25" t="n">
-        <v>111</v>
-      </c>
-      <c r="H25" t="n">
-        <v>2</v>
-      </c>
-      <c r="I25" t="n">
-        <v>27</v>
-      </c>
-      <c r="J25" t="n">
-        <v>5</v>
-      </c>
       <c r="K25" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M25" t="n">
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="N25" t="n">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="O25" t="n">
-        <v>100.1</v>
+        <v>101.3</v>
       </c>
       <c r="P25" t="n">
-        <v>0.1</v>
+        <v>1.3</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="R25" t="n">
-        <v>2475208</v>
+        <v>2231895</v>
       </c>
       <c r="S25" t="n">
-        <v>637992</v>
+        <v>1948104</v>
       </c>
       <c r="T25" t="n">
         <v>2</v>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>bboost, 3xc</t>
+          <t>wildcard</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D26" t="n">
-        <v>63.6</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F26" t="n">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="G26" t="n">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="H26" t="n">
         <v>2</v>
       </c>
       <c r="I26" t="n">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="J26" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K26" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L26" t="n">
         <v>0</v>
@@ -6604,29 +6604,29 @@
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="O26" t="n">
-        <v>101.7</v>
+        <v>100.1</v>
       </c>
       <c r="P26" t="n">
-        <v>1.7</v>
+        <v>0.1</v>
       </c>
       <c r="Q26" t="n">
-        <v>1.2</v>
+        <v>0.3</v>
       </c>
       <c r="R26" t="n">
-        <v>2513181</v>
+        <v>2475208</v>
       </c>
       <c r="S26" t="n">
-        <v>453361</v>
+        <v>637992</v>
       </c>
       <c r="T26" t="n">
         <v>2</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>wildcard</t>
+          <t>bboost, 3xc</t>
         </is>
       </c>
     </row>
@@ -6713,7 +6713,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="D28" t="n">
         <v>64.40000000000001</v>
@@ -6784,7 +6784,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D29" t="n">
         <v>58.6</v>
@@ -6855,7 +6855,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D30" t="n">
         <v>56.8</v>

</xml_diff>

<commit_message>
Update standings 2026-10-13 01:50 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -484,13 +484,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="3">
@@ -499,43 +499,43 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>83</v>
+        <v>61</v>
       </c>
       <c r="E3" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F4" t="n">
         <v>444</v>
@@ -556,13 +556,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="6">
@@ -580,13 +580,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>430</v>
+        <v>431</v>
       </c>
     </row>
     <row r="7">
@@ -604,13 +604,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="8">
@@ -628,13 +628,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="9">
@@ -652,13 +652,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="10">
@@ -667,22 +667,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="11">
@@ -691,22 +691,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="12">
@@ -787,40 +787,40 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -844,13 +844,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="18">
@@ -931,22 +931,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="22">
@@ -955,22 +955,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="23">
@@ -988,13 +988,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="24">
@@ -1003,19 +1003,19 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="F24" t="n">
         <v>387</v>
@@ -1027,22 +1027,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="E25" t="n">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="26">
@@ -1108,13 +1108,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="29">
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="30">
@@ -1156,13 +1156,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E30" t="n">
         <v>-8</v>
       </c>
       <c r="F30" t="n">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="31">
@@ -1618,45 +1618,45 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C3" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D3" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="E3" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="F3" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C4" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D4" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="E4" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="F4" t="n">
-        <v>58</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5">
@@ -1772,45 +1772,45 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="C10" t="n">
         <v>107</v>
       </c>
       <c r="D10" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="E10" t="n">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="F10" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="C11" t="n">
         <v>107</v>
       </c>
       <c r="D11" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E11" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="F11" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12">
@@ -1882,45 +1882,45 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="E15" t="n">
-        <v>69</v>
+        <v>91</v>
       </c>
       <c r="F15" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="D16" t="n">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>91</v>
+        <v>69</v>
       </c>
       <c r="F16" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17">
@@ -2014,45 +2014,45 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="C21" t="n">
-        <v>111</v>
+        <v>78</v>
       </c>
       <c r="D21" t="n">
-        <v>54</v>
+        <v>78</v>
       </c>
       <c r="E21" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="F21" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>41</v>
+        <v>62</v>
       </c>
       <c r="C22" t="n">
-        <v>78</v>
+        <v>111</v>
       </c>
       <c r="D22" t="n">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="E22" t="n">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="F22" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23">
@@ -2080,45 +2080,45 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C24" t="n">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E24" t="n">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="F24" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C25" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D25" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E25" t="n">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="F25" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26">
@@ -2590,7 +2590,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2605,7 +2605,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -3027,7 +3027,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -3038,7 +3038,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -3060,7 +3060,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -3071,7 +3071,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -3653,30 +3653,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>281617</v>
+        <v>545267</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1051323</v>
+        <v>604934</v>
       </c>
       <c r="H3" t="n">
-        <v>1076546</v>
+        <v>545267</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -3686,34 +3686,34 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E4" t="n">
-        <v>545267</v>
+        <v>281617</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>604934</v>
+        <v>1051323</v>
       </c>
       <c r="H4" t="n">
-        <v>545267</v>
+        <v>1076546</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -3912,30 +3912,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E10" t="n">
-        <v>410102</v>
+        <v>30971</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2088802</v>
+        <v>820221</v>
       </c>
       <c r="H10" t="n">
-        <v>5360778</v>
+        <v>58227</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -3949,30 +3949,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E11" t="n">
-        <v>30971</v>
+        <v>410102</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>820221</v>
+        <v>2088802</v>
       </c>
       <c r="H11" t="n">
-        <v>58227</v>
+        <v>5360778</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -4097,30 +4097,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E15" t="n">
-        <v>37120</v>
+        <v>28582</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2014/15</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1571193</v>
+        <v>881388</v>
       </c>
       <c r="H15" t="n">
-        <v>3349378</v>
+        <v>239490</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -4130,34 +4130,34 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E16" t="n">
-        <v>28582</v>
+        <v>37120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2021/22</t>
+          <t>2014/15</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>881388</v>
+        <v>1571193</v>
       </c>
       <c r="H16" t="n">
-        <v>239490</v>
+        <v>3349378</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -4319,30 +4319,30 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E21" t="n">
-        <v>31543</v>
+        <v>15288</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2022/23</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>820692</v>
+        <v>329510</v>
       </c>
       <c r="H21" t="n">
-        <v>1637750</v>
+        <v>538046</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -4356,30 +4356,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E22" t="n">
-        <v>15288</v>
+        <v>31543</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2020/21</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>329510</v>
+        <v>820692</v>
       </c>
       <c r="H22" t="n">
-        <v>538046</v>
+        <v>1637750</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -4430,19 +4430,19 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E24" t="n">
-        <v>334016</v>
+        <v>1320699</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -4450,14 +4450,14 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>2156629</v>
+        <v>2490743</v>
       </c>
       <c r="H24" t="n">
-        <v>2691725</v>
+        <v>1861933</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2024/25</t>
         </is>
       </c>
     </row>
@@ -4467,19 +4467,19 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E25" t="n">
-        <v>1320699</v>
+        <v>334016</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -4487,14 +4487,14 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>2490743</v>
+        <v>2156629</v>
       </c>
       <c r="H25" t="n">
-        <v>1861933</v>
+        <v>2691725</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2024/25</t>
+          <t>2025/26</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D2" t="n">
         <v>79</v>
@@ -4904,7 +4904,7 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="O2" t="n">
         <v>102.3</v>
@@ -4916,7 +4916,7 @@
         <v>2.4</v>
       </c>
       <c r="R2" t="n">
-        <v>11041</v>
+        <v>7626</v>
       </c>
       <c r="S2" t="n">
         <v>270274</v>
@@ -4933,34 +4933,34 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="D3" t="n">
-        <v>72.40000000000001</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
         <v>84</v>
       </c>
       <c r="G3" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="H3" t="n">
         <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="J3" t="n">
         <v>3</v>
@@ -4969,69 +4969,65 @@
         <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="O3" t="n">
-        <v>102.2</v>
+        <v>101.1</v>
       </c>
       <c r="P3" t="n">
-        <v>2.2</v>
+        <v>1.1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="R3" t="n">
-        <v>138579</v>
+        <v>148000</v>
       </c>
       <c r="S3" t="n">
-        <v>1229264</v>
+        <v>1461471</v>
       </c>
       <c r="T3" t="n">
-        <v>4</v>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>bboost, wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>444</v>
       </c>
       <c r="D4" t="n">
-        <v>76.59999999999999</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
         <v>84</v>
       </c>
       <c r="G4" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="H4" t="n">
         <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="J4" t="n">
         <v>3</v>
@@ -5040,33 +5036,37 @@
         <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N4" t="n">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="O4" t="n">
-        <v>101.1</v>
+        <v>102.2</v>
       </c>
       <c r="P4" t="n">
-        <v>1.1</v>
+        <v>2.2</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="R4" t="n">
-        <v>160619</v>
+        <v>148000</v>
       </c>
       <c r="S4" t="n">
-        <v>1461471</v>
+        <v>1229264</v>
       </c>
       <c r="T4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U4" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>bboost, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5080,7 +5080,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="D5" t="n">
         <v>68.8</v>
@@ -5125,7 +5125,7 @@
         <v>3.5</v>
       </c>
       <c r="R5" t="n">
-        <v>346688</v>
+        <v>286883</v>
       </c>
       <c r="S5" t="n">
         <v>5250200</v>
@@ -5151,7 +5151,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="D6" t="n">
         <v>70.8</v>
@@ -5196,7 +5196,7 @@
         <v>1.3</v>
       </c>
       <c r="R6" t="n">
-        <v>360389</v>
+        <v>337246</v>
       </c>
       <c r="S6" t="n">
         <v>266328</v>
@@ -5222,7 +5222,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D7" t="n">
         <v>68.8</v>
@@ -5255,7 +5255,7 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="O7" t="n">
         <v>101.2</v>
@@ -5267,7 +5267,7 @@
         <v>0.3</v>
       </c>
       <c r="R7" t="n">
-        <v>537268</v>
+        <v>506363</v>
       </c>
       <c r="S7" t="n">
         <v>5881370</v>
@@ -5293,7 +5293,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D8" t="n">
         <v>70.2</v>
@@ -5338,7 +5338,7 @@
         <v>1.9</v>
       </c>
       <c r="R8" t="n">
-        <v>693079</v>
+        <v>656597</v>
       </c>
       <c r="S8" t="n">
         <v>3046343</v>
@@ -5364,7 +5364,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D9" t="n">
         <v>70.2</v>
@@ -5409,7 +5409,7 @@
         <v>1</v>
       </c>
       <c r="R9" t="n">
-        <v>1095162</v>
+        <v>880298</v>
       </c>
       <c r="S9" t="n">
         <v>617418</v>
@@ -5426,25 +5426,25 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D10" t="n">
-        <v>66.40000000000001</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="E10" t="n">
         <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G10" t="n">
         <v>107</v>
@@ -5453,10 +5453,10 @@
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
@@ -5468,54 +5468,54 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="O10" t="n">
-        <v>101.3</v>
+        <v>101.4</v>
       </c>
       <c r="P10" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="R10" t="n">
-        <v>952624</v>
+        <v>907720</v>
       </c>
       <c r="S10" t="n">
-        <v>4185865</v>
+        <v>1034411</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard, bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D11" t="n">
-        <v>68.59999999999999</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="E11" t="n">
         <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G11" t="n">
         <v>107</v>
@@ -5524,10 +5524,10 @@
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
         <v>2</v>
@@ -5539,29 +5539,29 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="O11" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="P11" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="R11" t="n">
-        <v>952624</v>
+        <v>907720</v>
       </c>
       <c r="S11" t="n">
-        <v>1034411</v>
+        <v>4185865</v>
       </c>
       <c r="T11" t="n">
         <v>2</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard, bboost</t>
         </is>
       </c>
     </row>
@@ -5622,7 +5622,7 @@
         <v>0.4</v>
       </c>
       <c r="R12" t="n">
-        <v>1037797</v>
+        <v>990550</v>
       </c>
       <c r="S12" t="n">
         <v>2735246</v>
@@ -5681,7 +5681,7 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="O13" t="n">
         <v>101.6</v>
@@ -5693,7 +5693,7 @@
         <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>1220869</v>
+        <v>1077473</v>
       </c>
       <c r="S13" t="n">
         <v>3039834</v>
@@ -5764,7 +5764,7 @@
         <v>3.1</v>
       </c>
       <c r="R14" t="n">
-        <v>1131411</v>
+        <v>1081831</v>
       </c>
       <c r="S14" t="n">
         <v>878473</v>
@@ -5781,37 +5781,37 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D15" t="n">
-        <v>67.40000000000001</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="E15" t="n">
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="G15" t="n">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="H15" t="n">
         <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K15" t="n">
         <v>4</v>
@@ -5826,63 +5826,63 @@
         <v>56</v>
       </c>
       <c r="O15" t="n">
-        <v>101.4</v>
+        <v>102.2</v>
       </c>
       <c r="P15" t="n">
-        <v>1.4</v>
+        <v>2.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>2.3</v>
+        <v>0.1</v>
       </c>
       <c r="R15" t="n">
-        <v>1140818</v>
+        <v>1136211</v>
       </c>
       <c r="S15" t="n">
-        <v>101935</v>
+        <v>466127</v>
       </c>
       <c r="T15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="C16" t="n">
         <v>406</v>
       </c>
       <c r="D16" t="n">
-        <v>69.59999999999999</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="E16" t="n">
         <v>3</v>
       </c>
       <c r="F16" t="n">
+        <v>66</v>
+      </c>
+      <c r="G16" t="n">
         <v>90</v>
       </c>
-      <c r="G16" t="n">
-        <v>104</v>
-      </c>
       <c r="H16" t="n">
         <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="J16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K16" t="n">
         <v>4</v>
@@ -5894,29 +5894,29 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="O16" t="n">
-        <v>102.2</v>
+        <v>101.4</v>
       </c>
       <c r="P16" t="n">
-        <v>2.2</v>
+        <v>1.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.1</v>
+        <v>2.3</v>
       </c>
       <c r="R16" t="n">
-        <v>1187333</v>
+        <v>1182656</v>
       </c>
       <c r="S16" t="n">
-        <v>466127</v>
+        <v>101935</v>
       </c>
       <c r="T16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>bboost</t>
         </is>
       </c>
     </row>
@@ -5932,7 +5932,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="D17" t="n">
         <v>63.8</v>
@@ -5977,7 +5977,7 @@
         <v>0.6</v>
       </c>
       <c r="R17" t="n">
-        <v>1533467</v>
+        <v>1582314</v>
       </c>
       <c r="S17" t="n">
         <v>2489160</v>
@@ -6048,7 +6048,7 @@
         <v>1.3</v>
       </c>
       <c r="R18" t="n">
-        <v>1694595</v>
+        <v>1632614</v>
       </c>
       <c r="S18" t="n">
         <v>3009015</v>
@@ -6119,7 +6119,7 @@
         <v>4.6</v>
       </c>
       <c r="R19" t="n">
-        <v>1885922</v>
+        <v>1704855</v>
       </c>
       <c r="S19" t="n">
         <v>166751</v>
@@ -6178,7 +6178,7 @@
         <v>-8</v>
       </c>
       <c r="N20" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="O20" t="n">
         <v>100.9</v>
@@ -6190,7 +6190,7 @@
         <v>3.5</v>
       </c>
       <c r="R20" t="n">
-        <v>1797324</v>
+        <v>1850007</v>
       </c>
       <c r="S20" t="n">
         <v>3048395</v>
@@ -6207,37 +6207,37 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D21" t="n">
-        <v>66.8</v>
+        <v>64.2</v>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>117</v>
+        <v>93</v>
       </c>
       <c r="G21" t="n">
-        <v>111</v>
+        <v>78</v>
       </c>
       <c r="H21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I21" t="n">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="J21" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K21" t="n">
         <v>4</v>
@@ -6249,25 +6249,25 @@
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="O21" t="n">
-        <v>101.3</v>
+        <v>101.4</v>
       </c>
       <c r="P21" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="R21" t="n">
-        <v>2007432</v>
+        <v>2000463</v>
       </c>
       <c r="S21" t="n">
-        <v>1066412</v>
+        <v>3395267</v>
       </c>
       <c r="T21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
@@ -6278,37 +6278,37 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="D22" t="n">
-        <v>64.2</v>
+        <v>66.8</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="G22" t="n">
-        <v>78</v>
+        <v>111</v>
       </c>
       <c r="H22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I22" t="n">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K22" t="n">
         <v>4</v>
@@ -6320,25 +6320,25 @@
         <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>56</v>
+        <v>82</v>
       </c>
       <c r="O22" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="P22" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="R22" t="n">
-        <v>1946361</v>
+        <v>2062527</v>
       </c>
       <c r="S22" t="n">
-        <v>3395267</v>
+        <v>1066412</v>
       </c>
       <c r="T22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
@@ -6358,7 +6358,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D23" t="n">
         <v>62.2</v>
@@ -6403,7 +6403,7 @@
         <v>0.7</v>
       </c>
       <c r="R23" t="n">
-        <v>2308052</v>
+        <v>2108351</v>
       </c>
       <c r="S23" t="n">
         <v>614528</v>
@@ -6420,64 +6420,64 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mishra's 13</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="C24" t="n">
         <v>387</v>
       </c>
       <c r="D24" t="n">
-        <v>63.6</v>
+        <v>63.4</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="G24" t="n">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="H24" t="n">
         <v>2</v>
       </c>
       <c r="I24" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="J24" t="n">
         <v>3</v>
       </c>
       <c r="K24" t="n">
+        <v>7</v>
+      </c>
+      <c r="L24" t="n">
         <v>3</v>
       </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
       <c r="M24" t="n">
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="N24" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="O24" t="n">
-        <v>101.7</v>
+        <v>101.3</v>
       </c>
       <c r="P24" t="n">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
       <c r="Q24" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="R24" t="n">
-        <v>2513181</v>
+        <v>2289346</v>
       </c>
       <c r="S24" t="n">
-        <v>453361</v>
+        <v>1948104</v>
       </c>
       <c r="T24" t="n">
         <v>2</v>
@@ -6491,64 +6491,64 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>Mishra's 13</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D25" t="n">
-        <v>63.4</v>
+        <v>63.6</v>
       </c>
       <c r="E25" t="n">
         <v>2</v>
       </c>
       <c r="F25" t="n">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="G25" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="H25" t="n">
         <v>2</v>
       </c>
       <c r="I25" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="J25" t="n">
         <v>3</v>
       </c>
       <c r="K25" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L25" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="N25" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="O25" t="n">
-        <v>101.3</v>
+        <v>101.7</v>
       </c>
       <c r="P25" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="R25" t="n">
-        <v>2231895</v>
+        <v>2306156</v>
       </c>
       <c r="S25" t="n">
-        <v>1948104</v>
+        <v>453361</v>
       </c>
       <c r="T25" t="n">
         <v>2</v>
@@ -6616,7 +6616,7 @@
         <v>0.3</v>
       </c>
       <c r="R26" t="n">
-        <v>2475208</v>
+        <v>2534452</v>
       </c>
       <c r="S26" t="n">
         <v>637992</v>
@@ -6675,7 +6675,7 @@
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="O27" t="n">
         <v>100.6</v>
@@ -6687,7 +6687,7 @@
         <v>2.5</v>
       </c>
       <c r="R27" t="n">
-        <v>2524915</v>
+        <v>2584534</v>
       </c>
       <c r="S27" t="n">
         <v>1595922</v>
@@ -6713,7 +6713,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="D28" t="n">
         <v>64.40000000000001</v>
@@ -6758,7 +6758,7 @@
         <v>1.7</v>
       </c>
       <c r="R28" t="n">
-        <v>2871388</v>
+        <v>2791889</v>
       </c>
       <c r="S28" t="n">
         <v>4399137</v>
@@ -6784,7 +6784,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D29" t="n">
         <v>58.6</v>
@@ -6817,7 +6817,7 @@
         <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="O29" t="n">
         <v>101.1</v>
@@ -6829,7 +6829,7 @@
         <v>2.3</v>
       </c>
       <c r="R29" t="n">
-        <v>3013315</v>
+        <v>2932938</v>
       </c>
       <c r="S29" t="n">
         <v>3963132</v>
@@ -6855,7 +6855,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D30" t="n">
         <v>56.8</v>
@@ -6888,7 +6888,7 @@
         <v>-8</v>
       </c>
       <c r="N30" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="O30" t="n">
         <v>101.6</v>
@@ -6900,7 +6900,7 @@
         <v>1</v>
       </c>
       <c r="R30" t="n">
-        <v>5407173</v>
+        <v>5320703</v>
       </c>
       <c r="S30" t="n">
         <v>1952243</v>
@@ -6971,7 +6971,7 @@
         <v>1.2</v>
       </c>
       <c r="R31" t="n">
-        <v>5751989</v>
+        <v>5807661</v>
       </c>
       <c r="S31" t="n">
         <v>553038</v>
@@ -7042,7 +7042,7 @@
         <v>2.2</v>
       </c>
       <c r="R32" t="n">
-        <v>8713733</v>
+        <v>8737279</v>
       </c>
       <c r="S32" t="n">
         <v>216389</v>

</xml_diff>

<commit_message>
Update standings 2026-10-13 09:01 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -499,19 +499,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F3" t="n">
         <v>444</v>
@@ -523,19 +523,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="E4" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>444</v>
@@ -1618,45 +1618,45 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C3" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D3" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="E3" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="F3" t="n">
-        <v>58</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C4" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="E4" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="F4" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5">
@@ -2590,7 +2590,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2605,7 +2605,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -3653,30 +3653,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>545267</v>
+        <v>281617</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>604934</v>
+        <v>1051323</v>
       </c>
       <c r="H3" t="n">
-        <v>545267</v>
+        <v>1076546</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -3690,30 +3690,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>281617</v>
+        <v>545267</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1051323</v>
+        <v>604934</v>
       </c>
       <c r="H4" t="n">
-        <v>1076546</v>
+        <v>545267</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -4933,34 +4933,34 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>444</v>
       </c>
       <c r="D3" t="n">
-        <v>76.59999999999999</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
         <v>84</v>
       </c>
       <c r="G3" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="H3" t="n">
         <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="J3" t="n">
         <v>3</v>
@@ -4969,65 +4969,69 @@
         <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N3" t="n">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="O3" t="n">
-        <v>101.1</v>
+        <v>102.2</v>
       </c>
       <c r="P3" t="n">
-        <v>1.1</v>
+        <v>2.2</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="R3" t="n">
         <v>148000</v>
       </c>
       <c r="S3" t="n">
-        <v>1461471</v>
+        <v>1229264</v>
       </c>
       <c r="T3" t="n">
-        <v>2</v>
-      </c>
-      <c r="U3" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>bboost, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>444</v>
       </c>
       <c r="D4" t="n">
-        <v>72.40000000000001</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
         <v>84</v>
       </c>
       <c r="G4" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="H4" t="n">
         <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="J4" t="n">
         <v>3</v>
@@ -5036,37 +5040,33 @@
         <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="O4" t="n">
-        <v>102.2</v>
+        <v>101.1</v>
       </c>
       <c r="P4" t="n">
-        <v>2.2</v>
+        <v>1.1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="R4" t="n">
         <v>148000</v>
       </c>
       <c r="S4" t="n">
-        <v>1229264</v>
+        <v>1461471</v>
       </c>
       <c r="T4" t="n">
-        <v>4</v>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>bboost, wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-10-13 17:23 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -1060,13 +1060,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="27">
@@ -1180,13 +1180,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E31" t="n">
         <v>-4</v>
       </c>
       <c r="F31" t="n">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="32">
@@ -1204,13 +1204,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
   </sheetData>
@@ -1558,7 +1558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1592,6 +1592,11 @@
           <t>GW5</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>GW6</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1614,6 +1619,9 @@
       <c r="F2" t="n">
         <v>51</v>
       </c>
+      <c r="G2" t="n">
+        <v>79</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1636,6 +1644,9 @@
       <c r="F3" t="n">
         <v>47</v>
       </c>
+      <c r="G3" t="n">
+        <v>82</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1658,6 +1669,9 @@
       <c r="F4" t="n">
         <v>58</v>
       </c>
+      <c r="G4" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1680,6 +1694,9 @@
       <c r="F5" t="n">
         <v>61</v>
       </c>
+      <c r="G5" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1702,6 +1719,9 @@
       <c r="F6" t="n">
         <v>40</v>
       </c>
+      <c r="G6" t="n">
+        <v>77</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1724,6 +1744,9 @@
       <c r="F7" t="n">
         <v>60</v>
       </c>
+      <c r="G7" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1746,6 +1769,9 @@
       <c r="F8" t="n">
         <v>64</v>
       </c>
+      <c r="G8" t="n">
+        <v>68</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1768,6 +1794,9 @@
       <c r="F9" t="n">
         <v>46</v>
       </c>
+      <c r="G9" t="n">
+        <v>62</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1790,6 +1819,9 @@
       <c r="F10" t="n">
         <v>44</v>
       </c>
+      <c r="G10" t="n">
+        <v>69</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1812,6 +1844,9 @@
       <c r="F11" t="n">
         <v>52</v>
       </c>
+      <c r="G11" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1834,6 +1869,9 @@
       <c r="F12" t="n">
         <v>45</v>
       </c>
+      <c r="G12" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1856,6 +1894,9 @@
       <c r="F13" t="n">
         <v>48</v>
       </c>
+      <c r="G13" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1878,6 +1919,9 @@
       <c r="F14" t="n">
         <v>51</v>
       </c>
+      <c r="G14" t="n">
+        <v>68</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1900,6 +1944,9 @@
       <c r="F15" t="n">
         <v>43</v>
       </c>
+      <c r="G15" t="n">
+        <v>59</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1922,6 +1969,9 @@
       <c r="F16" t="n">
         <v>50</v>
       </c>
+      <c r="G16" t="n">
+        <v>69</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1944,6 +1994,9 @@
       <c r="F17" t="n">
         <v>49</v>
       </c>
+      <c r="G17" t="n">
+        <v>79</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1966,6 +2019,9 @@
       <c r="F18" t="n">
         <v>51</v>
       </c>
+      <c r="G18" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1988,6 +2044,9 @@
       <c r="F19" t="n">
         <v>32</v>
       </c>
+      <c r="G19" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2010,6 +2069,9 @@
       <c r="F20" t="n">
         <v>38</v>
       </c>
+      <c r="G20" t="n">
+        <v>69</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2032,6 +2094,9 @@
       <c r="F21" t="n">
         <v>55</v>
       </c>
+      <c r="G21" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2054,6 +2119,9 @@
       <c r="F22" t="n">
         <v>49</v>
       </c>
+      <c r="G22" t="n">
+        <v>56</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2076,6 +2144,9 @@
       <c r="F23" t="n">
         <v>48</v>
       </c>
+      <c r="G23" t="n">
+        <v>78</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2098,6 +2169,9 @@
       <c r="F24" t="n">
         <v>50</v>
       </c>
+      <c r="G24" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2120,6 +2194,9 @@
       <c r="F25" t="n">
         <v>48</v>
       </c>
+      <c r="G25" t="n">
+        <v>68</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2142,6 +2219,9 @@
       <c r="F26" t="n">
         <v>27</v>
       </c>
+      <c r="G26" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2164,6 +2244,9 @@
       <c r="F27" t="n">
         <v>45</v>
       </c>
+      <c r="G27" t="n">
+        <v>68</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2186,6 +2269,9 @@
       <c r="F28" t="n">
         <v>29</v>
       </c>
+      <c r="G28" t="n">
+        <v>57</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2208,6 +2294,9 @@
       <c r="F29" t="n">
         <v>46</v>
       </c>
+      <c r="G29" t="n">
+        <v>84</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2230,6 +2319,9 @@
       <c r="F30" t="n">
         <v>52</v>
       </c>
+      <c r="G30" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2252,6 +2344,9 @@
       <c r="F31" t="n">
         <v>46</v>
       </c>
+      <c r="G31" t="n">
+        <v>67</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2273,6 +2368,9 @@
       </c>
       <c r="F32" t="n">
         <v>46</v>
+      </c>
+      <c r="G32" t="n">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -2421,7 +2519,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C2" t="inlineStr"/>
     </row>
@@ -2432,346 +2530,346 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Abhay Rawat</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>93</v>
-      </c>
-      <c r="C7" t="inlineStr"/>
+        <v>106</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Abhay Rawat</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>90</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>105</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>90</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>102</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>90</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
+        <v>96</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>90</v>
-      </c>
-      <c r="C16" t="inlineStr"/>
+        <v>94</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>84</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>84</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>81</v>
-      </c>
-      <c r="C20" t="inlineStr"/>
+        <v>88</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="C21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>79</v>
-      </c>
-      <c r="C22" t="inlineStr"/>
+        <v>87</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Ashwin Jose</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="C23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="C24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="C25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Ashwin Jose</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="C26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="C27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="C28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Pranav Thomas</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>69</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="C29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="C30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="C31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Pranav Thomas</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C32" t="inlineStr"/>
     </row>
@@ -2828,7 +2926,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3" t="inlineStr"/>
     </row>
@@ -2839,7 +2937,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" t="inlineStr"/>
     </row>
@@ -2850,62 +2948,66 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Karan Khanna</t>
+          <t>Deepankar Sachdeva</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Deepankar Sachdeva</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Abhay Rawat</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>3</v>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Abhay Rawat</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -2916,11 +3018,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Aayush Khanna</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -2931,11 +3033,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Aayush Khanna</t>
+          <t>Aquib Razack</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -2946,121 +3048,117 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Aquib Razack</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sid Shaurya</t>
+          <t>Satweek Nayak</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Raveesh Kalra</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Satweek Nayak</t>
+          <t>Karan Khanna</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Pranshul Jain</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Raveesh Kalra</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>prateek gupta</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Abhinav Premsekhar</t>
+          <t>Pranav Thomas</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Sid Shaurya</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -3071,7 +3169,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -3082,7 +3180,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Pranshul Jain</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -3093,7 +3191,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -3104,7 +3202,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>prateek gupta</t>
+          <t>Abhinav Premsekhar</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -3115,7 +3213,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Pranav Thomas</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -3126,29 +3224,29 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Parakh Tripathy</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -3159,7 +3257,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Parakh Tripathy</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -4877,10 +4975,10 @@
         <v>79</v>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F2" t="n">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="G2" t="n">
         <v>126</v>
@@ -4916,7 +5014,7 @@
         <v>2.4</v>
       </c>
       <c r="R2" t="n">
-        <v>7626</v>
+        <v>8570</v>
       </c>
       <c r="S2" t="n">
         <v>270274</v>
@@ -4945,13 +5043,13 @@
         <v>444</v>
       </c>
       <c r="D3" t="n">
-        <v>72.40000000000001</v>
+        <v>74</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="G3" t="n">
         <v>107</v>
@@ -4987,7 +5085,7 @@
         <v>0.7</v>
       </c>
       <c r="R3" t="n">
-        <v>148000</v>
+        <v>161939</v>
       </c>
       <c r="S3" t="n">
         <v>1229264</v>
@@ -5016,13 +5114,13 @@
         <v>444</v>
       </c>
       <c r="D4" t="n">
-        <v>76.59999999999999</v>
+        <v>74</v>
       </c>
       <c r="E4" t="n">
         <v>5</v>
       </c>
       <c r="F4" t="n">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="G4" t="n">
         <v>116</v>
@@ -5058,7 +5156,7 @@
         <v>0.3</v>
       </c>
       <c r="R4" t="n">
-        <v>148000</v>
+        <v>161939</v>
       </c>
       <c r="S4" t="n">
         <v>1461471</v>
@@ -5083,13 +5181,13 @@
         <v>434</v>
       </c>
       <c r="D5" t="n">
-        <v>68.8</v>
+        <v>72.3</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="G5" t="n">
         <v>114</v>
@@ -5125,7 +5223,7 @@
         <v>3.5</v>
       </c>
       <c r="R5" t="n">
-        <v>286883</v>
+        <v>311734</v>
       </c>
       <c r="S5" t="n">
         <v>5250200</v>
@@ -5154,13 +5252,13 @@
         <v>431</v>
       </c>
       <c r="D6" t="n">
-        <v>70.8</v>
+        <v>71.8</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="G6" t="n">
         <v>103</v>
@@ -5196,7 +5294,7 @@
         <v>1.3</v>
       </c>
       <c r="R6" t="n">
-        <v>337246</v>
+        <v>366004</v>
       </c>
       <c r="S6" t="n">
         <v>266328</v>
@@ -5225,13 +5323,13 @@
         <v>424</v>
       </c>
       <c r="D7" t="n">
-        <v>68.8</v>
+        <v>70.7</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F7" t="n">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="G7" t="n">
         <v>118</v>
@@ -5267,7 +5365,7 @@
         <v>0.3</v>
       </c>
       <c r="R7" t="n">
-        <v>506363</v>
+        <v>547376</v>
       </c>
       <c r="S7" t="n">
         <v>5881370</v>
@@ -5296,13 +5394,13 @@
         <v>419</v>
       </c>
       <c r="D8" t="n">
-        <v>70.2</v>
+        <v>69.8</v>
       </c>
       <c r="E8" t="n">
         <v>2</v>
       </c>
       <c r="F8" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="G8" t="n">
         <v>113</v>
@@ -5338,7 +5436,7 @@
         <v>1.9</v>
       </c>
       <c r="R8" t="n">
-        <v>656597</v>
+        <v>708275</v>
       </c>
       <c r="S8" t="n">
         <v>3046343</v>
@@ -5367,13 +5465,13 @@
         <v>413</v>
       </c>
       <c r="D9" t="n">
-        <v>70.2</v>
+        <v>68.8</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="G9" t="n">
         <v>105</v>
@@ -5409,7 +5507,7 @@
         <v>1</v>
       </c>
       <c r="R9" t="n">
-        <v>880298</v>
+        <v>946821</v>
       </c>
       <c r="S9" t="n">
         <v>617418</v>
@@ -5438,13 +5536,13 @@
         <v>412</v>
       </c>
       <c r="D10" t="n">
-        <v>68.59999999999999</v>
+        <v>68.7</v>
       </c>
       <c r="E10" t="n">
         <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="G10" t="n">
         <v>107</v>
@@ -5480,7 +5578,7 @@
         <v>0.2</v>
       </c>
       <c r="R10" t="n">
-        <v>907720</v>
+        <v>976197</v>
       </c>
       <c r="S10" t="n">
         <v>1034411</v>
@@ -5509,13 +5607,13 @@
         <v>412</v>
       </c>
       <c r="D11" t="n">
-        <v>66.40000000000001</v>
+        <v>68.7</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="G11" t="n">
         <v>107</v>
@@ -5551,7 +5649,7 @@
         <v>0.4</v>
       </c>
       <c r="R11" t="n">
-        <v>907720</v>
+        <v>976197</v>
       </c>
       <c r="S11" t="n">
         <v>4185865</v>
@@ -5580,13 +5678,13 @@
         <v>410</v>
       </c>
       <c r="D12" t="n">
-        <v>64</v>
+        <v>68.3</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G12" t="n">
         <v>93</v>
@@ -5622,7 +5720,7 @@
         <v>0.4</v>
       </c>
       <c r="R12" t="n">
-        <v>990550</v>
+        <v>1064362</v>
       </c>
       <c r="S12" t="n">
         <v>2735246</v>
@@ -5651,13 +5749,13 @@
         <v>408</v>
       </c>
       <c r="D13" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E13" t="n">
         <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="G13" t="n">
         <v>118</v>
@@ -5693,7 +5791,7 @@
         <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>1077473</v>
+        <v>1156782</v>
       </c>
       <c r="S13" t="n">
         <v>3039834</v>
@@ -5728,7 +5826,7 @@
         <v>3</v>
       </c>
       <c r="F14" t="n">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="G14" t="n">
         <v>109</v>
@@ -5764,7 +5862,7 @@
         <v>3.1</v>
       </c>
       <c r="R14" t="n">
-        <v>1081831</v>
+        <v>1161332</v>
       </c>
       <c r="S14" t="n">
         <v>878473</v>
@@ -5793,13 +5891,13 @@
         <v>407</v>
       </c>
       <c r="D15" t="n">
-        <v>69.59999999999999</v>
+        <v>67.8</v>
       </c>
       <c r="E15" t="n">
         <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="G15" t="n">
         <v>104</v>
@@ -5835,7 +5933,7 @@
         <v>0.1</v>
       </c>
       <c r="R15" t="n">
-        <v>1136211</v>
+        <v>1219150</v>
       </c>
       <c r="S15" t="n">
         <v>466127</v>
@@ -5864,13 +5962,13 @@
         <v>406</v>
       </c>
       <c r="D16" t="n">
-        <v>67.40000000000001</v>
+        <v>67.7</v>
       </c>
       <c r="E16" t="n">
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G16" t="n">
         <v>90</v>
@@ -5906,13 +6004,13 @@
         <v>2.3</v>
       </c>
       <c r="R16" t="n">
-        <v>1182656</v>
+        <v>1268749</v>
       </c>
       <c r="S16" t="n">
-        <v>101935</v>
+        <v>128137</v>
       </c>
       <c r="T16" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
@@ -5935,13 +6033,13 @@
         <v>398</v>
       </c>
       <c r="D17" t="n">
-        <v>63.8</v>
+        <v>66.3</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="G17" t="n">
         <v>93</v>
@@ -5977,7 +6075,7 @@
         <v>0.6</v>
       </c>
       <c r="R17" t="n">
-        <v>1582314</v>
+        <v>1690121</v>
       </c>
       <c r="S17" t="n">
         <v>2489160</v>
@@ -6006,13 +6104,13 @@
         <v>397</v>
       </c>
       <c r="D18" t="n">
-        <v>67.40000000000001</v>
+        <v>66.2</v>
       </c>
       <c r="E18" t="n">
         <v>3</v>
       </c>
       <c r="F18" t="n">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="G18" t="n">
         <v>101</v>
@@ -6048,7 +6146,7 @@
         <v>1.3</v>
       </c>
       <c r="R18" t="n">
-        <v>1632614</v>
+        <v>1743174</v>
       </c>
       <c r="S18" t="n">
         <v>3009015</v>
@@ -6077,13 +6175,13 @@
         <v>396</v>
       </c>
       <c r="D19" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E19" t="n">
         <v>4</v>
       </c>
       <c r="F19" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="G19" t="n">
         <v>106</v>
@@ -6119,7 +6217,7 @@
         <v>4.6</v>
       </c>
       <c r="R19" t="n">
-        <v>1704855</v>
+        <v>1819175</v>
       </c>
       <c r="S19" t="n">
         <v>166751</v>
@@ -6148,13 +6246,13 @@
         <v>394</v>
       </c>
       <c r="D20" t="n">
-        <v>65</v>
+        <v>65.7</v>
       </c>
       <c r="E20" t="n">
         <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="G20" t="n">
         <v>97</v>
@@ -6190,7 +6288,7 @@
         <v>3.5</v>
       </c>
       <c r="R20" t="n">
-        <v>1850007</v>
+        <v>1971616</v>
       </c>
       <c r="S20" t="n">
         <v>3048395</v>
@@ -6219,13 +6317,13 @@
         <v>391</v>
       </c>
       <c r="D21" t="n">
-        <v>64.2</v>
+        <v>65.2</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F21" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="G21" t="n">
         <v>78</v>
@@ -6261,7 +6359,7 @@
         <v>0.5</v>
       </c>
       <c r="R21" t="n">
-        <v>2000463</v>
+        <v>2130542</v>
       </c>
       <c r="S21" t="n">
         <v>3395267</v>
@@ -6290,13 +6388,13 @@
         <v>390</v>
       </c>
       <c r="D22" t="n">
-        <v>66.8</v>
+        <v>65</v>
       </c>
       <c r="E22" t="n">
         <v>4</v>
       </c>
       <c r="F22" t="n">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="G22" t="n">
         <v>111</v>
@@ -6332,7 +6430,7 @@
         <v>0.1</v>
       </c>
       <c r="R22" t="n">
-        <v>2062527</v>
+        <v>2195350</v>
       </c>
       <c r="S22" t="n">
         <v>1066412</v>
@@ -6361,13 +6459,13 @@
         <v>389</v>
       </c>
       <c r="D23" t="n">
-        <v>62.2</v>
+        <v>64.8</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F23" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="G23" t="n">
         <v>80</v>
@@ -6403,13 +6501,13 @@
         <v>0.7</v>
       </c>
       <c r="R23" t="n">
-        <v>2108351</v>
+        <v>2243697</v>
       </c>
       <c r="S23" t="n">
-        <v>614528</v>
+        <v>1196618</v>
       </c>
       <c r="T23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U23" t="inlineStr">
         <is>
@@ -6432,13 +6530,13 @@
         <v>387</v>
       </c>
       <c r="D24" t="n">
-        <v>63.4</v>
+        <v>64.5</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F24" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G24" t="n">
         <v>102</v>
@@ -6474,7 +6572,7 @@
         <v>0.6</v>
       </c>
       <c r="R24" t="n">
-        <v>2289346</v>
+        <v>2432981</v>
       </c>
       <c r="S24" t="n">
         <v>1948104</v>
@@ -6503,13 +6601,13 @@
         <v>386</v>
       </c>
       <c r="D25" t="n">
-        <v>63.6</v>
+        <v>64.3</v>
       </c>
       <c r="E25" t="n">
         <v>2</v>
       </c>
       <c r="F25" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="G25" t="n">
         <v>96</v>
@@ -6545,7 +6643,7 @@
         <v>1.2</v>
       </c>
       <c r="R25" t="n">
-        <v>2306156</v>
+        <v>2451033</v>
       </c>
       <c r="S25" t="n">
         <v>453361</v>
@@ -6571,16 +6669,16 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="D26" t="n">
-        <v>65.40000000000001</v>
+        <v>64.2</v>
       </c>
       <c r="E26" t="n">
         <v>3</v>
       </c>
       <c r="F26" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G26" t="n">
         <v>111</v>
@@ -6604,7 +6702,7 @@
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="O26" t="n">
         <v>100.1</v>
@@ -6616,7 +6714,7 @@
         <v>0.3</v>
       </c>
       <c r="R26" t="n">
-        <v>2534452</v>
+        <v>2549625</v>
       </c>
       <c r="S26" t="n">
         <v>637992</v>
@@ -6645,13 +6743,13 @@
         <v>382</v>
       </c>
       <c r="D27" t="n">
-        <v>62.8</v>
+        <v>63.7</v>
       </c>
       <c r="E27" t="n">
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G27" t="n">
         <v>89</v>
@@ -6687,7 +6785,7 @@
         <v>2.5</v>
       </c>
       <c r="R27" t="n">
-        <v>2584534</v>
+        <v>2741982</v>
       </c>
       <c r="S27" t="n">
         <v>1595922</v>
@@ -6716,13 +6814,13 @@
         <v>379</v>
       </c>
       <c r="D28" t="n">
-        <v>64.40000000000001</v>
+        <v>63.2</v>
       </c>
       <c r="E28" t="n">
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="G28" t="n">
         <v>120</v>
@@ -6758,7 +6856,7 @@
         <v>1.7</v>
       </c>
       <c r="R28" t="n">
-        <v>2791889</v>
+        <v>2958093</v>
       </c>
       <c r="S28" t="n">
         <v>4399137</v>
@@ -6787,13 +6885,13 @@
         <v>377</v>
       </c>
       <c r="D29" t="n">
-        <v>58.6</v>
+        <v>62.8</v>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F29" t="n">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="G29" t="n">
         <v>101</v>
@@ -6829,7 +6927,7 @@
         <v>2.3</v>
       </c>
       <c r="R29" t="n">
-        <v>2932938</v>
+        <v>3104076</v>
       </c>
       <c r="S29" t="n">
         <v>3963132</v>
@@ -6858,13 +6956,13 @@
         <v>345</v>
       </c>
       <c r="D30" t="n">
-        <v>56.8</v>
+        <v>57.5</v>
       </c>
       <c r="E30" t="n">
         <v>2</v>
       </c>
       <c r="F30" t="n">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="G30" t="n">
         <v>89</v>
@@ -6900,7 +6998,7 @@
         <v>1</v>
       </c>
       <c r="R30" t="n">
-        <v>5320703</v>
+        <v>5544586</v>
       </c>
       <c r="S30" t="n">
         <v>1952243</v>
@@ -6926,16 +7024,16 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="D31" t="n">
-        <v>54.6</v>
+        <v>56.7</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="G31" t="n">
         <v>73</v>
@@ -6959,7 +7057,7 @@
         <v>-4</v>
       </c>
       <c r="N31" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="O31" t="n">
         <v>101.2</v>
@@ -6971,13 +7069,13 @@
         <v>1.2</v>
       </c>
       <c r="R31" t="n">
-        <v>5807661</v>
+        <v>5892305</v>
       </c>
       <c r="S31" t="n">
-        <v>553038</v>
+        <v>912089</v>
       </c>
       <c r="T31" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U31" t="inlineStr">
         <is>
@@ -6997,16 +7095,16 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D32" t="n">
-        <v>46.6</v>
+        <v>47.2</v>
       </c>
       <c r="E32" t="n">
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="G32" t="n">
         <v>55</v>
@@ -7030,7 +7128,7 @@
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="O32" t="n">
         <v>98.7</v>
@@ -7042,7 +7140,7 @@
         <v>2.2</v>
       </c>
       <c r="R32" t="n">
-        <v>8737279</v>
+        <v>8841683</v>
       </c>
       <c r="S32" t="n">
         <v>216389</v>

</xml_diff>

<commit_message>
Update standings 2026-10-13 22:20 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -667,16 +667,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -691,16 +691,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -1801,51 +1801,51 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="C10" t="n">
         <v>107</v>
       </c>
       <c r="D10" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E10" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="F10" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="G10" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="C11" t="n">
         <v>107</v>
       </c>
       <c r="D11" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="E11" t="n">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="F11" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="G11" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12">
@@ -4010,30 +4010,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E10" t="n">
-        <v>30971</v>
+        <v>410102</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>820221</v>
+        <v>2088802</v>
       </c>
       <c r="H10" t="n">
-        <v>58227</v>
+        <v>5360778</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -4047,30 +4047,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E11" t="n">
-        <v>410102</v>
+        <v>30971</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2088802</v>
+        <v>820221</v>
       </c>
       <c r="H11" t="n">
-        <v>5360778</v>
+        <v>58227</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -5524,12 +5524,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -5539,10 +5539,10 @@
         <v>68.7</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G10" t="n">
         <v>107</v>
@@ -5551,10 +5551,10 @@
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
@@ -5566,41 +5566,41 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="O10" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="P10" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="R10" t="n">
         <v>976197</v>
       </c>
       <c r="S10" t="n">
-        <v>1034411</v>
+        <v>4185865</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -5610,10 +5610,10 @@
         <v>68.7</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G11" t="n">
         <v>107</v>
@@ -5622,10 +5622,10 @@
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K11" t="n">
         <v>2</v>
@@ -5637,29 +5637,29 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="O11" t="n">
-        <v>101.3</v>
+        <v>101.4</v>
       </c>
       <c r="P11" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="R11" t="n">
         <v>976197</v>
       </c>
       <c r="S11" t="n">
-        <v>4185865</v>
+        <v>1034411</v>
       </c>
       <c r="T11" t="n">
         <v>2</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard, bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-14 03:47 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -499,19 +499,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="E3" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
         <v>444</v>
@@ -523,19 +523,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F4" t="n">
         <v>444</v>
@@ -667,16 +667,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -691,16 +691,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -1626,51 +1626,51 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C3" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D3" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="E3" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="F3" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="G3" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C4" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D4" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="E4" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="F4" t="n">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="G4" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5">
@@ -1801,51 +1801,51 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="C10" t="n">
         <v>107</v>
       </c>
       <c r="D10" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="E10" t="n">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="F10" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="G10" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="C11" t="n">
         <v>107</v>
       </c>
       <c r="D11" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E11" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="F11" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="G11" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12">
@@ -3751,30 +3751,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>281617</v>
+        <v>545267</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1051323</v>
+        <v>604934</v>
       </c>
       <c r="H3" t="n">
-        <v>1076546</v>
+        <v>545267</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -3788,30 +3788,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E4" t="n">
-        <v>545267</v>
+        <v>281617</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>604934</v>
+        <v>1051323</v>
       </c>
       <c r="H4" t="n">
-        <v>545267</v>
+        <v>1076546</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -4010,30 +4010,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E10" t="n">
-        <v>410102</v>
+        <v>30971</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2088802</v>
+        <v>820221</v>
       </c>
       <c r="H10" t="n">
-        <v>5360778</v>
+        <v>58227</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -4047,30 +4047,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E11" t="n">
-        <v>30971</v>
+        <v>410102</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>820221</v>
+        <v>2088802</v>
       </c>
       <c r="H11" t="n">
-        <v>58227</v>
+        <v>5360778</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -5031,12 +5031,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -5046,19 +5046,19 @@
         <v>74</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="G3" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="H3" t="n">
         <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="J3" t="n">
         <v>3</v>
@@ -5067,47 +5067,43 @@
         <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="O3" t="n">
-        <v>102.2</v>
+        <v>101.1</v>
       </c>
       <c r="P3" t="n">
-        <v>2.2</v>
+        <v>1.1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="R3" t="n">
         <v>161939</v>
       </c>
       <c r="S3" t="n">
-        <v>1229264</v>
+        <v>1461471</v>
       </c>
       <c r="T3" t="n">
-        <v>4</v>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>bboost, wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -5117,19 +5113,19 @@
         <v>74</v>
       </c>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="G4" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="H4" t="n">
         <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="J4" t="n">
         <v>3</v>
@@ -5138,33 +5134,37 @@
         <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N4" t="n">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="O4" t="n">
-        <v>101.1</v>
+        <v>102.2</v>
       </c>
       <c r="P4" t="n">
-        <v>1.1</v>
+        <v>2.2</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="R4" t="n">
         <v>161939</v>
       </c>
       <c r="S4" t="n">
-        <v>1461471</v>
+        <v>1229264</v>
       </c>
       <c r="T4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U4" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>bboost, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5524,12 +5524,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -5539,10 +5539,10 @@
         <v>68.7</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G10" t="n">
         <v>107</v>
@@ -5551,10 +5551,10 @@
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
@@ -5566,41 +5566,41 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="O10" t="n">
-        <v>101.3</v>
+        <v>101.4</v>
       </c>
       <c r="P10" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="R10" t="n">
         <v>976197</v>
       </c>
       <c r="S10" t="n">
-        <v>4185865</v>
+        <v>1034411</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard, bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -5610,10 +5610,10 @@
         <v>68.7</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G11" t="n">
         <v>107</v>
@@ -5622,10 +5622,10 @@
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
         <v>2</v>
@@ -5637,29 +5637,29 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="O11" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="P11" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="R11" t="n">
         <v>976197</v>
       </c>
       <c r="S11" t="n">
-        <v>1034411</v>
+        <v>4185865</v>
       </c>
       <c r="T11" t="n">
         <v>2</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard, bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-14 09:19 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -499,19 +499,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F3" t="n">
         <v>444</v>
@@ -523,19 +523,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="E4" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>444</v>
@@ -667,16 +667,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -691,16 +691,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -1626,51 +1626,51 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C3" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D3" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="E3" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="F3" t="n">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="G3" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C4" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="E4" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="F4" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="G4" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5">
@@ -1801,51 +1801,51 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="C10" t="n">
         <v>107</v>
       </c>
       <c r="D10" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E10" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="F10" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="G10" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="C11" t="n">
         <v>107</v>
       </c>
       <c r="D11" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="E11" t="n">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="F11" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="G11" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12">
@@ -3751,30 +3751,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>545267</v>
+        <v>281617</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>604934</v>
+        <v>1051323</v>
       </c>
       <c r="H3" t="n">
-        <v>545267</v>
+        <v>1076546</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -3788,30 +3788,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>281617</v>
+        <v>545267</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1051323</v>
+        <v>604934</v>
       </c>
       <c r="H4" t="n">
-        <v>1076546</v>
+        <v>545267</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -4010,30 +4010,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E10" t="n">
-        <v>30971</v>
+        <v>410102</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>820221</v>
+        <v>2088802</v>
       </c>
       <c r="H10" t="n">
-        <v>58227</v>
+        <v>5360778</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -4047,30 +4047,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E11" t="n">
-        <v>410102</v>
+        <v>30971</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2088802</v>
+        <v>820221</v>
       </c>
       <c r="H11" t="n">
-        <v>5360778</v>
+        <v>58227</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -5031,12 +5031,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -5046,19 +5046,19 @@
         <v>74</v>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="G3" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="H3" t="n">
         <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="J3" t="n">
         <v>3</v>
@@ -5067,43 +5067,47 @@
         <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N3" t="n">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="O3" t="n">
-        <v>101.1</v>
+        <v>102.2</v>
       </c>
       <c r="P3" t="n">
-        <v>1.1</v>
+        <v>2.2</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="R3" t="n">
         <v>161939</v>
       </c>
       <c r="S3" t="n">
-        <v>1461471</v>
+        <v>1229264</v>
       </c>
       <c r="T3" t="n">
-        <v>2</v>
-      </c>
-      <c r="U3" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>bboost, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -5113,19 +5117,19 @@
         <v>74</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="G4" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="H4" t="n">
         <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="J4" t="n">
         <v>3</v>
@@ -5134,37 +5138,33 @@
         <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="O4" t="n">
-        <v>102.2</v>
+        <v>101.1</v>
       </c>
       <c r="P4" t="n">
-        <v>2.2</v>
+        <v>1.1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="R4" t="n">
         <v>161939</v>
       </c>
       <c r="S4" t="n">
-        <v>1229264</v>
+        <v>1461471</v>
       </c>
       <c r="T4" t="n">
-        <v>4</v>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>bboost, wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5524,12 +5524,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -5539,10 +5539,10 @@
         <v>68.7</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G10" t="n">
         <v>107</v>
@@ -5551,10 +5551,10 @@
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
@@ -5566,41 +5566,41 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="O10" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="P10" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="R10" t="n">
         <v>976197</v>
       </c>
       <c r="S10" t="n">
-        <v>1034411</v>
+        <v>4185865</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -5610,10 +5610,10 @@
         <v>68.7</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G11" t="n">
         <v>107</v>
@@ -5622,10 +5622,10 @@
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K11" t="n">
         <v>2</v>
@@ -5637,29 +5637,29 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="O11" t="n">
-        <v>101.3</v>
+        <v>101.4</v>
       </c>
       <c r="P11" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="R11" t="n">
         <v>976197</v>
       </c>
       <c r="S11" t="n">
-        <v>4185865</v>
+        <v>1034411</v>
       </c>
       <c r="T11" t="n">
         <v>2</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard, bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-14 14:54 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -499,19 +499,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="E3" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
         <v>444</v>
@@ -523,19 +523,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F4" t="n">
         <v>444</v>
@@ -667,16 +667,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -691,16 +691,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -1626,51 +1626,51 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C3" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D3" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="E3" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="F3" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="G3" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C4" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D4" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="E4" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="F4" t="n">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="G4" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5">
@@ -1801,51 +1801,51 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="C10" t="n">
         <v>107</v>
       </c>
       <c r="D10" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="E10" t="n">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="F10" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="G10" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="C11" t="n">
         <v>107</v>
       </c>
       <c r="D11" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E11" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="F11" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="G11" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12">
@@ -3751,30 +3751,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>281617</v>
+        <v>545267</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1051323</v>
+        <v>604934</v>
       </c>
       <c r="H3" t="n">
-        <v>1076546</v>
+        <v>545267</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -3788,30 +3788,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E4" t="n">
-        <v>545267</v>
+        <v>281617</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>604934</v>
+        <v>1051323</v>
       </c>
       <c r="H4" t="n">
-        <v>545267</v>
+        <v>1076546</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -4010,30 +4010,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E10" t="n">
-        <v>410102</v>
+        <v>30971</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2088802</v>
+        <v>820221</v>
       </c>
       <c r="H10" t="n">
-        <v>5360778</v>
+        <v>58227</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -4047,30 +4047,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E11" t="n">
-        <v>30971</v>
+        <v>410102</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>820221</v>
+        <v>2088802</v>
       </c>
       <c r="H11" t="n">
-        <v>58227</v>
+        <v>5360778</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -5031,12 +5031,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -5046,19 +5046,19 @@
         <v>74</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="G3" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="H3" t="n">
         <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="J3" t="n">
         <v>3</v>
@@ -5067,47 +5067,43 @@
         <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="O3" t="n">
-        <v>102.2</v>
+        <v>101.1</v>
       </c>
       <c r="P3" t="n">
-        <v>2.2</v>
+        <v>1.1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="R3" t="n">
         <v>161939</v>
       </c>
       <c r="S3" t="n">
-        <v>1229264</v>
+        <v>1461471</v>
       </c>
       <c r="T3" t="n">
-        <v>4</v>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>bboost, wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -5117,19 +5113,19 @@
         <v>74</v>
       </c>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="G4" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="H4" t="n">
         <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="J4" t="n">
         <v>3</v>
@@ -5138,33 +5134,37 @@
         <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N4" t="n">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="O4" t="n">
-        <v>101.1</v>
+        <v>102.2</v>
       </c>
       <c r="P4" t="n">
-        <v>1.1</v>
+        <v>2.2</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="R4" t="n">
         <v>161939</v>
       </c>
       <c r="S4" t="n">
-        <v>1461471</v>
+        <v>1229264</v>
       </c>
       <c r="T4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U4" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>bboost, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5524,12 +5524,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -5539,10 +5539,10 @@
         <v>68.7</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G10" t="n">
         <v>107</v>
@@ -5551,10 +5551,10 @@
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
@@ -5566,41 +5566,41 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="O10" t="n">
-        <v>101.3</v>
+        <v>101.4</v>
       </c>
       <c r="P10" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="R10" t="n">
         <v>976197</v>
       </c>
       <c r="S10" t="n">
-        <v>4185865</v>
+        <v>1034411</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard, bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -5610,10 +5610,10 @@
         <v>68.7</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G11" t="n">
         <v>107</v>
@@ -5622,10 +5622,10 @@
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
         <v>2</v>
@@ -5637,29 +5637,29 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="O11" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="P11" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="R11" t="n">
         <v>976197</v>
       </c>
       <c r="S11" t="n">
-        <v>1034411</v>
+        <v>4185865</v>
       </c>
       <c r="T11" t="n">
         <v>2</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard, bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-15 00:18 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -499,19 +499,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F3" t="n">
         <v>444</v>
@@ -523,19 +523,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="E4" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>444</v>
@@ -1626,51 +1626,51 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C3" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D3" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="E3" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="F3" t="n">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="G3" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C4" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="E4" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="F4" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="G4" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5">
@@ -3751,30 +3751,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>545267</v>
+        <v>281617</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>604934</v>
+        <v>1051323</v>
       </c>
       <c r="H3" t="n">
-        <v>545267</v>
+        <v>1076546</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -3788,30 +3788,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>281617</v>
+        <v>545267</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1051323</v>
+        <v>604934</v>
       </c>
       <c r="H4" t="n">
-        <v>1076546</v>
+        <v>545267</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -5031,12 +5031,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -5046,19 +5046,19 @@
         <v>74</v>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="G3" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="H3" t="n">
         <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="J3" t="n">
         <v>3</v>
@@ -5067,43 +5067,47 @@
         <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N3" t="n">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="O3" t="n">
-        <v>101.1</v>
+        <v>102.2</v>
       </c>
       <c r="P3" t="n">
-        <v>1.1</v>
+        <v>2.2</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="R3" t="n">
         <v>161939</v>
       </c>
       <c r="S3" t="n">
-        <v>1461471</v>
+        <v>1229264</v>
       </c>
       <c r="T3" t="n">
-        <v>2</v>
-      </c>
-      <c r="U3" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>bboost, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -5113,19 +5117,19 @@
         <v>74</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="G4" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="H4" t="n">
         <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="J4" t="n">
         <v>3</v>
@@ -5134,37 +5138,33 @@
         <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="O4" t="n">
-        <v>102.2</v>
+        <v>101.1</v>
       </c>
       <c r="P4" t="n">
-        <v>2.2</v>
+        <v>1.1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="R4" t="n">
         <v>161939</v>
       </c>
       <c r="S4" t="n">
-        <v>1229264</v>
+        <v>1461471</v>
       </c>
       <c r="T4" t="n">
-        <v>4</v>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>bboost, wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-10-15 07:01 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -667,16 +667,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -691,16 +691,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -1801,51 +1801,51 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="C10" t="n">
         <v>107</v>
       </c>
       <c r="D10" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E10" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="F10" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="G10" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="C11" t="n">
         <v>107</v>
       </c>
       <c r="D11" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="E11" t="n">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="F11" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="G11" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12">
@@ -4010,30 +4010,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E10" t="n">
-        <v>30971</v>
+        <v>410102</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>820221</v>
+        <v>2088802</v>
       </c>
       <c r="H10" t="n">
-        <v>58227</v>
+        <v>5360778</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -4047,30 +4047,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E11" t="n">
-        <v>410102</v>
+        <v>30971</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2088802</v>
+        <v>820221</v>
       </c>
       <c r="H11" t="n">
-        <v>5360778</v>
+        <v>58227</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -5524,12 +5524,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -5539,10 +5539,10 @@
         <v>68.7</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G10" t="n">
         <v>107</v>
@@ -5551,10 +5551,10 @@
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
@@ -5566,41 +5566,41 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="O10" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="P10" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="R10" t="n">
         <v>976197</v>
       </c>
       <c r="S10" t="n">
-        <v>1034411</v>
+        <v>4185865</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -5610,10 +5610,10 @@
         <v>68.7</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G11" t="n">
         <v>107</v>
@@ -5622,10 +5622,10 @@
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K11" t="n">
         <v>2</v>
@@ -5637,29 +5637,29 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="O11" t="n">
-        <v>101.3</v>
+        <v>101.4</v>
       </c>
       <c r="P11" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="R11" t="n">
         <v>976197</v>
       </c>
       <c r="S11" t="n">
-        <v>4185865</v>
+        <v>1034411</v>
       </c>
       <c r="T11" t="n">
         <v>2</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard, bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-15 18:02 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -499,19 +499,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="E3" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
         <v>444</v>
@@ -523,19 +523,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F4" t="n">
         <v>444</v>
@@ -667,16 +667,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -691,16 +691,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -1626,51 +1626,51 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C3" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D3" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="E3" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="F3" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="G3" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C4" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D4" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="E4" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="F4" t="n">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="G4" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5">
@@ -1801,51 +1801,51 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="C10" t="n">
         <v>107</v>
       </c>
       <c r="D10" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="E10" t="n">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="F10" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="G10" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="C11" t="n">
         <v>107</v>
       </c>
       <c r="D11" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E11" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="F11" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="G11" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12">
@@ -3751,30 +3751,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>281617</v>
+        <v>545267</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1051323</v>
+        <v>604934</v>
       </c>
       <c r="H3" t="n">
-        <v>1076546</v>
+        <v>545267</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -3788,30 +3788,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E4" t="n">
-        <v>545267</v>
+        <v>281617</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>604934</v>
+        <v>1051323</v>
       </c>
       <c r="H4" t="n">
-        <v>545267</v>
+        <v>1076546</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -4010,30 +4010,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E10" t="n">
-        <v>410102</v>
+        <v>30971</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2088802</v>
+        <v>820221</v>
       </c>
       <c r="H10" t="n">
-        <v>5360778</v>
+        <v>58227</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -4047,30 +4047,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E11" t="n">
-        <v>30971</v>
+        <v>410102</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>820221</v>
+        <v>2088802</v>
       </c>
       <c r="H11" t="n">
-        <v>58227</v>
+        <v>5360778</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -5031,12 +5031,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -5046,19 +5046,19 @@
         <v>74</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="G3" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="H3" t="n">
         <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="J3" t="n">
         <v>3</v>
@@ -5067,47 +5067,43 @@
         <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="O3" t="n">
-        <v>102.2</v>
+        <v>101.1</v>
       </c>
       <c r="P3" t="n">
-        <v>2.2</v>
+        <v>1.1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="R3" t="n">
         <v>161939</v>
       </c>
       <c r="S3" t="n">
-        <v>1229264</v>
+        <v>1461471</v>
       </c>
       <c r="T3" t="n">
-        <v>4</v>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>bboost, wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -5117,19 +5113,19 @@
         <v>74</v>
       </c>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="G4" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="H4" t="n">
         <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="J4" t="n">
         <v>3</v>
@@ -5138,33 +5134,37 @@
         <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N4" t="n">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="O4" t="n">
-        <v>101.1</v>
+        <v>102.2</v>
       </c>
       <c r="P4" t="n">
-        <v>1.1</v>
+        <v>2.2</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="R4" t="n">
         <v>161939</v>
       </c>
       <c r="S4" t="n">
-        <v>1461471</v>
+        <v>1229264</v>
       </c>
       <c r="T4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U4" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>bboost, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5524,12 +5524,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -5539,10 +5539,10 @@
         <v>68.7</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G10" t="n">
         <v>107</v>
@@ -5551,10 +5551,10 @@
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
@@ -5566,41 +5566,41 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="O10" t="n">
-        <v>101.3</v>
+        <v>101.4</v>
       </c>
       <c r="P10" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="R10" t="n">
         <v>976197</v>
       </c>
       <c r="S10" t="n">
-        <v>4185865</v>
+        <v>1034411</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard, bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -5610,10 +5610,10 @@
         <v>68.7</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G11" t="n">
         <v>107</v>
@@ -5622,10 +5622,10 @@
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
         <v>2</v>
@@ -5637,29 +5637,29 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="O11" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="P11" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="R11" t="n">
         <v>976197</v>
       </c>
       <c r="S11" t="n">
-        <v>1034411</v>
+        <v>4185865</v>
       </c>
       <c r="T11" t="n">
         <v>2</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard, bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-15 22:54 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -499,19 +499,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F3" t="n">
         <v>444</v>
@@ -523,19 +523,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="E4" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>444</v>
@@ -1626,51 +1626,51 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C3" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D3" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="E3" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="F3" t="n">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="G3" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C4" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="E4" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="F4" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="G4" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5">
@@ -3751,30 +3751,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>545267</v>
+        <v>281617</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>604934</v>
+        <v>1051323</v>
       </c>
       <c r="H3" t="n">
-        <v>545267</v>
+        <v>1076546</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -3788,30 +3788,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>281617</v>
+        <v>545267</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1051323</v>
+        <v>604934</v>
       </c>
       <c r="H4" t="n">
-        <v>1076546</v>
+        <v>545267</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -5031,12 +5031,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -5046,19 +5046,19 @@
         <v>74</v>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="G3" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="H3" t="n">
         <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="J3" t="n">
         <v>3</v>
@@ -5067,43 +5067,47 @@
         <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N3" t="n">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="O3" t="n">
-        <v>101.1</v>
+        <v>102.2</v>
       </c>
       <c r="P3" t="n">
-        <v>1.1</v>
+        <v>2.2</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="R3" t="n">
         <v>161939</v>
       </c>
       <c r="S3" t="n">
-        <v>1461471</v>
+        <v>1229264</v>
       </c>
       <c r="T3" t="n">
-        <v>2</v>
-      </c>
-      <c r="U3" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>bboost, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -5113,19 +5117,19 @@
         <v>74</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="G4" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="H4" t="n">
         <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="J4" t="n">
         <v>3</v>
@@ -5134,37 +5138,33 @@
         <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="O4" t="n">
-        <v>102.2</v>
+        <v>101.1</v>
       </c>
       <c r="P4" t="n">
-        <v>2.2</v>
+        <v>1.1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="R4" t="n">
         <v>161939</v>
       </c>
       <c r="S4" t="n">
-        <v>1229264</v>
+        <v>1461471</v>
       </c>
       <c r="T4" t="n">
-        <v>4</v>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>bboost, wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-10-16 03:24 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -667,16 +667,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -691,16 +691,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -1801,51 +1801,51 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="C10" t="n">
         <v>107</v>
       </c>
       <c r="D10" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E10" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="F10" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="G10" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="C11" t="n">
         <v>107</v>
       </c>
       <c r="D11" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="E11" t="n">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="F11" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="G11" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12">
@@ -4010,30 +4010,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E10" t="n">
-        <v>30971</v>
+        <v>410102</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>820221</v>
+        <v>2088802</v>
       </c>
       <c r="H10" t="n">
-        <v>58227</v>
+        <v>5360778</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -4047,30 +4047,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E11" t="n">
-        <v>410102</v>
+        <v>30971</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2088802</v>
+        <v>820221</v>
       </c>
       <c r="H11" t="n">
-        <v>5360778</v>
+        <v>58227</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -5524,12 +5524,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -5539,10 +5539,10 @@
         <v>68.7</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G10" t="n">
         <v>107</v>
@@ -5551,10 +5551,10 @@
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
@@ -5566,41 +5566,41 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="O10" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="P10" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="R10" t="n">
         <v>976197</v>
       </c>
       <c r="S10" t="n">
-        <v>1034411</v>
+        <v>4185865</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -5610,10 +5610,10 @@
         <v>68.7</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G11" t="n">
         <v>107</v>
@@ -5622,10 +5622,10 @@
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K11" t="n">
         <v>2</v>
@@ -5637,29 +5637,29 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="O11" t="n">
-        <v>101.3</v>
+        <v>101.4</v>
       </c>
       <c r="P11" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="R11" t="n">
         <v>976197</v>
       </c>
       <c r="S11" t="n">
-        <v>4185865</v>
+        <v>1034411</v>
       </c>
       <c r="T11" t="n">
         <v>2</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard, bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-16 08:47 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -667,16 +667,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -691,16 +691,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -1801,51 +1801,51 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="C10" t="n">
         <v>107</v>
       </c>
       <c r="D10" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="E10" t="n">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="F10" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="G10" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="C11" t="n">
         <v>107</v>
       </c>
       <c r="D11" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E11" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="F11" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="G11" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12">
@@ -4010,30 +4010,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E10" t="n">
-        <v>410102</v>
+        <v>30971</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2088802</v>
+        <v>820221</v>
       </c>
       <c r="H10" t="n">
-        <v>5360778</v>
+        <v>58227</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -4047,30 +4047,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E11" t="n">
-        <v>30971</v>
+        <v>410102</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>820221</v>
+        <v>2088802</v>
       </c>
       <c r="H11" t="n">
-        <v>58227</v>
+        <v>5360778</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -5524,12 +5524,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -5539,10 +5539,10 @@
         <v>68.7</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G10" t="n">
         <v>107</v>
@@ -5551,10 +5551,10 @@
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
@@ -5566,41 +5566,41 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="O10" t="n">
-        <v>101.3</v>
+        <v>101.4</v>
       </c>
       <c r="P10" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="R10" t="n">
         <v>976197</v>
       </c>
       <c r="S10" t="n">
-        <v>4185865</v>
+        <v>1034411</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard, bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -5610,10 +5610,10 @@
         <v>68.7</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G11" t="n">
         <v>107</v>
@@ -5622,10 +5622,10 @@
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
         <v>2</v>
@@ -5637,29 +5637,29 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="O11" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="P11" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="R11" t="n">
         <v>976197</v>
       </c>
       <c r="S11" t="n">
-        <v>1034411</v>
+        <v>4185865</v>
       </c>
       <c r="T11" t="n">
         <v>2</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard, bboost</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-16 19:21 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -499,19 +499,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="E3" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
         <v>444</v>
@@ -523,19 +523,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F4" t="n">
         <v>444</v>
@@ -667,16 +667,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -691,16 +691,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -1626,51 +1626,51 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C3" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D3" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="E3" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="F3" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="G3" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C4" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D4" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="E4" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="F4" t="n">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="G4" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5">
@@ -1801,51 +1801,51 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="C10" t="n">
         <v>107</v>
       </c>
       <c r="D10" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E10" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="F10" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="G10" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="C11" t="n">
         <v>107</v>
       </c>
       <c r="D11" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="E11" t="n">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="F11" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="G11" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12">
@@ -3751,30 +3751,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>281617</v>
+        <v>545267</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1051323</v>
+        <v>604934</v>
       </c>
       <c r="H3" t="n">
-        <v>1076546</v>
+        <v>545267</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -3788,30 +3788,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E4" t="n">
-        <v>545267</v>
+        <v>281617</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>604934</v>
+        <v>1051323</v>
       </c>
       <c r="H4" t="n">
-        <v>545267</v>
+        <v>1076546</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -4010,30 +4010,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E10" t="n">
-        <v>30971</v>
+        <v>410102</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2018/19</t>
+          <t>2009/10</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>820221</v>
+        <v>2088802</v>
       </c>
       <c r="H10" t="n">
-        <v>58227</v>
+        <v>5360778</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -4047,30 +4047,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E11" t="n">
-        <v>410102</v>
+        <v>30971</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2009/10</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2088802</v>
+        <v>820221</v>
       </c>
       <c r="H11" t="n">
-        <v>5360778</v>
+        <v>58227</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -5031,12 +5031,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -5046,19 +5046,19 @@
         <v>74</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="G3" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="H3" t="n">
         <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="J3" t="n">
         <v>3</v>
@@ -5067,47 +5067,43 @@
         <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="O3" t="n">
-        <v>102.2</v>
+        <v>101.1</v>
       </c>
       <c r="P3" t="n">
-        <v>2.2</v>
+        <v>1.1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="R3" t="n">
         <v>161939</v>
       </c>
       <c r="S3" t="n">
-        <v>1229264</v>
+        <v>1461471</v>
       </c>
       <c r="T3" t="n">
-        <v>4</v>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>bboost, wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -5117,19 +5113,19 @@
         <v>74</v>
       </c>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="G4" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="H4" t="n">
         <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="J4" t="n">
         <v>3</v>
@@ -5138,33 +5134,37 @@
         <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N4" t="n">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="O4" t="n">
-        <v>101.1</v>
+        <v>102.2</v>
       </c>
       <c r="P4" t="n">
-        <v>1.1</v>
+        <v>2.2</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="R4" t="n">
         <v>161939</v>
       </c>
       <c r="S4" t="n">
-        <v>1461471</v>
+        <v>1229264</v>
       </c>
       <c r="T4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U4" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>bboost, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5524,12 +5524,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Yash Beohar</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Fluente in Football</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -5539,10 +5539,10 @@
         <v>68.7</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G10" t="n">
         <v>107</v>
@@ -5551,10 +5551,10 @@
         <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="J10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
         <v>2</v>
@@ -5566,41 +5566,41 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="O10" t="n">
-        <v>101.4</v>
+        <v>101.3</v>
       </c>
       <c r="P10" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="R10" t="n">
         <v>976197</v>
       </c>
       <c r="S10" t="n">
-        <v>1034411</v>
+        <v>4185865</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>bboost, wildcard</t>
+          <t>3xc, freehit, wildcard, bboost</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Yash Beohar</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>Fluente in Football</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -5610,10 +5610,10 @@
         <v>68.7</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G11" t="n">
         <v>107</v>
@@ -5622,10 +5622,10 @@
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K11" t="n">
         <v>2</v>
@@ -5637,29 +5637,29 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="O11" t="n">
-        <v>101.3</v>
+        <v>101.4</v>
       </c>
       <c r="P11" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="R11" t="n">
         <v>976197</v>
       </c>
       <c r="S11" t="n">
-        <v>4185865</v>
+        <v>1034411</v>
       </c>
       <c r="T11" t="n">
         <v>2</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>3xc, freehit, wildcard, bboost</t>
+          <t>bboost, wildcard</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update standings 2026-10-17 08:17 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -499,19 +499,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F3" t="n">
         <v>444</v>
@@ -523,19 +523,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="E4" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>444</v>
@@ -1626,51 +1626,51 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C3" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D3" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="E3" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="F3" t="n">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="G3" t="n">
-        <v>61</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C4" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="E4" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="F4" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="G4" t="n">
-        <v>82</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5">
@@ -3751,30 +3751,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>545267</v>
+        <v>281617</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2025/26</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>604934</v>
+        <v>1051323</v>
       </c>
       <c r="H3" t="n">
-        <v>545267</v>
+        <v>1076546</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -3788,30 +3788,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>281617</v>
+        <v>545267</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2019/20</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1051323</v>
+        <v>604934</v>
       </c>
       <c r="H4" t="n">
-        <v>1076546</v>
+        <v>545267</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -5031,12 +5031,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ajith Thomas Kuthukatt George</t>
+          <t>Anish Joshi</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Onside Offside</t>
+          <t>Fiery Raiders</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -5046,19 +5046,19 @@
         <v>74</v>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="G3" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="H3" t="n">
         <v>4</v>
       </c>
       <c r="I3" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="J3" t="n">
         <v>3</v>
@@ -5067,43 +5067,47 @@
         <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="N3" t="n">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="O3" t="n">
-        <v>101.1</v>
+        <v>102.2</v>
       </c>
       <c r="P3" t="n">
-        <v>1.1</v>
+        <v>2.2</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="R3" t="n">
         <v>161939</v>
       </c>
       <c r="S3" t="n">
-        <v>1461471</v>
+        <v>1229264</v>
       </c>
       <c r="T3" t="n">
-        <v>2</v>
-      </c>
-      <c r="U3" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>bboost, wildcard</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Anish Joshi</t>
+          <t>Ajith Thomas Kuthukatt George</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Fiery Raiders</t>
+          <t>Onside Offside</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -5113,19 +5117,19 @@
         <v>74</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="G4" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="H4" t="n">
         <v>4</v>
       </c>
       <c r="I4" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="J4" t="n">
         <v>3</v>
@@ -5134,37 +5138,33 @@
         <v>5</v>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="O4" t="n">
-        <v>102.2</v>
+        <v>101.1</v>
       </c>
       <c r="P4" t="n">
-        <v>2.2</v>
+        <v>1.1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="R4" t="n">
         <v>161939</v>
       </c>
       <c r="S4" t="n">
-        <v>1229264</v>
+        <v>1461471</v>
       </c>
       <c r="T4" t="n">
-        <v>4</v>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>bboost, wildcard</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">

</xml_diff>

<commit_message>
Update standings 2026-10-17 13:28 UTC
</commit_message>
<xml_diff>
--- a/docs/Laxmi_Chit_Fund_S5_audit.xlsx
+++ b/docs/Laxmi_Chit_Fund_S5_audit.xlsx
@@ -484,13 +484,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>474</v>
+        <v>480</v>
       </c>
     </row>
     <row r="3">
@@ -508,18 +508,18 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>82</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
         <v>-4</v>
       </c>
       <c r="F3" t="n">
-        <v>444</v>
+        <v>448</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -532,13 +532,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>61</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>444</v>
+        <v>448</v>
       </c>
     </row>
     <row r="5">
@@ -556,13 +556,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>434</v>
+        <v>438</v>
       </c>
     </row>
     <row r="6">
@@ -580,13 +580,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>77</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>431</v>
+        <v>435</v>
       </c>
     </row>
     <row r="7">
@@ -604,13 +604,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>424</v>
+        <v>430</v>
       </c>
     </row>
     <row r="8">
@@ -628,13 +628,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>419</v>
+        <v>423</v>
       </c>
     </row>
     <row r="9">
@@ -643,22 +643,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ShakeNBake</t>
+          <t>Goal Diggers FC</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>62</v>
+        <v>6</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>413</v>
+        <v>418</v>
       </c>
     </row>
     <row r="10">
@@ -667,27 +667,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Goal Diggers FC</t>
+          <t>ShakeNBake</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>412</v>
+        <v>417</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -700,13 +700,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>412</v>
+        <v>416</v>
       </c>
     </row>
     <row r="12">
@@ -724,18 +724,18 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>410</v>
+        <v>414</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -748,13 +748,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>63</v>
+        <v>6</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>408</v>
+        <v>414</v>
       </c>
     </row>
     <row r="14">
@@ -772,13 +772,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>68</v>
+        <v>6</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>408</v>
+        <v>414</v>
       </c>
     </row>
     <row r="15">
@@ -787,22 +787,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>KingOfKings Fc</t>
+          <t>Enzotic</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>59</v>
+        <v>6</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>407</v>
+        <v>412</v>
       </c>
     </row>
     <row r="16">
@@ -811,22 +811,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Enzotic</t>
+          <t>KingOfKings Fc</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>406</v>
+        <v>411</v>
       </c>
     </row>
     <row r="17">
@@ -844,13 +844,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>398</v>
+        <v>404</v>
       </c>
     </row>
     <row r="18">
@@ -868,13 +868,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>60</v>
+        <v>7</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="F18" t="n">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="19">
@@ -892,13 +892,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>51</v>
+        <v>2</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="20">
@@ -916,13 +916,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="E20" t="n">
         <v>-8</v>
       </c>
       <c r="F20" t="n">
-        <v>394</v>
+        <v>398</v>
       </c>
     </row>
     <row r="21">
@@ -931,22 +931,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>His Name is Diogo</t>
+          <t>Cold Palmer</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>70</v>
+        <v>6</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>391</v>
+        <v>396</v>
       </c>
     </row>
     <row r="22">
@@ -955,22 +955,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Cold Palmer</t>
+          <t>His Name is Diogo</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>56</v>
+        <v>4</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>390</v>
+        <v>395</v>
       </c>
     </row>
     <row r="23">
@@ -979,46 +979,46 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>fpl_26_27</t>
+          <t>Captn Magnifico</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>78</v>
+        <v>8</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>389</v>
+        <v>393</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Southall United</t>
+          <t>fpl_26_27</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>74</v>
+        <v>4</v>
       </c>
       <c r="E24" t="n">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>387</v>
+        <v>393</v>
       </c>
     </row>
     <row r="25">
@@ -1036,13 +1036,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>386</v>
+        <v>390</v>
       </c>
     </row>
     <row r="26">
@@ -1051,22 +1051,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Captn Magnifico</t>
+          <t>FC Teetotallers</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>58</v>
+        <v>6</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>385</v>
+        <v>388</v>
       </c>
     </row>
     <row r="27">
@@ -1075,22 +1075,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>FC Teetotallers</t>
+          <t>Southall United</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>-16</v>
       </c>
       <c r="F27" t="n">
-        <v>382</v>
+        <v>387</v>
       </c>
     </row>
     <row r="28">
@@ -1108,13 +1108,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>379</v>
+        <v>383</v>
       </c>
     </row>
     <row r="29">
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>84</v>
+        <v>4</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>377</v>
+        <v>381</v>
       </c>
     </row>
     <row r="30">
@@ -1147,22 +1147,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Redsbay</t>
+          <t>Slumber FC</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>61</v>
+        <v>8</v>
       </c>
       <c r="E30" t="n">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="F30" t="n">
-        <v>345</v>
+        <v>348</v>
       </c>
     </row>
     <row r="31">
@@ -1171,22 +1171,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Slumber FC</t>
+          <t>Redsbay</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>67</v>
+        <v>4</v>
       </c>
       <c r="E31" t="n">
-        <v>-4</v>
+        <v>-12</v>
       </c>
       <c r="F31" t="n">
-        <v>340</v>
+        <v>345</v>
       </c>
     </row>
     <row r="32">
@@ -1204,13 +1204,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>283</v>
+        <v>287</v>
       </c>
     </row>
   </sheetData>
@@ -1776,51 +1776,51 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Arshaq Razack</t>
+          <t>Varun Khurana</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="C9" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D9" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E9" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F9" t="n">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="G9" t="n">
-        <v>62</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Varun Khurana</t>
+          <t>Arshaq Razack</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="C10" t="n">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D10" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E10" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F10" t="n">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="G10" t="n">
-        <v>80</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11">
@@ -1926,51 +1926,51 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Abhiraj Singh</t>
+          <t>Abhishek Gupte</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>73</v>
       </c>
       <c r="C15" t="n">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="D15" t="n">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="E15" t="n">
-        <v>91</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="G15" t="n">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Abhishek Gupte</t>
+          <t>Abhiraj Singh</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>73</v>
       </c>
       <c r="C16" t="n">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="D16" t="n">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="E16" t="n">
-        <v>69</v>
+        <v>91</v>
       </c>
       <c r="F16" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="G16" t="n">
-        <v>69</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17">
@@ -2076,101 +2076,101 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Aditya Vaidya</t>
+          <t>Shivanshu Madan</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>41</v>
+        <v>62</v>
       </c>
       <c r="C21" t="n">
-        <v>78</v>
+        <v>111</v>
       </c>
       <c r="D21" t="n">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="E21" t="n">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="F21" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="G21" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Shivanshu Madan</t>
+          <t>Aditya Vaidya</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="C22" t="n">
-        <v>111</v>
+        <v>78</v>
       </c>
       <c r="D22" t="n">
-        <v>54</v>
+        <v>78</v>
       </c>
       <c r="E22" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="F22" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="G22" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="C23" t="n">
-        <v>80</v>
+        <v>111</v>
       </c>
       <c r="D23" t="n">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="E23" t="n">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="F23" t="n">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="G23" t="n">
-        <v>78</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C24" t="n">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="D24" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E24" t="n">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="F24" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G24" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
     </row>
     <row r="25">
@@ -2201,51 +2201,51 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="C26" t="n">
-        <v>111</v>
+        <v>89</v>
       </c>
       <c r="D26" t="n">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="E26" t="n">
-        <v>62</v>
+        <v>84</v>
       </c>
       <c r="F26" t="n">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="G26" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B27" t="n">
+        <v>53</v>
+      </c>
+      <c r="C27" t="n">
+        <v>102</v>
+      </c>
+      <c r="D27" t="n">
         <v>46</v>
       </c>
-      <c r="C27" t="n">
-        <v>89</v>
-      </c>
-      <c r="D27" t="n">
+      <c r="E27" t="n">
+        <v>66</v>
+      </c>
+      <c r="F27" t="n">
         <v>50</v>
       </c>
-      <c r="E27" t="n">
-        <v>84</v>
-      </c>
-      <c r="F27" t="n">
-        <v>45</v>
-      </c>
       <c r="G27" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28">
@@ -2301,51 +2301,51 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Nilay jain</t>
+          <t>Dean Jenkins</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="C30" t="n">
+        <v>73</v>
+      </c>
+      <c r="D30" t="n">
+        <v>32</v>
+      </c>
+      <c r="E30" t="n">
         <v>69</v>
       </c>
-      <c r="D30" t="n">
-        <v>37</v>
-      </c>
-      <c r="E30" t="n">
-        <v>89</v>
-      </c>
       <c r="F30" t="n">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="G30" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Dean Jenkins</t>
+          <t>Nilay jain</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="C31" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D31" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="E31" t="n">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="F31" t="n">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="G31" t="n">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32">
@@ -3103,7 +3103,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Rohan Agrawal</t>
+          <t>Aparnesh Mishra</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -3114,7 +3114,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Aparnesh Mishra</t>
+          <t>Rajit Das</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -3125,7 +3125,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Rajit Das</t>
+          <t>Rohan Agrawal</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -3213,7 +3213,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Karan Chopra</t>
+          <t>Naman Agrawal</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -3224,7 +3224,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Naman Agrawal</t>
+          <t>Karan Chopra</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -3784,7